<commit_message>
fix(rd-jachymov): situace-measured areas — terasa 9.23, dvorek 16.54, +venkovní schody na terénu
Legend (zpevněné plochy: dlažba [brick-hatch] vs terasa [line-hatch]) + situace měření corrected
the rough ODHAD (terasa 30 / dvorek 30):
- terasa (line-hatch, dřevěná): HSV1.005 podklad + PSV76.002 dřevo 30 → 9.23 m²
- anglický dvorek (brick-hatch dlažba): HSV1.004 30 → 16.54 m² (12.46 + 4.08)
- NEW HSV1.016: venkovní schody na terénu z betonových dílců — 8×175×280 + 5×175×280
  = 13 stupňů (TZ statika §3.2.5); code blank (Pattern 26 — família ÚRS not yet bound)

items 214 → 215. atomic_decomposition.py terasa/dvorek op qtys updated to match.
regenerate_all_views.py (9 steps) + assertions pass; completeness 0 gaps. Snapshot:
items_pre_terasa_area_fix.json.

https://claude.ai/code/session_01FskzLAZkXgJAwuN2cQQEdx
</commit_message>
<xml_diff>
--- a/test-data/RD_Jachymov_dum/outputs/Vykaz_vymer_RD_Jachymov_ATOMIC_WORKLIST_2026-05-27.xlsx
+++ b/test-data/RD_Jachymov_dum/outputs/Vykaz_vymer_RD_Jachymov_ATOMIC_WORKLIST_2026-05-27.xlsx
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>243</v>
+        <v>244</v>
       </c>
       <c r="C6" s="2">
         <f> carried 1:1 + decomposed children</f>
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -662,7 +662,7 @@
         </is>
       </c>
       <c r="B13" s="5" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="14">
@@ -1019,7 +1019,7 @@
         </is>
       </c>
       <c r="B50" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="52">
@@ -1079,7 +1079,7 @@
         </is>
       </c>
       <c r="B59" s="5" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
@@ -1681,7 +1681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K102"/>
+  <dimension ref="A1:K103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1757,7 +1757,7 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>━━ HSV-1 Zemní práce  (18 atomic operací) ━━</t>
+          <t>━━ HSV-1 Zemní práce  (19 atomic operací) ━━</t>
         </is>
       </c>
       <c r="B2" s="9" t="n"/>
@@ -1938,10 +1938,10 @@
         </is>
       </c>
       <c r="E6" s="16" t="n">
-        <v>30</v>
+        <v>16.54</v>
       </c>
       <c r="F6" s="15">
-        <f> HSV1.004 plocha dvorku 30 m²</f>
+        <f> HSV1.004 plocha dvorku 16.54 m² (situace 12.46 + 4.08, dlažba = brick-hatch)</f>
         <v/>
       </c>
       <c r="G6" s="15" t="inlineStr">
@@ -1990,10 +1990,10 @@
         </is>
       </c>
       <c r="E7" s="16" t="n">
-        <v>30</v>
+        <v>16.54</v>
       </c>
       <c r="F7" s="15">
-        <f> HSV1.004 plocha dvorku 30 m²</f>
+        <f> HSV1.004 plocha dvorku 16.54 m² (situace 12.46 + 4.08)</f>
         <v/>
       </c>
       <c r="G7" s="15" t="inlineStr">
@@ -2042,10 +2042,10 @@
         </is>
       </c>
       <c r="E8" s="16" t="n">
-        <v>30</v>
+        <v>16.54</v>
       </c>
       <c r="F8" s="15">
-        <f> HSV1.004 plocha 30 m²</f>
+        <f> HSV1.004 plocha 16.54 m²</f>
         <v/>
       </c>
       <c r="G8" s="15" t="inlineStr">
@@ -2094,10 +2094,10 @@
         </is>
       </c>
       <c r="E9" s="16" t="n">
-        <v>30</v>
+        <v>16.54</v>
       </c>
       <c r="F9" s="15">
-        <f> HSV1.004 plocha 30 m²</f>
+        <f> HSV1.004 plocha 16.54 m²</f>
         <v/>
       </c>
       <c r="G9" s="15" t="inlineStr">
@@ -2146,10 +2146,10 @@
         </is>
       </c>
       <c r="E10" s="19" t="n">
-        <v>30</v>
+        <v>9.23</v>
       </c>
       <c r="F10" s="18">
-        <f> HSV1.005 plocha terasy 30 m²</f>
+        <f> HSV1.005 plocha terasy 9.23 m² (situace měření, terasa = line-hatch)</f>
         <v/>
       </c>
       <c r="G10" s="18" t="inlineStr"/>
@@ -2194,10 +2194,10 @@
         </is>
       </c>
       <c r="E11" s="16" t="n">
-        <v>30</v>
+        <v>9.23</v>
       </c>
       <c r="F11" s="15">
-        <f> HSV1.005 plocha terasy 30 m²</f>
+        <f> HSV1.005 plocha terasy 9.23 m² (situace měření)</f>
         <v/>
       </c>
       <c r="G11" s="15" t="inlineStr">
@@ -2246,10 +2246,10 @@
         </is>
       </c>
       <c r="E12" s="16" t="n">
-        <v>30</v>
+        <v>9.23</v>
       </c>
       <c r="F12" s="15">
-        <f> HSV1.005 plocha 30 m²</f>
+        <f> HSV1.005 plocha 9.23 m²</f>
         <v/>
       </c>
       <c r="G12" s="15" t="inlineStr">
@@ -2298,10 +2298,10 @@
         </is>
       </c>
       <c r="E13" s="16" t="n">
-        <v>30</v>
+        <v>9.23</v>
       </c>
       <c r="F13" s="15">
-        <f> HSV1.005 plocha 30 m²</f>
+        <f> HSV1.005 plocha 9.23 m²</f>
         <v/>
       </c>
       <c r="G13" s="15" t="inlineStr">
@@ -2350,10 +2350,10 @@
         </is>
       </c>
       <c r="E14" s="16" t="n">
-        <v>30</v>
+        <v>9.23</v>
       </c>
       <c r="F14" s="15">
-        <f> HSV1.005 plocha 30 m²</f>
+        <f> HSV1.005 plocha 9.23 m²</f>
         <v/>
       </c>
       <c r="G14" s="15" t="inlineStr">
@@ -2669,70 +2669,70 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="17" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" s="18" t="inlineStr">
+        <is>
+          <t>HSV-1 Zemní práce</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>Venkovní schody na terénu z betonových dílců do betonového lože — rameno 1: 8×175×280 mm + rameno 2: 5×175×280 mm (13 stupňů), zahrada za opěrnou stěnou</t>
+        </is>
+      </c>
+      <c r="D21" s="17" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="E21" s="19" t="n">
+        <v>13</v>
+      </c>
+      <c r="F21" s="18" t="inlineStr">
+        <is>
+          <t>Situace měření 2026-05-29: rameno 1 = 8 stupňů + rameno 2 = 5 stupňů = 13 stupňů (175×280 mm)</t>
+        </is>
+      </c>
+      <c r="G21" s="18" t="inlineStr"/>
+      <c r="H21" s="17" t="inlineStr">
+        <is>
+          <t>❌ blank — ÚRS online</t>
+        </is>
+      </c>
+      <c r="I21" s="18" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV1.016</t>
+        </is>
+      </c>
+      <c r="J21" s="18" t="inlineStr">
+        <is>
+          <t>Venkovní schody na terénu</t>
+        </is>
+      </c>
+      <c r="K21" s="18" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
         <is>
           <t>━━ HSV-2 Základové a ŽB  (13 atomic operací) ━━</t>
         </is>
       </c>
-      <c r="B21" s="9" t="n"/>
-      <c r="C21" s="9" t="n"/>
-      <c r="D21" s="9" t="n"/>
-      <c r="E21" s="9" t="n"/>
-      <c r="F21" s="9" t="n"/>
-      <c r="G21" s="9" t="n"/>
-      <c r="H21" s="9" t="n"/>
-      <c r="I21" s="9" t="n"/>
-      <c r="J21" s="9" t="n"/>
-      <c r="K21" s="9" t="n"/>
-    </row>
-    <row r="22">
-      <c r="A22" s="10" t="n">
-        <v>19</v>
-      </c>
-      <c r="B22" s="11" t="inlineStr">
-        <is>
-          <t>HSV-2 Základové a ŽB</t>
-        </is>
-      </c>
-      <c r="C22" s="11" t="inlineStr">
-        <is>
-          <t>Bílá vana ČBS 02 — pata úhlové opěrné stěny 250×1200 mm × L=10 m, C25/30 XC3 XF1 XA1 CL0.4 Dmax22 S3</t>
-        </is>
-      </c>
-      <c r="D22" s="10" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="E22" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="F22" s="11" t="inlineStr">
-        <is>
-          <t>0.25 × 1.20 × 10 = 3.0</t>
-        </is>
-      </c>
-      <c r="G22" s="13" t="inlineStr">
-        <is>
-          <t>274321321</t>
-        </is>
-      </c>
-      <c r="H22" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I22" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV2.001</t>
-        </is>
-      </c>
-      <c r="J22" s="11" t="inlineStr"/>
-      <c r="K22" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
+      <c r="B22" s="9" t="n"/>
+      <c r="C22" s="9" t="n"/>
+      <c r="D22" s="9" t="n"/>
+      <c r="E22" s="9" t="n"/>
+      <c r="F22" s="9" t="n"/>
+      <c r="G22" s="9" t="n"/>
+      <c r="H22" s="9" t="n"/>
+      <c r="I22" s="9" t="n"/>
+      <c r="J22" s="9" t="n"/>
+      <c r="K22" s="9" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="10" t="n">
@@ -2745,7 +2745,7 @@
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>Bílá vana ČBS 02 — stěna úhlová tl. 250 mm × výška 2050 mm × L=10 m, beton C25/30 XC3 XF1 XA1 (trhliny max 0.20 mm)</t>
+          <t>Bílá vana ČBS 02 — pata úhlové opěrné stěny 250×1200 mm × L=10 m, C25/30 XC3 XF1 XA1 CL0.4 Dmax22 S3</t>
         </is>
       </c>
       <c r="D23" s="10" t="inlineStr">
@@ -2754,14 +2754,14 @@
         </is>
       </c>
       <c r="E23" s="12" t="n">
-        <v>5.12</v>
+        <v>3</v>
       </c>
       <c r="F23" s="11" t="inlineStr">
         <is>
-          <t>0.25 × 2.05 × 10 = 5.13</t>
-        </is>
-      </c>
-      <c r="G23" s="11" t="inlineStr">
+          <t>0.25 × 1.20 × 10 = 3.0</t>
+        </is>
+      </c>
+      <c r="G23" s="13" t="inlineStr">
         <is>
           <t>274321321</t>
         </is>
@@ -2773,7 +2773,7 @@
       </c>
       <c r="I23" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV2.002</t>
+          <t>260219_dum.HSV2.001</t>
         </is>
       </c>
       <c r="J23" s="11" t="inlineStr"/>
@@ -2784,190 +2784,190 @@
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="17" t="n">
+      <c r="A24" s="10" t="n">
         <v>21</v>
       </c>
-      <c r="B24" s="18" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>HSV-2 Základové a ŽB</t>
         </is>
       </c>
-      <c r="C24" s="18" t="inlineStr">
+      <c r="C24" s="11" t="inlineStr">
+        <is>
+          <t>Bílá vana ČBS 02 — stěna úhlová tl. 250 mm × výška 2050 mm × L=10 m, beton C25/30 XC3 XF1 XA1 (trhliny max 0.20 mm)</t>
+        </is>
+      </c>
+      <c r="D24" s="10" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="n">
+        <v>5.12</v>
+      </c>
+      <c r="F24" s="11" t="inlineStr">
+        <is>
+          <t>0.25 × 2.05 × 10 = 5.13</t>
+        </is>
+      </c>
+      <c r="G24" s="11" t="inlineStr">
+        <is>
+          <t>274321321</t>
+        </is>
+      </c>
+      <c r="H24" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I24" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV2.002</t>
+        </is>
+      </c>
+      <c r="J24" s="11" t="inlineStr"/>
+      <c r="K24" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="n">
+        <v>22</v>
+      </c>
+      <c r="B25" s="18" t="inlineStr">
+        <is>
+          <t>HSV-2 Základové a ŽB</t>
+        </is>
+      </c>
+      <c r="C25" s="18" t="inlineStr">
         <is>
           <t>Systémové oboustranné bednění bílé vany — DOKA Framax / PERI MAXIMO, vč. těsnění pracovních spár bobtnavý pásek bentonit (TZ §5.5)</t>
         </is>
       </c>
-      <c r="D24" s="17" t="inlineStr">
+      <c r="D25" s="17" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E24" s="19" t="n">
+      <c r="E25" s="19" t="n">
         <v>65</v>
       </c>
-      <c r="F24" s="18" t="inlineStr">
+      <c r="F25" s="18" t="inlineStr">
         <is>
           <t>2×2.05×10 (svislé) + 2×1.20×10 (pata) = 41 + 24 = 65</t>
         </is>
       </c>
-      <c r="G24" s="18" t="inlineStr"/>
-      <c r="H24" s="17" t="inlineStr">
+      <c r="G25" s="18" t="inlineStr"/>
+      <c r="H25" s="17" t="inlineStr">
         <is>
           <t>❌ blank — ÚRS online</t>
         </is>
       </c>
-      <c r="I24" s="18" t="inlineStr">
+      <c r="I25" s="18" t="inlineStr">
         <is>
           <t>260219_dum.HSV2.003</t>
         </is>
       </c>
-      <c r="J24" s="18" t="inlineStr"/>
-      <c r="K24" s="18" t="inlineStr">
+      <c r="J25" s="18" t="inlineStr"/>
+      <c r="K25" s="18" t="inlineStr">
         <is>
           <t>Carried 1:1 (atomic — no decomposition needed)  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="10" t="n">
-        <v>22</v>
-      </c>
-      <c r="B25" s="11" t="inlineStr">
+    <row r="26">
+      <c r="A26" s="10" t="n">
+        <v>23</v>
+      </c>
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>HSV-2 Základové a ŽB</t>
         </is>
       </c>
-      <c r="C25" s="11" t="inlineStr">
+      <c r="C26" s="11" t="inlineStr">
         <is>
           <t>Výztuž bílé vany B500B 120 kg/m³ (empirická sazba Methvin pro úhlové opěrné stěny W0)</t>
         </is>
       </c>
-      <c r="D25" s="10" t="inlineStr">
+      <c r="D26" s="10" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="E25" s="12" t="n">
+      <c r="E26" s="12" t="n">
         <v>975</v>
       </c>
-      <c r="F25" s="11" t="inlineStr">
+      <c r="F26" s="11" t="inlineStr">
         <is>
           <t>(3.0+5.13) × 120 = 976</t>
         </is>
       </c>
-      <c r="G25" s="13" t="inlineStr">
+      <c r="G26" s="13" t="inlineStr">
         <is>
           <t>273361821</t>
         </is>
       </c>
-      <c r="H25" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I25" s="11" t="inlineStr">
+      <c r="H26" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I26" s="11" t="inlineStr">
         <is>
           <t>260219_dum.HSV2.004</t>
         </is>
       </c>
-      <c r="J25" s="11" t="inlineStr"/>
-      <c r="K25" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="17" t="n">
-        <v>23</v>
-      </c>
-      <c r="B26" s="18" t="inlineStr">
+      <c r="J26" s="11" t="inlineStr"/>
+      <c r="K26" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="17" t="n">
+        <v>24</v>
+      </c>
+      <c r="B27" s="18" t="inlineStr">
         <is>
           <t>HSV-2 Základové a ŽB</t>
         </is>
       </c>
-      <c r="C26" s="18" t="inlineStr">
+      <c r="C27" s="18" t="inlineStr">
         <is>
           <t>Separační PE fólie pod základovou patou bílé vany (povinná dle ČBS 02)</t>
         </is>
       </c>
-      <c r="D26" s="17" t="inlineStr">
+      <c r="D27" s="17" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E26" s="19" t="n">
+      <c r="E27" s="19" t="n">
         <v>13.2</v>
       </c>
-      <c r="F26" s="18" t="inlineStr">
+      <c r="F27" s="18" t="inlineStr">
         <is>
           <t>1.20 × 10 × 1.10 přesah = 13.2</t>
         </is>
       </c>
-      <c r="G26" s="18" t="inlineStr"/>
-      <c r="H26" s="17" t="inlineStr">
+      <c r="G27" s="18" t="inlineStr"/>
+      <c r="H27" s="17" t="inlineStr">
         <is>
           <t>❌ blank — ÚRS online</t>
         </is>
       </c>
-      <c r="I26" s="18" t="inlineStr">
+      <c r="I27" s="18" t="inlineStr">
         <is>
           <t>260219_dum.HSV2.005</t>
         </is>
       </c>
-      <c r="J26" s="18" t="inlineStr"/>
-      <c r="K26" s="18" t="inlineStr">
+      <c r="J27" s="18" t="inlineStr"/>
+      <c r="K27" s="18" t="inlineStr">
         <is>
           <t>Carried 1:1 (atomic — no decomposition needed)  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="10" t="n">
-        <v>24</v>
-      </c>
-      <c r="B27" s="11" t="inlineStr">
-        <is>
-          <t>HSV-2 Základové a ŽB</t>
-        </is>
-      </c>
-      <c r="C27" s="11" t="inlineStr">
-        <is>
-          <t>Mokré ošetřování betonu bílé vany min. 7 dní dle ČSN EN 13670 + ČBS 02 (kontrola trhlin max 0.20 mm)</t>
-        </is>
-      </c>
-      <c r="D27" s="10" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E27" s="12" t="n">
-        <v>53</v>
-      </c>
-      <c r="F27" s="11" t="inlineStr">
-        <is>
-          <t>viditelná plocha BV pro ošetřování ~53</t>
-        </is>
-      </c>
-      <c r="G27" s="11" t="inlineStr">
-        <is>
-          <t>279351102</t>
-        </is>
-      </c>
-      <c r="H27" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I27" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV2.006</t>
-        </is>
-      </c>
-      <c r="J27" s="11" t="inlineStr"/>
-      <c r="K27" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
         </is>
       </c>
     </row>
@@ -2982,25 +2982,25 @@
       </c>
       <c r="C28" s="11" t="inlineStr">
         <is>
-          <t>ŽB pozední věnec 300×250 mm po obvodu nadezdívky 3.NP, beton C25/30 XC1 + výztuž 100 kg/m³</t>
+          <t>Mokré ošetřování betonu bílé vany min. 7 dní dle ČSN EN 13670 + ČBS 02 (kontrola trhlin max 0.20 mm)</t>
         </is>
       </c>
       <c r="D28" s="10" t="inlineStr">
         <is>
-          <t>m³</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E28" s="12" t="n">
-        <v>2.9</v>
+        <v>53</v>
       </c>
       <c r="F28" s="11" t="inlineStr">
         <is>
-          <t>0.30 × 0.25 × obvod 38.7 m (DXF km_R_návrh_tlustá 2 closed polygon area 91.28 m²) = 2.9 m³</t>
-        </is>
-      </c>
-      <c r="G28" s="13" t="inlineStr">
-        <is>
-          <t>274321311</t>
+          <t>viditelná plocha BV pro ošetřování ~53</t>
+        </is>
+      </c>
+      <c r="G28" s="11" t="inlineStr">
+        <is>
+          <t>279351102</t>
         </is>
       </c>
       <c r="H28" s="10" t="inlineStr">
@@ -3010,7 +3010,7 @@
       </c>
       <c r="I28" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV2.007</t>
+          <t>260219_dum.HSV2.006</t>
         </is>
       </c>
       <c r="J28" s="11" t="inlineStr"/>
@@ -3021,96 +3021,96 @@
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="17" t="n">
+      <c r="A29" s="10" t="n">
         <v>26</v>
       </c>
-      <c r="B29" s="18" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>HSV-2 Základové a ŽB</t>
         </is>
       </c>
-      <c r="C29" s="18" t="inlineStr">
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>ŽB pozední věnec 300×250 mm po obvodu nadezdívky 3.NP, beton C25/30 XC1 + výztuž 100 kg/m³</t>
+        </is>
+      </c>
+      <c r="D29" s="10" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="E29" s="12" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="F29" s="11" t="inlineStr">
+        <is>
+          <t>0.30 × 0.25 × obvod 38.7 m (DXF km_R_návrh_tlustá 2 closed polygon area 91.28 m²) = 2.9 m³</t>
+        </is>
+      </c>
+      <c r="G29" s="13" t="inlineStr">
+        <is>
+          <t>274321311</t>
+        </is>
+      </c>
+      <c r="H29" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I29" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV2.007</t>
+        </is>
+      </c>
+      <c r="J29" s="11" t="inlineStr"/>
+      <c r="K29" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="17" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" s="18" t="inlineStr">
+        <is>
+          <t>HSV-2 Základové a ŽB</t>
+        </is>
+      </c>
+      <c r="C30" s="18" t="inlineStr">
         <is>
           <t>Bednění pozedního věnce systémové oboustranné</t>
         </is>
       </c>
-      <c r="D29" s="17" t="inlineStr">
+      <c r="D30" s="17" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E29" s="19" t="n">
+      <c r="E30" s="19" t="n">
         <v>19.4</v>
       </c>
-      <c r="F29" s="18" t="inlineStr">
+      <c r="F30" s="18" t="inlineStr">
         <is>
           <t>2 (oboustranné) × 0.25 m výška × obvod 38.7 m (DXF) = 19.4 m²</t>
         </is>
       </c>
-      <c r="G29" s="18" t="inlineStr"/>
-      <c r="H29" s="17" t="inlineStr">
+      <c r="G30" s="18" t="inlineStr"/>
+      <c r="H30" s="17" t="inlineStr">
         <is>
           <t>❌ blank — ÚRS online</t>
         </is>
       </c>
-      <c r="I29" s="18" t="inlineStr">
+      <c r="I30" s="18" t="inlineStr">
         <is>
           <t>260219_dum.HSV2.008</t>
         </is>
       </c>
-      <c r="J29" s="18" t="inlineStr"/>
-      <c r="K29" s="18" t="inlineStr">
+      <c r="J30" s="18" t="inlineStr"/>
+      <c r="K30" s="18" t="inlineStr">
         <is>
           <t>Carried 1:1 (atomic — no decomposition needed)  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30">
-      <c r="A30" s="10" t="n">
-        <v>27</v>
-      </c>
-      <c r="B30" s="11" t="inlineStr">
-        <is>
-          <t>HSV-2 Základové a ŽB</t>
-        </is>
-      </c>
-      <c r="C30" s="11" t="inlineStr">
-        <is>
-          <t>Výztuž B500B věnce 100 kg/m³ (Methvin sazba pro pozední věnce)</t>
-        </is>
-      </c>
-      <c r="D30" s="10" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E30" s="12" t="n">
-        <v>310</v>
-      </c>
-      <c r="F30" s="11" t="inlineStr">
-        <is>
-          <t>3.1 × 100 = 310</t>
-        </is>
-      </c>
-      <c r="G30" s="11" t="inlineStr">
-        <is>
-          <t>273361821</t>
-        </is>
-      </c>
-      <c r="H30" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I30" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV2.009</t>
-        </is>
-      </c>
-      <c r="J30" s="11" t="inlineStr"/>
-      <c r="K30" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
         </is>
       </c>
     </row>
@@ -3125,25 +3125,25 @@
       </c>
       <c r="C31" s="11" t="inlineStr">
         <is>
-          <t>Nabetonávka stropu 2.NP/3.NP — beton C25/30 XC1 tl. 60 mm nad vlnu trapézového plechu 40S/160</t>
+          <t>Výztuž B500B věnce 100 kg/m³ (Methvin sazba pro pozední věnce)</t>
         </is>
       </c>
       <c r="D31" s="10" t="inlineStr">
         <is>
-          <t>m³</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E31" s="12" t="n">
-        <v>6.26</v>
+        <v>310</v>
       </c>
       <c r="F31" s="11" t="inlineStr">
         <is>
-          <t>104.4 m² × 0.06 m = 6.26</t>
-        </is>
-      </c>
-      <c r="G31" s="13" t="inlineStr">
-        <is>
-          <t>274321111</t>
+          <t>3.1 × 100 = 310</t>
+        </is>
+      </c>
+      <c r="G31" s="11" t="inlineStr">
+        <is>
+          <t>273361821</t>
         </is>
       </c>
       <c r="H31" s="10" t="inlineStr">
@@ -3153,14 +3153,10 @@
       </c>
       <c r="I31" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV2.010</t>
-        </is>
-      </c>
-      <c r="J31" s="11" t="inlineStr">
-        <is>
-          <t>S09</t>
-        </is>
-      </c>
+          <t>260219_dum.HSV2.009</t>
+        </is>
+      </c>
+      <c r="J31" s="11" t="inlineStr"/>
       <c r="K31" s="11" t="inlineStr">
         <is>
           <t>Carried 1:1 (atomic — no decomposition needed)</t>
@@ -3178,25 +3174,25 @@
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Výztuž nabetonávky kari síť 5/100/100 (cca 4.4 kg/m²)</t>
+          <t>Nabetonávka stropu 2.NP/3.NP — beton C25/30 XC1 tl. 60 mm nad vlnu trapézového plechu 40S/160</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="E32" s="12" t="n">
-        <v>459</v>
+        <v>6.26</v>
       </c>
       <c r="F32" s="11" t="inlineStr">
         <is>
-          <t>104.4 m² × 4.4 kg/m² = 459</t>
-        </is>
-      </c>
-      <c r="G32" s="11" t="inlineStr">
-        <is>
-          <t>273362441</t>
+          <t>104.4 m² × 0.06 m = 6.26</t>
+        </is>
+      </c>
+      <c r="G32" s="13" t="inlineStr">
+        <is>
+          <t>274321111</t>
         </is>
       </c>
       <c r="H32" s="10" t="inlineStr">
@@ -3206,7 +3202,7 @@
       </c>
       <c r="I32" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV2.011</t>
+          <t>260219_dum.HSV2.010</t>
         </is>
       </c>
       <c r="J32" s="11" t="inlineStr">
@@ -3231,25 +3227,25 @@
       </c>
       <c r="C33" s="11" t="inlineStr">
         <is>
-          <t>ŽB deska podlahy 1.NP na terénu tl. 150 mm, C25/30 XC2 + vyztužení kari 6/150/150 + okrajové pruty</t>
+          <t>Výztuž nabetonávky kari síť 5/100/100 (cca 4.4 kg/m²)</t>
         </is>
       </c>
       <c r="D33" s="10" t="inlineStr">
         <is>
-          <t>m³</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E33" s="12" t="n">
-        <v>10.96</v>
+        <v>459</v>
       </c>
       <c r="F33" s="11" t="inlineStr">
         <is>
-          <t>104.4 × 0.7 (rozsah 1.NP) × 0.15 = ~11.0</t>
-        </is>
-      </c>
-      <c r="G33" s="13" t="inlineStr">
-        <is>
-          <t>273321311</t>
+          <t>104.4 m² × 4.4 kg/m² = 459</t>
+        </is>
+      </c>
+      <c r="G33" s="11" t="inlineStr">
+        <is>
+          <t>273362441</t>
         </is>
       </c>
       <c r="H33" s="10" t="inlineStr">
@@ -3259,12 +3255,12 @@
       </c>
       <c r="I33" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV2.012</t>
+          <t>260219_dum.HSV2.011</t>
         </is>
       </c>
       <c r="J33" s="11" t="inlineStr">
         <is>
-          <t>S05</t>
+          <t>S09</t>
         </is>
       </c>
       <c r="K33" s="11" t="inlineStr">
@@ -3284,117 +3280,117 @@
       </c>
       <c r="C34" s="11" t="inlineStr">
         <is>
+          <t>ŽB deska podlahy 1.NP na terénu tl. 150 mm, C25/30 XC2 + vyztužení kari 6/150/150 + okrajové pruty</t>
+        </is>
+      </c>
+      <c r="D34" s="10" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="E34" s="12" t="n">
+        <v>10.96</v>
+      </c>
+      <c r="F34" s="11" t="inlineStr">
+        <is>
+          <t>104.4 × 0.7 (rozsah 1.NP) × 0.15 = ~11.0</t>
+        </is>
+      </c>
+      <c r="G34" s="13" t="inlineStr">
+        <is>
+          <t>273321311</t>
+        </is>
+      </c>
+      <c r="H34" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I34" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV2.012</t>
+        </is>
+      </c>
+      <c r="J34" s="11" t="inlineStr">
+        <is>
+          <t>S05</t>
+        </is>
+      </c>
+      <c r="K34" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="10" t="n">
+        <v>32</v>
+      </c>
+      <c r="B35" s="11" t="inlineStr">
+        <is>
+          <t>HSV-2 Základové a ŽB</t>
+        </is>
+      </c>
+      <c r="C35" s="11" t="inlineStr">
+        <is>
           <t>Výztuž ŽB desky 1.NP — kari 6/150/150 + B500B okrajové pruty (~75 kg/m³ Methvin)</t>
         </is>
       </c>
-      <c r="D34" s="10" t="inlineStr">
+      <c r="D35" s="10" t="inlineStr">
         <is>
           <t>kg</t>
         </is>
       </c>
-      <c r="E34" s="12" t="n">
+      <c r="E35" s="12" t="n">
         <v>825</v>
       </c>
-      <c r="F34" s="11" t="inlineStr">
+      <c r="F35" s="11" t="inlineStr">
         <is>
           <t>11.0 × 75 = 825</t>
         </is>
       </c>
-      <c r="G34" s="11" t="inlineStr">
+      <c r="G35" s="11" t="inlineStr">
         <is>
           <t>273361821</t>
         </is>
       </c>
-      <c r="H34" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I34" s="11" t="inlineStr">
+      <c r="H35" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I35" s="11" t="inlineStr">
         <is>
           <t>260219_dum.HSV2.013</t>
         </is>
       </c>
-      <c r="J34" s="11" t="inlineStr">
+      <c r="J35" s="11" t="inlineStr">
         <is>
           <t>S05</t>
         </is>
       </c>
-      <c r="K34" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="K35" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="8" t="inlineStr">
         <is>
           <t>━━ HSV-3 Svislé konstrukce  (7 atomic operací) ━━</t>
         </is>
       </c>
-      <c r="B35" s="9" t="n"/>
-      <c r="C35" s="9" t="n"/>
-      <c r="D35" s="9" t="n"/>
-      <c r="E35" s="9" t="n"/>
-      <c r="F35" s="9" t="n"/>
-      <c r="G35" s="9" t="n"/>
-      <c r="H35" s="9" t="n"/>
-      <c r="I35" s="9" t="n"/>
-      <c r="J35" s="9" t="n"/>
-      <c r="K35" s="9" t="n"/>
-    </row>
-    <row r="36">
-      <c r="A36" s="10" t="n">
-        <v>32</v>
-      </c>
-      <c r="B36" s="11" t="inlineStr">
-        <is>
-          <t>HSV-3 Svislé konstrukce</t>
-        </is>
-      </c>
-      <c r="C36" s="11" t="inlineStr">
-        <is>
-          <t>Lokální dozdívky a přizdívky z cihel plných pálených P10 na MVC M10 (uvedeno v TZ statika §4)</t>
-        </is>
-      </c>
-      <c r="D36" s="10" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="E36" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="F36" s="11" t="inlineStr">
-        <is>
-          <t>odhad — drobné dozdívky kolem nových otvorů 1.NP/2.NP</t>
-        </is>
-      </c>
-      <c r="G36" s="11" t="inlineStr">
-        <is>
-          <t>311232511</t>
-        </is>
-      </c>
-      <c r="H36" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I36" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV3.001</t>
-        </is>
-      </c>
-      <c r="J36" s="11" t="inlineStr">
-        <is>
-          <t>S01, S02</t>
-        </is>
-      </c>
-      <c r="K36" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
+      <c r="B36" s="9" t="n"/>
+      <c r="C36" s="9" t="n"/>
+      <c r="D36" s="9" t="n"/>
+      <c r="E36" s="9" t="n"/>
+      <c r="F36" s="9" t="n"/>
+      <c r="G36" s="9" t="n"/>
+      <c r="H36" s="9" t="n"/>
+      <c r="I36" s="9" t="n"/>
+      <c r="J36" s="9" t="n"/>
+      <c r="K36" s="9" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="10" t="n">
@@ -3407,40 +3403,40 @@
       </c>
       <c r="C37" s="11" t="inlineStr">
         <is>
-          <t>Nadezdívka 3.NP a čela vikýřů — Porotherm 30 Profi P10 na maltu pro tenké spáry, výška 2.65 m</t>
+          <t>Lokální dozdívky a přizdívky z cihel plných pálených P10 na MVC M10 (uvedeno v TZ statika §4)</t>
         </is>
       </c>
       <c r="D37" s="10" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="E37" s="12" t="n">
-        <v>71.8</v>
+        <v>4</v>
       </c>
       <c r="F37" s="11" t="inlineStr">
         <is>
-          <t>obvod 38.7 m (DXF km_R_návrh_tlustá 2) × výška 2.65 m × 0.7 (sníženo o štíty zachované — řadovka) = 71.8 m²</t>
-        </is>
-      </c>
-      <c r="G37" s="13" t="inlineStr">
-        <is>
-          <t>311321411</t>
+          <t>odhad — drobné dozdívky kolem nových otvorů 1.NP/2.NP</t>
+        </is>
+      </c>
+      <c r="G37" s="11" t="inlineStr">
+        <is>
+          <t>311232511</t>
         </is>
       </c>
       <c r="H37" s="10" t="inlineStr">
         <is>
-          <t>✓ verified</t>
+          <t>⚠ kandidát-verify</t>
         </is>
       </c>
       <c r="I37" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV3.002</t>
+          <t>260219_dum.HSV3.001</t>
         </is>
       </c>
       <c r="J37" s="11" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>S01, S02</t>
         </is>
       </c>
       <c r="K37" s="11" t="inlineStr">
@@ -3460,40 +3456,40 @@
       </c>
       <c r="C38" s="11" t="inlineStr">
         <is>
-          <t>Ocelové překlady IPN160 ve dvojici nad otvory pro nové dveře/okna v 1.NP a 2.NP (8 otvorů odhad)</t>
+          <t>Nadezdívka 3.NP a čela vikýřů — Porotherm 30 Profi P10 na maltu pro tenké spáry, výška 2.65 m</t>
         </is>
       </c>
       <c r="D38" s="10" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E38" s="12" t="n">
-        <v>8</v>
+        <v>71.8</v>
       </c>
       <c r="F38" s="11" t="inlineStr">
         <is>
-          <t>odhad 8 nových otvorů × 2 IPN160 (dvojice)</t>
+          <t>obvod 38.7 m (DXF km_R_návrh_tlustá 2) × výška 2.65 m × 0.7 (sníženo o štíty zachované — řadovka) = 71.8 m²</t>
         </is>
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t>317143112</t>
+          <t>311321411</t>
         </is>
       </c>
       <c r="H38" s="10" t="inlineStr">
         <is>
-          <t>⚠ kandidát-verify</t>
+          <t>✓ verified</t>
         </is>
       </c>
       <c r="I38" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV3.003</t>
+          <t>260219_dum.HSV3.002</t>
         </is>
       </c>
       <c r="J38" s="11" t="inlineStr">
         <is>
-          <t>S01</t>
+          <t>S12</t>
         </is>
       </c>
       <c r="K38" s="11" t="inlineStr">
@@ -3513,25 +3509,25 @@
       </c>
       <c r="C39" s="11" t="inlineStr">
         <is>
-          <t>Maltové uložení překladů IPN160 — MC25 tl. 50 mm + kari 5/100/100 (po obou stranách otvoru)</t>
+          <t>Ocelové překlady IPN160 ve dvojici nad otvory pro nové dveře/okna v 1.NP a 2.NP (8 otvorů odhad)</t>
         </is>
       </c>
       <c r="D39" s="10" t="inlineStr">
         <is>
-          <t>kpl</t>
+          <t>ks</t>
         </is>
       </c>
       <c r="E39" s="12" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F39" s="11" t="inlineStr">
         <is>
-          <t>8 otvorů × 2 strany = 16 uložení</t>
-        </is>
-      </c>
-      <c r="G39" s="11" t="inlineStr">
-        <is>
-          <t>317242421</t>
+          <t>odhad 8 nových otvorů × 2 IPN160 (dvojice)</t>
+        </is>
+      </c>
+      <c r="G39" s="13" t="inlineStr">
+        <is>
+          <t>317143112</t>
         </is>
       </c>
       <c r="H39" s="10" t="inlineStr">
@@ -3541,7 +3537,7 @@
       </c>
       <c r="I39" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV3.004</t>
+          <t>260219_dum.HSV3.003</t>
         </is>
       </c>
       <c r="J39" s="11" t="inlineStr">
@@ -3566,35 +3562,35 @@
       </c>
       <c r="C40" s="11" t="inlineStr">
         <is>
-          <t>Zesílení ostění úhelníky L100/10 dvojicí u otvoru u komínového tělesa (statická limitace)</t>
+          <t>Maltové uložení překladů IPN160 — MC25 tl. 50 mm + kari 5/100/100 (po obou stranách otvoru)</t>
         </is>
       </c>
       <c r="D40" s="10" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>kpl</t>
         </is>
       </c>
       <c r="E40" s="12" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="F40" s="11" t="inlineStr">
         <is>
-          <t>TZ statika §4 — 2× L100/10 (dvojice) na 2 strany otvoru = 4 ks</t>
+          <t>8 otvorů × 2 strany = 16 uložení</t>
         </is>
       </c>
       <c r="G40" s="11" t="inlineStr">
         <is>
-          <t>767131120</t>
+          <t>317242421</t>
         </is>
       </c>
       <c r="H40" s="10" t="inlineStr">
         <is>
-          <t>✓ verified</t>
+          <t>⚠ kandidát-verify</t>
         </is>
       </c>
       <c r="I40" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV3.005</t>
+          <t>260219_dum.HSV3.004</t>
         </is>
       </c>
       <c r="J40" s="11" t="inlineStr">
@@ -3619,37 +3615,42 @@
       </c>
       <c r="C41" s="11" t="inlineStr">
         <is>
-          <t>Dočasné podstojkování stávajících přiléhajících stropů při osazování IPN překladů (8 otvorů)</t>
+          <t>Zesílení ostění úhelníky L100/10 dvojicí u otvoru u komínového tělesa (statická limitace)</t>
         </is>
       </c>
       <c r="D41" s="10" t="inlineStr">
         <is>
-          <t>kpl</t>
+          <t>ks</t>
         </is>
       </c>
       <c r="E41" s="12" t="n">
-        <v>8</v>
-      </c>
-      <c r="F41" s="11">
-        <f> počet překladů (po jednom podstojkování per otvor)</f>
-        <v/>
-      </c>
-      <c r="G41" s="13" t="inlineStr">
-        <is>
-          <t>962081120</t>
+        <v>4</v>
+      </c>
+      <c r="F41" s="11" t="inlineStr">
+        <is>
+          <t>TZ statika §4 — 2× L100/10 (dvojice) na 2 strany otvoru = 4 ks</t>
+        </is>
+      </c>
+      <c r="G41" s="11" t="inlineStr">
+        <is>
+          <t>767131120</t>
         </is>
       </c>
       <c r="H41" s="10" t="inlineStr">
         <is>
-          <t>⚠ kandidát-verify</t>
+          <t>✓ verified</t>
         </is>
       </c>
       <c r="I41" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV3.006</t>
-        </is>
-      </c>
-      <c r="J41" s="11" t="inlineStr"/>
+          <t>260219_dum.HSV3.005</t>
+        </is>
+      </c>
+      <c r="J41" s="11" t="inlineStr">
+        <is>
+          <t>S01</t>
+        </is>
+      </c>
       <c r="K41" s="11" t="inlineStr">
         <is>
           <t>Carried 1:1 (atomic — no decomposition needed)</t>
@@ -3667,113 +3668,112 @@
       </c>
       <c r="C42" s="11" t="inlineStr">
         <is>
+          <t>Dočasné podstojkování stávajících přiléhajících stropů při osazování IPN překladů (8 otvorů)</t>
+        </is>
+      </c>
+      <c r="D42" s="10" t="inlineStr">
+        <is>
+          <t>kpl</t>
+        </is>
+      </c>
+      <c r="E42" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="F42" s="11">
+        <f> počet překladů (po jednom podstojkování per otvor)</f>
+        <v/>
+      </c>
+      <c r="G42" s="13" t="inlineStr">
+        <is>
+          <t>962081120</t>
+        </is>
+      </c>
+      <c r="H42" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I42" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV3.006</t>
+        </is>
+      </c>
+      <c r="J42" s="11" t="inlineStr"/>
+      <c r="K42" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="10" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="11" t="inlineStr">
+        <is>
+          <t>HSV-3 Svislé konstrukce</t>
+        </is>
+      </c>
+      <c r="C43" s="11" t="inlineStr">
+        <is>
           <t>Nové příčky z pórobetonových tvárnic 150 mm na lepidlo + dilatovány od stropu</t>
         </is>
       </c>
-      <c r="D42" s="10" t="inlineStr">
+      <c r="D43" s="10" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E42" s="12" t="n">
+      <c r="E43" s="12" t="n">
         <v>87.7</v>
       </c>
-      <c r="F42" s="11" t="inlineStr">
+      <c r="F43" s="11" t="inlineStr">
         <is>
           <t>podlahova_plocha × 0.4 (typický rozsah příček 30-50%)</t>
         </is>
       </c>
-      <c r="G42" s="13" t="inlineStr">
+      <c r="G43" s="13" t="inlineStr">
         <is>
           <t>342241211</t>
         </is>
       </c>
-      <c r="H42" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I42" s="11" t="inlineStr">
+      <c r="H43" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I43" s="11" t="inlineStr">
         <is>
           <t>260219_dum.HSV3.007</t>
         </is>
       </c>
-      <c r="J42" s="11" t="inlineStr">
+      <c r="J43" s="11" t="inlineStr">
         <is>
           <t>S02</t>
         </is>
       </c>
-      <c r="K42" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="K43" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="8" t="inlineStr">
         <is>
           <t>━━ HSV-4 Vodorovné  (14 atomic operací) ━━</t>
         </is>
       </c>
-      <c r="B43" s="9" t="n"/>
-      <c r="C43" s="9" t="n"/>
-      <c r="D43" s="9" t="n"/>
-      <c r="E43" s="9" t="n"/>
-      <c r="F43" s="9" t="n"/>
-      <c r="G43" s="9" t="n"/>
-      <c r="H43" s="9" t="n"/>
-      <c r="I43" s="9" t="n"/>
-      <c r="J43" s="9" t="n"/>
-      <c r="K43" s="9" t="n"/>
-    </row>
-    <row r="44">
-      <c r="A44" s="10" t="n">
-        <v>39</v>
-      </c>
-      <c r="B44" s="11" t="inlineStr">
-        <is>
-          <t>HSV-4 Vodorovné</t>
-        </is>
-      </c>
-      <c r="C44" s="11" t="inlineStr">
-        <is>
-          <t>Ocelová stropnice IPE180 1.NP v pozici nové příčky 2.NP — dodávka + montáž (1 ks × ~5 m)</t>
-        </is>
-      </c>
-      <c r="D44" s="10" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E44" s="12" t="n">
-        <v>94</v>
-      </c>
-      <c r="F44" s="11" t="inlineStr">
-        <is>
-          <t>1 ks × 5 m × 18.8 kg/m (IPE180 hmotnost) = 94</t>
-        </is>
-      </c>
-      <c r="G44" s="13" t="inlineStr">
-        <is>
-          <t>411321414</t>
-        </is>
-      </c>
-      <c r="H44" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I44" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV4.001</t>
-        </is>
-      </c>
-      <c r="J44" s="11" t="inlineStr"/>
-      <c r="K44" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
+      <c r="B44" s="9" t="n"/>
+      <c r="C44" s="9" t="n"/>
+      <c r="D44" s="9" t="n"/>
+      <c r="E44" s="9" t="n"/>
+      <c r="F44" s="9" t="n"/>
+      <c r="G44" s="9" t="n"/>
+      <c r="H44" s="9" t="n"/>
+      <c r="I44" s="9" t="n"/>
+      <c r="J44" s="9" t="n"/>
+      <c r="K44" s="9" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="10" t="n">
@@ -3786,7 +3786,7 @@
       </c>
       <c r="C45" s="11" t="inlineStr">
         <is>
-          <t>Ocelobetonový strop 2.NP/3.NP — stropnice IPE180 á 1000 mm × rozpon ~8 m × ~8 ks</t>
+          <t>Ocelová stropnice IPE180 1.NP v pozici nové příčky 2.NP — dodávka + montáž (1 ks × ~5 m)</t>
         </is>
       </c>
       <c r="D45" s="10" t="inlineStr">
@@ -3795,11 +3795,11 @@
         </is>
       </c>
       <c r="E45" s="12" t="n">
-        <v>1203</v>
+        <v>94</v>
       </c>
       <c r="F45" s="11" t="inlineStr">
         <is>
-          <t>8 ks × 8 m × 18.8 kg/m = 1203</t>
+          <t>1 ks × 5 m × 18.8 kg/m (IPE180 hmotnost) = 94</t>
         </is>
       </c>
       <c r="G45" s="13" t="inlineStr">
@@ -3814,14 +3814,10 @@
       </c>
       <c r="I45" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV4.002</t>
-        </is>
-      </c>
-      <c r="J45" s="11" t="inlineStr">
-        <is>
-          <t>S09</t>
-        </is>
-      </c>
+          <t>260219_dum.HSV4.001</t>
+        </is>
+      </c>
+      <c r="J45" s="11" t="inlineStr"/>
       <c r="K45" s="11" t="inlineStr">
         <is>
           <t>Carried 1:1 (atomic — no decomposition needed)</t>
@@ -3839,7 +3835,7 @@
       </c>
       <c r="C46" s="11" t="inlineStr">
         <is>
-          <t>Ocelobetonový strop — výztuha 2×HEA180 trakt do ulice (Fibichova), dl. ~10 m</t>
+          <t>Ocelobetonový strop 2.NP/3.NP — stropnice IPE180 á 1000 mm × rozpon ~8 m × ~8 ks</t>
         </is>
       </c>
       <c r="D46" s="10" t="inlineStr">
@@ -3848,11 +3844,11 @@
         </is>
       </c>
       <c r="E46" s="12" t="n">
-        <v>710</v>
+        <v>1203</v>
       </c>
       <c r="F46" s="11" t="inlineStr">
         <is>
-          <t>2 ks × 10 m × 35.5 kg/m (HEA180) = 710</t>
+          <t>8 ks × 8 m × 18.8 kg/m = 1203</t>
         </is>
       </c>
       <c r="G46" s="13" t="inlineStr">
@@ -3867,7 +3863,7 @@
       </c>
       <c r="I46" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV4.003</t>
+          <t>260219_dum.HSV4.002</t>
         </is>
       </c>
       <c r="J46" s="11" t="inlineStr">
@@ -3892,7 +3888,7 @@
       </c>
       <c r="C47" s="11" t="inlineStr">
         <is>
-          <t>Ocelobetonový strop — výztuha HEA200 dvorní trakt, dl. ~10 m</t>
+          <t>Ocelobetonový strop — výztuha 2×HEA180 trakt do ulice (Fibichova), dl. ~10 m</t>
         </is>
       </c>
       <c r="D47" s="10" t="inlineStr">
@@ -3901,14 +3897,14 @@
         </is>
       </c>
       <c r="E47" s="12" t="n">
-        <v>423</v>
+        <v>710</v>
       </c>
       <c r="F47" s="11" t="inlineStr">
         <is>
-          <t>1 ks × 10 m × 42.3 kg/m (HEA200) = 423</t>
-        </is>
-      </c>
-      <c r="G47" s="11" t="inlineStr">
+          <t>2 ks × 10 m × 35.5 kg/m (HEA180) = 710</t>
+        </is>
+      </c>
+      <c r="G47" s="13" t="inlineStr">
         <is>
           <t>411321414</t>
         </is>
@@ -3920,7 +3916,7 @@
       </c>
       <c r="I47" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV4.004</t>
+          <t>260219_dum.HSV4.003</t>
         </is>
       </c>
       <c r="J47" s="11" t="inlineStr">
@@ -3945,22 +3941,23 @@
       </c>
       <c r="C48" s="11" t="inlineStr">
         <is>
-          <t>Trapézový plech 40S/160 tl. 0.75 mm — dodávka + montáž na stropnice IPE180</t>
+          <t>Ocelobetonový strop — výztuha HEA200 dvorní trakt, dl. ~10 m</t>
         </is>
       </c>
       <c r="D48" s="10" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E48" s="12" t="n">
-        <v>104.4</v>
-      </c>
-      <c r="F48" s="11">
-        <f> zastavěna plocha 104.4 m² (celý strop 2.NP/3.NP)</f>
-        <v/>
-      </c>
-      <c r="G48" s="13" t="inlineStr">
+        <v>423</v>
+      </c>
+      <c r="F48" s="11" t="inlineStr">
+        <is>
+          <t>1 ks × 10 m × 42.3 kg/m (HEA200) = 423</t>
+        </is>
+      </c>
+      <c r="G48" s="11" t="inlineStr">
         <is>
           <t>411321414</t>
         </is>
@@ -3972,7 +3969,7 @@
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV4.005</t>
+          <t>260219_dum.HSV4.004</t>
         </is>
       </c>
       <c r="J48" s="11" t="inlineStr">
@@ -3997,7 +3994,7 @@
       </c>
       <c r="C49" s="11" t="inlineStr">
         <is>
-          <t>Protipožární SDK podhled pod trapézovým plechem (EI 30 dle PBŘ — ocelobeton + SDK)</t>
+          <t>Trapézový plech 40S/160 tl. 0.75 mm — dodávka + montáž na stropnice IPE180</t>
         </is>
       </c>
       <c r="D49" s="10" t="inlineStr">
@@ -4009,12 +4006,12 @@
         <v>104.4</v>
       </c>
       <c r="F49" s="11">
-        <f> plocha trapézu 104.4 m²</f>
+        <f> zastavěna plocha 104.4 m² (celý strop 2.NP/3.NP)</f>
         <v/>
       </c>
       <c r="G49" s="13" t="inlineStr">
         <is>
-          <t>342213131</t>
+          <t>411321414</t>
         </is>
       </c>
       <c r="H49" s="10" t="inlineStr">
@@ -4024,7 +4021,7 @@
       </c>
       <c r="I49" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV4.006</t>
+          <t>260219_dum.HSV4.005</t>
         </is>
       </c>
       <c r="J49" s="11" t="inlineStr">
@@ -4049,40 +4046,39 @@
       </c>
       <c r="C50" s="11" t="inlineStr">
         <is>
-          <t>Vyvezení původního zásypu z cihelné klenby 1.PP/1.NP — manuálně + odvoz</t>
+          <t>Protipožární SDK podhled pod trapézovým plechem (EI 30 dle PBŘ — ocelobeton + SDK)</t>
         </is>
       </c>
       <c r="D50" s="10" t="inlineStr">
         <is>
-          <t>m³</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E50" s="12" t="n">
-        <v>8</v>
-      </c>
-      <c r="F50" s="11" t="inlineStr">
-        <is>
-          <t>klenba ~50 m² × tl. zásypu 0.15 m = 7.5 (round 8)</t>
-        </is>
-      </c>
-      <c r="G50" s="11" t="inlineStr">
-        <is>
-          <t>974031150</t>
+        <v>104.4</v>
+      </c>
+      <c r="F50" s="11">
+        <f> plocha trapézu 104.4 m²</f>
+        <v/>
+      </c>
+      <c r="G50" s="13" t="inlineStr">
+        <is>
+          <t>342213131</t>
         </is>
       </c>
       <c r="H50" s="10" t="inlineStr">
         <is>
-          <t>✓ verified</t>
+          <t>⚠ kandidát-verify</t>
         </is>
       </c>
       <c r="I50" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV4.007</t>
+          <t>260219_dum.HSV4.006</t>
         </is>
       </c>
       <c r="J50" s="11" t="inlineStr">
         <is>
-          <t>S06</t>
+          <t>S09</t>
         </is>
       </c>
       <c r="K50" s="11" t="inlineStr">
@@ -4102,7 +4098,7 @@
       </c>
       <c r="C51" s="11" t="inlineStr">
         <is>
-          <t>Nový zásyp klenby 1.PP/1.NP — perlitbeton (lehký zásyp) tl. 100 mm</t>
+          <t>Vyvezení původního zásypu z cihelné klenby 1.PP/1.NP — manuálně + odvoz</t>
         </is>
       </c>
       <c r="D51" s="10" t="inlineStr">
@@ -4111,26 +4107,26 @@
         </is>
       </c>
       <c r="E51" s="12" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F51" s="11" t="inlineStr">
         <is>
-          <t>klenba 50 m² × 0.10 m perlitbeton = 5.0</t>
+          <t>klenba ~50 m² × tl. zásypu 0.15 m = 7.5 (round 8)</t>
         </is>
       </c>
       <c r="G51" s="11" t="inlineStr">
         <is>
-          <t>271223111</t>
+          <t>974031150</t>
         </is>
       </c>
       <c r="H51" s="10" t="inlineStr">
         <is>
-          <t>⚠ kandidát-verify</t>
+          <t>✓ verified</t>
         </is>
       </c>
       <c r="I51" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV4.008</t>
+          <t>260219_dum.HSV4.007</t>
         </is>
       </c>
       <c r="J51" s="11" t="inlineStr">
@@ -4155,25 +4151,25 @@
       </c>
       <c r="C52" s="11" t="inlineStr">
         <is>
-          <t>Plastická perlitbetonová roznášecí vrstva tl. 50 mm nad zásypem klenby</t>
+          <t>Nový zásyp klenby 1.PP/1.NP — perlitbeton (lehký zásyp) tl. 100 mm</t>
         </is>
       </c>
       <c r="D52" s="10" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="E52" s="12" t="n">
-        <v>50</v>
+        <v>5</v>
       </c>
       <c r="F52" s="11" t="inlineStr">
         <is>
-          <t>klenba 1.PP/1.NP plocha ~50 m²</t>
+          <t>klenba 50 m² × 0.10 m perlitbeton = 5.0</t>
         </is>
       </c>
       <c r="G52" s="11" t="inlineStr">
         <is>
-          <t>631321311</t>
+          <t>271223111</t>
         </is>
       </c>
       <c r="H52" s="10" t="inlineStr">
@@ -4183,7 +4179,7 @@
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV4.009</t>
+          <t>260219_dum.HSV4.008</t>
         </is>
       </c>
       <c r="J52" s="11" t="inlineStr">
@@ -4208,7 +4204,7 @@
       </c>
       <c r="C53" s="11" t="inlineStr">
         <is>
-          <t>Strop trámový 1.NP/2.NP — sejmutí podlah, demontáž záklopu a zásypu shora (zachovat prkenný záklop na trámech)</t>
+          <t>Plastická perlitbetonová roznášecí vrstva tl. 50 mm nad zásypem klenby</t>
         </is>
       </c>
       <c r="D53" s="10" t="inlineStr">
@@ -4217,16 +4213,16 @@
         </is>
       </c>
       <c r="E53" s="12" t="n">
-        <v>100</v>
+        <v>50</v>
       </c>
       <c r="F53" s="11" t="inlineStr">
         <is>
-          <t>podlahova_plocha_1NP+2NP ~100 m²</t>
+          <t>klenba 1.PP/1.NP plocha ~50 m²</t>
         </is>
       </c>
       <c r="G53" s="11" t="inlineStr">
         <is>
-          <t>974041141</t>
+          <t>631321311</t>
         </is>
       </c>
       <c r="H53" s="10" t="inlineStr">
@@ -4236,12 +4232,12 @@
       </c>
       <c r="I53" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV4.010</t>
+          <t>260219_dum.HSV4.009</t>
         </is>
       </c>
       <c r="J53" s="11" t="inlineStr">
         <is>
-          <t>S07</t>
+          <t>S06</t>
         </is>
       </c>
       <c r="K53" s="11" t="inlineStr">
@@ -4261,7 +4257,7 @@
       </c>
       <c r="C54" s="11" t="inlineStr">
         <is>
-          <t>Tepelná izolace minerální vata mezi trámy stropu 1.NP/2.NP, tl. 180 mm (= trám 60/180)</t>
+          <t>Strop trámový 1.NP/2.NP — sejmutí podlah, demontáž záklopu a zásypu shora (zachovat prkenný záklop na trámech)</t>
         </is>
       </c>
       <c r="D54" s="10" t="inlineStr">
@@ -4272,13 +4268,14 @@
       <c r="E54" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="F54" s="11">
-        <f> plocha stropu</f>
-        <v/>
-      </c>
-      <c r="G54" s="13" t="inlineStr">
-        <is>
-          <t>713121121</t>
+      <c r="F54" s="11" t="inlineStr">
+        <is>
+          <t>podlahova_plocha_1NP+2NP ~100 m²</t>
+        </is>
+      </c>
+      <c r="G54" s="11" t="inlineStr">
+        <is>
+          <t>974041141</t>
         </is>
       </c>
       <c r="H54" s="10" t="inlineStr">
@@ -4288,7 +4285,7 @@
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV4.011</t>
+          <t>260219_dum.HSV4.010</t>
         </is>
       </c>
       <c r="J54" s="11" t="inlineStr">
@@ -4313,7 +4310,7 @@
       </c>
       <c r="C55" s="11" t="inlineStr">
         <is>
-          <t>Protipožární SDK podhled zespodu trámového stropu (EI 30 dle PBŘ)</t>
+          <t>Tepelná izolace minerální vata mezi trámy stropu 1.NP/2.NP, tl. 180 mm (= trám 60/180)</t>
         </is>
       </c>
       <c r="D55" s="10" t="inlineStr">
@@ -4328,9 +4325,9 @@
         <f> plocha stropu</f>
         <v/>
       </c>
-      <c r="G55" s="11" t="inlineStr">
-        <is>
-          <t>342213131</t>
+      <c r="G55" s="13" t="inlineStr">
+        <is>
+          <t>713121121</t>
         </is>
       </c>
       <c r="H55" s="10" t="inlineStr">
@@ -4340,7 +4337,7 @@
       </c>
       <c r="I55" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV4.012</t>
+          <t>260219_dum.HSV4.011</t>
         </is>
       </c>
       <c r="J55" s="11" t="inlineStr">
@@ -4365,25 +4362,24 @@
       </c>
       <c r="C56" s="11" t="inlineStr">
         <is>
-          <t>Suchá podlahová skladba 1.NP/2.NP — zásyp Liapor pro vyrovnání tl. 50 mm</t>
+          <t>Protipožární SDK podhled zespodu trámového stropu (EI 30 dle PBŘ)</t>
         </is>
       </c>
       <c r="D56" s="10" t="inlineStr">
         <is>
-          <t>m³</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E56" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="F56" s="11" t="inlineStr">
-        <is>
-          <t>100 m² × 0.05 m = 5</t>
-        </is>
+        <v>100</v>
+      </c>
+      <c r="F56" s="11">
+        <f> plocha stropu</f>
+        <v/>
       </c>
       <c r="G56" s="11" t="inlineStr">
         <is>
-          <t>631311114</t>
+          <t>342213131</t>
         </is>
       </c>
       <c r="H56" s="10" t="inlineStr">
@@ -4393,7 +4389,7 @@
       </c>
       <c r="I56" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV4.013</t>
+          <t>260219_dum.HSV4.012</t>
         </is>
       </c>
       <c r="J56" s="11" t="inlineStr">
@@ -4418,112 +4414,116 @@
       </c>
       <c r="C57" s="11" t="inlineStr">
         <is>
+          <t>Suchá podlahová skladba 1.NP/2.NP — zásyp Liapor pro vyrovnání tl. 50 mm</t>
+        </is>
+      </c>
+      <c r="D57" s="10" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="E57" s="12" t="n">
+        <v>5</v>
+      </c>
+      <c r="F57" s="11" t="inlineStr">
+        <is>
+          <t>100 m² × 0.05 m = 5</t>
+        </is>
+      </c>
+      <c r="G57" s="11" t="inlineStr">
+        <is>
+          <t>631311114</t>
+        </is>
+      </c>
+      <c r="H57" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I57" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV4.013</t>
+        </is>
+      </c>
+      <c r="J57" s="11" t="inlineStr">
+        <is>
+          <t>S07</t>
+        </is>
+      </c>
+      <c r="K57" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="10" t="n">
+        <v>53</v>
+      </c>
+      <c r="B58" s="11" t="inlineStr">
+        <is>
+          <t>HSV-4 Vodorovné</t>
+        </is>
+      </c>
+      <c r="C58" s="11" t="inlineStr">
+        <is>
           <t>Suchá podlahová skladba — sádrovláknité dílce Fermacell tl. 25 mm (dva 12.5 mm vrstvy)</t>
         </is>
       </c>
-      <c r="D57" s="10" t="inlineStr">
+      <c r="D58" s="10" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E57" s="12" t="n">
+      <c r="E58" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="F57" s="11">
+      <c r="F58" s="11">
         <f> plocha stropu</f>
         <v/>
       </c>
-      <c r="G57" s="11" t="inlineStr">
+      <c r="G58" s="11" t="inlineStr">
         <is>
           <t>771421111</t>
         </is>
       </c>
-      <c r="H57" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I57" s="11" t="inlineStr">
+      <c r="H58" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I58" s="11" t="inlineStr">
         <is>
           <t>260219_dum.HSV4.014</t>
         </is>
       </c>
-      <c r="J57" s="11" t="inlineStr">
+      <c r="J58" s="11" t="inlineStr">
         <is>
           <t>S07</t>
         </is>
       </c>
-      <c r="K57" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" s="8" t="inlineStr">
+      <c r="K58" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="8" t="inlineStr">
         <is>
           <t>━━ HSV-5 Krov + střecha  (16 atomic operací) ━━</t>
         </is>
       </c>
-      <c r="B58" s="9" t="n"/>
-      <c r="C58" s="9" t="n"/>
-      <c r="D58" s="9" t="n"/>
-      <c r="E58" s="9" t="n"/>
-      <c r="F58" s="9" t="n"/>
-      <c r="G58" s="9" t="n"/>
-      <c r="H58" s="9" t="n"/>
-      <c r="I58" s="9" t="n"/>
-      <c r="J58" s="9" t="n"/>
-      <c r="K58" s="9" t="n"/>
-    </row>
-    <row r="59">
-      <c r="A59" s="10" t="n">
-        <v>53</v>
-      </c>
-      <c r="B59" s="11" t="inlineStr">
-        <is>
-          <t>HSV-5 Krov + střecha</t>
-        </is>
-      </c>
-      <c r="C59" s="11" t="inlineStr">
-        <is>
-          <t>Tesařský krov — krokve 100/180 mm á 800 mm, rezivo C24 fungicidní + protihmyzí (cca 2×12 krokví × ~6.5 m)</t>
-        </is>
-      </c>
-      <c r="D59" s="10" t="inlineStr">
-        <is>
-          <t>bm</t>
-        </is>
-      </c>
-      <c r="E59" s="12" t="n">
-        <v>156</v>
-      </c>
-      <c r="F59" s="11" t="inlineStr">
-        <is>
-          <t>(2 sklony × 12 krokví × 6.5 m délka) = 156</t>
-        </is>
-      </c>
-      <c r="G59" s="13" t="inlineStr">
-        <is>
-          <t>762331911</t>
-        </is>
-      </c>
-      <c r="H59" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I59" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV5.001</t>
-        </is>
-      </c>
-      <c r="J59" s="11" t="inlineStr"/>
-      <c r="K59" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
+      <c r="B59" s="9" t="n"/>
+      <c r="C59" s="9" t="n"/>
+      <c r="D59" s="9" t="n"/>
+      <c r="E59" s="9" t="n"/>
+      <c r="F59" s="9" t="n"/>
+      <c r="G59" s="9" t="n"/>
+      <c r="H59" s="9" t="n"/>
+      <c r="I59" s="9" t="n"/>
+      <c r="J59" s="9" t="n"/>
+      <c r="K59" s="9" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="10" t="n">
@@ -4536,7 +4536,7 @@
       </c>
       <c r="C60" s="11" t="inlineStr">
         <is>
-          <t>Tesařský krov — kleštiny dvojfošny 60/180 mm probíhající v oblasti spací části</t>
+          <t>Tesařský krov — krokve 100/180 mm á 800 mm, rezivo C24 fungicidní + protihmyzí (cca 2×12 krokví × ~6.5 m)</t>
         </is>
       </c>
       <c r="D60" s="10" t="inlineStr">
@@ -4545,16 +4545,16 @@
         </is>
       </c>
       <c r="E60" s="12" t="n">
-        <v>110</v>
+        <v>156</v>
       </c>
       <c r="F60" s="11" t="inlineStr">
         <is>
-          <t>11 pozic × 2 ks × ~5 m délka = 110</t>
+          <t>(2 sklony × 12 krokví × 6.5 m délka) = 156</t>
         </is>
       </c>
       <c r="G60" s="13" t="inlineStr">
         <is>
-          <t>762331912</t>
+          <t>762331911</t>
         </is>
       </c>
       <c r="H60" s="10" t="inlineStr">
@@ -4564,7 +4564,7 @@
       </c>
       <c r="I60" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.002</t>
+          <t>260219_dum.HSV5.001</t>
         </is>
       </c>
       <c r="J60" s="11" t="inlineStr"/>
@@ -4585,7 +4585,7 @@
       </c>
       <c r="C61" s="11" t="inlineStr">
         <is>
-          <t>Tesařský krov — pozednice 140/160 mm kotvená do ŽB věnce 3.NP</t>
+          <t>Tesařský krov — kleštiny dvojfošny 60/180 mm probíhající v oblasti spací části</t>
         </is>
       </c>
       <c r="D61" s="10" t="inlineStr">
@@ -4594,16 +4594,16 @@
         </is>
       </c>
       <c r="E61" s="12" t="n">
-        <v>19.4</v>
+        <v>110</v>
       </c>
       <c r="F61" s="11" t="inlineStr">
         <is>
-          <t>polovina obvodu (2 dlouhé strany) = ~20</t>
+          <t>11 pozic × 2 ks × ~5 m délka = 110</t>
         </is>
       </c>
       <c r="G61" s="13" t="inlineStr">
         <is>
-          <t>762331923</t>
+          <t>762331912</t>
         </is>
       </c>
       <c r="H61" s="10" t="inlineStr">
@@ -4613,7 +4613,7 @@
       </c>
       <c r="I61" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.003</t>
+          <t>260219_dum.HSV5.002</t>
         </is>
       </c>
       <c r="J61" s="11" t="inlineStr"/>
@@ -4634,7 +4634,7 @@
       </c>
       <c r="C62" s="11" t="inlineStr">
         <is>
-          <t>Tesařský krov — námětky 60/100 v dolní koncové části pro přesah střechy ~500 mm</t>
+          <t>Tesařský krov — pozednice 140/160 mm kotvená do ŽB věnce 3.NP</t>
         </is>
       </c>
       <c r="D62" s="10" t="inlineStr">
@@ -4643,16 +4643,16 @@
         </is>
       </c>
       <c r="E62" s="12" t="n">
-        <v>19.2</v>
+        <v>19.4</v>
       </c>
       <c r="F62" s="11" t="inlineStr">
         <is>
-          <t>24 krokví × 0.8 m námětek = 19.2</t>
-        </is>
-      </c>
-      <c r="G62" s="11" t="inlineStr">
-        <is>
-          <t>762331911</t>
+          <t>polovina obvodu (2 dlouhé strany) = ~20</t>
+        </is>
+      </c>
+      <c r="G62" s="13" t="inlineStr">
+        <is>
+          <t>762331923</t>
         </is>
       </c>
       <c r="H62" s="10" t="inlineStr">
@@ -4662,7 +4662,7 @@
       </c>
       <c r="I62" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.004</t>
+          <t>260219_dum.HSV5.003</t>
         </is>
       </c>
       <c r="J62" s="11" t="inlineStr"/>
@@ -4683,25 +4683,25 @@
       </c>
       <c r="C63" s="11" t="inlineStr">
         <is>
-          <t>Ocelová středová vaznice HEA160 — 2 ks × cca 10 m délka</t>
+          <t>Tesařský krov — námětky 60/100 v dolní koncové části pro přesah střechy ~500 mm</t>
         </is>
       </c>
       <c r="D63" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>bm</t>
         </is>
       </c>
       <c r="E63" s="12" t="n">
-        <v>608</v>
+        <v>19.2</v>
       </c>
       <c r="F63" s="11" t="inlineStr">
         <is>
-          <t>2 × 10 × 30.4 kg/m (HEA160) = 608</t>
-        </is>
-      </c>
-      <c r="G63" s="13" t="inlineStr">
-        <is>
-          <t>411321414</t>
+          <t>24 krokví × 0.8 m námětek = 19.2</t>
+        </is>
+      </c>
+      <c r="G63" s="11" t="inlineStr">
+        <is>
+          <t>762331911</t>
         </is>
       </c>
       <c r="H63" s="10" t="inlineStr">
@@ -4711,7 +4711,7 @@
       </c>
       <c r="I63" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.005</t>
+          <t>260219_dum.HSV5.004</t>
         </is>
       </c>
       <c r="J63" s="11" t="inlineStr"/>
@@ -4732,7 +4732,7 @@
       </c>
       <c r="C64" s="11" t="inlineStr">
         <is>
-          <t>Ocelové sloupky uzavřený profil 100×100×4 mm pod vaznice HEA160 (~6 ks × ~2.5 m výška)</t>
+          <t>Ocelová středová vaznice HEA160 — 2 ks × cca 10 m délka</t>
         </is>
       </c>
       <c r="D64" s="10" t="inlineStr">
@@ -4741,14 +4741,14 @@
         </is>
       </c>
       <c r="E64" s="12" t="n">
-        <v>176</v>
+        <v>608</v>
       </c>
       <c r="F64" s="11" t="inlineStr">
         <is>
-          <t>6 × 2.5 × 11.7 kg/m (RHS 100×100×4) = 176</t>
-        </is>
-      </c>
-      <c r="G64" s="11" t="inlineStr">
+          <t>2 × 10 × 30.4 kg/m (HEA160) = 608</t>
+        </is>
+      </c>
+      <c r="G64" s="13" t="inlineStr">
         <is>
           <t>411321414</t>
         </is>
@@ -4760,7 +4760,7 @@
       </c>
       <c r="I64" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.006</t>
+          <t>260219_dum.HSV5.005</t>
         </is>
       </c>
       <c r="J64" s="11" t="inlineStr"/>
@@ -4781,24 +4781,25 @@
       </c>
       <c r="C65" s="11" t="inlineStr">
         <is>
-          <t>Bednění z prken tl. 20 mm pod nadkrokevní PIR (biodeska/palubka)</t>
+          <t>Ocelové sloupky uzavřený profil 100×100×4 mm pod vaznice HEA160 (~6 ks × ~2.5 m výška)</t>
         </is>
       </c>
       <c r="D65" s="10" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E65" s="12" t="n">
-        <v>140.94</v>
-      </c>
-      <c r="F65" s="11">
-        <f> 141 m² (plocha střechy včetně sklonu + přesahy)</f>
-        <v/>
+        <v>176</v>
+      </c>
+      <c r="F65" s="11" t="inlineStr">
+        <is>
+          <t>6 × 2.5 × 11.7 kg/m (RHS 100×100×4) = 176</t>
+        </is>
       </c>
       <c r="G65" s="11" t="inlineStr">
         <is>
-          <t>762341711</t>
+          <t>411321414</t>
         </is>
       </c>
       <c r="H65" s="10" t="inlineStr">
@@ -4808,14 +4809,10 @@
       </c>
       <c r="I65" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.007</t>
-        </is>
-      </c>
-      <c r="J65" s="11" t="inlineStr">
-        <is>
-          <t>S10</t>
-        </is>
-      </c>
+          <t>260219_dum.HSV5.006</t>
+        </is>
+      </c>
+      <c r="J65" s="11" t="inlineStr"/>
       <c r="K65" s="11" t="inlineStr">
         <is>
           <t>Carried 1:1 (atomic — no decomposition needed)</t>
@@ -4833,7 +4830,7 @@
       </c>
       <c r="C66" s="11" t="inlineStr">
         <is>
-          <t>Parotěsná folie nad bedněním pod nadkrokevní PIR (např. Isover Vario nebo Tyvek Air guard)</t>
+          <t>Bednění z prken tl. 20 mm pod nadkrokevní PIR (biodeska/palubka)</t>
         </is>
       </c>
       <c r="D66" s="10" t="inlineStr">
@@ -4842,16 +4839,15 @@
         </is>
       </c>
       <c r="E66" s="12" t="n">
-        <v>155.034</v>
-      </c>
-      <c r="F66" s="11" t="inlineStr">
-        <is>
-          <t>141 × 1.1 přesah = 155</t>
-        </is>
+        <v>140.94</v>
+      </c>
+      <c r="F66" s="11">
+        <f> 141 m² (plocha střechy včetně sklonu + přesahy)</f>
+        <v/>
       </c>
       <c r="G66" s="11" t="inlineStr">
         <is>
-          <t>712311101</t>
+          <t>762341711</t>
         </is>
       </c>
       <c r="H66" s="10" t="inlineStr">
@@ -4861,7 +4857,7 @@
       </c>
       <c r="I66" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.008</t>
+          <t>260219_dum.HSV5.007</t>
         </is>
       </c>
       <c r="J66" s="11" t="inlineStr">
@@ -4886,7 +4882,7 @@
       </c>
       <c r="C67" s="11" t="inlineStr">
         <is>
-          <t>Nadkrokevní tepelná izolace PIR (polyisokyanurát) tl. 160 mm (λ=0,022 W/mK) — řez A-A S10 explicit</t>
+          <t>Parotěsná folie nad bedněním pod nadkrokevní PIR (např. Isover Vario nebo Tyvek Air guard)</t>
         </is>
       </c>
       <c r="D67" s="10" t="inlineStr">
@@ -4895,25 +4891,26 @@
         </is>
       </c>
       <c r="E67" s="12" t="n">
-        <v>140.94</v>
-      </c>
-      <c r="F67" s="11">
-        <f> 141 m² (plocha krytiny krov)</f>
-        <v/>
-      </c>
-      <c r="G67" s="13" t="inlineStr">
-        <is>
-          <t>713131811</t>
+        <v>155.034</v>
+      </c>
+      <c r="F67" s="11" t="inlineStr">
+        <is>
+          <t>141 × 1.1 přesah = 155</t>
+        </is>
+      </c>
+      <c r="G67" s="11" t="inlineStr">
+        <is>
+          <t>712311101</t>
         </is>
       </c>
       <c r="H67" s="10" t="inlineStr">
         <is>
-          <t>✓ verified</t>
+          <t>⚠ kandidát-verify</t>
         </is>
       </c>
       <c r="I67" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.009</t>
+          <t>260219_dum.HSV5.008</t>
         </is>
       </c>
       <c r="J67" s="11" t="inlineStr">
@@ -4938,7 +4935,7 @@
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>Doplňková hydroizolační difuzně otevřená folie nad PIR pod kontralatě</t>
+          <t>Nadkrokevní tepelná izolace PIR (polyisokyanurát) tl. 160 mm (λ=0,022 W/mK) — řez A-A S10 explicit</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr">
@@ -4947,26 +4944,25 @@
         </is>
       </c>
       <c r="E68" s="12" t="n">
-        <v>155.034</v>
-      </c>
-      <c r="F68" s="11" t="inlineStr">
-        <is>
-          <t>141 × 1.1 přesah = 155</t>
-        </is>
-      </c>
-      <c r="G68" s="11" t="inlineStr">
-        <is>
-          <t>712311111</t>
+        <v>140.94</v>
+      </c>
+      <c r="F68" s="11">
+        <f> 141 m² (plocha krytiny krov)</f>
+        <v/>
+      </c>
+      <c r="G68" s="13" t="inlineStr">
+        <is>
+          <t>713131811</t>
         </is>
       </c>
       <c r="H68" s="10" t="inlineStr">
         <is>
-          <t>⚠ kandidát-verify</t>
+          <t>✓ verified</t>
         </is>
       </c>
       <c r="I68" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.010</t>
+          <t>260219_dum.HSV5.009</t>
         </is>
       </c>
       <c r="J68" s="11" t="inlineStr">
@@ -4991,7 +4987,7 @@
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>Distanční kontralatě 40×60 mm pro vzduchovou mezeru nad PIR</t>
+          <t>Doplňková hydroizolační difuzně otevřená folie nad PIR pod kontralatě</t>
         </is>
       </c>
       <c r="D69" s="10" t="inlineStr">
@@ -5000,15 +4996,16 @@
         </is>
       </c>
       <c r="E69" s="12" t="n">
-        <v>140.94</v>
-      </c>
-      <c r="F69" s="11">
-        <f> 141 m²</f>
-        <v/>
+        <v>155.034</v>
+      </c>
+      <c r="F69" s="11" t="inlineStr">
+        <is>
+          <t>141 × 1.1 přesah = 155</t>
+        </is>
       </c>
       <c r="G69" s="11" t="inlineStr">
         <is>
-          <t>762331923</t>
+          <t>712311111</t>
         </is>
       </c>
       <c r="H69" s="10" t="inlineStr">
@@ -5018,7 +5015,7 @@
       </c>
       <c r="I69" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.011</t>
+          <t>260219_dum.HSV5.010</t>
         </is>
       </c>
       <c r="J69" s="11" t="inlineStr">
@@ -5043,7 +5040,7 @@
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>Bednění z prken tl. 25 mm pod plechovou hliníkovou krytinu (rozsah dle technologie krytiny)</t>
+          <t>Distanční kontralatě 40×60 mm pro vzduchovou mezeru nad PIR</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
@@ -5058,9 +5055,9 @@
         <f> 141 m²</f>
         <v/>
       </c>
-      <c r="G70" s="13" t="inlineStr">
-        <is>
-          <t>762341711</t>
+      <c r="G70" s="11" t="inlineStr">
+        <is>
+          <t>762331923</t>
         </is>
       </c>
       <c r="H70" s="10" t="inlineStr">
@@ -5070,7 +5067,7 @@
       </c>
       <c r="I70" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.012</t>
+          <t>260219_dum.HSV5.011</t>
         </is>
       </c>
       <c r="J70" s="11" t="inlineStr">
@@ -5095,7 +5092,7 @@
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>Plechová falcovaná HLINÍKOVÁ krytina (např. PREFA, Rheinzink, Lindab) + tlumící podložka</t>
+          <t>Bednění z prken tl. 25 mm pod plechovou hliníkovou krytinu (rozsah dle technologie krytiny)</t>
         </is>
       </c>
       <c r="D71" s="10" t="inlineStr">
@@ -5107,12 +5104,12 @@
         <v>140.94</v>
       </c>
       <c r="F71" s="11">
-        <f> 141 m² (vč. vikýřů přidat ~10%)</f>
+        <f> 141 m²</f>
         <v/>
       </c>
       <c r="G71" s="13" t="inlineStr">
         <is>
-          <t>765791121</t>
+          <t>762341711</t>
         </is>
       </c>
       <c r="H71" s="10" t="inlineStr">
@@ -5122,7 +5119,7 @@
       </c>
       <c r="I71" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.013</t>
+          <t>260219_dum.HSV5.012</t>
         </is>
       </c>
       <c r="J71" s="11" t="inlineStr">
@@ -5147,7 +5144,7 @@
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>Patro pro přespání v krovu — biodeska / OSB desky tl. 22 mm nad kleštinami</t>
+          <t>Plechová falcovaná HLINÍKOVÁ krytina (např. PREFA, Rheinzink, Lindab) + tlumící podložka</t>
         </is>
       </c>
       <c r="D72" s="10" t="inlineStr">
@@ -5156,16 +5153,15 @@
         </is>
       </c>
       <c r="E72" s="12" t="n">
-        <v>25</v>
-      </c>
-      <c r="F72" s="11" t="inlineStr">
-        <is>
-          <t>odhad — spací patro ~5 × 5 m</t>
-        </is>
-      </c>
-      <c r="G72" s="11" t="inlineStr">
-        <is>
-          <t>762341711</t>
+        <v>140.94</v>
+      </c>
+      <c r="F72" s="11">
+        <f> 141 m² (vč. vikýřů přidat ~10%)</f>
+        <v/>
+      </c>
+      <c r="G72" s="13" t="inlineStr">
+        <is>
+          <t>765791121</t>
         </is>
       </c>
       <c r="H72" s="10" t="inlineStr">
@@ -5175,12 +5171,12 @@
       </c>
       <c r="I72" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.014</t>
+          <t>260219_dum.HSV5.013</t>
         </is>
       </c>
       <c r="J72" s="11" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="K72" s="11" t="inlineStr">
@@ -5200,7 +5196,7 @@
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>Vikýře — zděná čela z Porotherm 30 (odhad 4 ks × ~3 m² stěna)</t>
+          <t>Patro pro přespání v krovu — biodeska / OSB desky tl. 22 mm nad kleštinami</t>
         </is>
       </c>
       <c r="D73" s="10" t="inlineStr">
@@ -5209,16 +5205,16 @@
         </is>
       </c>
       <c r="E73" s="12" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="F73" s="11" t="inlineStr">
         <is>
-          <t>4 vikýře × ~3 m² zděných čel = 12</t>
+          <t>odhad — spací patro ~5 × 5 m</t>
         </is>
       </c>
       <c r="G73" s="11" t="inlineStr">
         <is>
-          <t>311321411</t>
+          <t>762341711</t>
         </is>
       </c>
       <c r="H73" s="10" t="inlineStr">
@@ -5228,10 +5224,14 @@
       </c>
       <c r="I73" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.015</t>
-        </is>
-      </c>
-      <c r="J73" s="11" t="inlineStr"/>
+          <t>260219_dum.HSV5.014</t>
+        </is>
+      </c>
+      <c r="J73" s="11" t="inlineStr">
+        <is>
+          <t>S11</t>
+        </is>
+      </c>
       <c r="K73" s="11" t="inlineStr">
         <is>
           <t>Carried 1:1 (atomic — no decomposition needed)</t>
@@ -5249,204 +5249,204 @@
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
+          <t>Vikýře — zděná čela z Porotherm 30 (odhad 4 ks × ~3 m² stěna)</t>
+        </is>
+      </c>
+      <c r="D74" s="10" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E74" s="12" t="n">
+        <v>12</v>
+      </c>
+      <c r="F74" s="11" t="inlineStr">
+        <is>
+          <t>4 vikýře × ~3 m² zděných čel = 12</t>
+        </is>
+      </c>
+      <c r="G74" s="11" t="inlineStr">
+        <is>
+          <t>311321411</t>
+        </is>
+      </c>
+      <c r="H74" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I74" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV5.015</t>
+        </is>
+      </c>
+      <c r="J74" s="11" t="inlineStr"/>
+      <c r="K74" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="10" t="n">
+        <v>69</v>
+      </c>
+      <c r="B75" s="11" t="inlineStr">
+        <is>
+          <t>HSV-5 Krov + střecha</t>
+        </is>
+      </c>
+      <c r="C75" s="11" t="inlineStr">
+        <is>
           <t>Vikýře — provětrávaná fasáda min. vata + plech falcovaný hliník (4 vikýře × ~6 m² fasády)</t>
         </is>
       </c>
-      <c r="D74" s="10" t="inlineStr">
+      <c r="D75" s="10" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E74" s="12" t="n">
+      <c r="E75" s="12" t="n">
         <v>24</v>
       </c>
-      <c r="F74" s="11" t="inlineStr">
+      <c r="F75" s="11" t="inlineStr">
         <is>
           <t>4 vikýře × 2 strany × ~3 m² = 24</t>
         </is>
       </c>
-      <c r="G74" s="11" t="inlineStr">
+      <c r="G75" s="11" t="inlineStr">
         <is>
           <t>765791121</t>
         </is>
       </c>
-      <c r="H74" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I74" s="11" t="inlineStr">
+      <c r="H75" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I75" s="11" t="inlineStr">
         <is>
           <t>260219_dum.HSV5.016</t>
         </is>
       </c>
-      <c r="J74" s="11" t="inlineStr">
+      <c r="J75" s="11" t="inlineStr">
         <is>
           <t>S12b</t>
         </is>
       </c>
-      <c r="K74" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="75">
-      <c r="A75" s="8" t="inlineStr">
+      <c r="K75" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="8" t="inlineStr">
         <is>
           <t>━━ HSV-6 Bourací práce  (17 atomic operací) ━━</t>
         </is>
       </c>
-      <c r="B75" s="9" t="n"/>
-      <c r="C75" s="9" t="n"/>
-      <c r="D75" s="9" t="n"/>
-      <c r="E75" s="9" t="n"/>
-      <c r="F75" s="9" t="n"/>
-      <c r="G75" s="9" t="n"/>
-      <c r="H75" s="9" t="n"/>
-      <c r="I75" s="9" t="n"/>
-      <c r="J75" s="9" t="n"/>
-      <c r="K75" s="9" t="n"/>
-    </row>
-    <row r="76">
-      <c r="A76" s="10" t="n">
-        <v>69</v>
-      </c>
-      <c r="B76" s="11" t="inlineStr">
+      <c r="B76" s="9" t="n"/>
+      <c r="C76" s="9" t="n"/>
+      <c r="D76" s="9" t="n"/>
+      <c r="E76" s="9" t="n"/>
+      <c r="F76" s="9" t="n"/>
+      <c r="G76" s="9" t="n"/>
+      <c r="H76" s="9" t="n"/>
+      <c r="I76" s="9" t="n"/>
+      <c r="J76" s="9" t="n"/>
+      <c r="K76" s="9" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="B77" s="11" t="inlineStr">
         <is>
           <t>HSV-6 Bourací práce</t>
         </is>
       </c>
-      <c r="C76" s="11" t="inlineStr">
+      <c r="C77" s="11" t="inlineStr">
         <is>
           <t>Bourání kompletního stávajícího krovu vč. vikýřů — vaznicový s ležatou stolicí — manuálně, odvoz</t>
         </is>
       </c>
-      <c r="D76" s="10" t="inlineStr">
+      <c r="D77" s="10" t="inlineStr">
         <is>
           <t>m³</t>
         </is>
       </c>
-      <c r="E76" s="12" t="n">
+      <c r="E77" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="F76" s="11" t="inlineStr">
+      <c r="F77" s="11" t="inlineStr">
         <is>
           <t>TZ B m.10.e: 9 t dřeva × 0.75 t/m³ = 12 m³ dřeva</t>
         </is>
       </c>
-      <c r="G76" s="13" t="inlineStr">
+      <c r="G77" s="13" t="inlineStr">
         <is>
           <t>962041141</t>
         </is>
       </c>
-      <c r="H76" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I76" s="11" t="inlineStr">
+      <c r="H77" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I77" s="11" t="inlineStr">
         <is>
           <t>260219_dum.HSV6.001</t>
         </is>
       </c>
-      <c r="J76" s="11" t="inlineStr"/>
-      <c r="K76" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" s="17" t="n">
-        <v>70</v>
-      </c>
-      <c r="B77" s="18" t="inlineStr">
+      <c r="J77" s="11" t="inlineStr"/>
+      <c r="K77" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="17" t="n">
+        <v>71</v>
+      </c>
+      <c r="B78" s="18" t="inlineStr">
         <is>
           <t>HSV-6 Bourací práce</t>
         </is>
       </c>
-      <c r="C77" s="18" t="inlineStr">
+      <c r="C78" s="18" t="inlineStr">
         <is>
           <t>Bourání stávající plechové krytiny (manuálně, recyklace plechu)</t>
         </is>
       </c>
-      <c r="D77" s="17" t="inlineStr">
+      <c r="D78" s="17" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E77" s="19" t="n">
+      <c r="E78" s="19" t="n">
         <v>140.9</v>
       </c>
-      <c r="F77" s="18">
+      <c r="F78" s="18">
         <f> plocha krytiny ~141</f>
         <v/>
       </c>
-      <c r="G77" s="18" t="inlineStr"/>
-      <c r="H77" s="17" t="inlineStr">
+      <c r="G78" s="18" t="inlineStr"/>
+      <c r="H78" s="17" t="inlineStr">
         <is>
           <t>❌ blank — ÚRS online</t>
         </is>
       </c>
-      <c r="I77" s="18" t="inlineStr">
+      <c r="I78" s="18" t="inlineStr">
         <is>
           <t>260219_dum.HSV6.002</t>
         </is>
       </c>
-      <c r="J77" s="18" t="inlineStr"/>
-      <c r="K77" s="18" t="inlineStr">
+      <c r="J78" s="18" t="inlineStr"/>
+      <c r="K78" s="18" t="inlineStr">
         <is>
           <t>Carried 1:1 (atomic — no decomposition needed)  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="10" t="n">
-        <v>71</v>
-      </c>
-      <c r="B78" s="11" t="inlineStr">
-        <is>
-          <t>HSV-6 Bourací práce</t>
-        </is>
-      </c>
-      <c r="C78" s="11" t="inlineStr">
-        <is>
-          <t>Bourání zděných nadezdívek nad stropem 2.NP (mimo štítových stěn) — cihla pálená</t>
-        </is>
-      </c>
-      <c r="D78" s="10" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="E78" s="12" t="n">
-        <v>6</v>
-      </c>
-      <c r="F78" s="11" t="inlineStr">
-        <is>
-          <t>odhad — 3.NP nadezdívka půdy ~104 m² × 0.45 m výška ~6</t>
-        </is>
-      </c>
-      <c r="G78" s="11" t="inlineStr">
-        <is>
-          <t>962031132</t>
-        </is>
-      </c>
-      <c r="H78" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I78" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV6.003</t>
-        </is>
-      </c>
-      <c r="J78" s="11" t="inlineStr"/>
-      <c r="K78" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
         </is>
       </c>
     </row>
@@ -5461,24 +5461,25 @@
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>Bourání trámového stropu 2.NP/podkroví — kompletně (vč. zajištění schodiště)</t>
+          <t>Bourání zděných nadezdívek nad stropem 2.NP (mimo štítových stěn) — cihla pálená</t>
         </is>
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="E79" s="12" t="n">
-        <v>104.4</v>
-      </c>
-      <c r="F79" s="11">
-        <f> zastavěna 104.4 m²</f>
-        <v/>
+        <v>6</v>
+      </c>
+      <c r="F79" s="11" t="inlineStr">
+        <is>
+          <t>odhad — 3.NP nadezdívka půdy ~104 m² × 0.45 m výška ~6</t>
+        </is>
       </c>
       <c r="G79" s="11" t="inlineStr">
         <is>
-          <t>962041141</t>
+          <t>962031132</t>
         </is>
       </c>
       <c r="H79" s="10" t="inlineStr">
@@ -5488,7 +5489,7 @@
       </c>
       <c r="I79" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.004</t>
+          <t>260219_dum.HSV6.003</t>
         </is>
       </c>
       <c r="J79" s="11" t="inlineStr"/>
@@ -5509,7 +5510,7 @@
       </c>
       <c r="C80" s="11" t="inlineStr">
         <is>
-          <t>Bourání stávajících lehkých příček (cihla, sádrokarton, dřevo)</t>
+          <t>Bourání trámového stropu 2.NP/podkroví — kompletně (vč. zajištění schodiště)</t>
         </is>
       </c>
       <c r="D80" s="10" t="inlineStr">
@@ -5518,16 +5519,15 @@
         </is>
       </c>
       <c r="E80" s="12" t="n">
-        <v>80</v>
-      </c>
-      <c r="F80" s="11" t="inlineStr">
-        <is>
-          <t>odhad — interier 2 patra × ~40 m² příček = 80</t>
-        </is>
+        <v>104.4</v>
+      </c>
+      <c r="F80" s="11">
+        <f> zastavěna 104.4 m²</f>
+        <v/>
       </c>
       <c r="G80" s="11" t="inlineStr">
         <is>
-          <t>962031132</t>
+          <t>962041141</t>
         </is>
       </c>
       <c r="H80" s="10" t="inlineStr">
@@ -5537,7 +5537,7 @@
       </c>
       <c r="I80" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.005</t>
+          <t>260219_dum.HSV6.004</t>
         </is>
       </c>
       <c r="J80" s="11" t="inlineStr"/>
@@ -5558,20 +5558,20 @@
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>Bourání 8 nových otvorů v nosných cihelných zdech pro dveře/okna (~1.0 × 2.1 m)</t>
+          <t>Bourání stávajících lehkých příček (cihla, sádrokarton, dřevo)</t>
         </is>
       </c>
       <c r="D81" s="10" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E81" s="12" t="n">
-        <v>8</v>
+        <v>80</v>
       </c>
       <c r="F81" s="11" t="inlineStr">
         <is>
-          <t>odhad počtu nových otvorů (= počet IPN160 překladů)</t>
+          <t>odhad — interier 2 patra × ~40 m² příček = 80</t>
         </is>
       </c>
       <c r="G81" s="11" t="inlineStr">
@@ -5586,7 +5586,7 @@
       </c>
       <c r="I81" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.006</t>
+          <t>260219_dum.HSV6.005</t>
         </is>
       </c>
       <c r="J81" s="11" t="inlineStr"/>
@@ -5607,25 +5607,25 @@
       </c>
       <c r="C82" s="11" t="inlineStr">
         <is>
-          <t>Bourání keramických obkladů a zařizovacích předmětů v koupelnách 1.NP + 2.NP</t>
+          <t>Bourání 8 nových otvorů v nosných cihelných zdech pro dveře/okna (~1.0 × 2.1 m)</t>
         </is>
       </c>
       <c r="D82" s="10" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>ks</t>
         </is>
       </c>
       <c r="E82" s="12" t="n">
-        <v>60</v>
+        <v>8</v>
       </c>
       <c r="F82" s="11" t="inlineStr">
         <is>
-          <t>2 koupelny × ~30 m² obkladů = 60</t>
-        </is>
-      </c>
-      <c r="G82" s="13" t="inlineStr">
-        <is>
-          <t>781473810</t>
+          <t>odhad počtu nových otvorů (= počet IPN160 překladů)</t>
+        </is>
+      </c>
+      <c r="G82" s="11" t="inlineStr">
+        <is>
+          <t>962031132</t>
         </is>
       </c>
       <c r="H82" s="10" t="inlineStr">
@@ -5635,7 +5635,7 @@
       </c>
       <c r="I82" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.007</t>
+          <t>260219_dum.HSV6.006</t>
         </is>
       </c>
       <c r="J82" s="11" t="inlineStr"/>
@@ -5656,7 +5656,7 @@
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>Sejmutí podlah 1.NP a 2.NP — vč. nášlapů, podkladních vrstev</t>
+          <t>Bourání keramických obkladů a zařizovacích předmětů v koupelnách 1.NP + 2.NP</t>
         </is>
       </c>
       <c r="D83" s="10" t="inlineStr">
@@ -5665,16 +5665,16 @@
         </is>
       </c>
       <c r="E83" s="12" t="n">
-        <v>153.51</v>
+        <v>60</v>
       </c>
       <c r="F83" s="11" t="inlineStr">
         <is>
-          <t>podlahova × 0.7 = ~154 m² (bez 3.NP nového)</t>
-        </is>
-      </c>
-      <c r="G83" s="11" t="inlineStr">
-        <is>
-          <t>974031132</t>
+          <t>2 koupelny × ~30 m² obkladů = 60</t>
+        </is>
+      </c>
+      <c r="G83" s="13" t="inlineStr">
+        <is>
+          <t>781473810</t>
         </is>
       </c>
       <c r="H83" s="10" t="inlineStr">
@@ -5684,7 +5684,7 @@
       </c>
       <c r="I83" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.008</t>
+          <t>260219_dum.HSV6.007</t>
         </is>
       </c>
       <c r="J83" s="11" t="inlineStr"/>
@@ -5705,25 +5705,25 @@
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>Demontáž záklopu a zásypů stropu 1.NP (prkenný záklop na trámech zachován)</t>
+          <t>Sejmutí podlah 1.NP a 2.NP — vč. nášlapů, podkladních vrstev</t>
         </is>
       </c>
       <c r="D84" s="10" t="inlineStr">
         <is>
-          <t>m³</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E84" s="12" t="n">
-        <v>5</v>
+        <v>153.51</v>
       </c>
       <c r="F84" s="11" t="inlineStr">
         <is>
-          <t>100 m² × 0.05 m tl. zásypu = 5</t>
+          <t>podlahova × 0.7 = ~154 m² (bez 3.NP nového)</t>
         </is>
       </c>
       <c r="G84" s="11" t="inlineStr">
         <is>
-          <t>974041151</t>
+          <t>974031132</t>
         </is>
       </c>
       <c r="H84" s="10" t="inlineStr">
@@ -5733,7 +5733,7 @@
       </c>
       <c r="I84" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.009</t>
+          <t>260219_dum.HSV6.008</t>
         </is>
       </c>
       <c r="J84" s="11" t="inlineStr"/>
@@ -5754,25 +5754,25 @@
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Demontáž všech oken a dveří stávajících (recyklace)</t>
+          <t>Demontáž záklopu a zásypů stropu 1.NP (prkenný záklop na trámech zachován)</t>
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="E85" s="12" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="F85" s="11" t="inlineStr">
         <is>
-          <t>odhad — ~10 oken + ~15 dveří (vstupní + vnitřní)</t>
+          <t>100 m² × 0.05 m tl. zásypu = 5</t>
         </is>
       </c>
       <c r="G85" s="11" t="inlineStr">
         <is>
-          <t>968071120</t>
+          <t>974041151</t>
         </is>
       </c>
       <c r="H85" s="10" t="inlineStr">
@@ -5782,7 +5782,7 @@
       </c>
       <c r="I85" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.010</t>
+          <t>260219_dum.HSV6.009</t>
         </is>
       </c>
       <c r="J85" s="11" t="inlineStr"/>
@@ -5803,7 +5803,7 @@
       </c>
       <c r="C86" s="11" t="inlineStr">
         <is>
-          <t>Demontáž všech sanitárních zařizovacích předmětů (WC, umyvadla, baterie, sprcha)</t>
+          <t>Demontáž všech oken a dveří stávajících (recyklace)</t>
         </is>
       </c>
       <c r="D86" s="10" t="inlineStr">
@@ -5812,16 +5812,16 @@
         </is>
       </c>
       <c r="E86" s="12" t="n">
-        <v>12</v>
+        <v>25</v>
       </c>
       <c r="F86" s="11" t="inlineStr">
         <is>
-          <t>odhad — 2 koupelny × ~5 ks + WC + dřez = ~12</t>
+          <t>odhad — ~10 oken + ~15 dveří (vstupní + vnitřní)</t>
         </is>
       </c>
       <c r="G86" s="11" t="inlineStr">
         <is>
-          <t>725900001</t>
+          <t>968071120</t>
         </is>
       </c>
       <c r="H86" s="10" t="inlineStr">
@@ -5831,7 +5831,7 @@
       </c>
       <c r="I86" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.011</t>
+          <t>260219_dum.HSV6.010</t>
         </is>
       </c>
       <c r="J86" s="11" t="inlineStr"/>
@@ -5852,25 +5852,25 @@
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>Odvoz a likvidace stavební suti dle vyhl. 8/2021 Sb. — celková tonáž odpadů</t>
+          <t>Demontáž všech sanitárních zařizovacích předmětů (WC, umyvadla, baterie, sprcha)</t>
         </is>
       </c>
       <c r="D87" s="10" t="inlineStr">
         <is>
-          <t>t</t>
+          <t>ks</t>
         </is>
       </c>
       <c r="E87" s="12" t="n">
-        <v>56.5</v>
+        <v>12</v>
       </c>
       <c r="F87" s="11" t="inlineStr">
         <is>
-          <t>TZ B m.10.e: 46 (beton/cihly) + 9 (dřevo) + 0.1 (kov) + 0.1 (EPS) + 0.2 (sádra) + 1.0 (směs) = 56.4</t>
+          <t>odhad — 2 koupelny × ~5 ks + WC + dřez = ~12</t>
         </is>
       </c>
       <c r="G87" s="11" t="inlineStr">
         <is>
-          <t>997013501</t>
+          <t>725900001</t>
         </is>
       </c>
       <c r="H87" s="10" t="inlineStr">
@@ -5880,7 +5880,7 @@
       </c>
       <c r="I87" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.012</t>
+          <t>260219_dum.HSV6.011</t>
         </is>
       </c>
       <c r="J87" s="11" t="inlineStr"/>
@@ -5901,35 +5901,35 @@
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
-          <t>Demontáž stávajících dřevěných oken vč. rámů a parapetů — 16 ks (návrh všechna okna nová plastová trojsklem)</t>
+          <t>Odvoz a likvidace stavební suti dle vyhl. 8/2021 Sb. — celková tonáž odpadů</t>
         </is>
       </c>
       <c r="D88" s="10" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>t</t>
         </is>
       </c>
       <c r="E88" s="12" t="n">
-        <v>16</v>
+        <v>56.5</v>
       </c>
       <c r="F88" s="11" t="inlineStr">
         <is>
-          <t>DXF INSERT okno* total 16 ks (Path C Tier 4 — front 9 + back 7)</t>
-        </is>
-      </c>
-      <c r="G88" s="13" t="inlineStr">
-        <is>
-          <t>978013181</t>
+          <t>TZ B m.10.e: 46 (beton/cihly) + 9 (dřevo) + 0.1 (kov) + 0.1 (EPS) + 0.2 (sádra) + 1.0 (směs) = 56.4</t>
+        </is>
+      </c>
+      <c r="G88" s="11" t="inlineStr">
+        <is>
+          <t>997013501</t>
         </is>
       </c>
       <c r="H88" s="10" t="inlineStr">
         <is>
-          <t>✓ verified</t>
+          <t>⚠ kandidát-verify</t>
         </is>
       </c>
       <c r="I88" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.013</t>
+          <t>260219_dum.HSV6.012</t>
         </is>
       </c>
       <c r="J88" s="11" t="inlineStr"/>
@@ -5950,7 +5950,7 @@
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>Demontáž stávajících vstupních dveří + rámů — 2 ks (1× ulice Fibichova + 1× zahrada; návrh nové plastové vstupní dveře)</t>
+          <t>Demontáž stávajících dřevěných oken vč. rámů a parapetů — 16 ks (návrh všechna okna nová plastová trojsklem)</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr">
@@ -5959,11 +5959,11 @@
         </is>
       </c>
       <c r="E89" s="12" t="n">
-        <v>2</v>
+        <v>16</v>
       </c>
       <c r="F89" s="11" t="inlineStr">
         <is>
-          <t>DXF INSERT dveře = 2 (Path C Tier 4) + TZ ARS</t>
+          <t>DXF INSERT okno* total 16 ks (Path C Tier 4 — front 9 + back 7)</t>
         </is>
       </c>
       <c r="G89" s="13" t="inlineStr">
@@ -5978,7 +5978,7 @@
       </c>
       <c r="I89" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.014</t>
+          <t>260219_dum.HSV6.013</t>
         </is>
       </c>
       <c r="J89" s="11" t="inlineStr"/>
@@ -5999,7 +5999,7 @@
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>Demontáž stávajících vnitřních dveří vč. ocelových/dřevěných zárubní — odhad 15 ks (3 patra × ~5 dveří/patro per DXF SM__dveře layer)</t>
+          <t>Demontáž stávajících vstupních dveří + rámů — 2 ks (1× ulice Fibichova + 1× zahrada; návrh nové plastové vstupní dveře)</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr">
@@ -6008,26 +6008,26 @@
         </is>
       </c>
       <c r="E90" s="12" t="n">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="F90" s="11" t="inlineStr">
         <is>
-          <t>DXF SM__dveře polylines 102 / ~3 fáze / ~2.3 symbol per dveře ≈ 15 ks návrh (Path C confidence 0.65)</t>
-        </is>
-      </c>
-      <c r="G90" s="11" t="inlineStr">
-        <is>
-          <t>968072456</t>
+          <t>DXF INSERT dveře = 2 (Path C Tier 4) + TZ ARS</t>
+        </is>
+      </c>
+      <c r="G90" s="13" t="inlineStr">
+        <is>
+          <t>978013181</t>
         </is>
       </c>
       <c r="H90" s="10" t="inlineStr">
         <is>
-          <t>⚠ kandidát-verify</t>
+          <t>✓ verified</t>
         </is>
       </c>
       <c r="I90" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.015</t>
+          <t>260219_dum.HSV6.014</t>
         </is>
       </c>
       <c r="J90" s="11" t="inlineStr"/>
@@ -6048,25 +6048,25 @@
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>Bourání vrchní části stávajícího komínu v posledním podlaží (cihelné zdivo, ručně), vč. likvidace cihelné suti</t>
+          <t>Demontáž stávajících vnitřních dveří vč. ocelových/dřevěných zárubní — odhad 15 ks (3 patra × ~5 dveří/patro per DXF SM__dveře layer)</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t>m³</t>
+          <t>ks</t>
         </is>
       </c>
       <c r="E91" s="12" t="n">
-        <v>0.6</v>
+        <v>15</v>
       </c>
       <c r="F91" s="11" t="inlineStr">
         <is>
-          <t>průměr komín 0.50×0.50 × výška nad střechou ~2.4 m = 0.6 m³ (OPRAVA ChatGPT revize 2026-05-29: dříve 6.0 m³ = ×10 chybná inflace; skutečný objem 0.6 m³)</t>
-        </is>
-      </c>
-      <c r="G91" s="13" t="inlineStr">
-        <is>
-          <t>962024141</t>
+          <t>DXF SM__dveře polylines 102 / ~3 fáze / ~2.3 symbol per dveře ≈ 15 ks návrh (Path C confidence 0.65)</t>
+        </is>
+      </c>
+      <c r="G91" s="11" t="inlineStr">
+        <is>
+          <t>968072456</t>
         </is>
       </c>
       <c r="H91" s="10" t="inlineStr">
@@ -6076,7 +6076,7 @@
       </c>
       <c r="I91" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.016</t>
+          <t>260219_dum.HSV6.015</t>
         </is>
       </c>
       <c r="J91" s="11" t="inlineStr"/>
@@ -6097,7 +6097,7 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>Bourání stávajících opěrných zídek a venkovního schodiště v zahradě/dvoře — částečné, dle vyznačení v půdorysech bourání</t>
+          <t>Bourání vrchní části stávajícího komínu v posledním podlaží (cihelné zdivo, ručně), vč. likvidace cihelné suti</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
@@ -6106,16 +6106,16 @@
         </is>
       </c>
       <c r="E92" s="12" t="n">
-        <v>8</v>
+        <v>0.6</v>
       </c>
       <c r="F92" s="11" t="inlineStr">
         <is>
-          <t>odhad ze řez A-A bourání + půdorys bourání 1.NP/1.PP, ~8 m³ celkem (opěrné zídky + venkovní schodiště zahrada/dvůr)</t>
+          <t>průměr komín 0.50×0.50 × výška nad střechou ~2.4 m = 0.6 m³ (OPRAVA ChatGPT revize 2026-05-29: dříve 6.0 m³ = ×10 chybná inflace; skutečný objem 0.6 m³)</t>
         </is>
       </c>
       <c r="G92" s="13" t="inlineStr">
         <is>
-          <t>961044111</t>
+          <t>962024141</t>
         </is>
       </c>
       <c r="H92" s="10" t="inlineStr">
@@ -6125,7 +6125,7 @@
       </c>
       <c r="I92" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.017</t>
+          <t>260219_dum.HSV6.016</t>
         </is>
       </c>
       <c r="J92" s="11" t="inlineStr"/>
@@ -6136,124 +6136,121 @@
       </c>
     </row>
     <row r="93">
-      <c r="A93" s="8" t="inlineStr">
+      <c r="A93" s="10" t="n">
+        <v>86</v>
+      </c>
+      <c r="B93" s="11" t="inlineStr">
+        <is>
+          <t>HSV-6 Bourací práce</t>
+        </is>
+      </c>
+      <c r="C93" s="11" t="inlineStr">
+        <is>
+          <t>Bourání stávajících opěrných zídek a venkovního schodiště v zahradě/dvoře — částečné, dle vyznačení v půdorysech bourání</t>
+        </is>
+      </c>
+      <c r="D93" s="10" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="E93" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="F93" s="11" t="inlineStr">
+        <is>
+          <t>odhad ze řez A-A bourání + půdorys bourání 1.NP/1.PP, ~8 m³ celkem (opěrné zídky + venkovní schodiště zahrada/dvůr)</t>
+        </is>
+      </c>
+      <c r="G93" s="13" t="inlineStr">
+        <is>
+          <t>961044111</t>
+        </is>
+      </c>
+      <c r="H93" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I93" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV6.017</t>
+        </is>
+      </c>
+      <c r="J93" s="11" t="inlineStr"/>
+      <c r="K93" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="8" t="inlineStr">
         <is>
           <t>━━ HSV-7 Fasáda ETICS  (9 atomic operací) ━━</t>
         </is>
       </c>
-      <c r="B93" s="9" t="n"/>
-      <c r="C93" s="9" t="n"/>
-      <c r="D93" s="9" t="n"/>
-      <c r="E93" s="9" t="n"/>
-      <c r="F93" s="9" t="n"/>
-      <c r="G93" s="9" t="n"/>
-      <c r="H93" s="9" t="n"/>
-      <c r="I93" s="9" t="n"/>
-      <c r="J93" s="9" t="n"/>
-      <c r="K93" s="9" t="n"/>
-    </row>
-    <row r="94">
-      <c r="A94" s="10" t="n">
-        <v>86</v>
-      </c>
-      <c r="B94" s="11" t="inlineStr">
+      <c r="B94" s="9" t="n"/>
+      <c r="C94" s="9" t="n"/>
+      <c r="D94" s="9" t="n"/>
+      <c r="E94" s="9" t="n"/>
+      <c r="F94" s="9" t="n"/>
+      <c r="G94" s="9" t="n"/>
+      <c r="H94" s="9" t="n"/>
+      <c r="I94" s="9" t="n"/>
+      <c r="J94" s="9" t="n"/>
+      <c r="K94" s="9" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="10" t="n">
+        <v>87</v>
+      </c>
+      <c r="B95" s="11" t="inlineStr">
         <is>
           <t>HSV-7 Fasáda ETICS</t>
         </is>
       </c>
-      <c r="C94" s="11" t="inlineStr">
+      <c r="C95" s="11" t="inlineStr">
         <is>
           <t>Příprava fasádního podkladu — očištění tlakovou vodou, vyspravení omítek, fungicidní nátěr</t>
         </is>
       </c>
-      <c r="D94" s="10" t="inlineStr">
+      <c r="D95" s="10" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E94" s="12" t="n">
+      <c r="E95" s="12" t="n">
         <v>276.7</v>
       </c>
-      <c r="F94" s="11" t="inlineStr">
+      <c r="F95" s="11" t="inlineStr">
         <is>
           <t>obvod 38.7 m (DXF) × 0.55 (volná fasáda, štíty zachované) × výška 13.0 m = 276.7 m²</t>
         </is>
       </c>
-      <c r="G94" s="11" t="inlineStr">
+      <c r="G95" s="11" t="inlineStr">
         <is>
           <t>622401110</t>
         </is>
       </c>
-      <c r="H94" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I94" s="11" t="inlineStr">
+      <c r="H95" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I95" s="11" t="inlineStr">
         <is>
           <t>260219_dum.HSV7.001</t>
         </is>
       </c>
-      <c r="J94" s="11" t="inlineStr">
+      <c r="J95" s="11" t="inlineStr">
         <is>
           <t>S01</t>
         </is>
       </c>
-      <c r="K94" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="95">
-      <c r="A95" s="14" t="n">
-        <v>87</v>
-      </c>
-      <c r="B95" s="15" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda ETICS</t>
-        </is>
-      </c>
-      <c r="C95" s="15" t="inlineStr">
-        <is>
-          <t>Lepení + kotvení desek EPS 70F grey λ=0.032 tl. 160 mm — ETICS kontaktní zateplení fasády</t>
-        </is>
-      </c>
-      <c r="D95" s="14" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E95" s="16" t="n">
-        <v>276.7</v>
-      </c>
-      <c r="F95" s="15">
-        <f> HSV7.002 plocha fasády 276.7 m²</f>
-        <v/>
-      </c>
-      <c r="G95" s="15" t="inlineStr">
-        <is>
-          <t>713</t>
-        </is>
-      </c>
-      <c r="H95" s="14" t="inlineStr">
-        <is>
-          <t>⚠ família ??? (ÚRS online)</t>
-        </is>
-      </c>
-      <c r="I95" s="15" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.002 → HSV7.002a</t>
-        </is>
-      </c>
-      <c r="J95" s="15" t="inlineStr">
-        <is>
-          <t>S01, S12a</t>
-        </is>
-      </c>
-      <c r="K95" s="15" t="inlineStr">
-        <is>
-          <t>Lepení+kotvení EPS (713/622 família). Leaf dle tl. 160 mm — verify.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+      <c r="K95" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
         </is>
       </c>
     </row>
@@ -6268,7 +6265,7 @@
       </c>
       <c r="C96" s="15" t="inlineStr">
         <is>
-          <t>Armovací vrstva — výztužná síťka + lepicí stěrka (zatírací) na ETICS</t>
+          <t>Lepení + kotvení desek EPS 70F grey λ=0.032 tl. 160 mm — ETICS kontaktní zateplení fasády</t>
         </is>
       </c>
       <c r="D96" s="14" t="inlineStr">
@@ -6280,12 +6277,12 @@
         <v>276.7</v>
       </c>
       <c r="F96" s="15">
-        <f> HSV7.002 plocha 276.7 m²</f>
+        <f> HSV7.002 plocha fasády 276.7 m²</f>
         <v/>
       </c>
       <c r="G96" s="15" t="inlineStr">
         <is>
-          <t>622</t>
+          <t>713</t>
         </is>
       </c>
       <c r="H96" s="14" t="inlineStr">
@@ -6295,7 +6292,7 @@
       </c>
       <c r="I96" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.002 → HSV7.002b</t>
+          <t>260219_dum.HSV7.002 → HSV7.002a</t>
         </is>
       </c>
       <c r="J96" s="15" t="inlineStr">
@@ -6305,7 +6302,7 @@
       </c>
       <c r="K96" s="15" t="inlineStr">
         <is>
-          <t>Armovací vrstva síťka+stěrka (622 família). Finální omítka je samostatně HSV7.006.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+          <t>Lepení+kotvení EPS (713/622 família). Leaf dle tl. 160 mm — verify.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -6320,7 +6317,7 @@
       </c>
       <c r="C97" s="15" t="inlineStr">
         <is>
-          <t>Lepení + kotvení desek XPS λ=0.034 tl. 120 mm + soklový profil — ETICS sokl</t>
+          <t>Armovací vrstva — výztužná síťka + lepicí stěrka (zatírací) na ETICS</t>
         </is>
       </c>
       <c r="D97" s="14" t="inlineStr">
@@ -6329,15 +6326,15 @@
         </is>
       </c>
       <c r="E97" s="16" t="n">
-        <v>13.5</v>
+        <v>276.7</v>
       </c>
       <c r="F97" s="15">
-        <f> HSV7.003 plocha soklu 13.5 m²</f>
+        <f> HSV7.002 plocha 276.7 m²</f>
         <v/>
       </c>
       <c r="G97" s="15" t="inlineStr">
         <is>
-          <t>713</t>
+          <t>622</t>
         </is>
       </c>
       <c r="H97" s="14" t="inlineStr">
@@ -6347,17 +6344,17 @@
       </c>
       <c r="I97" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.003 → HSV7.003a</t>
+          <t>260219_dum.HSV7.002 → HSV7.002b</t>
         </is>
       </c>
       <c r="J97" s="15" t="inlineStr">
         <is>
-          <t>S01</t>
+          <t>S01, S12a</t>
         </is>
       </c>
       <c r="K97" s="15" t="inlineStr">
         <is>
-          <t>Sokl XPS lepení + soklový profil (713/622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+          <t>Armovací vrstva síťka+stěrka (622 família). Finální omítka je samostatně HSV7.006.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6369,7 @@
       </c>
       <c r="C98" s="15" t="inlineStr">
         <is>
-          <t>Cihelný obklad soklu spárovaný (na armovací vrstvu)</t>
+          <t>Lepení + kotvení desek XPS λ=0.034 tl. 120 mm + soklový profil — ETICS sokl</t>
         </is>
       </c>
       <c r="D98" s="14" t="inlineStr">
@@ -6389,7 +6386,7 @@
       </c>
       <c r="G98" s="15" t="inlineStr">
         <is>
-          <t>781</t>
+          <t>713</t>
         </is>
       </c>
       <c r="H98" s="14" t="inlineStr">
@@ -6399,7 +6396,7 @@
       </c>
       <c r="I98" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.003 → HSV7.003b</t>
+          <t>260219_dum.HSV7.003 → HSV7.003a</t>
         </is>
       </c>
       <c r="J98" s="15" t="inlineStr">
@@ -6409,7 +6406,7 @@
       </c>
       <c r="K98" s="15" t="inlineStr">
         <is>
-          <t>Cihelný obklad spárovaný (781 família obklady).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+          <t>Sokl XPS lepení + soklový profil (713/622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -6424,24 +6421,24 @@
       </c>
       <c r="C99" s="15" t="inlineStr">
         <is>
-          <t>Špalety oken — EPS přesah 35-40 mm lepení + kotvení</t>
+          <t>Cihelný obklad soklu spárovaný (na armovací vrstvu)</t>
         </is>
       </c>
       <c r="D99" s="14" t="inlineStr">
         <is>
-          <t>bm</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E99" s="16" t="n">
-        <v>82.2</v>
+        <v>13.5</v>
       </c>
       <c r="F99" s="15">
-        <f> HSV7.004 obvod špalet 82.2 bm</f>
+        <f> HSV7.003 plocha soklu 13.5 m²</f>
         <v/>
       </c>
       <c r="G99" s="15" t="inlineStr">
         <is>
-          <t>622</t>
+          <t>781</t>
         </is>
       </c>
       <c r="H99" s="14" t="inlineStr">
@@ -6451,17 +6448,17 @@
       </c>
       <c r="I99" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.004 → HSV7.004a</t>
+          <t>260219_dum.HSV7.003 → HSV7.003b</t>
         </is>
       </c>
       <c r="J99" s="15" t="inlineStr">
         <is>
-          <t>S01, S12a</t>
+          <t>S01</t>
         </is>
       </c>
       <c r="K99" s="15" t="inlineStr">
         <is>
-          <t>Špalety EPS přesah (622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+          <t>Cihelný obklad spárovaný (781 família obklady).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -6476,7 +6473,7 @@
       </c>
       <c r="C100" s="15" t="inlineStr">
         <is>
-          <t>Špalety oken — armovací vrstva síťka + omítka</t>
+          <t>Špalety oken — EPS přesah 35-40 mm lepení + kotvení</t>
         </is>
       </c>
       <c r="D100" s="14" t="inlineStr">
@@ -6488,85 +6485,84 @@
         <v>82.2</v>
       </c>
       <c r="F100" s="15">
+        <f> HSV7.004 obvod špalet 82.2 bm</f>
+        <v/>
+      </c>
+      <c r="G100" s="15" t="inlineStr">
+        <is>
+          <t>622</t>
+        </is>
+      </c>
+      <c r="H100" s="14" t="inlineStr">
+        <is>
+          <t>⚠ família ??? (ÚRS online)</t>
+        </is>
+      </c>
+      <c r="I100" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.004 → HSV7.004a</t>
+        </is>
+      </c>
+      <c r="J100" s="15" t="inlineStr">
+        <is>
+          <t>S01, S12a</t>
+        </is>
+      </c>
+      <c r="K100" s="15" t="inlineStr">
+        <is>
+          <t>Špalety EPS přesah (622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="14" t="n">
+        <v>93</v>
+      </c>
+      <c r="B101" s="15" t="inlineStr">
+        <is>
+          <t>HSV-7 Fasáda ETICS</t>
+        </is>
+      </c>
+      <c r="C101" s="15" t="inlineStr">
+        <is>
+          <t>Špalety oken — armovací vrstva síťka + omítka</t>
+        </is>
+      </c>
+      <c r="D101" s="14" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="E101" s="16" t="n">
+        <v>82.2</v>
+      </c>
+      <c r="F101" s="15">
         <f> HSV7.004 obvod 82.2 bm</f>
         <v/>
       </c>
-      <c r="G100" s="15" t="inlineStr">
+      <c r="G101" s="15" t="inlineStr">
         <is>
           <t>622</t>
         </is>
       </c>
-      <c r="H100" s="14" t="inlineStr">
+      <c r="H101" s="14" t="inlineStr">
         <is>
           <t>⚠ família ??? (ÚRS online)</t>
         </is>
       </c>
-      <c r="I100" s="15" t="inlineStr">
+      <c r="I101" s="15" t="inlineStr">
         <is>
           <t>260219_dum.HSV7.004 → HSV7.004b</t>
         </is>
       </c>
-      <c r="J100" s="15" t="inlineStr">
+      <c r="J101" s="15" t="inlineStr">
         <is>
           <t>S01, S12a</t>
         </is>
       </c>
-      <c r="K100" s="15" t="inlineStr">
+      <c r="K101" s="15" t="inlineStr">
         <is>
           <t>Armovací vrstva + omítka špalet (622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="10" t="n">
-        <v>93</v>
-      </c>
-      <c r="B101" s="11" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda ETICS</t>
-        </is>
-      </c>
-      <c r="C101" s="11" t="inlineStr">
-        <is>
-          <t>Profilace fasády — různé tloušťky EPS (kordony, šambrány, rámování oken) — paušál podle pohledů</t>
-        </is>
-      </c>
-      <c r="D101" s="10" t="inlineStr">
-        <is>
-          <t>soubor</t>
-        </is>
-      </c>
-      <c r="E101" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F101" s="11" t="inlineStr">
-        <is>
-          <t>paušál — dle pohledů NCS NZÚ</t>
-        </is>
-      </c>
-      <c r="G101" s="11" t="inlineStr">
-        <is>
-          <t>622221221</t>
-        </is>
-      </c>
-      <c r="H101" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I101" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.005</t>
-        </is>
-      </c>
-      <c r="J101" s="11" t="inlineStr">
-        <is>
-          <t>S01, S12a</t>
-        </is>
-      </c>
-      <c r="K101" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
         </is>
       </c>
     </row>
@@ -6581,43 +6577,96 @@
       </c>
       <c r="C102" s="11" t="inlineStr">
         <is>
+          <t>Profilace fasády — různé tloušťky EPS (kordony, šambrány, rámování oken) — paušál podle pohledů</t>
+        </is>
+      </c>
+      <c r="D102" s="10" t="inlineStr">
+        <is>
+          <t>soubor</t>
+        </is>
+      </c>
+      <c r="E102" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F102" s="11" t="inlineStr">
+        <is>
+          <t>paušál — dle pohledů NCS NZÚ</t>
+        </is>
+      </c>
+      <c r="G102" s="11" t="inlineStr">
+        <is>
+          <t>622221221</t>
+        </is>
+      </c>
+      <c r="H102" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I102" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.005</t>
+        </is>
+      </c>
+      <c r="J102" s="11" t="inlineStr">
+        <is>
+          <t>S01, S12a</t>
+        </is>
+      </c>
+      <c r="K102" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="10" t="n">
+        <v>95</v>
+      </c>
+      <c r="B103" s="11" t="inlineStr">
+        <is>
+          <t>HSV-7 Fasáda ETICS</t>
+        </is>
+      </c>
+      <c r="C103" s="11" t="inlineStr">
+        <is>
           <t>Tenkovrstvá pastovitá probarvená omítka, lomená bílá NCS NZÚ — finální vrstva ETICS</t>
         </is>
       </c>
-      <c r="D102" s="10" t="inlineStr">
+      <c r="D103" s="10" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E102" s="12" t="n">
+      <c r="E103" s="12" t="n">
         <v>290.2</v>
       </c>
-      <c r="F102" s="11" t="inlineStr">
+      <c r="F103" s="11" t="inlineStr">
         <is>
           <t>ETICS plocha 276.7 m² + sokl 13.5 m² = 290.2 m²</t>
         </is>
       </c>
-      <c r="G102" s="13" t="inlineStr">
+      <c r="G103" s="13" t="inlineStr">
         <is>
           <t>622521111</t>
         </is>
       </c>
-      <c r="H102" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I102" s="11" t="inlineStr">
+      <c r="H103" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I103" s="11" t="inlineStr">
         <is>
           <t>260219_dum.HSV7.006</t>
         </is>
       </c>
-      <c r="J102" s="11" t="inlineStr">
+      <c r="J103" s="11" t="inlineStr">
         <is>
           <t>S01, S12a, S12b</t>
         </is>
       </c>
-      <c r="K102" s="11" t="inlineStr">
+      <c r="K103" s="11" t="inlineStr">
         <is>
           <t>Carried 1:1 (atomic — no decomposition needed)</t>
         </is>
@@ -6626,13 +6675,13 @@
   </sheetData>
   <autoFilter ref="A1:K1"/>
   <mergeCells count="7">
-    <mergeCell ref="A58:K58"/>
-    <mergeCell ref="A35:K35"/>
-    <mergeCell ref="A21:K21"/>
-    <mergeCell ref="A43:K43"/>
+    <mergeCell ref="A22:K22"/>
+    <mergeCell ref="A59:K59"/>
     <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A93:K93"/>
-    <mergeCell ref="A75:K75"/>
+    <mergeCell ref="A76:K76"/>
+    <mergeCell ref="A36:K36"/>
+    <mergeCell ref="A44:K44"/>
+    <mergeCell ref="A94:K94"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -9126,10 +9175,10 @@
         </is>
       </c>
       <c r="E55" s="16" t="n">
-        <v>30</v>
+        <v>9.23</v>
       </c>
       <c r="F55" s="15">
-        <f> PSV76.002 plocha terasy 30 m²</f>
+        <f> PSV76.002 plocha terasy 9.23 m² (situace měření)</f>
         <v/>
       </c>
       <c r="G55" s="15" t="inlineStr">
@@ -9174,10 +9223,10 @@
         </is>
       </c>
       <c r="E56" s="16" t="n">
-        <v>30</v>
+        <v>9.23</v>
       </c>
       <c r="F56" s="15">
-        <f> PSV76.002 plocha terasy 30 m²</f>
+        <f> PSV76.002 plocha terasy 9.23 m² (situace měření)</f>
         <v/>
       </c>
       <c r="G56" s="15" t="inlineStr">
@@ -14878,7 +14927,7 @@
         </is>
       </c>
       <c r="E2" s="16" t="n">
-        <v>30</v>
+        <v>16.54</v>
       </c>
       <c r="F2" s="14" t="n">
         <v>4</v>
@@ -14911,7 +14960,7 @@
         </is>
       </c>
       <c r="E3" s="16" t="n">
-        <v>30</v>
+        <v>9.23</v>
       </c>
       <c r="F3" s="14" t="n">
         <v>5</v>
@@ -15076,7 +15125,7 @@
         </is>
       </c>
       <c r="E8" s="16" t="n">
-        <v>30</v>
+        <v>9.23</v>
       </c>
       <c r="F8" s="14" t="n">
         <v>2</v>

</xml_diff>

<commit_message>
fix(rd-jachymov): worklist notes — drop stale '636311 na terče/NE 762', reflect ŘEZ C-C + situace areas
ATOMIC_WORKLIST Souhrn/notes still said 'HSV1.005 terasa 636311 (na terče, NE 762)' +
'A2 korekce: dlaždice NA TERČE, NE 762 carpentry' — contradicted the corrected data
(dlaždice roznášecí POD terče 564 + dřevo 762 in PSV76.002, terasa 9.23 / dvorek 16.54).
Notes updated; regenerated (9 steps, assertions pass).

https://claude.ai/code/session_01FskzLAZkXgJAwuN2cQQEdx
</commit_message>
<xml_diff>
--- a/test-data/RD_Jachymov_dum/outputs/Vykaz_vymer_RD_Jachymov_ATOMIC_WORKLIST_2026-05-27.xlsx
+++ b/test-data/RD_Jachymov_dum/outputs/Vykaz_vymer_RD_Jachymov_ATOMIC_WORKLIST_2026-05-27.xlsx
@@ -1032,7 +1032,7 @@
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
         <is>
-          <t>• Reconciliation consensus: HSV1.004 dvorek 596811220 · HSV1.005 terasa 636311 (na terče, NE 762) · HSV2.003/008 bednění 274.</t>
+          <t>• Reconciliation consensus: HSV1.004 dvorek 596811220 · HSV1.005 terasa = podkladní skladba 564 (dlaždice ROZNÁŠECÍ POD terče, ŘEZ C-C) · dřevo 762 = PSV76.002 Truhlář · HSV2.003/008 bednění 274.</t>
         </is>
       </c>
     </row>
@@ -1649,7 +1649,7 @@
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
         <is>
-          <t>• Terasa A2 korekce: HSV1.005a = 636311 família (dlaždice NA TERČE, NE 762 carpentry)</t>
+          <t>• Terasa ŘEZ C-C oprava: dlaždice = roznášecí vrstva POD terče (564, NE '636311 na terče'); dřevěná pochozí vrstva (762) = PSV76.002 Truhlář (split-by-trade). Plochy situace: terasa 9.23 / dvorek 16.54 m².</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat(rd-jachymov): krov leaf-bind 762332xxx by průřez + montáž/materiál split (ÚRS)
Stage-3 leaf-binding for krov timber, unblocked via KROS catalog + STAVAGENT MCP.
Krov is classified by PRŮŘEZOVÁ PLOCHA (cm²) in group 762332 (vázané konstrukce
krovů pomocí ocelových spojek), not by element name:
- krokve 100/180 (180 cm²), kleštiny 2×60/180 (216), pozednice 140/160 (224) → 762332122
- námětky 60/100 (60 cm²) → 762332121
Replaces prior imprecise 762331xxx (krokve+námětky wrongly shared 762331911).

items.json HSV5.001-004: montáž code + status matched_catalog (MJ stays bm = catalog m).
atomic_decomposition.py: each split into montáž (762332xxx, m) + dodávka řeziva C24
(60512136, m³ incl. 10% prořez) per ÚRS. Companion note: pozednice kotvení do věnce
= CHYBÍ DETAIL; námětky material leaf needs short-length lookup.
items 215 (codes only, no count change); 9-step regen + assertion pass. Snapshot held.

https://claude.ai/code/session_01FskzLAZkXgJAwuN2cQQEdx
</commit_message>
<xml_diff>
--- a/test-data/RD_Jachymov_dum/outputs/Vykaz_vymer_RD_Jachymov_ATOMIC_WORKLIST_2026-05-27.xlsx
+++ b/test-data/RD_Jachymov_dum/outputs/Vykaz_vymer_RD_Jachymov_ATOMIC_WORKLIST_2026-05-27.xlsx
@@ -538,7 +538,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C119"/>
+  <dimension ref="A1:C120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>244</v>
+        <v>248</v>
       </c>
       <c r="C6" s="2">
         <f> carried 1:1 + decomposed children</f>
@@ -603,7 +603,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>47</v>
+        <v>55</v>
       </c>
     </row>
     <row r="9">
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -712,7 +712,7 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="19">
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
     </row>
     <row r="48">
@@ -999,7 +999,7 @@
         </is>
       </c>
       <c r="B48" s="5" t="n">
-        <v>171</v>
+        <v>167</v>
       </c>
     </row>
     <row r="49">
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>46</v>
+        <v>50</v>
       </c>
     </row>
     <row r="50">
@@ -1280,7 +1280,7 @@
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>713</t>
+          <t>605</t>
         </is>
       </c>
       <c r="B79" s="5" t="n">
@@ -1290,7 +1290,7 @@
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>974</t>
+          <t>713</t>
         </is>
       </c>
       <c r="B80" s="5" t="n">
@@ -1300,7 +1300,7 @@
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>997</t>
+          <t>974</t>
         </is>
       </c>
       <c r="B81" s="5" t="n">
@@ -1310,17 +1310,17 @@
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>031</t>
+          <t>997</t>
         </is>
       </c>
       <c r="B82" s="5" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>132</t>
+          <t>031</t>
         </is>
       </c>
       <c r="B83" s="5" t="n">
@@ -1330,7 +1330,7 @@
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>174</t>
+          <t>132</t>
         </is>
       </c>
       <c r="B84" s="5" t="n">
@@ -1340,7 +1340,7 @@
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>342</t>
+          <t>174</t>
         </is>
       </c>
       <c r="B85" s="5" t="n">
@@ -1350,7 +1350,7 @@
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>631</t>
+          <t>342</t>
         </is>
       </c>
       <c r="B86" s="5" t="n">
@@ -1360,17 +1360,17 @@
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>121</t>
+          <t>631</t>
         </is>
       </c>
       <c r="B87" s="5" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>131</t>
+          <t>121</t>
         </is>
       </c>
       <c r="B88" s="5" t="n">
@@ -1380,7 +1380,7 @@
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>212</t>
+          <t>131</t>
         </is>
       </c>
       <c r="B89" s="5" t="n">
@@ -1390,7 +1390,7 @@
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>317</t>
+          <t>212</t>
         </is>
       </c>
       <c r="B90" s="5" t="n">
@@ -1400,7 +1400,7 @@
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>693</t>
+          <t>317</t>
         </is>
       </c>
       <c r="B91" s="5" t="n">
@@ -1410,7 +1410,7 @@
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>722</t>
+          <t>693</t>
         </is>
       </c>
       <c r="B92" s="5" t="n">
@@ -1420,7 +1420,7 @@
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>732</t>
+          <t>722</t>
         </is>
       </c>
       <c r="B93" s="5" t="n">
@@ -1430,7 +1430,7 @@
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>765</t>
+          <t>732</t>
         </is>
       </c>
       <c r="B94" s="5" t="n">
@@ -1440,7 +1440,7 @@
     <row r="95">
       <c r="A95" s="4" t="inlineStr">
         <is>
-          <t>776</t>
+          <t>765</t>
         </is>
       </c>
       <c r="B95" s="5" t="n">
@@ -1450,7 +1450,7 @@
     <row r="96">
       <c r="A96" s="4" t="inlineStr">
         <is>
-          <t>968</t>
+          <t>776</t>
         </is>
       </c>
       <c r="B96" s="5" t="n">
@@ -1460,7 +1460,7 @@
     <row r="97">
       <c r="A97" s="4" t="inlineStr">
         <is>
-          <t>978</t>
+          <t>968</t>
         </is>
       </c>
       <c r="B97" s="5" t="n">
@@ -1470,17 +1470,17 @@
     <row r="98">
       <c r="A98" s="4" t="inlineStr">
         <is>
-          <t>012</t>
+          <t>978</t>
         </is>
       </c>
       <c r="B98" s="5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="99">
       <c r="A99" s="4" t="inlineStr">
         <is>
-          <t>151</t>
+          <t>012</t>
         </is>
       </c>
       <c r="B99" s="5" t="n">
@@ -1490,7 +1490,7 @@
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>181</t>
+          <t>151</t>
         </is>
       </c>
       <c r="B100" s="5" t="n">
@@ -1500,7 +1500,7 @@
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>271</t>
+          <t>181</t>
         </is>
       </c>
       <c r="B101" s="5" t="n">
@@ -1510,7 +1510,7 @@
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>279</t>
+          <t>271</t>
         </is>
       </c>
       <c r="B102" s="5" t="n">
@@ -1520,7 +1520,7 @@
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>375</t>
+          <t>279</t>
         </is>
       </c>
       <c r="B103" s="5" t="n">
@@ -1530,7 +1530,7 @@
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>596</t>
+          <t>375</t>
         </is>
       </c>
       <c r="B104" s="5" t="n">
@@ -1540,7 +1540,7 @@
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>721</t>
+          <t>596</t>
         </is>
       </c>
       <c r="B105" s="5" t="n">
@@ -1550,7 +1550,7 @@
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
         <is>
-          <t>734</t>
+          <t>721</t>
         </is>
       </c>
       <c r="B106" s="5" t="n">
@@ -1560,7 +1560,7 @@
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>783</t>
+          <t>734</t>
         </is>
       </c>
       <c r="B107" s="5" t="n">
@@ -1570,7 +1570,7 @@
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>783</t>
         </is>
       </c>
       <c r="B108" s="5" t="n">
@@ -1580,7 +1580,7 @@
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>966</t>
+          <t>961</t>
         </is>
       </c>
       <c r="B109" s="5" t="n">
@@ -1590,64 +1590,74 @@
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>996</t>
+          <t>966</t>
         </is>
       </c>
       <c r="B110" s="5" t="n">
         <v>1</v>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" s="3" t="inlineStr">
+    <row r="111">
+      <c r="A111" s="4" t="inlineStr">
+        <is>
+          <t>996</t>
+        </is>
+      </c>
+      <c r="B111" s="5" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="3" t="inlineStr">
         <is>
           <t>METODIKA + PATTERN COMPLIANCE</t>
-        </is>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="4" t="inlineStr">
-        <is>
-          <t>• HK212 028a..f princip: composite → atomic codeable operace (per vrstva / per fixture)</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>• Pattern 15 Work-First: atomic ops = codeable units, catalog matching downstream</t>
+          <t>• HK212 028a..f princip: composite → atomic codeable operace (per vrstva / per fixture)</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" s="4" t="inlineStr">
         <is>
-          <t>• Pattern 26: família-level URS kde leaf neznámý + status flag; 9 BLANK ops (NE 999/TBD)</t>
+          <t>• Pattern 15 Work-First: atomic ops = codeable units, catalog matching downstream</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" s="4" t="inlineStr">
         <is>
-          <t>• Pattern 28: (id, kapitola) compound key — řeší PSV76.003 ×3 + VRN.001 ×9 collisions</t>
+          <t>• Pattern 26: família-level URS kde leaf neznámý + status flag; 9 BLANK ops (NE 999/TBD)</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" s="4" t="inlineStr">
         <is>
-          <t>• Pattern 32: separate deliverable — items.json frozen + File A audit NEDOTČENO</t>
+          <t>• Pattern 28: (id, kapitola) compound key — řeší PSV76.003 ×3 + VRN.001 ×9 collisions</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" s="4" t="inlineStr">
         <is>
-          <t>• Traceability: každá atomic op → parent_frozen_item_id (100% coverage)</t>
+          <t>• Pattern 32: separate deliverable — items.json frozen + File A audit NEDOTČENO</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" s="4" t="inlineStr">
+        <is>
+          <t>• Traceability: každá atomic op → parent_frozen_item_id (100% coverage)</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" s="4" t="inlineStr">
         <is>
           <t>• Terasa ŘEZ C-C oprava: dlaždice = roznášecí vrstva POD terče (564, NE '636311 na terče'); dřevěná pochozí vrstva (762) = PSV76.002 Truhlář (split-by-trade). Plochy situace: terasa 9.23 / dvorek 16.54 m².</t>
         </is>
@@ -1656,7 +1666,6 @@
   </sheetData>
   <mergeCells count="15">
     <mergeCell ref="A115:C115"/>
-    <mergeCell ref="A112:C112"/>
     <mergeCell ref="A11:C11"/>
     <mergeCell ref="A116:C116"/>
     <mergeCell ref="A117:C117"/>
@@ -1664,6 +1673,7 @@
     <mergeCell ref="A118:C118"/>
     <mergeCell ref="A119:C119"/>
     <mergeCell ref="A56:C56"/>
+    <mergeCell ref="A120:C120"/>
     <mergeCell ref="A53:C53"/>
     <mergeCell ref="A114:C114"/>
     <mergeCell ref="A4:C4"/>
@@ -1681,7 +1691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K103"/>
+  <dimension ref="A1:K107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4511,7 +4521,7 @@
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>━━ HSV-5 Krov + střecha  (16 atomic operací) ━━</t>
+          <t>━━ HSV-5 Krov + střecha  (20 atomic operací) ━━</t>
         </is>
       </c>
       <c r="B59" s="9" t="n"/>
@@ -4526,401 +4536,386 @@
       <c r="K59" s="9" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="10" t="n">
+      <c r="A60" s="14" t="n">
         <v>54</v>
       </c>
-      <c r="B60" s="11" t="inlineStr">
+      <c r="B60" s="15" t="inlineStr">
         <is>
           <t>HSV-5 Krov + střecha</t>
         </is>
       </c>
-      <c r="C60" s="11" t="inlineStr">
-        <is>
-          <t>Tesařský krov — krokve 100/180 mm á 800 mm, rezivo C24 fungicidní + protihmyzí (cca 2×12 krokví × ~6.5 m)</t>
-        </is>
-      </c>
-      <c r="D60" s="10" t="inlineStr">
-        <is>
-          <t>bm</t>
-        </is>
-      </c>
-      <c r="E60" s="12" t="n">
+      <c r="C60" s="15" t="inlineStr">
+        <is>
+          <t>Montáž krokví 100/180 mm — vázaná konstrukce krovu pomocí ocelových spojek, hraněné řezivo (průřez 180 cm², přes 120 do 224)</t>
+        </is>
+      </c>
+      <c r="D60" s="14" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E60" s="16" t="n">
         <v>156</v>
       </c>
-      <c r="F60" s="11" t="inlineStr">
-        <is>
-          <t>(2 sklony × 12 krokví × 6.5 m délka) = 156</t>
-        </is>
-      </c>
-      <c r="G60" s="13" t="inlineStr">
-        <is>
-          <t>762331911</t>
-        </is>
-      </c>
-      <c r="H60" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I60" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV5.001</t>
-        </is>
-      </c>
-      <c r="J60" s="11" t="inlineStr"/>
-      <c r="K60" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+      <c r="F60" s="15">
+        <f> HSV5.001 délka krokví 156 bm</f>
+        <v/>
+      </c>
+      <c r="G60" s="15" t="inlineStr">
+        <is>
+          <t>762332122</t>
+        </is>
+      </c>
+      <c r="H60" s="14" t="inlineStr">
+        <is>
+          <t>✓ verified</t>
+        </is>
+      </c>
+      <c r="I60" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV5.001 → HSV5.001a</t>
+        </is>
+      </c>
+      <c r="J60" s="15" t="inlineStr"/>
+      <c r="K60" s="15" t="inlineStr">
+        <is>
+          <t>Montáž 762332122 (266 Kč/m, KROS). Materiál = op b.</t>
         </is>
       </c>
     </row>
     <row r="61">
-      <c r="A61" s="10" t="n">
+      <c r="A61" s="14" t="n">
         <v>55</v>
       </c>
-      <c r="B61" s="11" t="inlineStr">
+      <c r="B61" s="15" t="inlineStr">
         <is>
           <t>HSV-5 Krov + střecha</t>
         </is>
       </c>
-      <c r="C61" s="11" t="inlineStr">
-        <is>
-          <t>Tesařský krov — kleštiny dvojfošny 60/180 mm probíhající v oblasti spací části</t>
-        </is>
-      </c>
-      <c r="D61" s="10" t="inlineStr">
-        <is>
-          <t>bm</t>
-        </is>
-      </c>
-      <c r="E61" s="12" t="n">
+      <c r="C61" s="15" t="inlineStr">
+        <is>
+          <t>Dodávka hranolového řeziva C24 pro krokve 100/180 mm vč. 10 % prořezu (fungicidní + protihmyzí impregnace)</t>
+        </is>
+      </c>
+      <c r="D61" s="14" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="E61" s="16" t="n">
+        <v>3.09</v>
+      </c>
+      <c r="F61" s="15">
+        <f> 156 × 0.10 × 0.18 × 1.10 = 3.09 m³</f>
+        <v/>
+      </c>
+      <c r="G61" s="15" t="inlineStr">
+        <is>
+          <t>60512136</t>
+        </is>
+      </c>
+      <c r="H61" s="14" t="inlineStr">
+        <is>
+          <t>⚠ família ??? (ÚRS online)</t>
+        </is>
+      </c>
+      <c r="I61" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV5.001 → HSV5.001b</t>
+        </is>
+      </c>
+      <c r="J61" s="15" t="inlineStr"/>
+      <c r="K61" s="15" t="inlineStr">
+        <is>
+          <t>Hranol řezivo do 288 cm² (60512136). Impregnace dle TZ statika §6.2.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="14" t="n">
+        <v>56</v>
+      </c>
+      <c r="B62" s="15" t="inlineStr">
+        <is>
+          <t>HSV-5 Krov + střecha</t>
+        </is>
+      </c>
+      <c r="C62" s="15" t="inlineStr">
+        <is>
+          <t>Montáž kleštin 2×60/180 mm — vázaná konstrukce krovu pomocí ocelových spojek (průřez 216 cm², přes 120 do 224)</t>
+        </is>
+      </c>
+      <c r="D62" s="14" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E62" s="16" t="n">
         <v>110</v>
       </c>
-      <c r="F61" s="11" t="inlineStr">
-        <is>
-          <t>11 pozic × 2 ks × ~5 m délka = 110</t>
-        </is>
-      </c>
-      <c r="G61" s="13" t="inlineStr">
-        <is>
-          <t>762331912</t>
-        </is>
-      </c>
-      <c r="H61" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I61" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV5.002</t>
-        </is>
-      </c>
-      <c r="J61" s="11" t="inlineStr"/>
-      <c r="K61" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" s="10" t="n">
-        <v>56</v>
-      </c>
-      <c r="B62" s="11" t="inlineStr">
+      <c r="F62" s="15">
+        <f> HSV5.002 délka kleštin 110 bm</f>
+        <v/>
+      </c>
+      <c r="G62" s="15" t="inlineStr">
+        <is>
+          <t>762332122</t>
+        </is>
+      </c>
+      <c r="H62" s="14" t="inlineStr">
+        <is>
+          <t>✓ verified</t>
+        </is>
+      </c>
+      <c r="I62" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV5.002 → HSV5.002a</t>
+        </is>
+      </c>
+      <c r="J62" s="15" t="inlineStr"/>
+      <c r="K62" s="15" t="inlineStr">
+        <is>
+          <t>Montáž 762332122 (266 Kč/m). Materiál = op b.</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="14" t="n">
+        <v>57</v>
+      </c>
+      <c r="B63" s="15" t="inlineStr">
         <is>
           <t>HSV-5 Krov + střecha</t>
         </is>
       </c>
-      <c r="C62" s="11" t="inlineStr">
-        <is>
-          <t>Tesařský krov — pozednice 140/160 mm kotvená do ŽB věnce 3.NP</t>
-        </is>
-      </c>
-      <c r="D62" s="10" t="inlineStr">
-        <is>
-          <t>bm</t>
-        </is>
-      </c>
-      <c r="E62" s="12" t="n">
+      <c r="C63" s="15" t="inlineStr">
+        <is>
+          <t>Dodávka hranolového řeziva C24 pro kleštiny 2×60/180 mm vč. 10 % prořezu + impregnace</t>
+        </is>
+      </c>
+      <c r="D63" s="14" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="E63" s="16" t="n">
+        <v>1.31</v>
+      </c>
+      <c r="F63" s="15">
+        <f> 110 × 0.06 × 0.18 × 1.10 = 1.31 m³</f>
+        <v/>
+      </c>
+      <c r="G63" s="15" t="inlineStr">
+        <is>
+          <t>60512136</t>
+        </is>
+      </c>
+      <c r="H63" s="14" t="inlineStr">
+        <is>
+          <t>⚠ família ??? (ÚRS online)</t>
+        </is>
+      </c>
+      <c r="I63" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV5.002 → HSV5.002b</t>
+        </is>
+      </c>
+      <c r="J63" s="15" t="inlineStr"/>
+      <c r="K63" s="15" t="inlineStr">
+        <is>
+          <t>Hranol řezivo (60512136).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="14" t="n">
+        <v>58</v>
+      </c>
+      <c r="B64" s="15" t="inlineStr">
+        <is>
+          <t>HSV-5 Krov + střecha</t>
+        </is>
+      </c>
+      <c r="C64" s="15" t="inlineStr">
+        <is>
+          <t>Montáž pozednic 140/160 mm — vázaná konstrukce krovu pomocí ocelových spojek (průřez 224 cm², přes 120 do 224)</t>
+        </is>
+      </c>
+      <c r="D64" s="14" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E64" s="16" t="n">
         <v>19.4</v>
       </c>
-      <c r="F62" s="11" t="inlineStr">
-        <is>
-          <t>polovina obvodu (2 dlouhé strany) = ~20</t>
-        </is>
-      </c>
-      <c r="G62" s="13" t="inlineStr">
-        <is>
-          <t>762331923</t>
-        </is>
-      </c>
-      <c r="H62" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I62" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV5.003</t>
-        </is>
-      </c>
-      <c r="J62" s="11" t="inlineStr"/>
-      <c r="K62" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" s="10" t="n">
-        <v>57</v>
-      </c>
-      <c r="B63" s="11" t="inlineStr">
+      <c r="F64" s="15">
+        <f> HSV5.003 délka pozednic ~19.4 bm</f>
+        <v/>
+      </c>
+      <c r="G64" s="15" t="inlineStr">
+        <is>
+          <t>762332122</t>
+        </is>
+      </c>
+      <c r="H64" s="14" t="inlineStr">
+        <is>
+          <t>✓ verified</t>
+        </is>
+      </c>
+      <c r="I64" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV5.003 → HSV5.003a</t>
+        </is>
+      </c>
+      <c r="J64" s="15" t="inlineStr"/>
+      <c r="K64" s="15" t="inlineStr">
+        <is>
+          <t>Montáž 762332122. Kotvení do ŽB věnce = samostatně (CHYBÍ DETAIL — závitové tyče/kotvy).</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="14" t="n">
+        <v>59</v>
+      </c>
+      <c r="B65" s="15" t="inlineStr">
         <is>
           <t>HSV-5 Krov + střecha</t>
         </is>
       </c>
-      <c r="C63" s="11" t="inlineStr">
-        <is>
-          <t>Tesařský krov — námětky 60/100 v dolní koncové části pro přesah střechy ~500 mm</t>
-        </is>
-      </c>
-      <c r="D63" s="10" t="inlineStr">
-        <is>
-          <t>bm</t>
-        </is>
-      </c>
-      <c r="E63" s="12" t="n">
+      <c r="C65" s="15" t="inlineStr">
+        <is>
+          <t>Dodávka hranolového řeziva C24 pro pozednice 140/160 mm vč. 10 % prořezu + impregnace</t>
+        </is>
+      </c>
+      <c r="D65" s="14" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="E65" s="16" t="n">
+        <v>0.48</v>
+      </c>
+      <c r="F65" s="15">
+        <f> 19.4 × 0.14 × 0.16 × 1.10 = 0.48 m³</f>
+        <v/>
+      </c>
+      <c r="G65" s="15" t="inlineStr">
+        <is>
+          <t>60512136</t>
+        </is>
+      </c>
+      <c r="H65" s="14" t="inlineStr">
+        <is>
+          <t>⚠ família ??? (ÚRS online)</t>
+        </is>
+      </c>
+      <c r="I65" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV5.003 → HSV5.003b</t>
+        </is>
+      </c>
+      <c r="J65" s="15" t="inlineStr"/>
+      <c r="K65" s="15" t="inlineStr">
+        <is>
+          <t>Hranol řezivo (60512136).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="14" t="n">
+        <v>60</v>
+      </c>
+      <c r="B66" s="15" t="inlineStr">
+        <is>
+          <t>HSV-5 Krov + střecha</t>
+        </is>
+      </c>
+      <c r="C66" s="15" t="inlineStr">
+        <is>
+          <t>Montáž námětků 60/100 mm — vázaná konstrukce krovu pomocí ocelových spojek (průřez 60 cm², přes 50 do 120)</t>
+        </is>
+      </c>
+      <c r="D66" s="14" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E66" s="16" t="n">
         <v>19.2</v>
       </c>
-      <c r="F63" s="11" t="inlineStr">
-        <is>
-          <t>24 krokví × 0.8 m námětek = 19.2</t>
-        </is>
-      </c>
-      <c r="G63" s="11" t="inlineStr">
-        <is>
-          <t>762331911</t>
-        </is>
-      </c>
-      <c r="H63" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I63" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV5.004</t>
-        </is>
-      </c>
-      <c r="J63" s="11" t="inlineStr"/>
-      <c r="K63" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" s="10" t="n">
-        <v>58</v>
-      </c>
-      <c r="B64" s="11" t="inlineStr">
+      <c r="F66" s="15">
+        <f> HSV5.004 délka námětků 19.2 bm</f>
+        <v/>
+      </c>
+      <c r="G66" s="15" t="inlineStr">
+        <is>
+          <t>762332121</t>
+        </is>
+      </c>
+      <c r="H66" s="14" t="inlineStr">
+        <is>
+          <t>✓ verified</t>
+        </is>
+      </c>
+      <c r="I66" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV5.004 → HSV5.004a</t>
+        </is>
+      </c>
+      <c r="J66" s="15" t="inlineStr"/>
+      <c r="K66" s="15" t="inlineStr">
+        <is>
+          <t>Montáž 762332121 (206 Kč/m, KROS).</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="14" t="n">
+        <v>61</v>
+      </c>
+      <c r="B67" s="15" t="inlineStr">
         <is>
           <t>HSV-5 Krov + střecha</t>
         </is>
       </c>
-      <c r="C64" s="11" t="inlineStr">
-        <is>
-          <t>Ocelová středová vaznice HEA160 — 2 ks × cca 10 m délka</t>
-        </is>
-      </c>
-      <c r="D64" s="10" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E64" s="12" t="n">
-        <v>608</v>
-      </c>
-      <c r="F64" s="11" t="inlineStr">
-        <is>
-          <t>2 × 10 × 30.4 kg/m (HEA160) = 608</t>
-        </is>
-      </c>
-      <c r="G64" s="13" t="inlineStr">
-        <is>
-          <t>411321414</t>
-        </is>
-      </c>
-      <c r="H64" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I64" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV5.005</t>
-        </is>
-      </c>
-      <c r="J64" s="11" t="inlineStr"/>
-      <c r="K64" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" s="10" t="n">
-        <v>59</v>
-      </c>
-      <c r="B65" s="11" t="inlineStr">
-        <is>
-          <t>HSV-5 Krov + střecha</t>
-        </is>
-      </c>
-      <c r="C65" s="11" t="inlineStr">
-        <is>
-          <t>Ocelové sloupky uzavřený profil 100×100×4 mm pod vaznice HEA160 (~6 ks × ~2.5 m výška)</t>
-        </is>
-      </c>
-      <c r="D65" s="10" t="inlineStr">
-        <is>
-          <t>kg</t>
-        </is>
-      </c>
-      <c r="E65" s="12" t="n">
-        <v>176</v>
-      </c>
-      <c r="F65" s="11" t="inlineStr">
-        <is>
-          <t>6 × 2.5 × 11.7 kg/m (RHS 100×100×4) = 176</t>
-        </is>
-      </c>
-      <c r="G65" s="11" t="inlineStr">
-        <is>
-          <t>411321414</t>
-        </is>
-      </c>
-      <c r="H65" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I65" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV5.006</t>
-        </is>
-      </c>
-      <c r="J65" s="11" t="inlineStr"/>
-      <c r="K65" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" s="10" t="n">
-        <v>60</v>
-      </c>
-      <c r="B66" s="11" t="inlineStr">
-        <is>
-          <t>HSV-5 Krov + střecha</t>
-        </is>
-      </c>
-      <c r="C66" s="11" t="inlineStr">
-        <is>
-          <t>Bednění z prken tl. 20 mm pod nadkrokevní PIR (biodeska/palubka)</t>
-        </is>
-      </c>
-      <c r="D66" s="10" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E66" s="12" t="n">
-        <v>140.94</v>
-      </c>
-      <c r="F66" s="11">
-        <f> 141 m² (plocha střechy včetně sklonu + přesahy)</f>
+      <c r="C67" s="15" t="inlineStr">
+        <is>
+          <t>Dodávka hranolového řeziva C24 pro námětky 60/100 mm vč. 10 % prořezu + impregnace</t>
+        </is>
+      </c>
+      <c r="D67" s="14" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="E67" s="16" t="n">
+        <v>0.127</v>
+      </c>
+      <c r="F67" s="15">
+        <f> 19.2 × 0.06 × 0.10 × 1.10 = 0.127 m³</f>
         <v/>
       </c>
-      <c r="G66" s="11" t="inlineStr">
-        <is>
-          <t>762341711</t>
-        </is>
-      </c>
-      <c r="H66" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I66" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV5.007</t>
-        </is>
-      </c>
-      <c r="J66" s="11" t="inlineStr">
-        <is>
-          <t>S10</t>
-        </is>
-      </c>
-      <c r="K66" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" s="10" t="n">
-        <v>61</v>
-      </c>
-      <c r="B67" s="11" t="inlineStr">
-        <is>
-          <t>HSV-5 Krov + střecha</t>
-        </is>
-      </c>
-      <c r="C67" s="11" t="inlineStr">
-        <is>
-          <t>Parotěsná folie nad bedněním pod nadkrokevní PIR (např. Isover Vario nebo Tyvek Air guard)</t>
-        </is>
-      </c>
-      <c r="D67" s="10" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E67" s="12" t="n">
-        <v>155.034</v>
-      </c>
-      <c r="F67" s="11" t="inlineStr">
-        <is>
-          <t>141 × 1.1 přesah = 155</t>
-        </is>
-      </c>
-      <c r="G67" s="11" t="inlineStr">
-        <is>
-          <t>712311101</t>
-        </is>
-      </c>
-      <c r="H67" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I67" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV5.008</t>
-        </is>
-      </c>
-      <c r="J67" s="11" t="inlineStr">
-        <is>
-          <t>S10</t>
-        </is>
-      </c>
-      <c r="K67" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+      <c r="G67" s="15" t="inlineStr">
+        <is>
+          <t>605</t>
+        </is>
+      </c>
+      <c r="H67" s="14" t="inlineStr">
+        <is>
+          <t>⚠ família ??? (ÚRS online)</t>
+        </is>
+      </c>
+      <c r="I67" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV5.004 → HSV5.004b</t>
+        </is>
+      </c>
+      <c r="J67" s="15" t="inlineStr"/>
+      <c r="K67" s="15" t="inlineStr">
+        <is>
+          <t>Hranol řezivo 605 família — leaf dle krátké délky &lt;6 m (60512136 je 6-8 m). Verify.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -4935,41 +4930,38 @@
       </c>
       <c r="C68" s="11" t="inlineStr">
         <is>
-          <t>Nadkrokevní tepelná izolace PIR (polyisokyanurát) tl. 160 mm (λ=0,022 W/mK) — řez A-A S10 explicit</t>
+          <t>Ocelová středová vaznice HEA160 — 2 ks × cca 10 m délka</t>
         </is>
       </c>
       <c r="D68" s="10" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E68" s="12" t="n">
-        <v>140.94</v>
-      </c>
-      <c r="F68" s="11">
-        <f> 141 m² (plocha krytiny krov)</f>
-        <v/>
+        <v>608</v>
+      </c>
+      <c r="F68" s="11" t="inlineStr">
+        <is>
+          <t>2 × 10 × 30.4 kg/m (HEA160) = 608</t>
+        </is>
       </c>
       <c r="G68" s="13" t="inlineStr">
         <is>
-          <t>713131811</t>
+          <t>411321414</t>
         </is>
       </c>
       <c r="H68" s="10" t="inlineStr">
         <is>
-          <t>✓ verified</t>
+          <t>⚠ kandidát-verify</t>
         </is>
       </c>
       <c r="I68" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.009</t>
-        </is>
-      </c>
-      <c r="J68" s="11" t="inlineStr">
-        <is>
-          <t>S10</t>
-        </is>
-      </c>
+          <t>260219_dum.HSV5.005</t>
+        </is>
+      </c>
+      <c r="J68" s="11" t="inlineStr"/>
       <c r="K68" s="11" t="inlineStr">
         <is>
           <t>Carried 1:1 (atomic — no decomposition needed)</t>
@@ -4987,25 +4979,25 @@
       </c>
       <c r="C69" s="11" t="inlineStr">
         <is>
-          <t>Doplňková hydroizolační difuzně otevřená folie nad PIR pod kontralatě</t>
+          <t>Ocelové sloupky uzavřený profil 100×100×4 mm pod vaznice HEA160 (~6 ks × ~2.5 m výška)</t>
         </is>
       </c>
       <c r="D69" s="10" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>kg</t>
         </is>
       </c>
       <c r="E69" s="12" t="n">
-        <v>155.034</v>
+        <v>176</v>
       </c>
       <c r="F69" s="11" t="inlineStr">
         <is>
-          <t>141 × 1.1 přesah = 155</t>
+          <t>6 × 2.5 × 11.7 kg/m (RHS 100×100×4) = 176</t>
         </is>
       </c>
       <c r="G69" s="11" t="inlineStr">
         <is>
-          <t>712311111</t>
+          <t>411321414</t>
         </is>
       </c>
       <c r="H69" s="10" t="inlineStr">
@@ -5015,14 +5007,10 @@
       </c>
       <c r="I69" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.010</t>
-        </is>
-      </c>
-      <c r="J69" s="11" t="inlineStr">
-        <is>
-          <t>S10</t>
-        </is>
-      </c>
+          <t>260219_dum.HSV5.006</t>
+        </is>
+      </c>
+      <c r="J69" s="11" t="inlineStr"/>
       <c r="K69" s="11" t="inlineStr">
         <is>
           <t>Carried 1:1 (atomic — no decomposition needed)</t>
@@ -5040,7 +5028,7 @@
       </c>
       <c r="C70" s="11" t="inlineStr">
         <is>
-          <t>Distanční kontralatě 40×60 mm pro vzduchovou mezeru nad PIR</t>
+          <t>Bednění z prken tl. 20 mm pod nadkrokevní PIR (biodeska/palubka)</t>
         </is>
       </c>
       <c r="D70" s="10" t="inlineStr">
@@ -5052,12 +5040,12 @@
         <v>140.94</v>
       </c>
       <c r="F70" s="11">
-        <f> 141 m²</f>
+        <f> 141 m² (plocha střechy včetně sklonu + přesahy)</f>
         <v/>
       </c>
       <c r="G70" s="11" t="inlineStr">
         <is>
-          <t>762331923</t>
+          <t>762341711</t>
         </is>
       </c>
       <c r="H70" s="10" t="inlineStr">
@@ -5067,7 +5055,7 @@
       </c>
       <c r="I70" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.011</t>
+          <t>260219_dum.HSV5.007</t>
         </is>
       </c>
       <c r="J70" s="11" t="inlineStr">
@@ -5092,7 +5080,7 @@
       </c>
       <c r="C71" s="11" t="inlineStr">
         <is>
-          <t>Bednění z prken tl. 25 mm pod plechovou hliníkovou krytinu (rozsah dle technologie krytiny)</t>
+          <t>Parotěsná folie nad bedněním pod nadkrokevní PIR (např. Isover Vario nebo Tyvek Air guard)</t>
         </is>
       </c>
       <c r="D71" s="10" t="inlineStr">
@@ -5101,15 +5089,16 @@
         </is>
       </c>
       <c r="E71" s="12" t="n">
-        <v>140.94</v>
-      </c>
-      <c r="F71" s="11">
-        <f> 141 m²</f>
-        <v/>
-      </c>
-      <c r="G71" s="13" t="inlineStr">
-        <is>
-          <t>762341711</t>
+        <v>155.034</v>
+      </c>
+      <c r="F71" s="11" t="inlineStr">
+        <is>
+          <t>141 × 1.1 přesah = 155</t>
+        </is>
+      </c>
+      <c r="G71" s="11" t="inlineStr">
+        <is>
+          <t>712311101</t>
         </is>
       </c>
       <c r="H71" s="10" t="inlineStr">
@@ -5119,7 +5108,7 @@
       </c>
       <c r="I71" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.012</t>
+          <t>260219_dum.HSV5.008</t>
         </is>
       </c>
       <c r="J71" s="11" t="inlineStr">
@@ -5144,7 +5133,7 @@
       </c>
       <c r="C72" s="11" t="inlineStr">
         <is>
-          <t>Plechová falcovaná HLINÍKOVÁ krytina (např. PREFA, Rheinzink, Lindab) + tlumící podložka</t>
+          <t>Nadkrokevní tepelná izolace PIR (polyisokyanurát) tl. 160 mm (λ=0,022 W/mK) — řez A-A S10 explicit</t>
         </is>
       </c>
       <c r="D72" s="10" t="inlineStr">
@@ -5156,22 +5145,22 @@
         <v>140.94</v>
       </c>
       <c r="F72" s="11">
-        <f> 141 m² (vč. vikýřů přidat ~10%)</f>
+        <f> 141 m² (plocha krytiny krov)</f>
         <v/>
       </c>
       <c r="G72" s="13" t="inlineStr">
         <is>
-          <t>765791121</t>
+          <t>713131811</t>
         </is>
       </c>
       <c r="H72" s="10" t="inlineStr">
         <is>
-          <t>⚠ kandidát-verify</t>
+          <t>✓ verified</t>
         </is>
       </c>
       <c r="I72" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.013</t>
+          <t>260219_dum.HSV5.009</t>
         </is>
       </c>
       <c r="J72" s="11" t="inlineStr">
@@ -5196,7 +5185,7 @@
       </c>
       <c r="C73" s="11" t="inlineStr">
         <is>
-          <t>Patro pro přespání v krovu — biodeska / OSB desky tl. 22 mm nad kleštinami</t>
+          <t>Doplňková hydroizolační difuzně otevřená folie nad PIR pod kontralatě</t>
         </is>
       </c>
       <c r="D73" s="10" t="inlineStr">
@@ -5205,16 +5194,16 @@
         </is>
       </c>
       <c r="E73" s="12" t="n">
-        <v>25</v>
+        <v>155.034</v>
       </c>
       <c r="F73" s="11" t="inlineStr">
         <is>
-          <t>odhad — spací patro ~5 × 5 m</t>
+          <t>141 × 1.1 přesah = 155</t>
         </is>
       </c>
       <c r="G73" s="11" t="inlineStr">
         <is>
-          <t>762341711</t>
+          <t>712311111</t>
         </is>
       </c>
       <c r="H73" s="10" t="inlineStr">
@@ -5224,12 +5213,12 @@
       </c>
       <c r="I73" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.014</t>
+          <t>260219_dum.HSV5.010</t>
         </is>
       </c>
       <c r="J73" s="11" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="K73" s="11" t="inlineStr">
@@ -5249,7 +5238,7 @@
       </c>
       <c r="C74" s="11" t="inlineStr">
         <is>
-          <t>Vikýře — zděná čela z Porotherm 30 (odhad 4 ks × ~3 m² stěna)</t>
+          <t>Distanční kontralatě 40×60 mm pro vzduchovou mezeru nad PIR</t>
         </is>
       </c>
       <c r="D74" s="10" t="inlineStr">
@@ -5258,16 +5247,15 @@
         </is>
       </c>
       <c r="E74" s="12" t="n">
-        <v>12</v>
-      </c>
-      <c r="F74" s="11" t="inlineStr">
-        <is>
-          <t>4 vikýře × ~3 m² zděných čel = 12</t>
-        </is>
+        <v>140.94</v>
+      </c>
+      <c r="F74" s="11">
+        <f> 141 m²</f>
+        <v/>
       </c>
       <c r="G74" s="11" t="inlineStr">
         <is>
-          <t>311321411</t>
+          <t>762331923</t>
         </is>
       </c>
       <c r="H74" s="10" t="inlineStr">
@@ -5277,10 +5265,14 @@
       </c>
       <c r="I74" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.015</t>
-        </is>
-      </c>
-      <c r="J74" s="11" t="inlineStr"/>
+          <t>260219_dum.HSV5.011</t>
+        </is>
+      </c>
+      <c r="J74" s="11" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
       <c r="K74" s="11" t="inlineStr">
         <is>
           <t>Carried 1:1 (atomic — no decomposition needed)</t>
@@ -5298,7 +5290,7 @@
       </c>
       <c r="C75" s="11" t="inlineStr">
         <is>
-          <t>Vikýře — provětrávaná fasáda min. vata + plech falcovaný hliník (4 vikýře × ~6 m² fasády)</t>
+          <t>Bednění z prken tl. 25 mm pod plechovou hliníkovou krytinu (rozsah dle technologie krytiny)</t>
         </is>
       </c>
       <c r="D75" s="10" t="inlineStr">
@@ -5307,179 +5299,222 @@
         </is>
       </c>
       <c r="E75" s="12" t="n">
-        <v>24</v>
-      </c>
-      <c r="F75" s="11" t="inlineStr">
-        <is>
-          <t>4 vikýře × 2 strany × ~3 m² = 24</t>
-        </is>
-      </c>
-      <c r="G75" s="11" t="inlineStr">
+        <v>140.94</v>
+      </c>
+      <c r="F75" s="11">
+        <f> 141 m²</f>
+        <v/>
+      </c>
+      <c r="G75" s="13" t="inlineStr">
+        <is>
+          <t>762341711</t>
+        </is>
+      </c>
+      <c r="H75" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I75" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV5.012</t>
+        </is>
+      </c>
+      <c r="J75" s="11" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="K75" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="10" t="n">
+        <v>70</v>
+      </c>
+      <c r="B76" s="11" t="inlineStr">
+        <is>
+          <t>HSV-5 Krov + střecha</t>
+        </is>
+      </c>
+      <c r="C76" s="11" t="inlineStr">
+        <is>
+          <t>Plechová falcovaná HLINÍKOVÁ krytina (např. PREFA, Rheinzink, Lindab) + tlumící podložka</t>
+        </is>
+      </c>
+      <c r="D76" s="10" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E76" s="12" t="n">
+        <v>140.94</v>
+      </c>
+      <c r="F76" s="11">
+        <f> 141 m² (vč. vikýřů přidat ~10%)</f>
+        <v/>
+      </c>
+      <c r="G76" s="13" t="inlineStr">
         <is>
           <t>765791121</t>
         </is>
       </c>
-      <c r="H75" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I75" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV5.016</t>
-        </is>
-      </c>
-      <c r="J75" s="11" t="inlineStr">
-        <is>
-          <t>S12b</t>
-        </is>
-      </c>
-      <c r="K75" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="76">
-      <c r="A76" s="8" t="inlineStr">
-        <is>
-          <t>━━ HSV-6 Bourací práce  (17 atomic operací) ━━</t>
-        </is>
-      </c>
-      <c r="B76" s="9" t="n"/>
-      <c r="C76" s="9" t="n"/>
-      <c r="D76" s="9" t="n"/>
-      <c r="E76" s="9" t="n"/>
-      <c r="F76" s="9" t="n"/>
-      <c r="G76" s="9" t="n"/>
-      <c r="H76" s="9" t="n"/>
-      <c r="I76" s="9" t="n"/>
-      <c r="J76" s="9" t="n"/>
-      <c r="K76" s="9" t="n"/>
+      <c r="H76" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I76" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV5.013</t>
+        </is>
+      </c>
+      <c r="J76" s="11" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+      <c r="K76" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="10" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B77" s="11" t="inlineStr">
         <is>
-          <t>HSV-6 Bourací práce</t>
+          <t>HSV-5 Krov + střecha</t>
         </is>
       </c>
       <c r="C77" s="11" t="inlineStr">
         <is>
-          <t>Bourání kompletního stávajícího krovu vč. vikýřů — vaznicový s ležatou stolicí — manuálně, odvoz</t>
+          <t>Patro pro přespání v krovu — biodeska / OSB desky tl. 22 mm nad kleštinami</t>
         </is>
       </c>
       <c r="D77" s="10" t="inlineStr">
         <is>
-          <t>m³</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E77" s="12" t="n">
+        <v>25</v>
+      </c>
+      <c r="F77" s="11" t="inlineStr">
+        <is>
+          <t>odhad — spací patro ~5 × 5 m</t>
+        </is>
+      </c>
+      <c r="G77" s="11" t="inlineStr">
+        <is>
+          <t>762341711</t>
+        </is>
+      </c>
+      <c r="H77" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I77" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV5.014</t>
+        </is>
+      </c>
+      <c r="J77" s="11" t="inlineStr">
+        <is>
+          <t>S11</t>
+        </is>
+      </c>
+      <c r="K77" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="10" t="n">
+        <v>72</v>
+      </c>
+      <c r="B78" s="11" t="inlineStr">
+        <is>
+          <t>HSV-5 Krov + střecha</t>
+        </is>
+      </c>
+      <c r="C78" s="11" t="inlineStr">
+        <is>
+          <t>Vikýře — zděná čela z Porotherm 30 (odhad 4 ks × ~3 m² stěna)</t>
+        </is>
+      </c>
+      <c r="D78" s="10" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E78" s="12" t="n">
         <v>12</v>
       </c>
-      <c r="F77" s="11" t="inlineStr">
-        <is>
-          <t>TZ B m.10.e: 9 t dřeva × 0.75 t/m³ = 12 m³ dřeva</t>
-        </is>
-      </c>
-      <c r="G77" s="13" t="inlineStr">
-        <is>
-          <t>962041141</t>
-        </is>
-      </c>
-      <c r="H77" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I77" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV6.001</t>
-        </is>
-      </c>
-      <c r="J77" s="11" t="inlineStr"/>
-      <c r="K77" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="17" t="n">
-        <v>71</v>
-      </c>
-      <c r="B78" s="18" t="inlineStr">
-        <is>
-          <t>HSV-6 Bourací práce</t>
-        </is>
-      </c>
-      <c r="C78" s="18" t="inlineStr">
-        <is>
-          <t>Bourání stávající plechové krytiny (manuálně, recyklace plechu)</t>
-        </is>
-      </c>
-      <c r="D78" s="17" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E78" s="19" t="n">
-        <v>140.9</v>
-      </c>
-      <c r="F78" s="18">
-        <f> plocha krytiny ~141</f>
-        <v/>
-      </c>
-      <c r="G78" s="18" t="inlineStr"/>
-      <c r="H78" s="17" t="inlineStr">
-        <is>
-          <t>❌ blank — ÚRS online</t>
-        </is>
-      </c>
-      <c r="I78" s="18" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV6.002</t>
-        </is>
-      </c>
-      <c r="J78" s="18" t="inlineStr"/>
-      <c r="K78" s="18" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+      <c r="F78" s="11" t="inlineStr">
+        <is>
+          <t>4 vikýře × ~3 m² zděných čel = 12</t>
+        </is>
+      </c>
+      <c r="G78" s="11" t="inlineStr">
+        <is>
+          <t>311321411</t>
+        </is>
+      </c>
+      <c r="H78" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I78" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV5.015</t>
+        </is>
+      </c>
+      <c r="J78" s="11" t="inlineStr"/>
+      <c r="K78" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="10" t="n">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B79" s="11" t="inlineStr">
         <is>
-          <t>HSV-6 Bourací práce</t>
+          <t>HSV-5 Krov + střecha</t>
         </is>
       </c>
       <c r="C79" s="11" t="inlineStr">
         <is>
-          <t>Bourání zděných nadezdívek nad stropem 2.NP (mimo štítových stěn) — cihla pálená</t>
+          <t>Vikýře — provětrávaná fasáda min. vata + plech falcovaný hliník (4 vikýře × ~6 m² fasády)</t>
         </is>
       </c>
       <c r="D79" s="10" t="inlineStr">
         <is>
-          <t>m³</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E79" s="12" t="n">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="F79" s="11" t="inlineStr">
         <is>
-          <t>odhad — 3.NP nadezdívka půdy ~104 m² × 0.45 m výška ~6</t>
+          <t>4 vikýře × 2 strany × ~3 m² = 24</t>
         </is>
       </c>
       <c r="G79" s="11" t="inlineStr">
         <is>
-          <t>962031132</t>
+          <t>765791121</t>
         </is>
       </c>
       <c r="H79" s="10" t="inlineStr">
@@ -5489,10 +5524,14 @@
       </c>
       <c r="I79" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.003</t>
-        </is>
-      </c>
-      <c r="J79" s="11" t="inlineStr"/>
+          <t>260219_dum.HSV5.016</t>
+        </is>
+      </c>
+      <c r="J79" s="11" t="inlineStr">
+        <is>
+          <t>S12b</t>
+        </is>
+      </c>
       <c r="K79" s="11" t="inlineStr">
         <is>
           <t>Carried 1:1 (atomic — no decomposition needed)</t>
@@ -5500,52 +5539,21 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="10" t="n">
-        <v>73</v>
-      </c>
-      <c r="B80" s="11" t="inlineStr">
-        <is>
-          <t>HSV-6 Bourací práce</t>
-        </is>
-      </c>
-      <c r="C80" s="11" t="inlineStr">
-        <is>
-          <t>Bourání trámového stropu 2.NP/podkroví — kompletně (vč. zajištění schodiště)</t>
-        </is>
-      </c>
-      <c r="D80" s="10" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E80" s="12" t="n">
-        <v>104.4</v>
-      </c>
-      <c r="F80" s="11">
-        <f> zastavěna 104.4 m²</f>
-        <v/>
-      </c>
-      <c r="G80" s="11" t="inlineStr">
-        <is>
-          <t>962041141</t>
-        </is>
-      </c>
-      <c r="H80" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I80" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV6.004</t>
-        </is>
-      </c>
-      <c r="J80" s="11" t="inlineStr"/>
-      <c r="K80" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
+      <c r="A80" s="8" t="inlineStr">
+        <is>
+          <t>━━ HSV-6 Bourací práce  (17 atomic operací) ━━</t>
+        </is>
+      </c>
+      <c r="B80" s="9" t="n"/>
+      <c r="C80" s="9" t="n"/>
+      <c r="D80" s="9" t="n"/>
+      <c r="E80" s="9" t="n"/>
+      <c r="F80" s="9" t="n"/>
+      <c r="G80" s="9" t="n"/>
+      <c r="H80" s="9" t="n"/>
+      <c r="I80" s="9" t="n"/>
+      <c r="J80" s="9" t="n"/>
+      <c r="K80" s="9" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="10" t="n">
@@ -5558,25 +5566,25 @@
       </c>
       <c r="C81" s="11" t="inlineStr">
         <is>
-          <t>Bourání stávajících lehkých příček (cihla, sádrokarton, dřevo)</t>
+          <t>Bourání kompletního stávajícího krovu vč. vikýřů — vaznicový s ležatou stolicí — manuálně, odvoz</t>
         </is>
       </c>
       <c r="D81" s="10" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="E81" s="12" t="n">
-        <v>80</v>
+        <v>12</v>
       </c>
       <c r="F81" s="11" t="inlineStr">
         <is>
-          <t>odhad — interier 2 patra × ~40 m² příček = 80</t>
-        </is>
-      </c>
-      <c r="G81" s="11" t="inlineStr">
-        <is>
-          <t>962031132</t>
+          <t>TZ B m.10.e: 9 t dřeva × 0.75 t/m³ = 12 m³ dřeva</t>
+        </is>
+      </c>
+      <c r="G81" s="13" t="inlineStr">
+        <is>
+          <t>962041141</t>
         </is>
       </c>
       <c r="H81" s="10" t="inlineStr">
@@ -5586,7 +5594,7 @@
       </c>
       <c r="I81" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.005</t>
+          <t>260219_dum.HSV6.001</t>
         </is>
       </c>
       <c r="J81" s="11" t="inlineStr"/>
@@ -5597,51 +5605,46 @@
       </c>
     </row>
     <row r="82">
-      <c r="A82" s="10" t="n">
+      <c r="A82" s="17" t="n">
         <v>75</v>
       </c>
-      <c r="B82" s="11" t="inlineStr">
+      <c r="B82" s="18" t="inlineStr">
         <is>
           <t>HSV-6 Bourací práce</t>
         </is>
       </c>
-      <c r="C82" s="11" t="inlineStr">
-        <is>
-          <t>Bourání 8 nových otvorů v nosných cihelných zdech pro dveře/okna (~1.0 × 2.1 m)</t>
-        </is>
-      </c>
-      <c r="D82" s="10" t="inlineStr">
-        <is>
-          <t>ks</t>
-        </is>
-      </c>
-      <c r="E82" s="12" t="n">
-        <v>8</v>
-      </c>
-      <c r="F82" s="11" t="inlineStr">
-        <is>
-          <t>odhad počtu nových otvorů (= počet IPN160 překladů)</t>
-        </is>
-      </c>
-      <c r="G82" s="11" t="inlineStr">
-        <is>
-          <t>962031132</t>
-        </is>
-      </c>
-      <c r="H82" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I82" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV6.006</t>
-        </is>
-      </c>
-      <c r="J82" s="11" t="inlineStr"/>
-      <c r="K82" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+      <c r="C82" s="18" t="inlineStr">
+        <is>
+          <t>Bourání stávající plechové krytiny (manuálně, recyklace plechu)</t>
+        </is>
+      </c>
+      <c r="D82" s="17" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E82" s="19" t="n">
+        <v>140.9</v>
+      </c>
+      <c r="F82" s="18">
+        <f> plocha krytiny ~141</f>
+        <v/>
+      </c>
+      <c r="G82" s="18" t="inlineStr"/>
+      <c r="H82" s="17" t="inlineStr">
+        <is>
+          <t>❌ blank — ÚRS online</t>
+        </is>
+      </c>
+      <c r="I82" s="18" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV6.002</t>
+        </is>
+      </c>
+      <c r="J82" s="18" t="inlineStr"/>
+      <c r="K82" s="18" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -5656,25 +5659,25 @@
       </c>
       <c r="C83" s="11" t="inlineStr">
         <is>
-          <t>Bourání keramických obkladů a zařizovacích předmětů v koupelnách 1.NP + 2.NP</t>
+          <t>Bourání zděných nadezdívek nad stropem 2.NP (mimo štítových stěn) — cihla pálená</t>
         </is>
       </c>
       <c r="D83" s="10" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="E83" s="12" t="n">
-        <v>60</v>
+        <v>6</v>
       </c>
       <c r="F83" s="11" t="inlineStr">
         <is>
-          <t>2 koupelny × ~30 m² obkladů = 60</t>
-        </is>
-      </c>
-      <c r="G83" s="13" t="inlineStr">
-        <is>
-          <t>781473810</t>
+          <t>odhad — 3.NP nadezdívka půdy ~104 m² × 0.45 m výška ~6</t>
+        </is>
+      </c>
+      <c r="G83" s="11" t="inlineStr">
+        <is>
+          <t>962031132</t>
         </is>
       </c>
       <c r="H83" s="10" t="inlineStr">
@@ -5684,7 +5687,7 @@
       </c>
       <c r="I83" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.007</t>
+          <t>260219_dum.HSV6.003</t>
         </is>
       </c>
       <c r="J83" s="11" t="inlineStr"/>
@@ -5705,7 +5708,7 @@
       </c>
       <c r="C84" s="11" t="inlineStr">
         <is>
-          <t>Sejmutí podlah 1.NP a 2.NP — vč. nášlapů, podkladních vrstev</t>
+          <t>Bourání trámového stropu 2.NP/podkroví — kompletně (vč. zajištění schodiště)</t>
         </is>
       </c>
       <c r="D84" s="10" t="inlineStr">
@@ -5714,16 +5717,15 @@
         </is>
       </c>
       <c r="E84" s="12" t="n">
-        <v>153.51</v>
-      </c>
-      <c r="F84" s="11" t="inlineStr">
-        <is>
-          <t>podlahova × 0.7 = ~154 m² (bez 3.NP nového)</t>
-        </is>
+        <v>104.4</v>
+      </c>
+      <c r="F84" s="11">
+        <f> zastavěna 104.4 m²</f>
+        <v/>
       </c>
       <c r="G84" s="11" t="inlineStr">
         <is>
-          <t>974031132</t>
+          <t>962041141</t>
         </is>
       </c>
       <c r="H84" s="10" t="inlineStr">
@@ -5733,7 +5735,7 @@
       </c>
       <c r="I84" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.008</t>
+          <t>260219_dum.HSV6.004</t>
         </is>
       </c>
       <c r="J84" s="11" t="inlineStr"/>
@@ -5754,25 +5756,25 @@
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Demontáž záklopu a zásypů stropu 1.NP (prkenný záklop na trámech zachován)</t>
+          <t>Bourání stávajících lehkých příček (cihla, sádrokarton, dřevo)</t>
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t>m³</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E85" s="12" t="n">
-        <v>5</v>
+        <v>80</v>
       </c>
       <c r="F85" s="11" t="inlineStr">
         <is>
-          <t>100 m² × 0.05 m tl. zásypu = 5</t>
+          <t>odhad — interier 2 patra × ~40 m² příček = 80</t>
         </is>
       </c>
       <c r="G85" s="11" t="inlineStr">
         <is>
-          <t>974041151</t>
+          <t>962031132</t>
         </is>
       </c>
       <c r="H85" s="10" t="inlineStr">
@@ -5782,7 +5784,7 @@
       </c>
       <c r="I85" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.009</t>
+          <t>260219_dum.HSV6.005</t>
         </is>
       </c>
       <c r="J85" s="11" t="inlineStr"/>
@@ -5803,7 +5805,7 @@
       </c>
       <c r="C86" s="11" t="inlineStr">
         <is>
-          <t>Demontáž všech oken a dveří stávajících (recyklace)</t>
+          <t>Bourání 8 nových otvorů v nosných cihelných zdech pro dveře/okna (~1.0 × 2.1 m)</t>
         </is>
       </c>
       <c r="D86" s="10" t="inlineStr">
@@ -5812,16 +5814,16 @@
         </is>
       </c>
       <c r="E86" s="12" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="F86" s="11" t="inlineStr">
         <is>
-          <t>odhad — ~10 oken + ~15 dveří (vstupní + vnitřní)</t>
+          <t>odhad počtu nových otvorů (= počet IPN160 překladů)</t>
         </is>
       </c>
       <c r="G86" s="11" t="inlineStr">
         <is>
-          <t>968071120</t>
+          <t>962031132</t>
         </is>
       </c>
       <c r="H86" s="10" t="inlineStr">
@@ -5831,7 +5833,7 @@
       </c>
       <c r="I86" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.010</t>
+          <t>260219_dum.HSV6.006</t>
         </is>
       </c>
       <c r="J86" s="11" t="inlineStr"/>
@@ -5852,25 +5854,25 @@
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>Demontáž všech sanitárních zařizovacích předmětů (WC, umyvadla, baterie, sprcha)</t>
+          <t>Bourání keramických obkladů a zařizovacích předmětů v koupelnách 1.NP + 2.NP</t>
         </is>
       </c>
       <c r="D87" s="10" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E87" s="12" t="n">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="F87" s="11" t="inlineStr">
         <is>
-          <t>odhad — 2 koupelny × ~5 ks + WC + dřez = ~12</t>
-        </is>
-      </c>
-      <c r="G87" s="11" t="inlineStr">
-        <is>
-          <t>725900001</t>
+          <t>2 koupelny × ~30 m² obkladů = 60</t>
+        </is>
+      </c>
+      <c r="G87" s="13" t="inlineStr">
+        <is>
+          <t>781473810</t>
         </is>
       </c>
       <c r="H87" s="10" t="inlineStr">
@@ -5880,7 +5882,7 @@
       </c>
       <c r="I87" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.011</t>
+          <t>260219_dum.HSV6.007</t>
         </is>
       </c>
       <c r="J87" s="11" t="inlineStr"/>
@@ -5901,25 +5903,25 @@
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
-          <t>Odvoz a likvidace stavební suti dle vyhl. 8/2021 Sb. — celková tonáž odpadů</t>
+          <t>Sejmutí podlah 1.NP a 2.NP — vč. nášlapů, podkladních vrstev</t>
         </is>
       </c>
       <c r="D88" s="10" t="inlineStr">
         <is>
-          <t>t</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E88" s="12" t="n">
-        <v>56.5</v>
+        <v>153.51</v>
       </c>
       <c r="F88" s="11" t="inlineStr">
         <is>
-          <t>TZ B m.10.e: 46 (beton/cihly) + 9 (dřevo) + 0.1 (kov) + 0.1 (EPS) + 0.2 (sádra) + 1.0 (směs) = 56.4</t>
+          <t>podlahova × 0.7 = ~154 m² (bez 3.NP nového)</t>
         </is>
       </c>
       <c r="G88" s="11" t="inlineStr">
         <is>
-          <t>997013501</t>
+          <t>974031132</t>
         </is>
       </c>
       <c r="H88" s="10" t="inlineStr">
@@ -5929,7 +5931,7 @@
       </c>
       <c r="I88" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.012</t>
+          <t>260219_dum.HSV6.008</t>
         </is>
       </c>
       <c r="J88" s="11" t="inlineStr"/>
@@ -5950,35 +5952,35 @@
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>Demontáž stávajících dřevěných oken vč. rámů a parapetů — 16 ks (návrh všechna okna nová plastová trojsklem)</t>
+          <t>Demontáž záklopu a zásypů stropu 1.NP (prkenný záklop na trámech zachován)</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="E89" s="12" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="F89" s="11" t="inlineStr">
         <is>
-          <t>DXF INSERT okno* total 16 ks (Path C Tier 4 — front 9 + back 7)</t>
-        </is>
-      </c>
-      <c r="G89" s="13" t="inlineStr">
-        <is>
-          <t>978013181</t>
+          <t>100 m² × 0.05 m tl. zásypu = 5</t>
+        </is>
+      </c>
+      <c r="G89" s="11" t="inlineStr">
+        <is>
+          <t>974041151</t>
         </is>
       </c>
       <c r="H89" s="10" t="inlineStr">
         <is>
-          <t>✓ verified</t>
+          <t>⚠ kandidát-verify</t>
         </is>
       </c>
       <c r="I89" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.013</t>
+          <t>260219_dum.HSV6.009</t>
         </is>
       </c>
       <c r="J89" s="11" t="inlineStr"/>
@@ -5999,7 +6001,7 @@
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>Demontáž stávajících vstupních dveří + rámů — 2 ks (1× ulice Fibichova + 1× zahrada; návrh nové plastové vstupní dveře)</t>
+          <t>Demontáž všech oken a dveří stávajících (recyklace)</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr">
@@ -6008,26 +6010,26 @@
         </is>
       </c>
       <c r="E90" s="12" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="F90" s="11" t="inlineStr">
         <is>
-          <t>DXF INSERT dveře = 2 (Path C Tier 4) + TZ ARS</t>
-        </is>
-      </c>
-      <c r="G90" s="13" t="inlineStr">
-        <is>
-          <t>978013181</t>
+          <t>odhad — ~10 oken + ~15 dveří (vstupní + vnitřní)</t>
+        </is>
+      </c>
+      <c r="G90" s="11" t="inlineStr">
+        <is>
+          <t>968071120</t>
         </is>
       </c>
       <c r="H90" s="10" t="inlineStr">
         <is>
-          <t>✓ verified</t>
+          <t>⚠ kandidát-verify</t>
         </is>
       </c>
       <c r="I90" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.014</t>
+          <t>260219_dum.HSV6.010</t>
         </is>
       </c>
       <c r="J90" s="11" t="inlineStr"/>
@@ -6048,7 +6050,7 @@
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>Demontáž stávajících vnitřních dveří vč. ocelových/dřevěných zárubní — odhad 15 ks (3 patra × ~5 dveří/patro per DXF SM__dveře layer)</t>
+          <t>Demontáž všech sanitárních zařizovacích předmětů (WC, umyvadla, baterie, sprcha)</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
@@ -6057,16 +6059,16 @@
         </is>
       </c>
       <c r="E91" s="12" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F91" s="11" t="inlineStr">
         <is>
-          <t>DXF SM__dveře polylines 102 / ~3 fáze / ~2.3 symbol per dveře ≈ 15 ks návrh (Path C confidence 0.65)</t>
+          <t>odhad — 2 koupelny × ~5 ks + WC + dřez = ~12</t>
         </is>
       </c>
       <c r="G91" s="11" t="inlineStr">
         <is>
-          <t>968072456</t>
+          <t>725900001</t>
         </is>
       </c>
       <c r="H91" s="10" t="inlineStr">
@@ -6076,7 +6078,7 @@
       </c>
       <c r="I91" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.015</t>
+          <t>260219_dum.HSV6.011</t>
         </is>
       </c>
       <c r="J91" s="11" t="inlineStr"/>
@@ -6097,25 +6099,25 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>Bourání vrchní části stávajícího komínu v posledním podlaží (cihelné zdivo, ručně), vč. likvidace cihelné suti</t>
+          <t>Odvoz a likvidace stavební suti dle vyhl. 8/2021 Sb. — celková tonáž odpadů</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t>m³</t>
+          <t>t</t>
         </is>
       </c>
       <c r="E92" s="12" t="n">
-        <v>0.6</v>
+        <v>56.5</v>
       </c>
       <c r="F92" s="11" t="inlineStr">
         <is>
-          <t>průměr komín 0.50×0.50 × výška nad střechou ~2.4 m = 0.6 m³ (OPRAVA ChatGPT revize 2026-05-29: dříve 6.0 m³ = ×10 chybná inflace; skutečný objem 0.6 m³)</t>
-        </is>
-      </c>
-      <c r="G92" s="13" t="inlineStr">
-        <is>
-          <t>962024141</t>
+          <t>TZ B m.10.e: 46 (beton/cihly) + 9 (dřevo) + 0.1 (kov) + 0.1 (EPS) + 0.2 (sádra) + 1.0 (směs) = 56.4</t>
+        </is>
+      </c>
+      <c r="G92" s="11" t="inlineStr">
+        <is>
+          <t>997013501</t>
         </is>
       </c>
       <c r="H92" s="10" t="inlineStr">
@@ -6125,7 +6127,7 @@
       </c>
       <c r="I92" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.016</t>
+          <t>260219_dum.HSV6.012</t>
         </is>
       </c>
       <c r="J92" s="11" t="inlineStr"/>
@@ -6146,35 +6148,35 @@
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>Bourání stávajících opěrných zídek a venkovního schodiště v zahradě/dvoře — částečné, dle vyznačení v půdorysech bourání</t>
+          <t>Demontáž stávajících dřevěných oken vč. rámů a parapetů — 16 ks (návrh všechna okna nová plastová trojsklem)</t>
         </is>
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t>m³</t>
+          <t>ks</t>
         </is>
       </c>
       <c r="E93" s="12" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F93" s="11" t="inlineStr">
         <is>
-          <t>odhad ze řez A-A bourání + půdorys bourání 1.NP/1.PP, ~8 m³ celkem (opěrné zídky + venkovní schodiště zahrada/dvůr)</t>
+          <t>DXF INSERT okno* total 16 ks (Path C Tier 4 — front 9 + back 7)</t>
         </is>
       </c>
       <c r="G93" s="13" t="inlineStr">
         <is>
-          <t>961044111</t>
+          <t>978013181</t>
         </is>
       </c>
       <c r="H93" s="10" t="inlineStr">
         <is>
-          <t>⚠ kandidát-verify</t>
+          <t>✓ verified</t>
         </is>
       </c>
       <c r="I93" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.017</t>
+          <t>260219_dum.HSV6.013</t>
         </is>
       </c>
       <c r="J93" s="11" t="inlineStr"/>
@@ -6185,280 +6187,268 @@
       </c>
     </row>
     <row r="94">
-      <c r="A94" s="8" t="inlineStr">
-        <is>
-          <t>━━ HSV-7 Fasáda ETICS  (9 atomic operací) ━━</t>
-        </is>
-      </c>
-      <c r="B94" s="9" t="n"/>
-      <c r="C94" s="9" t="n"/>
-      <c r="D94" s="9" t="n"/>
-      <c r="E94" s="9" t="n"/>
-      <c r="F94" s="9" t="n"/>
-      <c r="G94" s="9" t="n"/>
-      <c r="H94" s="9" t="n"/>
-      <c r="I94" s="9" t="n"/>
-      <c r="J94" s="9" t="n"/>
-      <c r="K94" s="9" t="n"/>
+      <c r="A94" s="10" t="n">
+        <v>87</v>
+      </c>
+      <c r="B94" s="11" t="inlineStr">
+        <is>
+          <t>HSV-6 Bourací práce</t>
+        </is>
+      </c>
+      <c r="C94" s="11" t="inlineStr">
+        <is>
+          <t>Demontáž stávajících vstupních dveří + rámů — 2 ks (1× ulice Fibichova + 1× zahrada; návrh nové plastové vstupní dveře)</t>
+        </is>
+      </c>
+      <c r="D94" s="10" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="E94" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F94" s="11" t="inlineStr">
+        <is>
+          <t>DXF INSERT dveře = 2 (Path C Tier 4) + TZ ARS</t>
+        </is>
+      </c>
+      <c r="G94" s="13" t="inlineStr">
+        <is>
+          <t>978013181</t>
+        </is>
+      </c>
+      <c r="H94" s="10" t="inlineStr">
+        <is>
+          <t>✓ verified</t>
+        </is>
+      </c>
+      <c r="I94" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV6.014</t>
+        </is>
+      </c>
+      <c r="J94" s="11" t="inlineStr"/>
+      <c r="K94" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="10" t="n">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B95" s="11" t="inlineStr">
         <is>
+          <t>HSV-6 Bourací práce</t>
+        </is>
+      </c>
+      <c r="C95" s="11" t="inlineStr">
+        <is>
+          <t>Demontáž stávajících vnitřních dveří vč. ocelových/dřevěných zárubní — odhad 15 ks (3 patra × ~5 dveří/patro per DXF SM__dveře layer)</t>
+        </is>
+      </c>
+      <c r="D95" s="10" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="E95" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="F95" s="11" t="inlineStr">
+        <is>
+          <t>DXF SM__dveře polylines 102 / ~3 fáze / ~2.3 symbol per dveře ≈ 15 ks návrh (Path C confidence 0.65)</t>
+        </is>
+      </c>
+      <c r="G95" s="11" t="inlineStr">
+        <is>
+          <t>968072456</t>
+        </is>
+      </c>
+      <c r="H95" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I95" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV6.015</t>
+        </is>
+      </c>
+      <c r="J95" s="11" t="inlineStr"/>
+      <c r="K95" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="10" t="n">
+        <v>89</v>
+      </c>
+      <c r="B96" s="11" t="inlineStr">
+        <is>
+          <t>HSV-6 Bourací práce</t>
+        </is>
+      </c>
+      <c r="C96" s="11" t="inlineStr">
+        <is>
+          <t>Bourání vrchní části stávajícího komínu v posledním podlaží (cihelné zdivo, ručně), vč. likvidace cihelné suti</t>
+        </is>
+      </c>
+      <c r="D96" s="10" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="E96" s="12" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F96" s="11" t="inlineStr">
+        <is>
+          <t>průměr komín 0.50×0.50 × výška nad střechou ~2.4 m = 0.6 m³ (OPRAVA ChatGPT revize 2026-05-29: dříve 6.0 m³ = ×10 chybná inflace; skutečný objem 0.6 m³)</t>
+        </is>
+      </c>
+      <c r="G96" s="13" t="inlineStr">
+        <is>
+          <t>962024141</t>
+        </is>
+      </c>
+      <c r="H96" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I96" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV6.016</t>
+        </is>
+      </c>
+      <c r="J96" s="11" t="inlineStr"/>
+      <c r="K96" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="10" t="n">
+        <v>90</v>
+      </c>
+      <c r="B97" s="11" t="inlineStr">
+        <is>
+          <t>HSV-6 Bourací práce</t>
+        </is>
+      </c>
+      <c r="C97" s="11" t="inlineStr">
+        <is>
+          <t>Bourání stávajících opěrných zídek a venkovního schodiště v zahradě/dvoře — částečné, dle vyznačení v půdorysech bourání</t>
+        </is>
+      </c>
+      <c r="D97" s="10" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="E97" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="F97" s="11" t="inlineStr">
+        <is>
+          <t>odhad ze řez A-A bourání + půdorys bourání 1.NP/1.PP, ~8 m³ celkem (opěrné zídky + venkovní schodiště zahrada/dvůr)</t>
+        </is>
+      </c>
+      <c r="G97" s="13" t="inlineStr">
+        <is>
+          <t>961044111</t>
+        </is>
+      </c>
+      <c r="H97" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I97" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV6.017</t>
+        </is>
+      </c>
+      <c r="J97" s="11" t="inlineStr"/>
+      <c r="K97" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="8" t="inlineStr">
+        <is>
+          <t>━━ HSV-7 Fasáda ETICS  (9 atomic operací) ━━</t>
+        </is>
+      </c>
+      <c r="B98" s="9" t="n"/>
+      <c r="C98" s="9" t="n"/>
+      <c r="D98" s="9" t="n"/>
+      <c r="E98" s="9" t="n"/>
+      <c r="F98" s="9" t="n"/>
+      <c r="G98" s="9" t="n"/>
+      <c r="H98" s="9" t="n"/>
+      <c r="I98" s="9" t="n"/>
+      <c r="J98" s="9" t="n"/>
+      <c r="K98" s="9" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="10" t="n">
+        <v>91</v>
+      </c>
+      <c r="B99" s="11" t="inlineStr">
+        <is>
           <t>HSV-7 Fasáda ETICS</t>
         </is>
       </c>
-      <c r="C95" s="11" t="inlineStr">
+      <c r="C99" s="11" t="inlineStr">
         <is>
           <t>Příprava fasádního podkladu — očištění tlakovou vodou, vyspravení omítek, fungicidní nátěr</t>
         </is>
       </c>
-      <c r="D95" s="10" t="inlineStr">
+      <c r="D99" s="10" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E95" s="12" t="n">
+      <c r="E99" s="12" t="n">
         <v>276.7</v>
       </c>
-      <c r="F95" s="11" t="inlineStr">
+      <c r="F99" s="11" t="inlineStr">
         <is>
           <t>obvod 38.7 m (DXF) × 0.55 (volná fasáda, štíty zachované) × výška 13.0 m = 276.7 m²</t>
         </is>
       </c>
-      <c r="G95" s="11" t="inlineStr">
+      <c r="G99" s="11" t="inlineStr">
         <is>
           <t>622401110</t>
         </is>
       </c>
-      <c r="H95" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I95" s="11" t="inlineStr">
+      <c r="H99" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I99" s="11" t="inlineStr">
         <is>
           <t>260219_dum.HSV7.001</t>
         </is>
       </c>
-      <c r="J95" s="11" t="inlineStr">
+      <c r="J99" s="11" t="inlineStr">
         <is>
           <t>S01</t>
         </is>
       </c>
-      <c r="K95" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="96">
-      <c r="A96" s="14" t="n">
-        <v>88</v>
-      </c>
-      <c r="B96" s="15" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda ETICS</t>
-        </is>
-      </c>
-      <c r="C96" s="15" t="inlineStr">
-        <is>
-          <t>Lepení + kotvení desek EPS 70F grey λ=0.032 tl. 160 mm — ETICS kontaktní zateplení fasády</t>
-        </is>
-      </c>
-      <c r="D96" s="14" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E96" s="16" t="n">
-        <v>276.7</v>
-      </c>
-      <c r="F96" s="15">
-        <f> HSV7.002 plocha fasády 276.7 m²</f>
-        <v/>
-      </c>
-      <c r="G96" s="15" t="inlineStr">
-        <is>
-          <t>713</t>
-        </is>
-      </c>
-      <c r="H96" s="14" t="inlineStr">
-        <is>
-          <t>⚠ família ??? (ÚRS online)</t>
-        </is>
-      </c>
-      <c r="I96" s="15" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.002 → HSV7.002a</t>
-        </is>
-      </c>
-      <c r="J96" s="15" t="inlineStr">
-        <is>
-          <t>S01, S12a</t>
-        </is>
-      </c>
-      <c r="K96" s="15" t="inlineStr">
-        <is>
-          <t>Lepení+kotvení EPS (713/622 família). Leaf dle tl. 160 mm — verify.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
-        </is>
-      </c>
-    </row>
-    <row r="97">
-      <c r="A97" s="14" t="n">
-        <v>89</v>
-      </c>
-      <c r="B97" s="15" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda ETICS</t>
-        </is>
-      </c>
-      <c r="C97" s="15" t="inlineStr">
-        <is>
-          <t>Armovací vrstva — výztužná síťka + lepicí stěrka (zatírací) na ETICS</t>
-        </is>
-      </c>
-      <c r="D97" s="14" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E97" s="16" t="n">
-        <v>276.7</v>
-      </c>
-      <c r="F97" s="15">
-        <f> HSV7.002 plocha 276.7 m²</f>
-        <v/>
-      </c>
-      <c r="G97" s="15" t="inlineStr">
-        <is>
-          <t>622</t>
-        </is>
-      </c>
-      <c r="H97" s="14" t="inlineStr">
-        <is>
-          <t>⚠ família ??? (ÚRS online)</t>
-        </is>
-      </c>
-      <c r="I97" s="15" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.002 → HSV7.002b</t>
-        </is>
-      </c>
-      <c r="J97" s="15" t="inlineStr">
-        <is>
-          <t>S01, S12a</t>
-        </is>
-      </c>
-      <c r="K97" s="15" t="inlineStr">
-        <is>
-          <t>Armovací vrstva síťka+stěrka (622 família). Finální omítka je samostatně HSV7.006.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
-        </is>
-      </c>
-    </row>
-    <row r="98">
-      <c r="A98" s="14" t="n">
-        <v>90</v>
-      </c>
-      <c r="B98" s="15" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda ETICS</t>
-        </is>
-      </c>
-      <c r="C98" s="15" t="inlineStr">
-        <is>
-          <t>Lepení + kotvení desek XPS λ=0.034 tl. 120 mm + soklový profil — ETICS sokl</t>
-        </is>
-      </c>
-      <c r="D98" s="14" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E98" s="16" t="n">
-        <v>13.5</v>
-      </c>
-      <c r="F98" s="15">
-        <f> HSV7.003 plocha soklu 13.5 m²</f>
-        <v/>
-      </c>
-      <c r="G98" s="15" t="inlineStr">
-        <is>
-          <t>713</t>
-        </is>
-      </c>
-      <c r="H98" s="14" t="inlineStr">
-        <is>
-          <t>⚠ família ??? (ÚRS online)</t>
-        </is>
-      </c>
-      <c r="I98" s="15" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.003 → HSV7.003a</t>
-        </is>
-      </c>
-      <c r="J98" s="15" t="inlineStr">
-        <is>
-          <t>S01</t>
-        </is>
-      </c>
-      <c r="K98" s="15" t="inlineStr">
-        <is>
-          <t>Sokl XPS lepení + soklový profil (713/622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
-        </is>
-      </c>
-    </row>
-    <row r="99">
-      <c r="A99" s="14" t="n">
-        <v>91</v>
-      </c>
-      <c r="B99" s="15" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda ETICS</t>
-        </is>
-      </c>
-      <c r="C99" s="15" t="inlineStr">
-        <is>
-          <t>Cihelný obklad soklu spárovaný (na armovací vrstvu)</t>
-        </is>
-      </c>
-      <c r="D99" s="14" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E99" s="16" t="n">
-        <v>13.5</v>
-      </c>
-      <c r="F99" s="15">
-        <f> HSV7.003 plocha soklu 13.5 m²</f>
-        <v/>
-      </c>
-      <c r="G99" s="15" t="inlineStr">
-        <is>
-          <t>781</t>
-        </is>
-      </c>
-      <c r="H99" s="14" t="inlineStr">
-        <is>
-          <t>⚠ família ??? (ÚRS online)</t>
-        </is>
-      </c>
-      <c r="I99" s="15" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.003 → HSV7.003b</t>
-        </is>
-      </c>
-      <c r="J99" s="15" t="inlineStr">
-        <is>
-          <t>S01</t>
-        </is>
-      </c>
-      <c r="K99" s="15" t="inlineStr">
-        <is>
-          <t>Cihelný obklad spárovaný (781 família obklady).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+      <c r="K99" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
         </is>
       </c>
     </row>
@@ -6473,24 +6463,24 @@
       </c>
       <c r="C100" s="15" t="inlineStr">
         <is>
-          <t>Špalety oken — EPS přesah 35-40 mm lepení + kotvení</t>
+          <t>Lepení + kotvení desek EPS 70F grey λ=0.032 tl. 160 mm — ETICS kontaktní zateplení fasády</t>
         </is>
       </c>
       <c r="D100" s="14" t="inlineStr">
         <is>
-          <t>bm</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E100" s="16" t="n">
-        <v>82.2</v>
+        <v>276.7</v>
       </c>
       <c r="F100" s="15">
-        <f> HSV7.004 obvod špalet 82.2 bm</f>
+        <f> HSV7.002 plocha fasády 276.7 m²</f>
         <v/>
       </c>
       <c r="G100" s="15" t="inlineStr">
         <is>
-          <t>622</t>
+          <t>713</t>
         </is>
       </c>
       <c r="H100" s="14" t="inlineStr">
@@ -6500,7 +6490,7 @@
       </c>
       <c r="I100" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.004 → HSV7.004a</t>
+          <t>260219_dum.HSV7.002 → HSV7.002a</t>
         </is>
       </c>
       <c r="J100" s="15" t="inlineStr">
@@ -6510,7 +6500,7 @@
       </c>
       <c r="K100" s="15" t="inlineStr">
         <is>
-          <t>Špalety EPS přesah (622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+          <t>Lepení+kotvení EPS (713/622 família). Leaf dle tl. 160 mm — verify.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -6525,148 +6515,356 @@
       </c>
       <c r="C101" s="15" t="inlineStr">
         <is>
+          <t>Armovací vrstva — výztužná síťka + lepicí stěrka (zatírací) na ETICS</t>
+        </is>
+      </c>
+      <c r="D101" s="14" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E101" s="16" t="n">
+        <v>276.7</v>
+      </c>
+      <c r="F101" s="15">
+        <f> HSV7.002 plocha 276.7 m²</f>
+        <v/>
+      </c>
+      <c r="G101" s="15" t="inlineStr">
+        <is>
+          <t>622</t>
+        </is>
+      </c>
+      <c r="H101" s="14" t="inlineStr">
+        <is>
+          <t>⚠ família ??? (ÚRS online)</t>
+        </is>
+      </c>
+      <c r="I101" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.002 → HSV7.002b</t>
+        </is>
+      </c>
+      <c r="J101" s="15" t="inlineStr">
+        <is>
+          <t>S01, S12a</t>
+        </is>
+      </c>
+      <c r="K101" s="15" t="inlineStr">
+        <is>
+          <t>Armovací vrstva síťka+stěrka (622 família). Finální omítka je samostatně HSV7.006.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="14" t="n">
+        <v>94</v>
+      </c>
+      <c r="B102" s="15" t="inlineStr">
+        <is>
+          <t>HSV-7 Fasáda ETICS</t>
+        </is>
+      </c>
+      <c r="C102" s="15" t="inlineStr">
+        <is>
+          <t>Lepení + kotvení desek XPS λ=0.034 tl. 120 mm + soklový profil — ETICS sokl</t>
+        </is>
+      </c>
+      <c r="D102" s="14" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E102" s="16" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F102" s="15">
+        <f> HSV7.003 plocha soklu 13.5 m²</f>
+        <v/>
+      </c>
+      <c r="G102" s="15" t="inlineStr">
+        <is>
+          <t>713</t>
+        </is>
+      </c>
+      <c r="H102" s="14" t="inlineStr">
+        <is>
+          <t>⚠ família ??? (ÚRS online)</t>
+        </is>
+      </c>
+      <c r="I102" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.003 → HSV7.003a</t>
+        </is>
+      </c>
+      <c r="J102" s="15" t="inlineStr">
+        <is>
+          <t>S01</t>
+        </is>
+      </c>
+      <c r="K102" s="15" t="inlineStr">
+        <is>
+          <t>Sokl XPS lepení + soklový profil (713/622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="14" t="n">
+        <v>95</v>
+      </c>
+      <c r="B103" s="15" t="inlineStr">
+        <is>
+          <t>HSV-7 Fasáda ETICS</t>
+        </is>
+      </c>
+      <c r="C103" s="15" t="inlineStr">
+        <is>
+          <t>Cihelný obklad soklu spárovaný (na armovací vrstvu)</t>
+        </is>
+      </c>
+      <c r="D103" s="14" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E103" s="16" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F103" s="15">
+        <f> HSV7.003 plocha soklu 13.5 m²</f>
+        <v/>
+      </c>
+      <c r="G103" s="15" t="inlineStr">
+        <is>
+          <t>781</t>
+        </is>
+      </c>
+      <c r="H103" s="14" t="inlineStr">
+        <is>
+          <t>⚠ família ??? (ÚRS online)</t>
+        </is>
+      </c>
+      <c r="I103" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.003 → HSV7.003b</t>
+        </is>
+      </c>
+      <c r="J103" s="15" t="inlineStr">
+        <is>
+          <t>S01</t>
+        </is>
+      </c>
+      <c r="K103" s="15" t="inlineStr">
+        <is>
+          <t>Cihelný obklad spárovaný (781 família obklady).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" s="14" t="n">
+        <v>96</v>
+      </c>
+      <c r="B104" s="15" t="inlineStr">
+        <is>
+          <t>HSV-7 Fasáda ETICS</t>
+        </is>
+      </c>
+      <c r="C104" s="15" t="inlineStr">
+        <is>
+          <t>Špalety oken — EPS přesah 35-40 mm lepení + kotvení</t>
+        </is>
+      </c>
+      <c r="D104" s="14" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="E104" s="16" t="n">
+        <v>82.2</v>
+      </c>
+      <c r="F104" s="15">
+        <f> HSV7.004 obvod špalet 82.2 bm</f>
+        <v/>
+      </c>
+      <c r="G104" s="15" t="inlineStr">
+        <is>
+          <t>622</t>
+        </is>
+      </c>
+      <c r="H104" s="14" t="inlineStr">
+        <is>
+          <t>⚠ família ??? (ÚRS online)</t>
+        </is>
+      </c>
+      <c r="I104" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.004 → HSV7.004a</t>
+        </is>
+      </c>
+      <c r="J104" s="15" t="inlineStr">
+        <is>
+          <t>S01, S12a</t>
+        </is>
+      </c>
+      <c r="K104" s="15" t="inlineStr">
+        <is>
+          <t>Špalety EPS přesah (622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="14" t="n">
+        <v>97</v>
+      </c>
+      <c r="B105" s="15" t="inlineStr">
+        <is>
+          <t>HSV-7 Fasáda ETICS</t>
+        </is>
+      </c>
+      <c r="C105" s="15" t="inlineStr">
+        <is>
           <t>Špalety oken — armovací vrstva síťka + omítka</t>
         </is>
       </c>
-      <c r="D101" s="14" t="inlineStr">
+      <c r="D105" s="14" t="inlineStr">
         <is>
           <t>bm</t>
         </is>
       </c>
-      <c r="E101" s="16" t="n">
+      <c r="E105" s="16" t="n">
         <v>82.2</v>
       </c>
-      <c r="F101" s="15">
+      <c r="F105" s="15">
         <f> HSV7.004 obvod 82.2 bm</f>
         <v/>
       </c>
-      <c r="G101" s="15" t="inlineStr">
+      <c r="G105" s="15" t="inlineStr">
         <is>
           <t>622</t>
         </is>
       </c>
-      <c r="H101" s="14" t="inlineStr">
+      <c r="H105" s="14" t="inlineStr">
         <is>
           <t>⚠ família ??? (ÚRS online)</t>
         </is>
       </c>
-      <c r="I101" s="15" t="inlineStr">
+      <c r="I105" s="15" t="inlineStr">
         <is>
           <t>260219_dum.HSV7.004 → HSV7.004b</t>
         </is>
       </c>
-      <c r="J101" s="15" t="inlineStr">
+      <c r="J105" s="15" t="inlineStr">
         <is>
           <t>S01, S12a</t>
         </is>
       </c>
-      <c r="K101" s="15" t="inlineStr">
+      <c r="K105" s="15" t="inlineStr">
         <is>
           <t>Armovací vrstva + omítka špalet (622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" s="10" t="n">
-        <v>94</v>
-      </c>
-      <c r="B102" s="11" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="10" t="n">
+        <v>98</v>
+      </c>
+      <c r="B106" s="11" t="inlineStr">
         <is>
           <t>HSV-7 Fasáda ETICS</t>
         </is>
       </c>
-      <c r="C102" s="11" t="inlineStr">
+      <c r="C106" s="11" t="inlineStr">
         <is>
           <t>Profilace fasády — různé tloušťky EPS (kordony, šambrány, rámování oken) — paušál podle pohledů</t>
         </is>
       </c>
-      <c r="D102" s="10" t="inlineStr">
+      <c r="D106" s="10" t="inlineStr">
         <is>
           <t>soubor</t>
         </is>
       </c>
-      <c r="E102" s="12" t="n">
+      <c r="E106" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F102" s="11" t="inlineStr">
+      <c r="F106" s="11" t="inlineStr">
         <is>
           <t>paušál — dle pohledů NCS NZÚ</t>
         </is>
       </c>
-      <c r="G102" s="11" t="inlineStr">
+      <c r="G106" s="11" t="inlineStr">
         <is>
           <t>622221221</t>
         </is>
       </c>
-      <c r="H102" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I102" s="11" t="inlineStr">
+      <c r="H106" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I106" s="11" t="inlineStr">
         <is>
           <t>260219_dum.HSV7.005</t>
         </is>
       </c>
-      <c r="J102" s="11" t="inlineStr">
+      <c r="J106" s="11" t="inlineStr">
         <is>
           <t>S01, S12a</t>
         </is>
       </c>
-      <c r="K102" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="10" t="n">
-        <v>95</v>
-      </c>
-      <c r="B103" s="11" t="inlineStr">
+      <c r="K106" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="10" t="n">
+        <v>99</v>
+      </c>
+      <c r="B107" s="11" t="inlineStr">
         <is>
           <t>HSV-7 Fasáda ETICS</t>
         </is>
       </c>
-      <c r="C103" s="11" t="inlineStr">
+      <c r="C107" s="11" t="inlineStr">
         <is>
           <t>Tenkovrstvá pastovitá probarvená omítka, lomená bílá NCS NZÚ — finální vrstva ETICS</t>
         </is>
       </c>
-      <c r="D103" s="10" t="inlineStr">
+      <c r="D107" s="10" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E103" s="12" t="n">
+      <c r="E107" s="12" t="n">
         <v>290.2</v>
       </c>
-      <c r="F103" s="11" t="inlineStr">
+      <c r="F107" s="11" t="inlineStr">
         <is>
           <t>ETICS plocha 276.7 m² + sokl 13.5 m² = 290.2 m²</t>
         </is>
       </c>
-      <c r="G103" s="13" t="inlineStr">
+      <c r="G107" s="13" t="inlineStr">
         <is>
           <t>622521111</t>
         </is>
       </c>
-      <c r="H103" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I103" s="11" t="inlineStr">
+      <c r="H107" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I107" s="11" t="inlineStr">
         <is>
           <t>260219_dum.HSV7.006</t>
         </is>
       </c>
-      <c r="J103" s="11" t="inlineStr">
+      <c r="J107" s="11" t="inlineStr">
         <is>
           <t>S01, S12a, S12b</t>
         </is>
       </c>
-      <c r="K103" s="11" t="inlineStr">
+      <c r="K107" s="11" t="inlineStr">
         <is>
           <t>Carried 1:1 (atomic — no decomposition needed)</t>
         </is>
@@ -6678,10 +6876,10 @@
     <mergeCell ref="A22:K22"/>
     <mergeCell ref="A59:K59"/>
     <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A76:K76"/>
+    <mergeCell ref="A98:K98"/>
     <mergeCell ref="A36:K36"/>
     <mergeCell ref="A44:K44"/>
-    <mergeCell ref="A94:K94"/>
+    <mergeCell ref="A80:K80"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -14856,7 +15054,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -14974,83 +15172,83 @@
     <row r="4">
       <c r="A4" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.002</t>
+          <t>260219_dum.HSV5.001</t>
         </is>
       </c>
       <c r="B4" s="15" t="inlineStr">
         <is>
-          <t>HSV-7 Fasáda ETICS</t>
+          <t>HSV-5 Krov + střecha</t>
         </is>
       </c>
       <c r="C4" s="15" t="inlineStr">
         <is>
-          <t xml:space="preserve">ETICS kontaktní zateplení — EPS 70F grey λ=0.032 tl. 160 mm + síťka + lepidlo + zatírací stěrka (řez S01+S12a explicit, </t>
+          <t>Tesařský krov — krokve 100/180 mm á 800 mm, rezivo C24 fungicidní + protihmyzí (cca 2×12 krokví × ~6.5 m)</t>
         </is>
       </c>
       <c r="D4" s="14" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>bm</t>
         </is>
       </c>
       <c r="E4" s="16" t="n">
-        <v>276.7</v>
+        <v>156</v>
       </c>
       <c r="F4" s="14" t="n">
         <v>2</v>
       </c>
       <c r="G4" s="15" t="inlineStr">
         <is>
-          <t>HSV7.002a, HSV7.002b</t>
+          <t>HSV5.001a, HSV5.001b</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.003</t>
+          <t>260219_dum.HSV5.002</t>
         </is>
       </c>
       <c r="B5" s="15" t="inlineStr">
         <is>
-          <t>HSV-7 Fasáda ETICS</t>
+          <t>HSV-5 Krov + střecha</t>
         </is>
       </c>
       <c r="C5" s="15" t="inlineStr">
         <is>
-          <t>ETICS sokl — XPS λ=0.034 tl. 120 mm + soklový profil + cihelný obklad spárovaný</t>
+          <t>Tesařský krov — kleštiny dvojfošny 60/180 mm probíhající v oblasti spací části</t>
         </is>
       </c>
       <c r="D5" s="14" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>bm</t>
         </is>
       </c>
       <c r="E5" s="16" t="n">
-        <v>13.5</v>
+        <v>110</v>
       </c>
       <c r="F5" s="14" t="n">
         <v>2</v>
       </c>
       <c r="G5" s="15" t="inlineStr">
         <is>
-          <t>HSV7.003a, HSV7.003b</t>
+          <t>HSV5.002a, HSV5.002b</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.004</t>
+          <t>260219_dum.HSV5.003</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>HSV-7 Fasáda ETICS</t>
+          <t>HSV-5 Krov + střecha</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>Špalety oken — EPS přesah 35-40 mm + síťka + omítka</t>
+          <t>Tesařský krov — pozednice 140/160 mm kotvená do ŽB věnce 3.NP</t>
         </is>
       </c>
       <c r="D6" s="14" t="inlineStr">
@@ -15059,31 +15257,31 @@
         </is>
       </c>
       <c r="E6" s="16" t="n">
-        <v>82.2</v>
+        <v>19.4</v>
       </c>
       <c r="F6" s="14" t="n">
         <v>2</v>
       </c>
       <c r="G6" s="15" t="inlineStr">
         <is>
-          <t>HSV7.004a, HSV7.004b</t>
+          <t>HSV5.003a, HSV5.003b</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV76.003</t>
+          <t>260219_dum.HSV5.004</t>
         </is>
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>PSV-76 Klempíř</t>
+          <t>HSV-5 Krov + střecha</t>
         </is>
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>Dešťové svody Pzn 100 mm + žlaby — 4 svody × ~14 m + žlaby per obvod střechy</t>
+          <t>Tesařský krov — námětky 60/100 v dolní koncové části pro přesah střechy ~500 mm</t>
         </is>
       </c>
       <c r="D7" s="14" t="inlineStr">
@@ -15092,31 +15290,31 @@
         </is>
       </c>
       <c r="E7" s="16" t="n">
-        <v>43.5</v>
+        <v>19.2</v>
       </c>
       <c r="F7" s="14" t="n">
         <v>2</v>
       </c>
       <c r="G7" s="15" t="inlineStr">
         <is>
-          <t>PSV76.003a, PSV76.003b</t>
+          <t>HSV5.004a, HSV5.004b</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV76.002</t>
+          <t>260219_dum.HSV7.002</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>PSV-76 Truhlář</t>
+          <t>HSV-7 Fasáda ETICS</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>Dřevěná terasa za opěrnou stěnou — prkna garapa 145×25 mm na dřevěném roštu z hranolů 50 mm na rektifikovatelných terčíc</t>
+          <t xml:space="preserve">ETICS kontaktní zateplení — EPS 70F grey λ=0.032 tl. 160 mm + síťka + lepidlo + zatírací stěrka (řez S01+S12a explicit, </t>
         </is>
       </c>
       <c r="D8" s="14" t="inlineStr">
@@ -15125,31 +15323,31 @@
         </is>
       </c>
       <c r="E8" s="16" t="n">
-        <v>9.23</v>
+        <v>276.7</v>
       </c>
       <c r="F8" s="14" t="n">
         <v>2</v>
       </c>
       <c r="G8" s="15" t="inlineStr">
         <is>
-          <t>PSV76.002a, PSV76.002b</t>
+          <t>HSV7.002a, HSV7.002b</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV77.002</t>
+          <t>260219_dum.HSV7.003</t>
         </is>
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>PSV-77 Podlahy</t>
+          <t>HSV-7 Fasáda ETICS</t>
         </is>
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>Nášlapná vrstva keramická dlažba lepená — koupelny + WC + spíž + komora (NÁDRŽ NP)</t>
+          <t>ETICS sokl — XPS λ=0.034 tl. 120 mm + soklový profil + cihelný obklad spárovaný</t>
         </is>
       </c>
       <c r="D9" s="14" t="inlineStr">
@@ -15165,90 +15363,90 @@
       </c>
       <c r="G9" s="15" t="inlineStr">
         <is>
-          <t>PSV77.002a, PSV77.002b</t>
+          <t>HSV7.003a, HSV7.003b</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV77.003</t>
+          <t>260219_dum.HSV7.004</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>PSV-77 Podlahy</t>
+          <t>HSV-7 Fasáda ETICS</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
-          <t>Nášlapná vrstva keramická dlažba — 1.PP technické místnosti (sušárna + sklepy + schodiště + chodba)</t>
+          <t>Špalety oken — EPS přesah 35-40 mm + síťka + omítka</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>bm</t>
         </is>
       </c>
       <c r="E10" s="16" t="n">
-        <v>32.4</v>
+        <v>82.2</v>
       </c>
       <c r="F10" s="14" t="n">
         <v>2</v>
       </c>
       <c r="G10" s="15" t="inlineStr">
         <is>
-          <t>PSV77.003a, PSV77.003b</t>
+          <t>HSV7.004a, HSV7.004b</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV78.001</t>
+          <t>260219_dum.PSV76.003</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>PSV-78 Povrchové úpravy</t>
+          <t>PSV-76 Klempíř</t>
         </is>
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>Omítka jádrová vápenocementová tl. 15 mm + štuková povrchová úprava na stěnách 1.PP (stávající vyspravené + nové zděné)</t>
+          <t>Dešťové svody Pzn 100 mm + žlaby — 4 svody × ~14 m + žlaby per obvod střechy</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>bm</t>
         </is>
       </c>
       <c r="E11" s="16" t="n">
-        <v>78.2</v>
+        <v>43.5</v>
       </c>
       <c r="F11" s="14" t="n">
         <v>2</v>
       </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>PSV78.001a, PSV78.001b</t>
+          <t>PSV76.003a, PSV76.003b</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV78.002</t>
+          <t>260219_dum.PSV76.002</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>PSV-78 Povrchové úpravy</t>
+          <t>PSV-76 Truhlář</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>Omítka jádrová vápenocementová tl. 15 mm + štuková povrchová úprava na stěnách 1.NP (stávající vyspravené + nové zděné)</t>
+          <t>Dřevěná terasa za opěrnou stěnou — prkna garapa 145×25 mm na dřevěném roštu z hranolů 50 mm na rektifikovatelných terčíc</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
@@ -15257,31 +15455,31 @@
         </is>
       </c>
       <c r="E12" s="16" t="n">
-        <v>208.4</v>
+        <v>9.23</v>
       </c>
       <c r="F12" s="14" t="n">
         <v>2</v>
       </c>
       <c r="G12" s="15" t="inlineStr">
         <is>
-          <t>PSV78.002a, PSV78.002b</t>
+          <t>PSV76.002a, PSV76.002b</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV78.003</t>
+          <t>260219_dum.PSV77.002</t>
         </is>
       </c>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>PSV-78 Povrchové úpravy</t>
+          <t>PSV-77 Podlahy</t>
         </is>
       </c>
       <c r="C13" s="15" t="inlineStr">
         <is>
-          <t>Omítka jádrová vápenocementová tl. 15 mm + štuková povrchová úprava na stěnách 2.NP (stávající vyspravené + nové zděné)</t>
+          <t>Nášlapná vrstva keramická dlažba lepená — koupelny + WC + spíž + komora (NÁDRŽ NP)</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
@@ -15290,31 +15488,31 @@
         </is>
       </c>
       <c r="E13" s="16" t="n">
-        <v>201.6</v>
+        <v>13.5</v>
       </c>
       <c r="F13" s="14" t="n">
         <v>2</v>
       </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
-          <t>PSV78.003a, PSV78.003b</t>
+          <t>PSV77.002a, PSV77.002b</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV78.004</t>
+          <t>260219_dum.PSV77.003</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>PSV-78 Povrchové úpravy</t>
+          <t>PSV-77 Podlahy</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>Omítka jádrová vápenocementová tl. 15 mm + štuková povrchová úprava na stěnách 3.NP (stávající vyspravené + nové zděné)</t>
+          <t>Nášlapná vrstva keramická dlažba — 1.PP technické místnosti (sušárna + sklepy + schodiště + chodba)</t>
         </is>
       </c>
       <c r="D14" s="14" t="inlineStr">
@@ -15323,177 +15521,309 @@
         </is>
       </c>
       <c r="E14" s="16" t="n">
-        <v>179.1</v>
+        <v>32.4</v>
       </c>
       <c r="F14" s="14" t="n">
         <v>2</v>
       </c>
       <c r="G14" s="15" t="inlineStr">
         <is>
-          <t>PSV78.004a, PSV78.004b</t>
+          <t>PSV77.003a, PSV77.003b</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV72.004</t>
+          <t>260219_dum.PSV78.001</t>
         </is>
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>PSV-72 ZTI</t>
+          <t>PSV-78 Povrchové úpravy</t>
         </is>
       </c>
       <c r="C15" s="15" t="inlineStr">
         <is>
-          <t>Sanitární keramika dodávka + montáž v koupelně 1.05 1.NP: 1× vana (DXF) + 1× umyvadlo (DXF) + 1× WC (TZ standard)</t>
+          <t>Omítka jádrová vápenocementová tl. 15 mm + štuková povrchová úprava na stěnách 1.PP (stávající vyspravené + nové zděné)</t>
         </is>
       </c>
       <c r="D15" s="14" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E15" s="16" t="n">
-        <v>0</v>
+        <v>78.2</v>
       </c>
       <c r="F15" s="14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G15" s="15" t="inlineStr">
         <is>
-          <t>PSV72.004a, PSV72.004b, PSV72.004c</t>
+          <t>PSV78.001a, PSV78.001b</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV72.005</t>
+          <t>260219_dum.PSV78.002</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>PSV-72 ZTI</t>
+          <t>PSV-78 Povrchové úpravy</t>
         </is>
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>Sanitární keramika dodávka + montáž v koupelně 2.03 2.NP: 1× umyvadlo (DXF) + 1× WC (TZ standard) + 1× sprcha (TZ standa</t>
+          <t>Omítka jádrová vápenocementová tl. 15 mm + štuková povrchová úprava na stěnách 1.NP (stávající vyspravené + nové zděné)</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E16" s="16" t="n">
-        <v>0</v>
+        <v>208.4</v>
       </c>
       <c r="F16" s="14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G16" s="15" t="inlineStr">
         <is>
-          <t>PSV72.005a, PSV72.005b, PSV72.005c</t>
+          <t>PSV78.002a, PSV78.002b</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV72.006</t>
+          <t>260219_dum.PSV78.003</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>PSV-72 ZTI</t>
+          <t>PSV-78 Povrchové úpravy</t>
         </is>
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
-          <t>Sanitární keramika dodávka + montáž v koupelně 3.04 3.NP: 1× WC (DXF) + 1× umyvadlo (TZ standard) + 1× sprcha (TZ standa</t>
+          <t>Omítka jádrová vápenocementová tl. 15 mm + štuková povrchová úprava na stěnách 2.NP (stávající vyspravené + nové zděné)</t>
         </is>
       </c>
       <c r="D17" s="14" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E17" s="16" t="n">
-        <v>0</v>
+        <v>201.6</v>
       </c>
       <c r="F17" s="14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
-          <t>PSV72.006a, PSV72.006b, PSV72.006c</t>
+          <t>PSV78.003a, PSV78.003b</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV72.008</t>
+          <t>260219_dum.PSV78.004</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>PSV-72 ZTI</t>
+          <t>PSV-78 Povrchové úpravy</t>
         </is>
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
-          <t>Vodovodní baterie (WC ventil + páková umyvadlová + sprchové + dřezové + termostat sprchové) — ~15 ks + drobné instalační</t>
+          <t>Omítka jádrová vápenocementová tl. 15 mm + štuková povrchová úprava na stěnách 3.NP (stávající vyspravené + nové zděné)</t>
         </is>
       </c>
       <c r="D18" s="14" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E18" s="16" t="n">
-        <v>15</v>
+        <v>179.1</v>
       </c>
       <c r="F18" s="14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G18" s="15" t="inlineStr">
         <is>
-          <t>PSV72.008a, PSV72.008b, PSV72.008c, PSV72.008d</t>
+          <t>PSV78.004a, PSV78.004b</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV1.015</t>
+          <t>260219_dum.PSV72.004</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
         <is>
-          <t>HSV-1 Zemní práce</t>
+          <t>PSV-72 ZTI</t>
         </is>
       </c>
       <c r="C19" s="15" t="inlineStr">
         <is>
-          <t>Drenáž za opěrnou stěnou (bílou vanou) — drenážní trubka DN100 vlnitá perforovaná + štěrkový obsyp 16/32 + geotextilie +</t>
+          <t>Sanitární keramika dodávka + montáž v koupelně 1.05 1.NP: 1× vana (DXF) + 1× umyvadlo (DXF) + 1× WC (TZ standard)</t>
         </is>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>set</t>
         </is>
       </c>
       <c r="E19" s="16" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="F19" s="14" t="n">
         <v>3</v>
       </c>
       <c r="G19" s="15" t="inlineStr">
+        <is>
+          <t>PSV72.004a, PSV72.004b, PSV72.004c</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.PSV72.005</t>
+        </is>
+      </c>
+      <c r="B20" s="15" t="inlineStr">
+        <is>
+          <t>PSV-72 ZTI</t>
+        </is>
+      </c>
+      <c r="C20" s="15" t="inlineStr">
+        <is>
+          <t>Sanitární keramika dodávka + montáž v koupelně 2.03 2.NP: 1× umyvadlo (DXF) + 1× WC (TZ standard) + 1× sprcha (TZ standa</t>
+        </is>
+      </c>
+      <c r="D20" s="14" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="E20" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="G20" s="15" t="inlineStr">
+        <is>
+          <t>PSV72.005a, PSV72.005b, PSV72.005c</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.PSV72.006</t>
+        </is>
+      </c>
+      <c r="B21" s="15" t="inlineStr">
+        <is>
+          <t>PSV-72 ZTI</t>
+        </is>
+      </c>
+      <c r="C21" s="15" t="inlineStr">
+        <is>
+          <t>Sanitární keramika dodávka + montáž v koupelně 3.04 3.NP: 1× WC (DXF) + 1× umyvadlo (TZ standard) + 1× sprcha (TZ standa</t>
+        </is>
+      </c>
+      <c r="D21" s="14" t="inlineStr">
+        <is>
+          <t>set</t>
+        </is>
+      </c>
+      <c r="E21" s="16" t="n">
+        <v>0</v>
+      </c>
+      <c r="F21" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="G21" s="15" t="inlineStr">
+        <is>
+          <t>PSV72.006a, PSV72.006b, PSV72.006c</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.PSV72.008</t>
+        </is>
+      </c>
+      <c r="B22" s="15" t="inlineStr">
+        <is>
+          <t>PSV-72 ZTI</t>
+        </is>
+      </c>
+      <c r="C22" s="15" t="inlineStr">
+        <is>
+          <t>Vodovodní baterie (WC ventil + páková umyvadlová + sprchové + dřezové + termostat sprchové) — ~15 ks + drobné instalační</t>
+        </is>
+      </c>
+      <c r="D22" s="14" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="E22" s="16" t="n">
+        <v>15</v>
+      </c>
+      <c r="F22" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="G22" s="15" t="inlineStr">
+        <is>
+          <t>PSV72.008a, PSV72.008b, PSV72.008c, PSV72.008d</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV1.015</t>
+        </is>
+      </c>
+      <c r="B23" s="15" t="inlineStr">
+        <is>
+          <t>HSV-1 Zemní práce</t>
+        </is>
+      </c>
+      <c r="C23" s="15" t="inlineStr">
+        <is>
+          <t>Drenáž za opěrnou stěnou (bílou vanou) — drenážní trubka DN100 vlnitá perforovaná + štěrkový obsyp 16/32 + geotextilie +</t>
+        </is>
+      </c>
+      <c r="D23" s="14" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E23" s="16" t="n">
+        <v>12</v>
+      </c>
+      <c r="F23" s="14" t="n">
+        <v>3</v>
+      </c>
+      <c r="G23" s="15" t="inlineStr">
         <is>
           <t>HSV1.015a, HSV1.015b, HSV1.015c</t>
         </is>

</xml_diff>

<commit_message>
feat(rd-jachymov): add krov svorníky tesařských spojů (762085112) + materiál split
Closes spojovací-prostředky-krovu companion gap from krov leaf-binding.
NEW HSV5.017: Montáž svorníků/šroubů tesařských spojů 762085112 (50 ks) — spoje
kleštin 2×60/180 s krokvemi (11 pozic × 2 konce × 2 = 44 + rezerva ≈ 50 ks).
Materiál split (atomic): tyč závitová Pz 4.6 M12 31197004 (14 m), matice DIN 934-8 M12
3111006 (1×100 ks), podložka DIN 440 D12 31121004 (1×100 ks). Source KROS + MCP.

Status OVĚŘIT (mnozstvi_conf 0.6): průměr M12/M16 + pevnost 4.6/8.8 + délka + počet
dle statiky. NEZAHRNUJE kotvení pozednice (samostatně) / úhelníky 762086111 / hřebíky.
items 215 → 216; 9-step regen + assertion pass; snapshot held.

https://claude.ai/code/session_01FskzLAZkXgJAwuN2cQQEdx
</commit_message>
<xml_diff>
--- a/test-data/RD_Jachymov_dum/outputs/Vykaz_vymer_RD_Jachymov_ATOMIC_WORKLIST_2026-05-27.xlsx
+++ b/test-data/RD_Jachymov_dum/outputs/Vykaz_vymer_RD_Jachymov_ATOMIC_WORKLIST_2026-05-27.xlsx
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>248</v>
+        <v>252</v>
       </c>
       <c r="C6" s="2">
         <f> carried 1:1 + decomposed children</f>
@@ -603,7 +603,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
     </row>
     <row r="9">
@@ -712,7 +712,7 @@
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
     </row>
     <row r="19">
@@ -989,7 +989,7 @@
         </is>
       </c>
       <c r="B47" s="5" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="48">
@@ -1009,7 +1009,7 @@
         </is>
       </c>
       <c r="B49" s="5" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="50">
@@ -1114,7 +1114,7 @@
         </is>
       </c>
       <c r="B62" s="5" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="63">
@@ -1140,7 +1140,7 @@
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>411</t>
+          <t>311</t>
         </is>
       </c>
       <c r="B65" s="5" t="n">
@@ -1150,37 +1150,37 @@
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>962</t>
+          <t>411</t>
         </is>
       </c>
       <c r="B66" s="5" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>733</t>
+          <t>962</t>
         </is>
       </c>
       <c r="B67" s="5" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>733</t>
         </is>
       </c>
       <c r="B68" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>311</t>
+          <t>210</t>
         </is>
       </c>
       <c r="B69" s="5" t="n">
@@ -1691,7 +1691,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K107"/>
+  <dimension ref="A1:K111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -4521,7 +4521,7 @@
     <row r="59">
       <c r="A59" s="8" t="inlineStr">
         <is>
-          <t>━━ HSV-5 Krov + střecha  (20 atomic operací) ━━</t>
+          <t>━━ HSV-5 Krov + střecha  (24 atomic operací) ━━</t>
         </is>
       </c>
       <c r="B59" s="9" t="n"/>
@@ -5539,211 +5539,229 @@
       </c>
     </row>
     <row r="80">
-      <c r="A80" s="8" t="inlineStr">
+      <c r="A80" s="14" t="n">
+        <v>74</v>
+      </c>
+      <c r="B80" s="15" t="inlineStr">
+        <is>
+          <t>HSV-5 Krov + střecha</t>
+        </is>
+      </c>
+      <c r="C80" s="15" t="inlineStr">
+        <is>
+          <t>Montáž svorníků/šroubů tesařských spojů krovu délky přes 150 do 300 mm — spoje kleštin 2×60/180 s krokvemi</t>
+        </is>
+      </c>
+      <c r="D80" s="14" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="E80" s="16" t="n">
+        <v>50</v>
+      </c>
+      <c r="F80" s="15">
+        <f> HSV5.017 počet svorníků 50 ks (11 pozic × 2 konce × 2)</f>
+        <v/>
+      </c>
+      <c r="G80" s="15" t="inlineStr">
+        <is>
+          <t>762085112</t>
+        </is>
+      </c>
+      <c r="H80" s="14" t="inlineStr">
+        <is>
+          <t>✓ verified</t>
+        </is>
+      </c>
+      <c r="I80" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV5.017 → HSV5.017a</t>
+        </is>
+      </c>
+      <c r="J80" s="15" t="inlineStr">
+        <is>
+          <t>Krov — spojovací prostředky</t>
+        </is>
+      </c>
+      <c r="K80" s="15" t="inlineStr">
+        <is>
+          <t>Montáž 762085112. OVĚŘIT M12/M16 + délku dle statiky/tesařského detailu.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="14" t="n">
+        <v>75</v>
+      </c>
+      <c r="B81" s="15" t="inlineStr">
+        <is>
+          <t>HSV-5 Krov + střecha</t>
+        </is>
+      </c>
+      <c r="C81" s="15" t="inlineStr">
+        <is>
+          <t>Tyč závitová Pz 4.6 M12 — materiál svorníků krovu</t>
+        </is>
+      </c>
+      <c r="D81" s="14" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
+      <c r="E81" s="16" t="n">
+        <v>14</v>
+      </c>
+      <c r="F81" s="15">
+        <f> 50 ks × 0.25 m × 1.10 prořez = 13.75 → 14 m</f>
+        <v/>
+      </c>
+      <c r="G81" s="15" t="inlineStr">
+        <is>
+          <t>31197004</t>
+        </is>
+      </c>
+      <c r="H81" s="14" t="inlineStr">
+        <is>
+          <t>⚠ família ??? (ÚRS online)</t>
+        </is>
+      </c>
+      <c r="I81" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV5.017 → HSV5.017b</t>
+        </is>
+      </c>
+      <c r="J81" s="15" t="inlineStr">
+        <is>
+          <t>Krov — spojovací prostředky</t>
+        </is>
+      </c>
+      <c r="K81" s="15" t="inlineStr">
+        <is>
+          <t>Materiál svorníku (31197004).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="14" t="n">
+        <v>76</v>
+      </c>
+      <c r="B82" s="15" t="inlineStr">
+        <is>
+          <t>HSV-5 Krov + střecha</t>
+        </is>
+      </c>
+      <c r="C82" s="15" t="inlineStr">
+        <is>
+          <t>Matice přesná šestihranná Pz DIN 934-8 M12</t>
+        </is>
+      </c>
+      <c r="D82" s="14" t="inlineStr">
+        <is>
+          <t>100 ks</t>
+        </is>
+      </c>
+      <c r="E82" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F82" s="15">
+        <f> 50 svorníků × 2 = 100 ks = 1×100ks</f>
+        <v/>
+      </c>
+      <c r="G82" s="15" t="inlineStr">
+        <is>
+          <t>3111006</t>
+        </is>
+      </c>
+      <c r="H82" s="14" t="inlineStr">
+        <is>
+          <t>⚠ família ??? (ÚRS online)</t>
+        </is>
+      </c>
+      <c r="I82" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV5.017 → HSV5.017c</t>
+        </is>
+      </c>
+      <c r="J82" s="15" t="inlineStr">
+        <is>
+          <t>Krov — spojovací prostředky</t>
+        </is>
+      </c>
+      <c r="K82" s="15" t="inlineStr">
+        <is>
+          <t>Matice (3111006), 2 na svorník.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="14" t="n">
+        <v>77</v>
+      </c>
+      <c r="B83" s="15" t="inlineStr">
+        <is>
+          <t>HSV-5 Krov + střecha</t>
+        </is>
+      </c>
+      <c r="C83" s="15" t="inlineStr">
+        <is>
+          <t>Podložka pod dřevěnou konstrukci DIN 440 D 12 mm</t>
+        </is>
+      </c>
+      <c r="D83" s="14" t="inlineStr">
+        <is>
+          <t>100 ks</t>
+        </is>
+      </c>
+      <c r="E83" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F83" s="15">
+        <f> 50 svorníků × 2 = 100 ks = 1×100ks</f>
+        <v/>
+      </c>
+      <c r="G83" s="15" t="inlineStr">
+        <is>
+          <t>31121004</t>
+        </is>
+      </c>
+      <c r="H83" s="14" t="inlineStr">
+        <is>
+          <t>⚠ família ??? (ÚRS online)</t>
+        </is>
+      </c>
+      <c r="I83" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV5.017 → HSV5.017d</t>
+        </is>
+      </c>
+      <c r="J83" s="15" t="inlineStr">
+        <is>
+          <t>Krov — spojovací prostředky</t>
+        </is>
+      </c>
+      <c r="K83" s="15" t="inlineStr">
+        <is>
+          <t>Podložka (31121004), 2 na svorník.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="8" t="inlineStr">
         <is>
           <t>━━ HSV-6 Bourací práce  (17 atomic operací) ━━</t>
         </is>
       </c>
-      <c r="B80" s="9" t="n"/>
-      <c r="C80" s="9" t="n"/>
-      <c r="D80" s="9" t="n"/>
-      <c r="E80" s="9" t="n"/>
-      <c r="F80" s="9" t="n"/>
-      <c r="G80" s="9" t="n"/>
-      <c r="H80" s="9" t="n"/>
-      <c r="I80" s="9" t="n"/>
-      <c r="J80" s="9" t="n"/>
-      <c r="K80" s="9" t="n"/>
-    </row>
-    <row r="81">
-      <c r="A81" s="10" t="n">
-        <v>74</v>
-      </c>
-      <c r="B81" s="11" t="inlineStr">
-        <is>
-          <t>HSV-6 Bourací práce</t>
-        </is>
-      </c>
-      <c r="C81" s="11" t="inlineStr">
-        <is>
-          <t>Bourání kompletního stávajícího krovu vč. vikýřů — vaznicový s ležatou stolicí — manuálně, odvoz</t>
-        </is>
-      </c>
-      <c r="D81" s="10" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="E81" s="12" t="n">
-        <v>12</v>
-      </c>
-      <c r="F81" s="11" t="inlineStr">
-        <is>
-          <t>TZ B m.10.e: 9 t dřeva × 0.75 t/m³ = 12 m³ dřeva</t>
-        </is>
-      </c>
-      <c r="G81" s="13" t="inlineStr">
-        <is>
-          <t>962041141</t>
-        </is>
-      </c>
-      <c r="H81" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I81" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV6.001</t>
-        </is>
-      </c>
-      <c r="J81" s="11" t="inlineStr"/>
-      <c r="K81" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="17" t="n">
-        <v>75</v>
-      </c>
-      <c r="B82" s="18" t="inlineStr">
-        <is>
-          <t>HSV-6 Bourací práce</t>
-        </is>
-      </c>
-      <c r="C82" s="18" t="inlineStr">
-        <is>
-          <t>Bourání stávající plechové krytiny (manuálně, recyklace plechu)</t>
-        </is>
-      </c>
-      <c r="D82" s="17" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E82" s="19" t="n">
-        <v>140.9</v>
-      </c>
-      <c r="F82" s="18">
-        <f> plocha krytiny ~141</f>
-        <v/>
-      </c>
-      <c r="G82" s="18" t="inlineStr"/>
-      <c r="H82" s="17" t="inlineStr">
-        <is>
-          <t>❌ blank — ÚRS online</t>
-        </is>
-      </c>
-      <c r="I82" s="18" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV6.002</t>
-        </is>
-      </c>
-      <c r="J82" s="18" t="inlineStr"/>
-      <c r="K82" s="18" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
-        </is>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="10" t="n">
-        <v>76</v>
-      </c>
-      <c r="B83" s="11" t="inlineStr">
-        <is>
-          <t>HSV-6 Bourací práce</t>
-        </is>
-      </c>
-      <c r="C83" s="11" t="inlineStr">
-        <is>
-          <t>Bourání zděných nadezdívek nad stropem 2.NP (mimo štítových stěn) — cihla pálená</t>
-        </is>
-      </c>
-      <c r="D83" s="10" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="E83" s="12" t="n">
-        <v>6</v>
-      </c>
-      <c r="F83" s="11" t="inlineStr">
-        <is>
-          <t>odhad — 3.NP nadezdívka půdy ~104 m² × 0.45 m výška ~6</t>
-        </is>
-      </c>
-      <c r="G83" s="11" t="inlineStr">
-        <is>
-          <t>962031132</t>
-        </is>
-      </c>
-      <c r="H83" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I83" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV6.003</t>
-        </is>
-      </c>
-      <c r="J83" s="11" t="inlineStr"/>
-      <c r="K83" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="10" t="n">
-        <v>77</v>
-      </c>
-      <c r="B84" s="11" t="inlineStr">
-        <is>
-          <t>HSV-6 Bourací práce</t>
-        </is>
-      </c>
-      <c r="C84" s="11" t="inlineStr">
-        <is>
-          <t>Bourání trámového stropu 2.NP/podkroví — kompletně (vč. zajištění schodiště)</t>
-        </is>
-      </c>
-      <c r="D84" s="10" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E84" s="12" t="n">
-        <v>104.4</v>
-      </c>
-      <c r="F84" s="11">
-        <f> zastavěna 104.4 m²</f>
-        <v/>
-      </c>
-      <c r="G84" s="11" t="inlineStr">
-        <is>
-          <t>962041141</t>
-        </is>
-      </c>
-      <c r="H84" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I84" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV6.004</t>
-        </is>
-      </c>
-      <c r="J84" s="11" t="inlineStr"/>
-      <c r="K84" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
+      <c r="B84" s="9" t="n"/>
+      <c r="C84" s="9" t="n"/>
+      <c r="D84" s="9" t="n"/>
+      <c r="E84" s="9" t="n"/>
+      <c r="F84" s="9" t="n"/>
+      <c r="G84" s="9" t="n"/>
+      <c r="H84" s="9" t="n"/>
+      <c r="I84" s="9" t="n"/>
+      <c r="J84" s="9" t="n"/>
+      <c r="K84" s="9" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="10" t="n">
@@ -5756,25 +5774,25 @@
       </c>
       <c r="C85" s="11" t="inlineStr">
         <is>
-          <t>Bourání stávajících lehkých příček (cihla, sádrokarton, dřevo)</t>
+          <t>Bourání kompletního stávajícího krovu vč. vikýřů — vaznicový s ležatou stolicí — manuálně, odvoz</t>
         </is>
       </c>
       <c r="D85" s="10" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="E85" s="12" t="n">
-        <v>80</v>
+        <v>12</v>
       </c>
       <c r="F85" s="11" t="inlineStr">
         <is>
-          <t>odhad — interier 2 patra × ~40 m² příček = 80</t>
-        </is>
-      </c>
-      <c r="G85" s="11" t="inlineStr">
-        <is>
-          <t>962031132</t>
+          <t>TZ B m.10.e: 9 t dřeva × 0.75 t/m³ = 12 m³ dřeva</t>
+        </is>
+      </c>
+      <c r="G85" s="13" t="inlineStr">
+        <is>
+          <t>962041141</t>
         </is>
       </c>
       <c r="H85" s="10" t="inlineStr">
@@ -5784,7 +5802,7 @@
       </c>
       <c r="I85" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.005</t>
+          <t>260219_dum.HSV6.001</t>
         </is>
       </c>
       <c r="J85" s="11" t="inlineStr"/>
@@ -5795,51 +5813,46 @@
       </c>
     </row>
     <row r="86">
-      <c r="A86" s="10" t="n">
+      <c r="A86" s="17" t="n">
         <v>79</v>
       </c>
-      <c r="B86" s="11" t="inlineStr">
+      <c r="B86" s="18" t="inlineStr">
         <is>
           <t>HSV-6 Bourací práce</t>
         </is>
       </c>
-      <c r="C86" s="11" t="inlineStr">
-        <is>
-          <t>Bourání 8 nových otvorů v nosných cihelných zdech pro dveře/okna (~1.0 × 2.1 m)</t>
-        </is>
-      </c>
-      <c r="D86" s="10" t="inlineStr">
-        <is>
-          <t>ks</t>
-        </is>
-      </c>
-      <c r="E86" s="12" t="n">
-        <v>8</v>
-      </c>
-      <c r="F86" s="11" t="inlineStr">
-        <is>
-          <t>odhad počtu nových otvorů (= počet IPN160 překladů)</t>
-        </is>
-      </c>
-      <c r="G86" s="11" t="inlineStr">
-        <is>
-          <t>962031132</t>
-        </is>
-      </c>
-      <c r="H86" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I86" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV6.006</t>
-        </is>
-      </c>
-      <c r="J86" s="11" t="inlineStr"/>
-      <c r="K86" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+      <c r="C86" s="18" t="inlineStr">
+        <is>
+          <t>Bourání stávající plechové krytiny (manuálně, recyklace plechu)</t>
+        </is>
+      </c>
+      <c r="D86" s="17" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E86" s="19" t="n">
+        <v>140.9</v>
+      </c>
+      <c r="F86" s="18">
+        <f> plocha krytiny ~141</f>
+        <v/>
+      </c>
+      <c r="G86" s="18" t="inlineStr"/>
+      <c r="H86" s="17" t="inlineStr">
+        <is>
+          <t>❌ blank — ÚRS online</t>
+        </is>
+      </c>
+      <c r="I86" s="18" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV6.002</t>
+        </is>
+      </c>
+      <c r="J86" s="18" t="inlineStr"/>
+      <c r="K86" s="18" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -5854,25 +5867,25 @@
       </c>
       <c r="C87" s="11" t="inlineStr">
         <is>
-          <t>Bourání keramických obkladů a zařizovacích předmětů v koupelnách 1.NP + 2.NP</t>
+          <t>Bourání zděných nadezdívek nad stropem 2.NP (mimo štítových stěn) — cihla pálená</t>
         </is>
       </c>
       <c r="D87" s="10" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="E87" s="12" t="n">
-        <v>60</v>
+        <v>6</v>
       </c>
       <c r="F87" s="11" t="inlineStr">
         <is>
-          <t>2 koupelny × ~30 m² obkladů = 60</t>
-        </is>
-      </c>
-      <c r="G87" s="13" t="inlineStr">
-        <is>
-          <t>781473810</t>
+          <t>odhad — 3.NP nadezdívka půdy ~104 m² × 0.45 m výška ~6</t>
+        </is>
+      </c>
+      <c r="G87" s="11" t="inlineStr">
+        <is>
+          <t>962031132</t>
         </is>
       </c>
       <c r="H87" s="10" t="inlineStr">
@@ -5882,7 +5895,7 @@
       </c>
       <c r="I87" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.007</t>
+          <t>260219_dum.HSV6.003</t>
         </is>
       </c>
       <c r="J87" s="11" t="inlineStr"/>
@@ -5903,7 +5916,7 @@
       </c>
       <c r="C88" s="11" t="inlineStr">
         <is>
-          <t>Sejmutí podlah 1.NP a 2.NP — vč. nášlapů, podkladních vrstev</t>
+          <t>Bourání trámového stropu 2.NP/podkroví — kompletně (vč. zajištění schodiště)</t>
         </is>
       </c>
       <c r="D88" s="10" t="inlineStr">
@@ -5912,16 +5925,15 @@
         </is>
       </c>
       <c r="E88" s="12" t="n">
-        <v>153.51</v>
-      </c>
-      <c r="F88" s="11" t="inlineStr">
-        <is>
-          <t>podlahova × 0.7 = ~154 m² (bez 3.NP nového)</t>
-        </is>
+        <v>104.4</v>
+      </c>
+      <c r="F88" s="11">
+        <f> zastavěna 104.4 m²</f>
+        <v/>
       </c>
       <c r="G88" s="11" t="inlineStr">
         <is>
-          <t>974031132</t>
+          <t>962041141</t>
         </is>
       </c>
       <c r="H88" s="10" t="inlineStr">
@@ -5931,7 +5943,7 @@
       </c>
       <c r="I88" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.008</t>
+          <t>260219_dum.HSV6.004</t>
         </is>
       </c>
       <c r="J88" s="11" t="inlineStr"/>
@@ -5952,25 +5964,25 @@
       </c>
       <c r="C89" s="11" t="inlineStr">
         <is>
-          <t>Demontáž záklopu a zásypů stropu 1.NP (prkenný záklop na trámech zachován)</t>
+          <t>Bourání stávajících lehkých příček (cihla, sádrokarton, dřevo)</t>
         </is>
       </c>
       <c r="D89" s="10" t="inlineStr">
         <is>
-          <t>m³</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E89" s="12" t="n">
-        <v>5</v>
+        <v>80</v>
       </c>
       <c r="F89" s="11" t="inlineStr">
         <is>
-          <t>100 m² × 0.05 m tl. zásypu = 5</t>
+          <t>odhad — interier 2 patra × ~40 m² příček = 80</t>
         </is>
       </c>
       <c r="G89" s="11" t="inlineStr">
         <is>
-          <t>974041151</t>
+          <t>962031132</t>
         </is>
       </c>
       <c r="H89" s="10" t="inlineStr">
@@ -5980,7 +5992,7 @@
       </c>
       <c r="I89" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.009</t>
+          <t>260219_dum.HSV6.005</t>
         </is>
       </c>
       <c r="J89" s="11" t="inlineStr"/>
@@ -6001,7 +6013,7 @@
       </c>
       <c r="C90" s="11" t="inlineStr">
         <is>
-          <t>Demontáž všech oken a dveří stávajících (recyklace)</t>
+          <t>Bourání 8 nových otvorů v nosných cihelných zdech pro dveře/okna (~1.0 × 2.1 m)</t>
         </is>
       </c>
       <c r="D90" s="10" t="inlineStr">
@@ -6010,16 +6022,16 @@
         </is>
       </c>
       <c r="E90" s="12" t="n">
-        <v>25</v>
+        <v>8</v>
       </c>
       <c r="F90" s="11" t="inlineStr">
         <is>
-          <t>odhad — ~10 oken + ~15 dveří (vstupní + vnitřní)</t>
+          <t>odhad počtu nových otvorů (= počet IPN160 překladů)</t>
         </is>
       </c>
       <c r="G90" s="11" t="inlineStr">
         <is>
-          <t>968071120</t>
+          <t>962031132</t>
         </is>
       </c>
       <c r="H90" s="10" t="inlineStr">
@@ -6029,7 +6041,7 @@
       </c>
       <c r="I90" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.010</t>
+          <t>260219_dum.HSV6.006</t>
         </is>
       </c>
       <c r="J90" s="11" t="inlineStr"/>
@@ -6050,25 +6062,25 @@
       </c>
       <c r="C91" s="11" t="inlineStr">
         <is>
-          <t>Demontáž všech sanitárních zařizovacích předmětů (WC, umyvadla, baterie, sprcha)</t>
+          <t>Bourání keramických obkladů a zařizovacích předmětů v koupelnách 1.NP + 2.NP</t>
         </is>
       </c>
       <c r="D91" s="10" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E91" s="12" t="n">
-        <v>12</v>
+        <v>60</v>
       </c>
       <c r="F91" s="11" t="inlineStr">
         <is>
-          <t>odhad — 2 koupelny × ~5 ks + WC + dřez = ~12</t>
-        </is>
-      </c>
-      <c r="G91" s="11" t="inlineStr">
-        <is>
-          <t>725900001</t>
+          <t>2 koupelny × ~30 m² obkladů = 60</t>
+        </is>
+      </c>
+      <c r="G91" s="13" t="inlineStr">
+        <is>
+          <t>781473810</t>
         </is>
       </c>
       <c r="H91" s="10" t="inlineStr">
@@ -6078,7 +6090,7 @@
       </c>
       <c r="I91" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.011</t>
+          <t>260219_dum.HSV6.007</t>
         </is>
       </c>
       <c r="J91" s="11" t="inlineStr"/>
@@ -6099,25 +6111,25 @@
       </c>
       <c r="C92" s="11" t="inlineStr">
         <is>
-          <t>Odvoz a likvidace stavební suti dle vyhl. 8/2021 Sb. — celková tonáž odpadů</t>
+          <t>Sejmutí podlah 1.NP a 2.NP — vč. nášlapů, podkladních vrstev</t>
         </is>
       </c>
       <c r="D92" s="10" t="inlineStr">
         <is>
-          <t>t</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E92" s="12" t="n">
-        <v>56.5</v>
+        <v>153.51</v>
       </c>
       <c r="F92" s="11" t="inlineStr">
         <is>
-          <t>TZ B m.10.e: 46 (beton/cihly) + 9 (dřevo) + 0.1 (kov) + 0.1 (EPS) + 0.2 (sádra) + 1.0 (směs) = 56.4</t>
+          <t>podlahova × 0.7 = ~154 m² (bez 3.NP nového)</t>
         </is>
       </c>
       <c r="G92" s="11" t="inlineStr">
         <is>
-          <t>997013501</t>
+          <t>974031132</t>
         </is>
       </c>
       <c r="H92" s="10" t="inlineStr">
@@ -6127,7 +6139,7 @@
       </c>
       <c r="I92" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.012</t>
+          <t>260219_dum.HSV6.008</t>
         </is>
       </c>
       <c r="J92" s="11" t="inlineStr"/>
@@ -6148,35 +6160,35 @@
       </c>
       <c r="C93" s="11" t="inlineStr">
         <is>
-          <t>Demontáž stávajících dřevěných oken vč. rámů a parapetů — 16 ks (návrh všechna okna nová plastová trojsklem)</t>
+          <t>Demontáž záklopu a zásypů stropu 1.NP (prkenný záklop na trámech zachován)</t>
         </is>
       </c>
       <c r="D93" s="10" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="E93" s="12" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="F93" s="11" t="inlineStr">
         <is>
-          <t>DXF INSERT okno* total 16 ks (Path C Tier 4 — front 9 + back 7)</t>
-        </is>
-      </c>
-      <c r="G93" s="13" t="inlineStr">
-        <is>
-          <t>978013181</t>
+          <t>100 m² × 0.05 m tl. zásypu = 5</t>
+        </is>
+      </c>
+      <c r="G93" s="11" t="inlineStr">
+        <is>
+          <t>974041151</t>
         </is>
       </c>
       <c r="H93" s="10" t="inlineStr">
         <is>
-          <t>✓ verified</t>
+          <t>⚠ kandidát-verify</t>
         </is>
       </c>
       <c r="I93" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.013</t>
+          <t>260219_dum.HSV6.009</t>
         </is>
       </c>
       <c r="J93" s="11" t="inlineStr"/>
@@ -6197,7 +6209,7 @@
       </c>
       <c r="C94" s="11" t="inlineStr">
         <is>
-          <t>Demontáž stávajících vstupních dveří + rámů — 2 ks (1× ulice Fibichova + 1× zahrada; návrh nové plastové vstupní dveře)</t>
+          <t>Demontáž všech oken a dveří stávajících (recyklace)</t>
         </is>
       </c>
       <c r="D94" s="10" t="inlineStr">
@@ -6206,26 +6218,26 @@
         </is>
       </c>
       <c r="E94" s="12" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="F94" s="11" t="inlineStr">
         <is>
-          <t>DXF INSERT dveře = 2 (Path C Tier 4) + TZ ARS</t>
-        </is>
-      </c>
-      <c r="G94" s="13" t="inlineStr">
-        <is>
-          <t>978013181</t>
+          <t>odhad — ~10 oken + ~15 dveří (vstupní + vnitřní)</t>
+        </is>
+      </c>
+      <c r="G94" s="11" t="inlineStr">
+        <is>
+          <t>968071120</t>
         </is>
       </c>
       <c r="H94" s="10" t="inlineStr">
         <is>
-          <t>✓ verified</t>
+          <t>⚠ kandidát-verify</t>
         </is>
       </c>
       <c r="I94" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.014</t>
+          <t>260219_dum.HSV6.010</t>
         </is>
       </c>
       <c r="J94" s="11" t="inlineStr"/>
@@ -6246,7 +6258,7 @@
       </c>
       <c r="C95" s="11" t="inlineStr">
         <is>
-          <t>Demontáž stávajících vnitřních dveří vč. ocelových/dřevěných zárubní — odhad 15 ks (3 patra × ~5 dveří/patro per DXF SM__dveře layer)</t>
+          <t>Demontáž všech sanitárních zařizovacích předmětů (WC, umyvadla, baterie, sprcha)</t>
         </is>
       </c>
       <c r="D95" s="10" t="inlineStr">
@@ -6255,16 +6267,16 @@
         </is>
       </c>
       <c r="E95" s="12" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F95" s="11" t="inlineStr">
         <is>
-          <t>DXF SM__dveře polylines 102 / ~3 fáze / ~2.3 symbol per dveře ≈ 15 ks návrh (Path C confidence 0.65)</t>
+          <t>odhad — 2 koupelny × ~5 ks + WC + dřez = ~12</t>
         </is>
       </c>
       <c r="G95" s="11" t="inlineStr">
         <is>
-          <t>968072456</t>
+          <t>725900001</t>
         </is>
       </c>
       <c r="H95" s="10" t="inlineStr">
@@ -6274,7 +6286,7 @@
       </c>
       <c r="I95" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.015</t>
+          <t>260219_dum.HSV6.011</t>
         </is>
       </c>
       <c r="J95" s="11" t="inlineStr"/>
@@ -6295,25 +6307,25 @@
       </c>
       <c r="C96" s="11" t="inlineStr">
         <is>
-          <t>Bourání vrchní části stávajícího komínu v posledním podlaží (cihelné zdivo, ručně), vč. likvidace cihelné suti</t>
+          <t>Odvoz a likvidace stavební suti dle vyhl. 8/2021 Sb. — celková tonáž odpadů</t>
         </is>
       </c>
       <c r="D96" s="10" t="inlineStr">
         <is>
-          <t>m³</t>
+          <t>t</t>
         </is>
       </c>
       <c r="E96" s="12" t="n">
-        <v>0.6</v>
+        <v>56.5</v>
       </c>
       <c r="F96" s="11" t="inlineStr">
         <is>
-          <t>průměr komín 0.50×0.50 × výška nad střechou ~2.4 m = 0.6 m³ (OPRAVA ChatGPT revize 2026-05-29: dříve 6.0 m³ = ×10 chybná inflace; skutečný objem 0.6 m³)</t>
-        </is>
-      </c>
-      <c r="G96" s="13" t="inlineStr">
-        <is>
-          <t>962024141</t>
+          <t>TZ B m.10.e: 46 (beton/cihly) + 9 (dřevo) + 0.1 (kov) + 0.1 (EPS) + 0.2 (sádra) + 1.0 (směs) = 56.4</t>
+        </is>
+      </c>
+      <c r="G96" s="11" t="inlineStr">
+        <is>
+          <t>997013501</t>
         </is>
       </c>
       <c r="H96" s="10" t="inlineStr">
@@ -6323,7 +6335,7 @@
       </c>
       <c r="I96" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.016</t>
+          <t>260219_dum.HSV6.012</t>
         </is>
       </c>
       <c r="J96" s="11" t="inlineStr"/>
@@ -6344,35 +6356,35 @@
       </c>
       <c r="C97" s="11" t="inlineStr">
         <is>
-          <t>Bourání stávajících opěrných zídek a venkovního schodiště v zahradě/dvoře — částečné, dle vyznačení v půdorysech bourání</t>
+          <t>Demontáž stávajících dřevěných oken vč. rámů a parapetů — 16 ks (návrh všechna okna nová plastová trojsklem)</t>
         </is>
       </c>
       <c r="D97" s="10" t="inlineStr">
         <is>
-          <t>m³</t>
+          <t>ks</t>
         </is>
       </c>
       <c r="E97" s="12" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="F97" s="11" t="inlineStr">
         <is>
-          <t>odhad ze řez A-A bourání + půdorys bourání 1.NP/1.PP, ~8 m³ celkem (opěrné zídky + venkovní schodiště zahrada/dvůr)</t>
+          <t>DXF INSERT okno* total 16 ks (Path C Tier 4 — front 9 + back 7)</t>
         </is>
       </c>
       <c r="G97" s="13" t="inlineStr">
         <is>
-          <t>961044111</t>
+          <t>978013181</t>
         </is>
       </c>
       <c r="H97" s="10" t="inlineStr">
         <is>
-          <t>⚠ kandidát-verify</t>
+          <t>✓ verified</t>
         </is>
       </c>
       <c r="I97" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.017</t>
+          <t>260219_dum.HSV6.013</t>
         </is>
       </c>
       <c r="J97" s="11" t="inlineStr"/>
@@ -6383,280 +6395,268 @@
       </c>
     </row>
     <row r="98">
-      <c r="A98" s="8" t="inlineStr">
-        <is>
-          <t>━━ HSV-7 Fasáda ETICS  (9 atomic operací) ━━</t>
-        </is>
-      </c>
-      <c r="B98" s="9" t="n"/>
-      <c r="C98" s="9" t="n"/>
-      <c r="D98" s="9" t="n"/>
-      <c r="E98" s="9" t="n"/>
-      <c r="F98" s="9" t="n"/>
-      <c r="G98" s="9" t="n"/>
-      <c r="H98" s="9" t="n"/>
-      <c r="I98" s="9" t="n"/>
-      <c r="J98" s="9" t="n"/>
-      <c r="K98" s="9" t="n"/>
+      <c r="A98" s="10" t="n">
+        <v>91</v>
+      </c>
+      <c r="B98" s="11" t="inlineStr">
+        <is>
+          <t>HSV-6 Bourací práce</t>
+        </is>
+      </c>
+      <c r="C98" s="11" t="inlineStr">
+        <is>
+          <t>Demontáž stávajících vstupních dveří + rámů — 2 ks (1× ulice Fibichova + 1× zahrada; návrh nové plastové vstupní dveře)</t>
+        </is>
+      </c>
+      <c r="D98" s="10" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="E98" s="12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F98" s="11" t="inlineStr">
+        <is>
+          <t>DXF INSERT dveře = 2 (Path C Tier 4) + TZ ARS</t>
+        </is>
+      </c>
+      <c r="G98" s="13" t="inlineStr">
+        <is>
+          <t>978013181</t>
+        </is>
+      </c>
+      <c r="H98" s="10" t="inlineStr">
+        <is>
+          <t>✓ verified</t>
+        </is>
+      </c>
+      <c r="I98" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV6.014</t>
+        </is>
+      </c>
+      <c r="J98" s="11" t="inlineStr"/>
+      <c r="K98" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="10" t="n">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B99" s="11" t="inlineStr">
         <is>
+          <t>HSV-6 Bourací práce</t>
+        </is>
+      </c>
+      <c r="C99" s="11" t="inlineStr">
+        <is>
+          <t>Demontáž stávajících vnitřních dveří vč. ocelových/dřevěných zárubní — odhad 15 ks (3 patra × ~5 dveří/patro per DXF SM__dveře layer)</t>
+        </is>
+      </c>
+      <c r="D99" s="10" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="E99" s="12" t="n">
+        <v>15</v>
+      </c>
+      <c r="F99" s="11" t="inlineStr">
+        <is>
+          <t>DXF SM__dveře polylines 102 / ~3 fáze / ~2.3 symbol per dveře ≈ 15 ks návrh (Path C confidence 0.65)</t>
+        </is>
+      </c>
+      <c r="G99" s="11" t="inlineStr">
+        <is>
+          <t>968072456</t>
+        </is>
+      </c>
+      <c r="H99" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I99" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV6.015</t>
+        </is>
+      </c>
+      <c r="J99" s="11" t="inlineStr"/>
+      <c r="K99" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="10" t="n">
+        <v>93</v>
+      </c>
+      <c r="B100" s="11" t="inlineStr">
+        <is>
+          <t>HSV-6 Bourací práce</t>
+        </is>
+      </c>
+      <c r="C100" s="11" t="inlineStr">
+        <is>
+          <t>Bourání vrchní části stávajícího komínu v posledním podlaží (cihelné zdivo, ručně), vč. likvidace cihelné suti</t>
+        </is>
+      </c>
+      <c r="D100" s="10" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="E100" s="12" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F100" s="11" t="inlineStr">
+        <is>
+          <t>průměr komín 0.50×0.50 × výška nad střechou ~2.4 m = 0.6 m³ (OPRAVA ChatGPT revize 2026-05-29: dříve 6.0 m³ = ×10 chybná inflace; skutečný objem 0.6 m³)</t>
+        </is>
+      </c>
+      <c r="G100" s="13" t="inlineStr">
+        <is>
+          <t>962024141</t>
+        </is>
+      </c>
+      <c r="H100" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I100" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV6.016</t>
+        </is>
+      </c>
+      <c r="J100" s="11" t="inlineStr"/>
+      <c r="K100" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="10" t="n">
+        <v>94</v>
+      </c>
+      <c r="B101" s="11" t="inlineStr">
+        <is>
+          <t>HSV-6 Bourací práce</t>
+        </is>
+      </c>
+      <c r="C101" s="11" t="inlineStr">
+        <is>
+          <t>Bourání stávajících opěrných zídek a venkovního schodiště v zahradě/dvoře — částečné, dle vyznačení v půdorysech bourání</t>
+        </is>
+      </c>
+      <c r="D101" s="10" t="inlineStr">
+        <is>
+          <t>m³</t>
+        </is>
+      </c>
+      <c r="E101" s="12" t="n">
+        <v>8</v>
+      </c>
+      <c r="F101" s="11" t="inlineStr">
+        <is>
+          <t>odhad ze řez A-A bourání + půdorys bourání 1.NP/1.PP, ~8 m³ celkem (opěrné zídky + venkovní schodiště zahrada/dvůr)</t>
+        </is>
+      </c>
+      <c r="G101" s="13" t="inlineStr">
+        <is>
+          <t>961044111</t>
+        </is>
+      </c>
+      <c r="H101" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I101" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV6.017</t>
+        </is>
+      </c>
+      <c r="J101" s="11" t="inlineStr"/>
+      <c r="K101" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="8" t="inlineStr">
+        <is>
+          <t>━━ HSV-7 Fasáda ETICS  (9 atomic operací) ━━</t>
+        </is>
+      </c>
+      <c r="B102" s="9" t="n"/>
+      <c r="C102" s="9" t="n"/>
+      <c r="D102" s="9" t="n"/>
+      <c r="E102" s="9" t="n"/>
+      <c r="F102" s="9" t="n"/>
+      <c r="G102" s="9" t="n"/>
+      <c r="H102" s="9" t="n"/>
+      <c r="I102" s="9" t="n"/>
+      <c r="J102" s="9" t="n"/>
+      <c r="K102" s="9" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="10" t="n">
+        <v>95</v>
+      </c>
+      <c r="B103" s="11" t="inlineStr">
+        <is>
           <t>HSV-7 Fasáda ETICS</t>
         </is>
       </c>
-      <c r="C99" s="11" t="inlineStr">
+      <c r="C103" s="11" t="inlineStr">
         <is>
           <t>Příprava fasádního podkladu — očištění tlakovou vodou, vyspravení omítek, fungicidní nátěr</t>
         </is>
       </c>
-      <c r="D99" s="10" t="inlineStr">
+      <c r="D103" s="10" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E99" s="12" t="n">
+      <c r="E103" s="12" t="n">
         <v>276.7</v>
       </c>
-      <c r="F99" s="11" t="inlineStr">
+      <c r="F103" s="11" t="inlineStr">
         <is>
           <t>obvod 38.7 m (DXF) × 0.55 (volná fasáda, štíty zachované) × výška 13.0 m = 276.7 m²</t>
         </is>
       </c>
-      <c r="G99" s="11" t="inlineStr">
+      <c r="G103" s="11" t="inlineStr">
         <is>
           <t>622401110</t>
         </is>
       </c>
-      <c r="H99" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I99" s="11" t="inlineStr">
+      <c r="H103" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I103" s="11" t="inlineStr">
         <is>
           <t>260219_dum.HSV7.001</t>
         </is>
       </c>
-      <c r="J99" s="11" t="inlineStr">
+      <c r="J103" s="11" t="inlineStr">
         <is>
           <t>S01</t>
         </is>
       </c>
-      <c r="K99" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="100">
-      <c r="A100" s="14" t="n">
-        <v>92</v>
-      </c>
-      <c r="B100" s="15" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda ETICS</t>
-        </is>
-      </c>
-      <c r="C100" s="15" t="inlineStr">
-        <is>
-          <t>Lepení + kotvení desek EPS 70F grey λ=0.032 tl. 160 mm — ETICS kontaktní zateplení fasády</t>
-        </is>
-      </c>
-      <c r="D100" s="14" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E100" s="16" t="n">
-        <v>276.7</v>
-      </c>
-      <c r="F100" s="15">
-        <f> HSV7.002 plocha fasády 276.7 m²</f>
-        <v/>
-      </c>
-      <c r="G100" s="15" t="inlineStr">
-        <is>
-          <t>713</t>
-        </is>
-      </c>
-      <c r="H100" s="14" t="inlineStr">
-        <is>
-          <t>⚠ família ??? (ÚRS online)</t>
-        </is>
-      </c>
-      <c r="I100" s="15" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.002 → HSV7.002a</t>
-        </is>
-      </c>
-      <c r="J100" s="15" t="inlineStr">
-        <is>
-          <t>S01, S12a</t>
-        </is>
-      </c>
-      <c r="K100" s="15" t="inlineStr">
-        <is>
-          <t>Lepení+kotvení EPS (713/622 família). Leaf dle tl. 160 mm — verify.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="14" t="n">
-        <v>93</v>
-      </c>
-      <c r="B101" s="15" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda ETICS</t>
-        </is>
-      </c>
-      <c r="C101" s="15" t="inlineStr">
-        <is>
-          <t>Armovací vrstva — výztužná síťka + lepicí stěrka (zatírací) na ETICS</t>
-        </is>
-      </c>
-      <c r="D101" s="14" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E101" s="16" t="n">
-        <v>276.7</v>
-      </c>
-      <c r="F101" s="15">
-        <f> HSV7.002 plocha 276.7 m²</f>
-        <v/>
-      </c>
-      <c r="G101" s="15" t="inlineStr">
-        <is>
-          <t>622</t>
-        </is>
-      </c>
-      <c r="H101" s="14" t="inlineStr">
-        <is>
-          <t>⚠ família ??? (ÚRS online)</t>
-        </is>
-      </c>
-      <c r="I101" s="15" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.002 → HSV7.002b</t>
-        </is>
-      </c>
-      <c r="J101" s="15" t="inlineStr">
-        <is>
-          <t>S01, S12a</t>
-        </is>
-      </c>
-      <c r="K101" s="15" t="inlineStr">
-        <is>
-          <t>Armovací vrstva síťka+stěrka (622 família). Finální omítka je samostatně HSV7.006.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
-        </is>
-      </c>
-    </row>
-    <row r="102">
-      <c r="A102" s="14" t="n">
-        <v>94</v>
-      </c>
-      <c r="B102" s="15" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda ETICS</t>
-        </is>
-      </c>
-      <c r="C102" s="15" t="inlineStr">
-        <is>
-          <t>Lepení + kotvení desek XPS λ=0.034 tl. 120 mm + soklový profil — ETICS sokl</t>
-        </is>
-      </c>
-      <c r="D102" s="14" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E102" s="16" t="n">
-        <v>13.5</v>
-      </c>
-      <c r="F102" s="15">
-        <f> HSV7.003 plocha soklu 13.5 m²</f>
-        <v/>
-      </c>
-      <c r="G102" s="15" t="inlineStr">
-        <is>
-          <t>713</t>
-        </is>
-      </c>
-      <c r="H102" s="14" t="inlineStr">
-        <is>
-          <t>⚠ família ??? (ÚRS online)</t>
-        </is>
-      </c>
-      <c r="I102" s="15" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.003 → HSV7.003a</t>
-        </is>
-      </c>
-      <c r="J102" s="15" t="inlineStr">
-        <is>
-          <t>S01</t>
-        </is>
-      </c>
-      <c r="K102" s="15" t="inlineStr">
-        <is>
-          <t>Sokl XPS lepení + soklový profil (713/622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
-        </is>
-      </c>
-    </row>
-    <row r="103">
-      <c r="A103" s="14" t="n">
-        <v>95</v>
-      </c>
-      <c r="B103" s="15" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda ETICS</t>
-        </is>
-      </c>
-      <c r="C103" s="15" t="inlineStr">
-        <is>
-          <t>Cihelný obklad soklu spárovaný (na armovací vrstvu)</t>
-        </is>
-      </c>
-      <c r="D103" s="14" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E103" s="16" t="n">
-        <v>13.5</v>
-      </c>
-      <c r="F103" s="15">
-        <f> HSV7.003 plocha soklu 13.5 m²</f>
-        <v/>
-      </c>
-      <c r="G103" s="15" t="inlineStr">
-        <is>
-          <t>781</t>
-        </is>
-      </c>
-      <c r="H103" s="14" t="inlineStr">
-        <is>
-          <t>⚠ família ??? (ÚRS online)</t>
-        </is>
-      </c>
-      <c r="I103" s="15" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.003 → HSV7.003b</t>
-        </is>
-      </c>
-      <c r="J103" s="15" t="inlineStr">
-        <is>
-          <t>S01</t>
-        </is>
-      </c>
-      <c r="K103" s="15" t="inlineStr">
-        <is>
-          <t>Cihelný obklad spárovaný (781 família obklady).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+      <c r="K103" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
         </is>
       </c>
     </row>
@@ -6671,24 +6671,24 @@
       </c>
       <c r="C104" s="15" t="inlineStr">
         <is>
-          <t>Špalety oken — EPS přesah 35-40 mm lepení + kotvení</t>
+          <t>Lepení + kotvení desek EPS 70F grey λ=0.032 tl. 160 mm — ETICS kontaktní zateplení fasády</t>
         </is>
       </c>
       <c r="D104" s="14" t="inlineStr">
         <is>
-          <t>bm</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E104" s="16" t="n">
-        <v>82.2</v>
+        <v>276.7</v>
       </c>
       <c r="F104" s="15">
-        <f> HSV7.004 obvod špalet 82.2 bm</f>
+        <f> HSV7.002 plocha fasády 276.7 m²</f>
         <v/>
       </c>
       <c r="G104" s="15" t="inlineStr">
         <is>
-          <t>622</t>
+          <t>713</t>
         </is>
       </c>
       <c r="H104" s="14" t="inlineStr">
@@ -6698,7 +6698,7 @@
       </c>
       <c r="I104" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.004 → HSV7.004a</t>
+          <t>260219_dum.HSV7.002 → HSV7.002a</t>
         </is>
       </c>
       <c r="J104" s="15" t="inlineStr">
@@ -6708,7 +6708,7 @@
       </c>
       <c r="K104" s="15" t="inlineStr">
         <is>
-          <t>Špalety EPS přesah (622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+          <t>Lepení+kotvení EPS (713/622 família). Leaf dle tl. 160 mm — verify.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -6723,148 +6723,356 @@
       </c>
       <c r="C105" s="15" t="inlineStr">
         <is>
+          <t>Armovací vrstva — výztužná síťka + lepicí stěrka (zatírací) na ETICS</t>
+        </is>
+      </c>
+      <c r="D105" s="14" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E105" s="16" t="n">
+        <v>276.7</v>
+      </c>
+      <c r="F105" s="15">
+        <f> HSV7.002 plocha 276.7 m²</f>
+        <v/>
+      </c>
+      <c r="G105" s="15" t="inlineStr">
+        <is>
+          <t>622</t>
+        </is>
+      </c>
+      <c r="H105" s="14" t="inlineStr">
+        <is>
+          <t>⚠ família ??? (ÚRS online)</t>
+        </is>
+      </c>
+      <c r="I105" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.002 → HSV7.002b</t>
+        </is>
+      </c>
+      <c r="J105" s="15" t="inlineStr">
+        <is>
+          <t>S01, S12a</t>
+        </is>
+      </c>
+      <c r="K105" s="15" t="inlineStr">
+        <is>
+          <t>Armovací vrstva síťka+stěrka (622 família). Finální omítka je samostatně HSV7.006.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="14" t="n">
+        <v>98</v>
+      </c>
+      <c r="B106" s="15" t="inlineStr">
+        <is>
+          <t>HSV-7 Fasáda ETICS</t>
+        </is>
+      </c>
+      <c r="C106" s="15" t="inlineStr">
+        <is>
+          <t>Lepení + kotvení desek XPS λ=0.034 tl. 120 mm + soklový profil — ETICS sokl</t>
+        </is>
+      </c>
+      <c r="D106" s="14" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E106" s="16" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F106" s="15">
+        <f> HSV7.003 plocha soklu 13.5 m²</f>
+        <v/>
+      </c>
+      <c r="G106" s="15" t="inlineStr">
+        <is>
+          <t>713</t>
+        </is>
+      </c>
+      <c r="H106" s="14" t="inlineStr">
+        <is>
+          <t>⚠ família ??? (ÚRS online)</t>
+        </is>
+      </c>
+      <c r="I106" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.003 → HSV7.003a</t>
+        </is>
+      </c>
+      <c r="J106" s="15" t="inlineStr">
+        <is>
+          <t>S01</t>
+        </is>
+      </c>
+      <c r="K106" s="15" t="inlineStr">
+        <is>
+          <t>Sokl XPS lepení + soklový profil (713/622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="14" t="n">
+        <v>99</v>
+      </c>
+      <c r="B107" s="15" t="inlineStr">
+        <is>
+          <t>HSV-7 Fasáda ETICS</t>
+        </is>
+      </c>
+      <c r="C107" s="15" t="inlineStr">
+        <is>
+          <t>Cihelný obklad soklu spárovaný (na armovací vrstvu)</t>
+        </is>
+      </c>
+      <c r="D107" s="14" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E107" s="16" t="n">
+        <v>13.5</v>
+      </c>
+      <c r="F107" s="15">
+        <f> HSV7.003 plocha soklu 13.5 m²</f>
+        <v/>
+      </c>
+      <c r="G107" s="15" t="inlineStr">
+        <is>
+          <t>781</t>
+        </is>
+      </c>
+      <c r="H107" s="14" t="inlineStr">
+        <is>
+          <t>⚠ família ??? (ÚRS online)</t>
+        </is>
+      </c>
+      <c r="I107" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.003 → HSV7.003b</t>
+        </is>
+      </c>
+      <c r="J107" s="15" t="inlineStr">
+        <is>
+          <t>S01</t>
+        </is>
+      </c>
+      <c r="K107" s="15" t="inlineStr">
+        <is>
+          <t>Cihelný obklad spárovaný (781 família obklady).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="B108" s="15" t="inlineStr">
+        <is>
+          <t>HSV-7 Fasáda ETICS</t>
+        </is>
+      </c>
+      <c r="C108" s="15" t="inlineStr">
+        <is>
+          <t>Špalety oken — EPS přesah 35-40 mm lepení + kotvení</t>
+        </is>
+      </c>
+      <c r="D108" s="14" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="E108" s="16" t="n">
+        <v>82.2</v>
+      </c>
+      <c r="F108" s="15">
+        <f> HSV7.004 obvod špalet 82.2 bm</f>
+        <v/>
+      </c>
+      <c r="G108" s="15" t="inlineStr">
+        <is>
+          <t>622</t>
+        </is>
+      </c>
+      <c r="H108" s="14" t="inlineStr">
+        <is>
+          <t>⚠ família ??? (ÚRS online)</t>
+        </is>
+      </c>
+      <c r="I108" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.004 → HSV7.004a</t>
+        </is>
+      </c>
+      <c r="J108" s="15" t="inlineStr">
+        <is>
+          <t>S01, S12a</t>
+        </is>
+      </c>
+      <c r="K108" s="15" t="inlineStr">
+        <is>
+          <t>Špalety EPS přesah (622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="14" t="n">
+        <v>101</v>
+      </c>
+      <c r="B109" s="15" t="inlineStr">
+        <is>
+          <t>HSV-7 Fasáda ETICS</t>
+        </is>
+      </c>
+      <c r="C109" s="15" t="inlineStr">
+        <is>
           <t>Špalety oken — armovací vrstva síťka + omítka</t>
         </is>
       </c>
-      <c r="D105" s="14" t="inlineStr">
+      <c r="D109" s="14" t="inlineStr">
         <is>
           <t>bm</t>
         </is>
       </c>
-      <c r="E105" s="16" t="n">
+      <c r="E109" s="16" t="n">
         <v>82.2</v>
       </c>
-      <c r="F105" s="15">
+      <c r="F109" s="15">
         <f> HSV7.004 obvod 82.2 bm</f>
         <v/>
       </c>
-      <c r="G105" s="15" t="inlineStr">
+      <c r="G109" s="15" t="inlineStr">
         <is>
           <t>622</t>
         </is>
       </c>
-      <c r="H105" s="14" t="inlineStr">
+      <c r="H109" s="14" t="inlineStr">
         <is>
           <t>⚠ família ??? (ÚRS online)</t>
         </is>
       </c>
-      <c r="I105" s="15" t="inlineStr">
+      <c r="I109" s="15" t="inlineStr">
         <is>
           <t>260219_dum.HSV7.004 → HSV7.004b</t>
         </is>
       </c>
-      <c r="J105" s="15" t="inlineStr">
+      <c r="J109" s="15" t="inlineStr">
         <is>
           <t>S01, S12a</t>
         </is>
       </c>
-      <c r="K105" s="15" t="inlineStr">
+      <c r="K109" s="15" t="inlineStr">
         <is>
           <t>Armovací vrstva + omítka špalet (622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="10" t="n">
-        <v>98</v>
-      </c>
-      <c r="B106" s="11" t="inlineStr">
+    <row r="110">
+      <c r="A110" s="10" t="n">
+        <v>102</v>
+      </c>
+      <c r="B110" s="11" t="inlineStr">
         <is>
           <t>HSV-7 Fasáda ETICS</t>
         </is>
       </c>
-      <c r="C106" s="11" t="inlineStr">
+      <c r="C110" s="11" t="inlineStr">
         <is>
           <t>Profilace fasády — různé tloušťky EPS (kordony, šambrány, rámování oken) — paušál podle pohledů</t>
         </is>
       </c>
-      <c r="D106" s="10" t="inlineStr">
+      <c r="D110" s="10" t="inlineStr">
         <is>
           <t>soubor</t>
         </is>
       </c>
-      <c r="E106" s="12" t="n">
+      <c r="E110" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="F106" s="11" t="inlineStr">
+      <c r="F110" s="11" t="inlineStr">
         <is>
           <t>paušál — dle pohledů NCS NZÚ</t>
         </is>
       </c>
-      <c r="G106" s="11" t="inlineStr">
+      <c r="G110" s="11" t="inlineStr">
         <is>
           <t>622221221</t>
         </is>
       </c>
-      <c r="H106" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I106" s="11" t="inlineStr">
+      <c r="H110" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I110" s="11" t="inlineStr">
         <is>
           <t>260219_dum.HSV7.005</t>
         </is>
       </c>
-      <c r="J106" s="11" t="inlineStr">
+      <c r="J110" s="11" t="inlineStr">
         <is>
           <t>S01, S12a</t>
         </is>
       </c>
-      <c r="K106" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="107">
-      <c r="A107" s="10" t="n">
-        <v>99</v>
-      </c>
-      <c r="B107" s="11" t="inlineStr">
+      <c r="K110" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="10" t="n">
+        <v>103</v>
+      </c>
+      <c r="B111" s="11" t="inlineStr">
         <is>
           <t>HSV-7 Fasáda ETICS</t>
         </is>
       </c>
-      <c r="C107" s="11" t="inlineStr">
+      <c r="C111" s="11" t="inlineStr">
         <is>
           <t>Tenkovrstvá pastovitá probarvená omítka, lomená bílá NCS NZÚ — finální vrstva ETICS</t>
         </is>
       </c>
-      <c r="D107" s="10" t="inlineStr">
+      <c r="D111" s="10" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E107" s="12" t="n">
+      <c r="E111" s="12" t="n">
         <v>290.2</v>
       </c>
-      <c r="F107" s="11" t="inlineStr">
+      <c r="F111" s="11" t="inlineStr">
         <is>
           <t>ETICS plocha 276.7 m² + sokl 13.5 m² = 290.2 m²</t>
         </is>
       </c>
-      <c r="G107" s="13" t="inlineStr">
+      <c r="G111" s="13" t="inlineStr">
         <is>
           <t>622521111</t>
         </is>
       </c>
-      <c r="H107" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I107" s="11" t="inlineStr">
+      <c r="H111" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I111" s="11" t="inlineStr">
         <is>
           <t>260219_dum.HSV7.006</t>
         </is>
       </c>
-      <c r="J107" s="11" t="inlineStr">
+      <c r="J111" s="11" t="inlineStr">
         <is>
           <t>S01, S12a, S12b</t>
         </is>
       </c>
-      <c r="K107" s="11" t="inlineStr">
+      <c r="K111" s="11" t="inlineStr">
         <is>
           <t>Carried 1:1 (atomic — no decomposition needed)</t>
         </is>
@@ -6876,10 +7084,10 @@
     <mergeCell ref="A22:K22"/>
     <mergeCell ref="A59:K59"/>
     <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A98:K98"/>
+    <mergeCell ref="A84:K84"/>
     <mergeCell ref="A36:K36"/>
     <mergeCell ref="A44:K44"/>
-    <mergeCell ref="A80:K80"/>
+    <mergeCell ref="A102:K102"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -15054,7 +15262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -15826,6 +16034,39 @@
       <c r="G23" s="15" t="inlineStr">
         <is>
           <t>HSV1.015a, HSV1.015b, HSV1.015c</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV5.017</t>
+        </is>
+      </c>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>HSV-5 Krov + střecha</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>Montáž svorníků / šroubů tesařských spojů krovu délky přes 150 do 300 mm — spojení kleštin 2×60/180 mm s krokvemi (svorn</t>
+        </is>
+      </c>
+      <c r="D24" s="14" t="inlineStr">
+        <is>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="E24" s="16" t="n">
+        <v>50</v>
+      </c>
+      <c r="F24" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="G24" s="15" t="inlineStr">
+        <is>
+          <t>HSV5.017a, HSV5.017b, HSV5.017c, HSV5.017d</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(rd-jachymov): schema — unique entity ids (Pattern 28), renumber 26 dup ids
Commit 2/2 of skladby workflow. Fixes systemic duplicate-id bug: id=objekt.KAPITOLA.seq
with seq restarting per subkapitola caused collisions (PSV71.001/002 ×2, PSV76.001-004 ×4,
VRN.001/002/003 ×many, sklad VRN.001 ×3).

Deterministic block-scheme renumber per (objekt, id-prefix) WITH collisions: distinct
kapitola strings ordered by first appearance; rank0 keeps numeric suffix, rank k≥1 →
k*100+local. Non-numeric (PM01/PM02) untouched. Prefixes without collisions untouched.
26 ids renumbered (e.g. PSV76 Klempíř→101-104, Zámečnictví→201-204, Truhlář→301-302;
PSV71 TI→101-102; VRN per-kapitola blocks). 2 atomic_decomposition keys auto-updated
(PSV76.002/Truhlář→302, PSV76.003/Klempíř→103) — terasa + dešťové svody decomp intact.

Verify: 228 items, 228 unique ids, 0 duplicates. 9-step regen + assert pass.

https://claude.ai/code/session_01FskzLAZkXgJAwuN2cQQEdx
</commit_message>
<xml_diff>
--- a/test-data/RD_Jachymov_dum/outputs/Vykaz_vymer_RD_Jachymov_ATOMIC_WORKLIST_2026-05-27.xlsx
+++ b/test-data/RD_Jachymov_dum/outputs/Vykaz_vymer_RD_Jachymov_ATOMIC_WORKLIST_2026-05-27.xlsx
@@ -8383,7 +8383,7 @@
       </c>
       <c r="I7" s="18" t="inlineStr">
         <is>
-          <t>260219_dum.PSV71.001</t>
+          <t>260219_dum.PSV71.101</t>
         </is>
       </c>
       <c r="J7" s="18" t="inlineStr"/>
@@ -8427,7 +8427,7 @@
       </c>
       <c r="I8" s="18" t="inlineStr">
         <is>
-          <t>260219_dum.PSV71.002</t>
+          <t>260219_dum.PSV71.102</t>
         </is>
       </c>
       <c r="J8" s="18" t="inlineStr">
@@ -10294,7 +10294,7 @@
       </c>
       <c r="I48" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.PSV76.001</t>
+          <t>260219_dum.PSV76.101</t>
         </is>
       </c>
       <c r="J48" s="11" t="inlineStr"/>
@@ -10342,7 +10342,7 @@
       </c>
       <c r="I49" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.PSV76.002</t>
+          <t>260219_dum.PSV76.102</t>
         </is>
       </c>
       <c r="J49" s="11" t="inlineStr"/>
@@ -10391,7 +10391,7 @@
       </c>
       <c r="I50" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV76.003 → PSV76.003a</t>
+          <t>260219_dum.PSV76.103 → PSV76.103a</t>
         </is>
       </c>
       <c r="J50" s="15" t="inlineStr"/>
@@ -10439,7 +10439,7 @@
       </c>
       <c r="I51" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV76.003 → PSV76.003b</t>
+          <t>260219_dum.PSV76.103 → PSV76.103b</t>
         </is>
       </c>
       <c r="J51" s="15" t="inlineStr"/>
@@ -10488,7 +10488,7 @@
       </c>
       <c r="I52" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.PSV76.004</t>
+          <t>260219_dum.PSV76.104</t>
         </is>
       </c>
       <c r="J52" s="11" t="inlineStr"/>
@@ -10554,7 +10554,7 @@
       </c>
       <c r="I54" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.PSV76.001</t>
+          <t>260219_dum.PSV76.301</t>
         </is>
       </c>
       <c r="J54" s="11" t="inlineStr"/>
@@ -10602,7 +10602,7 @@
       </c>
       <c r="I55" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV76.002 → PSV76.002a</t>
+          <t>260219_dum.PSV76.302 → PSV76.302a</t>
         </is>
       </c>
       <c r="J55" s="15" t="inlineStr"/>
@@ -10650,7 +10650,7 @@
       </c>
       <c r="I56" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV76.002 → PSV76.002b</t>
+          <t>260219_dum.PSV76.302 → PSV76.302b</t>
         </is>
       </c>
       <c r="J56" s="15" t="inlineStr"/>
@@ -11321,7 +11321,7 @@
       </c>
       <c r="I71" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.PSV76.001</t>
+          <t>260219_dum.PSV76.201</t>
         </is>
       </c>
       <c r="J71" s="11" t="inlineStr"/>
@@ -11370,7 +11370,7 @@
       </c>
       <c r="I72" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.PSV76.002</t>
+          <t>260219_dum.PSV76.202</t>
         </is>
       </c>
       <c r="J72" s="11" t="inlineStr"/>
@@ -11419,7 +11419,7 @@
       </c>
       <c r="I73" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.PSV76.003</t>
+          <t>260219_dum.PSV76.203</t>
         </is>
       </c>
       <c r="J73" s="11" t="inlineStr"/>
@@ -11468,7 +11468,7 @@
       </c>
       <c r="I74" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.PSV76.004</t>
+          <t>260219_dum.PSV76.204</t>
         </is>
       </c>
       <c r="J74" s="11" t="inlineStr"/>
@@ -13764,7 +13764,7 @@
       </c>
       <c r="I8" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.VRN.001</t>
+          <t>260219_dum.VRN.101</t>
         </is>
       </c>
       <c r="J8" s="11" t="inlineStr"/>
@@ -13813,7 +13813,7 @@
       </c>
       <c r="I9" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.VRN.002</t>
+          <t>260219_dum.VRN.102</t>
         </is>
       </c>
       <c r="J9" s="11" t="inlineStr"/>
@@ -13862,7 +13862,7 @@
       </c>
       <c r="I10" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.VRN.003</t>
+          <t>260219_dum.VRN.103</t>
         </is>
       </c>
       <c r="J10" s="11" t="inlineStr"/>
@@ -13928,7 +13928,7 @@
       </c>
       <c r="I12" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.VRN.001</t>
+          <t>260219_dum.VRN.201</t>
         </is>
       </c>
       <c r="J12" s="11" t="inlineStr"/>
@@ -13994,7 +13994,7 @@
       </c>
       <c r="I14" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.VRN.001</t>
+          <t>260219_dum.VRN.301</t>
         </is>
       </c>
       <c r="J14" s="11" t="inlineStr"/>
@@ -14043,7 +14043,7 @@
       </c>
       <c r="I15" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.VRN.002</t>
+          <t>260219_dum.VRN.302</t>
         </is>
       </c>
       <c r="J15" s="11" t="inlineStr"/>
@@ -14109,7 +14109,7 @@
       </c>
       <c r="I17" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.VRN.001</t>
+          <t>260219_dum.VRN.401</t>
         </is>
       </c>
       <c r="J17" s="11" t="inlineStr"/>
@@ -14158,7 +14158,7 @@
       </c>
       <c r="I18" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.VRN.002</t>
+          <t>260219_dum.VRN.402</t>
         </is>
       </c>
       <c r="J18" s="11" t="inlineStr"/>
@@ -14224,7 +14224,7 @@
       </c>
       <c r="I20" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.VRN.001</t>
+          <t>260219_dum.VRN.501</t>
         </is>
       </c>
       <c r="J20" s="11" t="inlineStr"/>
@@ -14290,7 +14290,7 @@
       </c>
       <c r="I22" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.VRN.001</t>
+          <t>260219_dum.VRN.601</t>
         </is>
       </c>
       <c r="J22" s="11" t="inlineStr"/>
@@ -14356,7 +14356,7 @@
       </c>
       <c r="I24" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.VRN.001</t>
+          <t>260219_dum.VRN.701</t>
         </is>
       </c>
       <c r="J24" s="11" t="inlineStr"/>
@@ -14422,7 +14422,7 @@
       </c>
       <c r="I26" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.VRN.001</t>
+          <t>260219_dum.VRN.801</t>
         </is>
       </c>
       <c r="J26" s="11" t="inlineStr"/>
@@ -16165,7 +16165,7 @@
       </c>
       <c r="I37" s="11" t="inlineStr">
         <is>
-          <t>260217_sklad.VRN.001</t>
+          <t>260217_sklad.VRN.101</t>
         </is>
       </c>
       <c r="J37" s="11" t="inlineStr"/>
@@ -16231,7 +16231,7 @@
       </c>
       <c r="I39" s="11" t="inlineStr">
         <is>
-          <t>260217_sklad.VRN.001</t>
+          <t>260217_sklad.VRN.201</t>
         </is>
       </c>
       <c r="J39" s="11" t="inlineStr"/>
@@ -16647,7 +16647,7 @@
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV76.003</t>
+          <t>260219_dum.PSV76.103</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
@@ -16673,14 +16673,14 @@
       </c>
       <c r="G12" s="15" t="inlineStr">
         <is>
-          <t>PSV76.003a, PSV76.003b</t>
+          <t>PSV76.103a, PSV76.103b</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV76.002</t>
+          <t>260219_dum.PSV76.302</t>
         </is>
       </c>
       <c r="B13" s="15" t="inlineStr">
@@ -16706,7 +16706,7 @@
       </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
-          <t>PSV76.002a, PSV76.002b</t>
+          <t>PSV76.302a, PSV76.302b</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(rd-jachymov): F2 dedup demontáž oken (remove aggregate) + F3 vyjasnění #33 (234→233)
F2 — remove HSV6.010 'Demontáž všech oken a dveří' (aggregate 25 ks) that double-counted
the detailed HSV6.013 (okna 16) + HSV6.014 (vstupní 2) + HSV6.015 (vnitřní 15) = 33 ks.
Aggregate also undercounted (25<33). No atomic entry, no cross-ref → clean delete.
Detail wins (ChatGPT correct). items 234→233.

F3 — pažení sklad VERIFY: statika D.2.1 §4.2 says 'jáma svahovaná, sklon 1:0,5' →
sklad cut solved by SVAHOVÁNÍ not pažení (HSV1.006 pažení do 2m is DŮM). No contradiction,
no blind change. Open point → vyjasnění #33: verify HSV1.002 výkop volume includes 1:0,5
battering in prudký svah + utility-trench pažení dle BOZP.

F1 (411321414 ×8) SKIPPED — legit code-sharing, not a bug.
10-step regen + assert docx 30==queue 30. snapshot items_pre_f2f3.json.

https://claude.ai/code/session_01FskzLAZkXgJAwuN2cQQEdx
</commit_message>
<xml_diff>
--- a/test-data/RD_Jachymov_dum/outputs/Vykaz_vymer_RD_Jachymov_ATOMIC_WORKLIST_2026-05-27.xlsx
+++ b/test-data/RD_Jachymov_dum/outputs/Vykaz_vymer_RD_Jachymov_ATOMIC_WORKLIST_2026-05-27.xlsx
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="C6" s="2">
         <f> carried 1:1 + decomposed children</f>
@@ -628,7 +628,7 @@
         </is>
       </c>
       <c r="B9" s="5" t="n">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
@@ -732,7 +732,7 @@
         </is>
       </c>
       <c r="B20" s="5" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="21">
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="B52" s="5" t="n">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="53">
@@ -1490,7 +1490,7 @@
     <row r="100">
       <c r="A100" s="4" t="inlineStr">
         <is>
-          <t>968</t>
+          <t>978</t>
         </is>
       </c>
       <c r="B100" s="5" t="n">
@@ -1500,17 +1500,17 @@
     <row r="101">
       <c r="A101" s="4" t="inlineStr">
         <is>
-          <t>978</t>
+          <t>012</t>
         </is>
       </c>
       <c r="B101" s="5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" s="4" t="inlineStr">
         <is>
-          <t>012</t>
+          <t>151</t>
         </is>
       </c>
       <c r="B102" s="5" t="n">
@@ -1520,7 +1520,7 @@
     <row r="103">
       <c r="A103" s="4" t="inlineStr">
         <is>
-          <t>151</t>
+          <t>181</t>
         </is>
       </c>
       <c r="B103" s="5" t="n">
@@ -1530,7 +1530,7 @@
     <row r="104">
       <c r="A104" s="4" t="inlineStr">
         <is>
-          <t>181</t>
+          <t>271</t>
         </is>
       </c>
       <c r="B104" s="5" t="n">
@@ -1540,7 +1540,7 @@
     <row r="105">
       <c r="A105" s="4" t="inlineStr">
         <is>
-          <t>271</t>
+          <t>279</t>
         </is>
       </c>
       <c r="B105" s="5" t="n">
@@ -1550,7 +1550,7 @@
     <row r="106">
       <c r="A106" s="4" t="inlineStr">
         <is>
-          <t>279</t>
+          <t>375</t>
         </is>
       </c>
       <c r="B106" s="5" t="n">
@@ -1560,7 +1560,7 @@
     <row r="107">
       <c r="A107" s="4" t="inlineStr">
         <is>
-          <t>375</t>
+          <t>596</t>
         </is>
       </c>
       <c r="B107" s="5" t="n">
@@ -1570,7 +1570,7 @@
     <row r="108">
       <c r="A108" s="4" t="inlineStr">
         <is>
-          <t>596</t>
+          <t>721</t>
         </is>
       </c>
       <c r="B108" s="5" t="n">
@@ -1580,7 +1580,7 @@
     <row r="109">
       <c r="A109" s="4" t="inlineStr">
         <is>
-          <t>721</t>
+          <t>734</t>
         </is>
       </c>
       <c r="B109" s="5" t="n">
@@ -1590,7 +1590,7 @@
     <row r="110">
       <c r="A110" s="4" t="inlineStr">
         <is>
-          <t>734</t>
+          <t>765</t>
         </is>
       </c>
       <c r="B110" s="5" t="n">
@@ -1600,7 +1600,7 @@
     <row r="111">
       <c r="A111" s="4" t="inlineStr">
         <is>
-          <t>765</t>
+          <t>783</t>
         </is>
       </c>
       <c r="B111" s="5" t="n">
@@ -1610,7 +1610,7 @@
     <row r="112">
       <c r="A112" s="4" t="inlineStr">
         <is>
-          <t>783</t>
+          <t>961</t>
         </is>
       </c>
       <c r="B112" s="5" t="n">
@@ -1620,7 +1620,7 @@
     <row r="113">
       <c r="A113" s="4" t="inlineStr">
         <is>
-          <t>961</t>
+          <t>966</t>
         </is>
       </c>
       <c r="B113" s="5" t="n">
@@ -1630,7 +1630,7 @@
     <row r="114">
       <c r="A114" s="4" t="inlineStr">
         <is>
-          <t>966</t>
+          <t>968</t>
         </is>
       </c>
       <c r="B114" s="5" t="n">
@@ -1731,7 +1731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K132"/>
+  <dimension ref="A1:K131"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -6468,7 +6468,7 @@
     <row r="98">
       <c r="A98" s="8" t="inlineStr">
         <is>
-          <t>━━ HSV-6 Bourací práce  (18 atomic operací) ━━</t>
+          <t>━━ HSV-6 Bourací práce  (17 atomic operací) ━━</t>
         </is>
       </c>
       <c r="B98" s="9" t="n"/>
@@ -6928,7 +6928,7 @@
       </c>
       <c r="C108" s="11" t="inlineStr">
         <is>
-          <t>Demontáž všech oken a dveří stávajících (recyklace)</t>
+          <t>Demontáž všech sanitárních zařizovacích předmětů (WC, umyvadla, baterie, sprcha)</t>
         </is>
       </c>
       <c r="D108" s="10" t="inlineStr">
@@ -6937,16 +6937,16 @@
         </is>
       </c>
       <c r="E108" s="12" t="n">
-        <v>25</v>
+        <v>12</v>
       </c>
       <c r="F108" s="11" t="inlineStr">
         <is>
-          <t>odhad — ~10 oken + ~15 dveří (vstupní + vnitřní)</t>
+          <t>odhad — 2 koupelny × ~5 ks + WC + dřez = ~12</t>
         </is>
       </c>
       <c r="G108" s="11" t="inlineStr">
         <is>
-          <t>968071120</t>
+          <t>725900001</t>
         </is>
       </c>
       <c r="H108" s="10" t="inlineStr">
@@ -6956,7 +6956,7 @@
       </c>
       <c r="I108" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.010</t>
+          <t>260219_dum.HSV6.011</t>
         </is>
       </c>
       <c r="J108" s="11" t="inlineStr"/>
@@ -6977,25 +6977,25 @@
       </c>
       <c r="C109" s="11" t="inlineStr">
         <is>
-          <t>Demontáž všech sanitárních zařizovacích předmětů (WC, umyvadla, baterie, sprcha)</t>
+          <t>Odvoz a likvidace stavební suti dle vyhl. 8/2021 Sb. — celková tonáž odpadů</t>
         </is>
       </c>
       <c r="D109" s="10" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>t</t>
         </is>
       </c>
       <c r="E109" s="12" t="n">
-        <v>12</v>
+        <v>56.5</v>
       </c>
       <c r="F109" s="11" t="inlineStr">
         <is>
-          <t>odhad — 2 koupelny × ~5 ks + WC + dřez = ~12</t>
+          <t>TZ B m.10.e: 46 (beton/cihly) + 9 (dřevo) + 0.1 (kov) + 0.1 (EPS) + 0.2 (sádra) + 1.0 (směs) = 56.4</t>
         </is>
       </c>
       <c r="G109" s="11" t="inlineStr">
         <is>
-          <t>725900001</t>
+          <t>997013501</t>
         </is>
       </c>
       <c r="H109" s="10" t="inlineStr">
@@ -7005,7 +7005,7 @@
       </c>
       <c r="I109" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.011</t>
+          <t>260219_dum.HSV6.012</t>
         </is>
       </c>
       <c r="J109" s="11" t="inlineStr"/>
@@ -7026,35 +7026,35 @@
       </c>
       <c r="C110" s="11" t="inlineStr">
         <is>
-          <t>Odvoz a likvidace stavební suti dle vyhl. 8/2021 Sb. — celková tonáž odpadů</t>
+          <t>Demontáž stávajících dřevěných oken vč. rámů a parapetů — 16 ks (návrh všechna okna nová plastová trojsklem)</t>
         </is>
       </c>
       <c r="D110" s="10" t="inlineStr">
         <is>
-          <t>t</t>
+          <t>ks</t>
         </is>
       </c>
       <c r="E110" s="12" t="n">
-        <v>56.5</v>
+        <v>16</v>
       </c>
       <c r="F110" s="11" t="inlineStr">
         <is>
-          <t>TZ B m.10.e: 46 (beton/cihly) + 9 (dřevo) + 0.1 (kov) + 0.1 (EPS) + 0.2 (sádra) + 1.0 (směs) = 56.4</t>
-        </is>
-      </c>
-      <c r="G110" s="11" t="inlineStr">
-        <is>
-          <t>997013501</t>
+          <t>DXF INSERT okno* total 16 ks (Path C Tier 4 — front 9 + back 7)</t>
+        </is>
+      </c>
+      <c r="G110" s="13" t="inlineStr">
+        <is>
+          <t>978013181</t>
         </is>
       </c>
       <c r="H110" s="10" t="inlineStr">
         <is>
-          <t>⚠ kandidát-verify</t>
+          <t>✓ verified</t>
         </is>
       </c>
       <c r="I110" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.012</t>
+          <t>260219_dum.HSV6.013</t>
         </is>
       </c>
       <c r="J110" s="11" t="inlineStr"/>
@@ -7075,7 +7075,7 @@
       </c>
       <c r="C111" s="11" t="inlineStr">
         <is>
-          <t>Demontáž stávajících dřevěných oken vč. rámů a parapetů — 16 ks (návrh všechna okna nová plastová trojsklem)</t>
+          <t>Demontáž stávajících vstupních dveří + rámů — 2 ks (1× ulice Fibichova + 1× zahrada; návrh nové plastové vstupní dveře)</t>
         </is>
       </c>
       <c r="D111" s="10" t="inlineStr">
@@ -7084,11 +7084,11 @@
         </is>
       </c>
       <c r="E111" s="12" t="n">
-        <v>16</v>
+        <v>2</v>
       </c>
       <c r="F111" s="11" t="inlineStr">
         <is>
-          <t>DXF INSERT okno* total 16 ks (Path C Tier 4 — front 9 + back 7)</t>
+          <t>DXF INSERT dveře = 2 (Path C Tier 4) + TZ ARS</t>
         </is>
       </c>
       <c r="G111" s="13" t="inlineStr">
@@ -7103,7 +7103,7 @@
       </c>
       <c r="I111" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.013</t>
+          <t>260219_dum.HSV6.014</t>
         </is>
       </c>
       <c r="J111" s="11" t="inlineStr"/>
@@ -7124,7 +7124,7 @@
       </c>
       <c r="C112" s="11" t="inlineStr">
         <is>
-          <t>Demontáž stávajících vstupních dveří + rámů — 2 ks (1× ulice Fibichova + 1× zahrada; návrh nové plastové vstupní dveře)</t>
+          <t>Demontáž stávajících vnitřních dveří vč. ocelových/dřevěných zárubní — odhad 15 ks (3 patra × ~5 dveří/patro per DXF SM__dveře layer)</t>
         </is>
       </c>
       <c r="D112" s="10" t="inlineStr">
@@ -7133,26 +7133,26 @@
         </is>
       </c>
       <c r="E112" s="12" t="n">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="F112" s="11" t="inlineStr">
         <is>
-          <t>DXF INSERT dveře = 2 (Path C Tier 4) + TZ ARS</t>
-        </is>
-      </c>
-      <c r="G112" s="13" t="inlineStr">
-        <is>
-          <t>978013181</t>
+          <t>DXF SM__dveře polylines 102 / ~3 fáze / ~2.3 symbol per dveře ≈ 15 ks návrh (Path C confidence 0.65)</t>
+        </is>
+      </c>
+      <c r="G112" s="11" t="inlineStr">
+        <is>
+          <t>968072456</t>
         </is>
       </c>
       <c r="H112" s="10" t="inlineStr">
         <is>
-          <t>✓ verified</t>
+          <t>⚠ kandidát-verify</t>
         </is>
       </c>
       <c r="I112" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.014</t>
+          <t>260219_dum.HSV6.015</t>
         </is>
       </c>
       <c r="J112" s="11" t="inlineStr"/>
@@ -7173,25 +7173,25 @@
       </c>
       <c r="C113" s="11" t="inlineStr">
         <is>
-          <t>Demontáž stávajících vnitřních dveří vč. ocelových/dřevěných zárubní — odhad 15 ks (3 patra × ~5 dveří/patro per DXF SM__dveře layer)</t>
+          <t>Bourání vrchní části stávajícího komínu v posledním podlaží (cihelné zdivo, ručně), vč. likvidace cihelné suti</t>
         </is>
       </c>
       <c r="D113" s="10" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>m³</t>
         </is>
       </c>
       <c r="E113" s="12" t="n">
-        <v>15</v>
+        <v>0.6</v>
       </c>
       <c r="F113" s="11" t="inlineStr">
         <is>
-          <t>DXF SM__dveře polylines 102 / ~3 fáze / ~2.3 symbol per dveře ≈ 15 ks návrh (Path C confidence 0.65)</t>
-        </is>
-      </c>
-      <c r="G113" s="11" t="inlineStr">
-        <is>
-          <t>968072456</t>
+          <t>průměr komín 0.50×0.50 × výška nad střechou ~2.4 m = 0.6 m³ (OPRAVA ChatGPT revize 2026-05-29: dříve 6.0 m³ = ×10 chybná inflace; skutečný objem 0.6 m³)</t>
+        </is>
+      </c>
+      <c r="G113" s="13" t="inlineStr">
+        <is>
+          <t>962024141</t>
         </is>
       </c>
       <c r="H113" s="10" t="inlineStr">
@@ -7201,7 +7201,7 @@
       </c>
       <c r="I113" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.015</t>
+          <t>260219_dum.HSV6.016</t>
         </is>
       </c>
       <c r="J113" s="11" t="inlineStr"/>
@@ -7222,7 +7222,7 @@
       </c>
       <c r="C114" s="11" t="inlineStr">
         <is>
-          <t>Bourání vrchní části stávajícího komínu v posledním podlaží (cihelné zdivo, ručně), vč. likvidace cihelné suti</t>
+          <t>Bourání stávajících opěrných zídek a venkovního schodiště v zahradě/dvoře — částečné, dle vyznačení v půdorysech bourání</t>
         </is>
       </c>
       <c r="D114" s="10" t="inlineStr">
@@ -7231,16 +7231,16 @@
         </is>
       </c>
       <c r="E114" s="12" t="n">
-        <v>0.6</v>
+        <v>8</v>
       </c>
       <c r="F114" s="11" t="inlineStr">
         <is>
-          <t>průměr komín 0.50×0.50 × výška nad střechou ~2.4 m = 0.6 m³ (OPRAVA ChatGPT revize 2026-05-29: dříve 6.0 m³ = ×10 chybná inflace; skutečný objem 0.6 m³)</t>
+          <t>odhad ze řez A-A bourání + půdorys bourání 1.NP/1.PP, ~8 m³ celkem (opěrné zídky + venkovní schodiště zahrada/dvůr)</t>
         </is>
       </c>
       <c r="G114" s="13" t="inlineStr">
         <is>
-          <t>962024141</t>
+          <t>961044111</t>
         </is>
       </c>
       <c r="H114" s="10" t="inlineStr">
@@ -7250,7 +7250,7 @@
       </c>
       <c r="I114" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.016</t>
+          <t>260219_dum.HSV6.017</t>
         </is>
       </c>
       <c r="J114" s="11" t="inlineStr"/>
@@ -7261,169 +7261,172 @@
       </c>
     </row>
     <row r="115">
-      <c r="A115" s="10" t="n">
+      <c r="A115" s="17" t="n">
         <v>108</v>
       </c>
-      <c r="B115" s="11" t="inlineStr">
+      <c r="B115" s="18" t="inlineStr">
         <is>
           <t>HSV-6 Bourací práce</t>
         </is>
       </c>
-      <c r="C115" s="11" t="inlineStr">
-        <is>
-          <t>Bourání stávajících opěrných zídek a venkovního schodiště v zahradě/dvoře — částečné, dle vyznačení v půdorysech bourání</t>
-        </is>
-      </c>
-      <c r="D115" s="10" t="inlineStr">
-        <is>
-          <t>m³</t>
-        </is>
-      </c>
-      <c r="E115" s="12" t="n">
-        <v>8</v>
-      </c>
-      <c r="F115" s="11" t="inlineStr">
-        <is>
-          <t>odhad ze řez A-A bourání + půdorys bourání 1.NP/1.PP, ~8 m³ celkem (opěrné zídky + venkovní schodiště zahrada/dvůr)</t>
-        </is>
-      </c>
-      <c r="G115" s="13" t="inlineStr">
-        <is>
-          <t>961044111</t>
-        </is>
-      </c>
-      <c r="H115" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I115" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV6.017</t>
-        </is>
-      </c>
-      <c r="J115" s="11" t="inlineStr"/>
-      <c r="K115" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="116">
-      <c r="A116" s="17" t="n">
-        <v>109</v>
-      </c>
-      <c r="B116" s="18" t="inlineStr">
-        <is>
-          <t>HSV-6 Bourací práce</t>
-        </is>
-      </c>
-      <c r="C116" s="18" t="inlineStr">
+      <c r="C115" s="18" t="inlineStr">
         <is>
           <t>Demontáž vnějšího keram. obkladu suterénu (sokl) 20 mm</t>
         </is>
       </c>
-      <c r="D116" s="17" t="inlineStr">
+      <c r="D115" s="17" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E116" s="19" t="n">
+      <c r="E115" s="19" t="n">
         <v>23</v>
       </c>
-      <c r="F116" s="18">
+      <c r="F115" s="18">
         <f> obvod 38.7 × 0.6 ≈ 23 (OVĚŘIT)</f>
         <v/>
       </c>
-      <c r="G116" s="18" t="inlineStr"/>
-      <c r="H116" s="17" t="inlineStr">
+      <c r="G115" s="18" t="inlineStr"/>
+      <c r="H115" s="17" t="inlineStr">
         <is>
           <t>❌ blank — ÚRS online</t>
         </is>
       </c>
-      <c r="I116" s="18" t="inlineStr">
+      <c r="I115" s="18" t="inlineStr">
         <is>
           <t>260219_dum.HSV6.018 → HSV6.018a</t>
         </is>
       </c>
-      <c r="J116" s="18" t="inlineStr">
+      <c r="J115" s="18" t="inlineStr">
         <is>
           <t>S03</t>
         </is>
       </c>
-      <c r="K116" s="18" t="inlineStr">
+      <c r="K115" s="18" t="inlineStr">
         <is>
           <t>Bourání.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
+    <row r="116">
+      <c r="A116" s="8" t="inlineStr">
+        <is>
+          <t>━━ HSV-7 Fasáda ETICS  (9 atomic operací) ━━</t>
+        </is>
+      </c>
+      <c r="B116" s="9" t="n"/>
+      <c r="C116" s="9" t="n"/>
+      <c r="D116" s="9" t="n"/>
+      <c r="E116" s="9" t="n"/>
+      <c r="F116" s="9" t="n"/>
+      <c r="G116" s="9" t="n"/>
+      <c r="H116" s="9" t="n"/>
+      <c r="I116" s="9" t="n"/>
+      <c r="J116" s="9" t="n"/>
+      <c r="K116" s="9" t="n"/>
+    </row>
     <row r="117">
-      <c r="A117" s="8" t="inlineStr">
-        <is>
-          <t>━━ HSV-7 Fasáda ETICS  (9 atomic operací) ━━</t>
-        </is>
-      </c>
-      <c r="B117" s="9" t="n"/>
-      <c r="C117" s="9" t="n"/>
-      <c r="D117" s="9" t="n"/>
-      <c r="E117" s="9" t="n"/>
-      <c r="F117" s="9" t="n"/>
-      <c r="G117" s="9" t="n"/>
-      <c r="H117" s="9" t="n"/>
-      <c r="I117" s="9" t="n"/>
-      <c r="J117" s="9" t="n"/>
-      <c r="K117" s="9" t="n"/>
+      <c r="A117" s="10" t="n">
+        <v>109</v>
+      </c>
+      <c r="B117" s="11" t="inlineStr">
+        <is>
+          <t>HSV-7 Fasáda ETICS</t>
+        </is>
+      </c>
+      <c r="C117" s="11" t="inlineStr">
+        <is>
+          <t>Příprava fasádního podkladu — očištění tlakovou vodou, vyspravení omítek, fungicidní nátěr</t>
+        </is>
+      </c>
+      <c r="D117" s="10" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E117" s="12" t="n">
+        <v>276.7</v>
+      </c>
+      <c r="F117" s="11" t="inlineStr">
+        <is>
+          <t>obvod 38.7 m (DXF) × 0.55 (volná fasáda, štíty zachované) × výška 13.0 m = 276.7 m²</t>
+        </is>
+      </c>
+      <c r="G117" s="11" t="inlineStr">
+        <is>
+          <t>622401110</t>
+        </is>
+      </c>
+      <c r="H117" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I117" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.001</t>
+        </is>
+      </c>
+      <c r="J117" s="11" t="inlineStr">
+        <is>
+          <t>S01</t>
+        </is>
+      </c>
+      <c r="K117" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
     </row>
     <row r="118">
-      <c r="A118" s="10" t="n">
+      <c r="A118" s="14" t="n">
         <v>110</v>
       </c>
-      <c r="B118" s="11" t="inlineStr">
+      <c r="B118" s="15" t="inlineStr">
         <is>
           <t>HSV-7 Fasáda ETICS</t>
         </is>
       </c>
-      <c r="C118" s="11" t="inlineStr">
-        <is>
-          <t>Příprava fasádního podkladu — očištění tlakovou vodou, vyspravení omítek, fungicidní nátěr</t>
-        </is>
-      </c>
-      <c r="D118" s="10" t="inlineStr">
+      <c r="C118" s="15" t="inlineStr">
+        <is>
+          <t>Lepení + kotvení desek EPS 70F grey λ=0.032 tl. 160 mm — ETICS kontaktní zateplení fasády</t>
+        </is>
+      </c>
+      <c r="D118" s="14" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E118" s="12" t="n">
+      <c r="E118" s="16" t="n">
         <v>276.7</v>
       </c>
-      <c r="F118" s="11" t="inlineStr">
-        <is>
-          <t>obvod 38.7 m (DXF) × 0.55 (volná fasáda, štíty zachované) × výška 13.0 m = 276.7 m²</t>
-        </is>
-      </c>
-      <c r="G118" s="11" t="inlineStr">
-        <is>
-          <t>622401110</t>
-        </is>
-      </c>
-      <c r="H118" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I118" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.001</t>
-        </is>
-      </c>
-      <c r="J118" s="11" t="inlineStr">
-        <is>
-          <t>S01</t>
-        </is>
-      </c>
-      <c r="K118" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+      <c r="F118" s="15">
+        <f> HSV7.002 plocha fasády 276.7 m²</f>
+        <v/>
+      </c>
+      <c r="G118" s="15" t="inlineStr">
+        <is>
+          <t>713</t>
+        </is>
+      </c>
+      <c r="H118" s="14" t="inlineStr">
+        <is>
+          <t>⚠ família ??? (ÚRS online)</t>
+        </is>
+      </c>
+      <c r="I118" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.002 → HSV7.002a</t>
+        </is>
+      </c>
+      <c r="J118" s="15" t="inlineStr">
+        <is>
+          <t>S01, S12a</t>
+        </is>
+      </c>
+      <c r="K118" s="15" t="inlineStr">
+        <is>
+          <t>Lepení+kotvení EPS (713/622 família). Leaf dle tl. 160 mm — verify.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -7438,7 +7441,7 @@
       </c>
       <c r="C119" s="15" t="inlineStr">
         <is>
-          <t>Lepení + kotvení desek EPS 70F grey λ=0.032 tl. 160 mm — ETICS kontaktní zateplení fasády</t>
+          <t>Armovací vrstva — výztužná síťka + lepicí stěrka (zatírací) na ETICS</t>
         </is>
       </c>
       <c r="D119" s="14" t="inlineStr">
@@ -7450,12 +7453,12 @@
         <v>276.7</v>
       </c>
       <c r="F119" s="15">
-        <f> HSV7.002 plocha fasády 276.7 m²</f>
+        <f> HSV7.002 plocha 276.7 m²</f>
         <v/>
       </c>
       <c r="G119" s="15" t="inlineStr">
         <is>
-          <t>713</t>
+          <t>622</t>
         </is>
       </c>
       <c r="H119" s="14" t="inlineStr">
@@ -7465,7 +7468,7 @@
       </c>
       <c r="I119" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.002 → HSV7.002a</t>
+          <t>260219_dum.HSV7.002 → HSV7.002b</t>
         </is>
       </c>
       <c r="J119" s="15" t="inlineStr">
@@ -7475,7 +7478,7 @@
       </c>
       <c r="K119" s="15" t="inlineStr">
         <is>
-          <t>Lepení+kotvení EPS (713/622 família). Leaf dle tl. 160 mm — verify.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+          <t>Armovací vrstva síťka+stěrka (622 família). Finální omítka je samostatně HSV7.006.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -7490,7 +7493,7 @@
       </c>
       <c r="C120" s="15" t="inlineStr">
         <is>
-          <t>Armovací vrstva — výztužná síťka + lepicí stěrka (zatírací) na ETICS</t>
+          <t>Lepení + kotvení desek XPS λ=0.034 tl. 120 mm + soklový profil — ETICS sokl</t>
         </is>
       </c>
       <c r="D120" s="14" t="inlineStr">
@@ -7499,15 +7502,15 @@
         </is>
       </c>
       <c r="E120" s="16" t="n">
-        <v>276.7</v>
+        <v>13.5</v>
       </c>
       <c r="F120" s="15">
-        <f> HSV7.002 plocha 276.7 m²</f>
+        <f> HSV7.003 plocha soklu 13.5 m²</f>
         <v/>
       </c>
       <c r="G120" s="15" t="inlineStr">
         <is>
-          <t>622</t>
+          <t>713</t>
         </is>
       </c>
       <c r="H120" s="14" t="inlineStr">
@@ -7517,17 +7520,17 @@
       </c>
       <c r="I120" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.002 → HSV7.002b</t>
+          <t>260219_dum.HSV7.003 → HSV7.003a</t>
         </is>
       </c>
       <c r="J120" s="15" t="inlineStr">
         <is>
-          <t>S01, S12a</t>
+          <t>S01</t>
         </is>
       </c>
       <c r="K120" s="15" t="inlineStr">
         <is>
-          <t>Armovací vrstva síťka+stěrka (622 família). Finální omítka je samostatně HSV7.006.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+          <t>Sokl XPS lepení + soklový profil (713/622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -7542,7 +7545,7 @@
       </c>
       <c r="C121" s="15" t="inlineStr">
         <is>
-          <t>Lepení + kotvení desek XPS λ=0.034 tl. 120 mm + soklový profil — ETICS sokl</t>
+          <t>Cihelný obklad soklu spárovaný (na armovací vrstvu)</t>
         </is>
       </c>
       <c r="D121" s="14" t="inlineStr">
@@ -7559,7 +7562,7 @@
       </c>
       <c r="G121" s="15" t="inlineStr">
         <is>
-          <t>713</t>
+          <t>781</t>
         </is>
       </c>
       <c r="H121" s="14" t="inlineStr">
@@ -7569,7 +7572,7 @@
       </c>
       <c r="I121" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.003 → HSV7.003a</t>
+          <t>260219_dum.HSV7.003 → HSV7.003b</t>
         </is>
       </c>
       <c r="J121" s="15" t="inlineStr">
@@ -7579,7 +7582,7 @@
       </c>
       <c r="K121" s="15" t="inlineStr">
         <is>
-          <t>Sokl XPS lepení + soklový profil (713/622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+          <t>Cihelný obklad spárovaný (781 família obklady).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -7594,24 +7597,24 @@
       </c>
       <c r="C122" s="15" t="inlineStr">
         <is>
-          <t>Cihelný obklad soklu spárovaný (na armovací vrstvu)</t>
+          <t>Špalety oken — EPS přesah 35-40 mm lepení + kotvení</t>
         </is>
       </c>
       <c r="D122" s="14" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>bm</t>
         </is>
       </c>
       <c r="E122" s="16" t="n">
-        <v>13.5</v>
+        <v>82.2</v>
       </c>
       <c r="F122" s="15">
-        <f> HSV7.003 plocha soklu 13.5 m²</f>
+        <f> HSV7.004 obvod špalet 82.2 bm</f>
         <v/>
       </c>
       <c r="G122" s="15" t="inlineStr">
         <is>
-          <t>781</t>
+          <t>622</t>
         </is>
       </c>
       <c r="H122" s="14" t="inlineStr">
@@ -7621,17 +7624,17 @@
       </c>
       <c r="I122" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.003 → HSV7.003b</t>
+          <t>260219_dum.HSV7.004 → HSV7.004a</t>
         </is>
       </c>
       <c r="J122" s="15" t="inlineStr">
         <is>
-          <t>S01</t>
+          <t>S01, S12a</t>
         </is>
       </c>
       <c r="K122" s="15" t="inlineStr">
         <is>
-          <t>Cihelný obklad spárovaný (781 família obklady).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+          <t>Špalety EPS přesah (622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -7646,7 +7649,7 @@
       </c>
       <c r="C123" s="15" t="inlineStr">
         <is>
-          <t>Špalety oken — EPS přesah 35-40 mm lepení + kotvení</t>
+          <t>Špalety oken — armovací vrstva síťka + omítka</t>
         </is>
       </c>
       <c r="D123" s="14" t="inlineStr">
@@ -7658,84 +7661,85 @@
         <v>82.2</v>
       </c>
       <c r="F123" s="15">
-        <f> HSV7.004 obvod špalet 82.2 bm</f>
-        <v/>
-      </c>
-      <c r="G123" s="15" t="inlineStr">
-        <is>
-          <t>622</t>
-        </is>
-      </c>
-      <c r="H123" s="14" t="inlineStr">
-        <is>
-          <t>⚠ família ??? (ÚRS online)</t>
-        </is>
-      </c>
-      <c r="I123" s="15" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.004 → HSV7.004a</t>
-        </is>
-      </c>
-      <c r="J123" s="15" t="inlineStr">
-        <is>
-          <t>S01, S12a</t>
-        </is>
-      </c>
-      <c r="K123" s="15" t="inlineStr">
-        <is>
-          <t>Špalety EPS přesah (622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="14" t="n">
-        <v>116</v>
-      </c>
-      <c r="B124" s="15" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda ETICS</t>
-        </is>
-      </c>
-      <c r="C124" s="15" t="inlineStr">
-        <is>
-          <t>Špalety oken — armovací vrstva síťka + omítka</t>
-        </is>
-      </c>
-      <c r="D124" s="14" t="inlineStr">
-        <is>
-          <t>bm</t>
-        </is>
-      </c>
-      <c r="E124" s="16" t="n">
-        <v>82.2</v>
-      </c>
-      <c r="F124" s="15">
         <f> HSV7.004 obvod 82.2 bm</f>
         <v/>
       </c>
-      <c r="G124" s="15" t="inlineStr">
+      <c r="G123" s="15" t="inlineStr">
         <is>
           <t>622</t>
         </is>
       </c>
-      <c r="H124" s="14" t="inlineStr">
+      <c r="H123" s="14" t="inlineStr">
         <is>
           <t>⚠ família ??? (ÚRS online)</t>
         </is>
       </c>
-      <c r="I124" s="15" t="inlineStr">
+      <c r="I123" s="15" t="inlineStr">
         <is>
           <t>260219_dum.HSV7.004 → HSV7.004b</t>
         </is>
       </c>
-      <c r="J124" s="15" t="inlineStr">
+      <c r="J123" s="15" t="inlineStr">
         <is>
           <t>S01, S12a</t>
         </is>
       </c>
-      <c r="K124" s="15" t="inlineStr">
+      <c r="K123" s="15" t="inlineStr">
         <is>
           <t>Armovací vrstva + omítka špalet (622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="10" t="n">
+        <v>116</v>
+      </c>
+      <c r="B124" s="11" t="inlineStr">
+        <is>
+          <t>HSV-7 Fasáda ETICS</t>
+        </is>
+      </c>
+      <c r="C124" s="11" t="inlineStr">
+        <is>
+          <t>Profilace fasády — různé tloušťky EPS (kordony, šambrány, rámování oken) — paušál podle pohledů</t>
+        </is>
+      </c>
+      <c r="D124" s="10" t="inlineStr">
+        <is>
+          <t>soubor</t>
+        </is>
+      </c>
+      <c r="E124" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F124" s="11" t="inlineStr">
+        <is>
+          <t>paušál — dle pohledů NCS NZÚ</t>
+        </is>
+      </c>
+      <c r="G124" s="11" t="inlineStr">
+        <is>
+          <t>622221221</t>
+        </is>
+      </c>
+      <c r="H124" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I124" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.005</t>
+        </is>
+      </c>
+      <c r="J124" s="11" t="inlineStr">
+        <is>
+          <t>S01, S12a</t>
+        </is>
+      </c>
+      <c r="K124" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
         </is>
       </c>
     </row>
@@ -7750,25 +7754,25 @@
       </c>
       <c r="C125" s="11" t="inlineStr">
         <is>
-          <t>Profilace fasády — různé tloušťky EPS (kordony, šambrány, rámování oken) — paušál podle pohledů</t>
+          <t>Tenkovrstvá pastovitá probarvená omítka, lomená bílá NCS NZÚ — finální vrstva ETICS</t>
         </is>
       </c>
       <c r="D125" s="10" t="inlineStr">
         <is>
-          <t>soubor</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E125" s="12" t="n">
-        <v>1</v>
+        <v>290.2</v>
       </c>
       <c r="F125" s="11" t="inlineStr">
         <is>
-          <t>paušál — dle pohledů NCS NZÚ</t>
-        </is>
-      </c>
-      <c r="G125" s="11" t="inlineStr">
-        <is>
-          <t>622221221</t>
+          <t>ETICS plocha 276.7 m² + sokl 13.5 m² = 290.2 m²</t>
+        </is>
+      </c>
+      <c r="G125" s="13" t="inlineStr">
+        <is>
+          <t>622521111</t>
         </is>
       </c>
       <c r="H125" s="10" t="inlineStr">
@@ -7778,12 +7782,12 @@
       </c>
       <c r="I125" s="11" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.005</t>
+          <t>260219_dum.HSV7.006</t>
         </is>
       </c>
       <c r="J125" s="11" t="inlineStr">
         <is>
-          <t>S01, S12a</t>
+          <t>S01, S12a, S12b</t>
         </is>
       </c>
       <c r="K125" s="11" t="inlineStr">
@@ -7793,74 +7797,69 @@
       </c>
     </row>
     <row r="126">
-      <c r="A126" s="10" t="n">
+      <c r="A126" s="8" t="inlineStr">
+        <is>
+          <t>━━ HSV-7 Fasáda + zateplení  (5 atomic operací) ━━</t>
+        </is>
+      </c>
+      <c r="B126" s="9" t="n"/>
+      <c r="C126" s="9" t="n"/>
+      <c r="D126" s="9" t="n"/>
+      <c r="E126" s="9" t="n"/>
+      <c r="F126" s="9" t="n"/>
+      <c r="G126" s="9" t="n"/>
+      <c r="H126" s="9" t="n"/>
+      <c r="I126" s="9" t="n"/>
+      <c r="J126" s="9" t="n"/>
+      <c r="K126" s="9" t="n"/>
+    </row>
+    <row r="127">
+      <c r="A127" s="17" t="n">
         <v>118</v>
       </c>
-      <c r="B126" s="11" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda ETICS</t>
-        </is>
-      </c>
-      <c r="C126" s="11" t="inlineStr">
-        <is>
-          <t>Tenkovrstvá pastovitá probarvená omítka, lomená bílá NCS NZÚ — finální vrstva ETICS</t>
-        </is>
-      </c>
-      <c r="D126" s="10" t="inlineStr">
+      <c r="B127" s="18" t="inlineStr">
+        <is>
+          <t>HSV-7 Fasáda + zateplení</t>
+        </is>
+      </c>
+      <c r="C127" s="18" t="inlineStr">
+        <is>
+          <t>Montáž sanační izolační desky Styrcon 200 + armovací — sokl S03</t>
+        </is>
+      </c>
+      <c r="D127" s="17" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E126" s="12" t="n">
-        <v>290.2</v>
-      </c>
-      <c r="F126" s="11" t="inlineStr">
-        <is>
-          <t>ETICS plocha 276.7 m² + sokl 13.5 m² = 290.2 m²</t>
-        </is>
-      </c>
-      <c r="G126" s="13" t="inlineStr">
-        <is>
-          <t>622521111</t>
-        </is>
-      </c>
-      <c r="H126" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I126" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.006</t>
-        </is>
-      </c>
-      <c r="J126" s="11" t="inlineStr">
-        <is>
-          <t>S01, S12a, S12b</t>
-        </is>
-      </c>
-      <c r="K126" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="8" t="inlineStr">
-        <is>
-          <t>━━ HSV-7 Fasáda + zateplení  (5 atomic operací) ━━</t>
-        </is>
-      </c>
-      <c r="B127" s="9" t="n"/>
-      <c r="C127" s="9" t="n"/>
-      <c r="D127" s="9" t="n"/>
-      <c r="E127" s="9" t="n"/>
-      <c r="F127" s="9" t="n"/>
-      <c r="G127" s="9" t="n"/>
-      <c r="H127" s="9" t="n"/>
-      <c r="I127" s="9" t="n"/>
-      <c r="J127" s="9" t="n"/>
-      <c r="K127" s="9" t="n"/>
+      <c r="E127" s="19" t="n">
+        <v>23</v>
+      </c>
+      <c r="F127" s="18">
+        <f> obvod 38.7 × 0.6 ≈ 23 (OVĚŘIT)</f>
+        <v/>
+      </c>
+      <c r="G127" s="18" t="inlineStr"/>
+      <c r="H127" s="17" t="inlineStr">
+        <is>
+          <t>❌ blank — ÚRS online</t>
+        </is>
+      </c>
+      <c r="I127" s="18" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.007 → HSV7.007a</t>
+        </is>
+      </c>
+      <c r="J127" s="18" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="K127" s="18" t="inlineStr">
+        <is>
+          <t>Montáž.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="17" t="n">
@@ -7873,7 +7872,7 @@
       </c>
       <c r="C128" s="18" t="inlineStr">
         <is>
-          <t>Montáž sanační izolační desky Styrcon 200 + armovací — sokl S03</t>
+          <t>Sanační deska Styrcon 200 + lepící tmel + armovací stěrka+tkanina — materiál</t>
         </is>
       </c>
       <c r="D128" s="17" t="inlineStr">
@@ -7882,10 +7881,10 @@
         </is>
       </c>
       <c r="E128" s="19" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F128" s="18">
-        <f> obvod 38.7 × 0.6 ≈ 23 (OVĚŘIT)</f>
+        <f> 23 × 1.05</f>
         <v/>
       </c>
       <c r="G128" s="18" t="inlineStr"/>
@@ -7896,7 +7895,7 @@
       </c>
       <c r="I128" s="18" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.007 → HSV7.007a</t>
+          <t>260219_dum.HSV7.007 → HSV7.007b</t>
         </is>
       </c>
       <c r="J128" s="18" t="inlineStr">
@@ -7906,7 +7905,7 @@
       </c>
       <c r="K128" s="18" t="inlineStr">
         <is>
-          <t>Montáž.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+          <t>Materiál.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -7921,7 +7920,7 @@
       </c>
       <c r="C129" s="18" t="inlineStr">
         <is>
-          <t>Sanační deska Styrcon 200 + lepící tmel + armovací stěrka+tkanina — materiál</t>
+          <t>Drenážní nopová folie 20 mm — dodávka+montáž, sokl pod terénem S03a</t>
         </is>
       </c>
       <c r="D129" s="17" t="inlineStr">
@@ -7930,10 +7929,10 @@
         </is>
       </c>
       <c r="E129" s="19" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F129" s="18">
-        <f> 23 × 1.05</f>
+        <f> 23 × 1.10</f>
         <v/>
       </c>
       <c r="G129" s="18" t="inlineStr"/>
@@ -7944,7 +7943,7 @@
       </c>
       <c r="I129" s="18" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.007 → HSV7.007b</t>
+          <t>260219_dum.HSV7.008 → HSV7.008a</t>
         </is>
       </c>
       <c r="J129" s="18" t="inlineStr">
@@ -7954,7 +7953,7 @@
       </c>
       <c r="K129" s="18" t="inlineStr">
         <is>
-          <t>Materiál.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+          <t>Montáž+materiál.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -7969,7 +7968,7 @@
       </c>
       <c r="C130" s="18" t="inlineStr">
         <is>
-          <t>Drenážní nopová folie 20 mm — dodávka+montáž, sokl pod terénem S03a</t>
+          <t>Kotevní rošt 40 mm provětraného soklu — montáž+materiál S03b</t>
         </is>
       </c>
       <c r="D130" s="17" t="inlineStr">
@@ -7978,10 +7977,10 @@
         </is>
       </c>
       <c r="E130" s="19" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="F130" s="18">
-        <f> 23 × 1.10</f>
+        <f> 23 (OVĚŘIT)</f>
         <v/>
       </c>
       <c r="G130" s="18" t="inlineStr"/>
@@ -7992,7 +7991,7 @@
       </c>
       <c r="I130" s="18" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.008 → HSV7.008a</t>
+          <t>260219_dum.HSV7.009 → HSV7.009a</t>
         </is>
       </c>
       <c r="J130" s="18" t="inlineStr">
@@ -8002,105 +8001,57 @@
       </c>
       <c r="K130" s="18" t="inlineStr">
         <is>
-          <t>Montáž+materiál.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+          <t>Rošt.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
     <row r="131">
-      <c r="A131" s="17" t="n">
+      <c r="A131" s="14" t="n">
         <v>122</v>
       </c>
-      <c r="B131" s="18" t="inlineStr">
+      <c r="B131" s="15" t="inlineStr">
         <is>
           <t>HSV-7 Fasáda + zateplení</t>
         </is>
       </c>
-      <c r="C131" s="18" t="inlineStr">
-        <is>
-          <t>Kotevní rošt 40 mm provětraného soklu — montáž+materiál S03b</t>
-        </is>
-      </c>
-      <c r="D131" s="17" t="inlineStr">
+      <c r="C131" s="15" t="inlineStr">
+        <is>
+          <t>Keramický obklad soklu 20 mm — montáž+materiál</t>
+        </is>
+      </c>
+      <c r="D131" s="14" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E131" s="19" t="n">
-        <v>23</v>
-      </c>
-      <c r="F131" s="18">
-        <f> 23 (OVĚŘIT)</f>
-        <v/>
-      </c>
-      <c r="G131" s="18" t="inlineStr"/>
-      <c r="H131" s="17" t="inlineStr">
-        <is>
-          <t>❌ blank — ÚRS online</t>
-        </is>
-      </c>
-      <c r="I131" s="18" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.009 → HSV7.009a</t>
-        </is>
-      </c>
-      <c r="J131" s="18" t="inlineStr">
-        <is>
-          <t>S03</t>
-        </is>
-      </c>
-      <c r="K131" s="18" t="inlineStr">
-        <is>
-          <t>Rošt.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="14" t="n">
-        <v>123</v>
-      </c>
-      <c r="B132" s="15" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda + zateplení</t>
-        </is>
-      </c>
-      <c r="C132" s="15" t="inlineStr">
-        <is>
-          <t>Keramický obklad soklu 20 mm — montáž+materiál</t>
-        </is>
-      </c>
-      <c r="D132" s="14" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E132" s="16" t="n">
+      <c r="E131" s="16" t="n">
         <v>24</v>
       </c>
-      <c r="F132" s="15">
+      <c r="F131" s="15">
         <f> 23 × 1.05</f>
         <v/>
       </c>
-      <c r="G132" s="15" t="inlineStr">
+      <c r="G131" s="15" t="inlineStr">
         <is>
           <t>781</t>
         </is>
       </c>
-      <c r="H132" s="14" t="inlineStr">
+      <c r="H131" s="14" t="inlineStr">
         <is>
           <t>⚠ família ??? (ÚRS online)</t>
         </is>
       </c>
-      <c r="I132" s="15" t="inlineStr">
+      <c r="I131" s="15" t="inlineStr">
         <is>
           <t>260219_dum.HSV7.009 → HSV7.009b</t>
         </is>
       </c>
-      <c r="J132" s="15" t="inlineStr">
+      <c r="J131" s="15" t="inlineStr">
         <is>
           <t>S03</t>
         </is>
       </c>
-      <c r="K132" s="15" t="inlineStr">
+      <c r="K131" s="15" t="inlineStr">
         <is>
           <t>Obklad.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
@@ -8110,13 +8061,13 @@
   <autoFilter ref="A1:K1"/>
   <mergeCells count="8">
     <mergeCell ref="A22:K22"/>
-    <mergeCell ref="A127:K127"/>
     <mergeCell ref="A2:K2"/>
-    <mergeCell ref="A117:K117"/>
     <mergeCell ref="A98:K98"/>
     <mergeCell ref="A68:K68"/>
     <mergeCell ref="A44:K44"/>
+    <mergeCell ref="A116:K116"/>
     <mergeCell ref="A36:K36"/>
+    <mergeCell ref="A126:K126"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -18134,7 +18085,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E14"/>
+  <dimension ref="A1:E15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18454,27 +18405,52 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="14" t="inlineStr">
+      <c r="A14" s="17" t="n">
+        <v>33</v>
+      </c>
+      <c r="B14" s="18" t="inlineStr">
+        <is>
+          <t>minor</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>Sklad výkop — svahovaná jáma 1:0,5 v prudkém svahu (hloubka &gt;2 m)</t>
+        </is>
+      </c>
+      <c r="D14" s="18" t="inlineStr">
+        <is>
+          <t>NEPŘIDÁNO (verify-first)</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t>Statiku/projektante: potvrďte, že objem výkopu skladu počítá se svahováním 1:0,5 + je dostupný prostor pro svah v prudkém svahu; pažení jen rýhy přípojek dle BOZP?</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>PM05</t>
         </is>
       </c>
-      <c r="B14" s="15" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="C14" s="15" t="inlineStr">
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <t>Okapový chodník + obvodová drenáž domu — NOT_IN_TZ (žádná zmínka v TZ)</t>
         </is>
       </c>
-      <c r="D14" s="15" t="inlineStr">
+      <c r="D15" s="15" t="inlineStr">
         <is>
           <t>SKIP (rekonstrukce — možná existuje)</t>
         </is>
       </c>
-      <c r="E14" s="15" t="inlineStr">
+      <c r="E15" s="15" t="inlineStr">
         <is>
           <t>Volitelné: ověřit zda okapový chodník po obvodu domu je v scope (mimo BV drenáž HSV1.015). Pokud ano → HSV-1 položka.</t>
         </is>

</xml_diff>

<commit_message>
feat(rd-jachymov): split ETICS armovací vrstva po vrstvách + ÚRS 622142001 (síťka)
User-provided leaf code from KROS catalog. HSV7.002 armovací vrstva (was bundled
'síťka + stěrka', urs=622 family) → split into 2 atomic layers (P41):
  b) Armovací vrstva ETICS — lepicí/stěrková hmota (zatírací) + vmáčknutí tkaniny (622 family)
  c) Výztužná síťka — sklovláknité pletivo vtlačené do tmelu, stěn → ÚRS 622142001 (leaf_verified)

622142001 user-verified from KROS (Pletivo vnějších ploch sklovláknité, stěn, m²).
Atomic ops 281→282. items unchanged (233). 10-step regen + assert 30==queue 30.
snapshot items_pre_armovaci_split.json.

https://claude.ai/code/session_01FskzLAZkXgJAwuN2cQQEdx
</commit_message>
<xml_diff>
--- a/test-data/RD_Jachymov_dum/outputs/Vykaz_vymer_RD_Jachymov_ATOMIC_WORKLIST_2026-05-27.xlsx
+++ b/test-data/RD_Jachymov_dum/outputs/Vykaz_vymer_RD_Jachymov_ATOMIC_WORKLIST_2026-05-27.xlsx
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>280</v>
+        <v>281</v>
       </c>
       <c r="C6" s="2">
         <f> carried 1:1 + decomposed children</f>
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="9">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23">
@@ -1029,7 +1029,7 @@
         </is>
       </c>
       <c r="B51" s="5" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="52">
@@ -1220,7 +1220,7 @@
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>733</t>
+          <t>622</t>
         </is>
       </c>
       <c r="B73" s="5" t="n">
@@ -1230,7 +1230,7 @@
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>781</t>
+          <t>733</t>
         </is>
       </c>
       <c r="B74" s="5" t="n">
@@ -1240,17 +1240,17 @@
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>781</t>
         </is>
       </c>
       <c r="B75" s="5" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>622</t>
+          <t>210</t>
         </is>
       </c>
       <c r="B76" s="5" t="n">
@@ -1731,7 +1731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K131"/>
+  <dimension ref="A1:K132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -7311,7 +7311,7 @@
     <row r="116">
       <c r="A116" s="8" t="inlineStr">
         <is>
-          <t>━━ HSV-7 Fasáda ETICS  (9 atomic operací) ━━</t>
+          <t>━━ HSV-7 Fasáda ETICS  (10 atomic operací) ━━</t>
         </is>
       </c>
       <c r="B116" s="9" t="n"/>
@@ -7441,7 +7441,7 @@
       </c>
       <c r="C119" s="15" t="inlineStr">
         <is>
-          <t>Armovací vrstva — výztužná síťka + lepicí stěrka (zatírací) na ETICS</t>
+          <t>Armovací vrstva ETICS — lepicí/stěrková hmota (zatírací) + vmáčknutí tkaniny</t>
         </is>
       </c>
       <c r="D119" s="14" t="inlineStr">
@@ -7478,7 +7478,7 @@
       </c>
       <c r="K119" s="15" t="inlineStr">
         <is>
-          <t>Armovací vrstva síťka+stěrka (622 família). Finální omítka je samostatně HSV7.006.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+          <t>Stěrková hmota armovací vrstvy (622 família). Pletivo viz suffix c.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -7493,7 +7493,7 @@
       </c>
       <c r="C120" s="15" t="inlineStr">
         <is>
-          <t>Lepení + kotvení desek XPS λ=0.034 tl. 120 mm + soklový profil — ETICS sokl</t>
+          <t>Výztužná síťka — sklovláknité pletivo vtlačené do tmelu, stěn (ETICS)</t>
         </is>
       </c>
       <c r="D120" s="14" t="inlineStr">
@@ -7502,35 +7502,35 @@
         </is>
       </c>
       <c r="E120" s="16" t="n">
-        <v>13.5</v>
+        <v>276.7</v>
       </c>
       <c r="F120" s="15">
-        <f> HSV7.003 plocha soklu 13.5 m²</f>
+        <f> HSV7.002 plocha 276.7 m² (přesahy v spotřebě)</f>
         <v/>
       </c>
       <c r="G120" s="15" t="inlineStr">
         <is>
-          <t>713</t>
+          <t>622142001</t>
         </is>
       </c>
       <c r="H120" s="14" t="inlineStr">
         <is>
-          <t>⚠ família ??? (ÚRS online)</t>
+          <t>✓ verified</t>
         </is>
       </c>
       <c r="I120" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.003 → HSV7.003a</t>
+          <t>260219_dum.HSV7.002 → HSV7.002c</t>
         </is>
       </c>
       <c r="J120" s="15" t="inlineStr">
         <is>
-          <t>S01</t>
+          <t>S01, S12a</t>
         </is>
       </c>
       <c r="K120" s="15" t="inlineStr">
         <is>
-          <t>Sokl XPS lepení + soklový profil (713/622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+          <t>ÚRS 622142001 — uživatelem ověřeno z KROS katalogu (Pletivo vnějších ploch sklovláknité, stěn, m²).</t>
         </is>
       </c>
     </row>
@@ -7545,7 +7545,7 @@
       </c>
       <c r="C121" s="15" t="inlineStr">
         <is>
-          <t>Cihelný obklad soklu spárovaný (na armovací vrstvu)</t>
+          <t>Lepení + kotvení desek XPS λ=0.034 tl. 120 mm + soklový profil — ETICS sokl</t>
         </is>
       </c>
       <c r="D121" s="14" t="inlineStr">
@@ -7562,7 +7562,7 @@
       </c>
       <c r="G121" s="15" t="inlineStr">
         <is>
-          <t>781</t>
+          <t>713</t>
         </is>
       </c>
       <c r="H121" s="14" t="inlineStr">
@@ -7572,7 +7572,7 @@
       </c>
       <c r="I121" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.003 → HSV7.003b</t>
+          <t>260219_dum.HSV7.003 → HSV7.003a</t>
         </is>
       </c>
       <c r="J121" s="15" t="inlineStr">
@@ -7582,7 +7582,7 @@
       </c>
       <c r="K121" s="15" t="inlineStr">
         <is>
-          <t>Cihelný obklad spárovaný (781 família obklady).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+          <t>Sokl XPS lepení + soklový profil (713/622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -7597,24 +7597,24 @@
       </c>
       <c r="C122" s="15" t="inlineStr">
         <is>
-          <t>Špalety oken — EPS přesah 35-40 mm lepení + kotvení</t>
+          <t>Cihelný obklad soklu spárovaný (na armovací vrstvu)</t>
         </is>
       </c>
       <c r="D122" s="14" t="inlineStr">
         <is>
-          <t>bm</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E122" s="16" t="n">
-        <v>82.2</v>
+        <v>13.5</v>
       </c>
       <c r="F122" s="15">
-        <f> HSV7.004 obvod špalet 82.2 bm</f>
+        <f> HSV7.003 plocha soklu 13.5 m²</f>
         <v/>
       </c>
       <c r="G122" s="15" t="inlineStr">
         <is>
-          <t>622</t>
+          <t>781</t>
         </is>
       </c>
       <c r="H122" s="14" t="inlineStr">
@@ -7624,17 +7624,17 @@
       </c>
       <c r="I122" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.004 → HSV7.004a</t>
+          <t>260219_dum.HSV7.003 → HSV7.003b</t>
         </is>
       </c>
       <c r="J122" s="15" t="inlineStr">
         <is>
-          <t>S01, S12a</t>
+          <t>S01</t>
         </is>
       </c>
       <c r="K122" s="15" t="inlineStr">
         <is>
-          <t>Špalety EPS přesah (622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+          <t>Cihelný obklad spárovaný (781 família obklady).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -7649,7 +7649,7 @@
       </c>
       <c r="C123" s="15" t="inlineStr">
         <is>
-          <t>Špalety oken — armovací vrstva síťka + omítka</t>
+          <t>Špalety oken — EPS přesah 35-40 mm lepení + kotvení</t>
         </is>
       </c>
       <c r="D123" s="14" t="inlineStr">
@@ -7661,85 +7661,84 @@
         <v>82.2</v>
       </c>
       <c r="F123" s="15">
+        <f> HSV7.004 obvod špalet 82.2 bm</f>
+        <v/>
+      </c>
+      <c r="G123" s="15" t="inlineStr">
+        <is>
+          <t>622</t>
+        </is>
+      </c>
+      <c r="H123" s="14" t="inlineStr">
+        <is>
+          <t>⚠ família ??? (ÚRS online)</t>
+        </is>
+      </c>
+      <c r="I123" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.004 → HSV7.004a</t>
+        </is>
+      </c>
+      <c r="J123" s="15" t="inlineStr">
+        <is>
+          <t>S01, S12a</t>
+        </is>
+      </c>
+      <c r="K123" s="15" t="inlineStr">
+        <is>
+          <t>Špalety EPS přesah (622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="14" t="n">
+        <v>116</v>
+      </c>
+      <c r="B124" s="15" t="inlineStr">
+        <is>
+          <t>HSV-7 Fasáda ETICS</t>
+        </is>
+      </c>
+      <c r="C124" s="15" t="inlineStr">
+        <is>
+          <t>Špalety oken — armovací vrstva síťka + omítka</t>
+        </is>
+      </c>
+      <c r="D124" s="14" t="inlineStr">
+        <is>
+          <t>bm</t>
+        </is>
+      </c>
+      <c r="E124" s="16" t="n">
+        <v>82.2</v>
+      </c>
+      <c r="F124" s="15">
         <f> HSV7.004 obvod 82.2 bm</f>
         <v/>
       </c>
-      <c r="G123" s="15" t="inlineStr">
+      <c r="G124" s="15" t="inlineStr">
         <is>
           <t>622</t>
         </is>
       </c>
-      <c r="H123" s="14" t="inlineStr">
+      <c r="H124" s="14" t="inlineStr">
         <is>
           <t>⚠ família ??? (ÚRS online)</t>
         </is>
       </c>
-      <c r="I123" s="15" t="inlineStr">
+      <c r="I124" s="15" t="inlineStr">
         <is>
           <t>260219_dum.HSV7.004 → HSV7.004b</t>
         </is>
       </c>
-      <c r="J123" s="15" t="inlineStr">
+      <c r="J124" s="15" t="inlineStr">
         <is>
           <t>S01, S12a</t>
         </is>
       </c>
-      <c r="K123" s="15" t="inlineStr">
+      <c r="K124" s="15" t="inlineStr">
         <is>
           <t>Armovací vrstva + omítka špalet (622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="10" t="n">
-        <v>116</v>
-      </c>
-      <c r="B124" s="11" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda ETICS</t>
-        </is>
-      </c>
-      <c r="C124" s="11" t="inlineStr">
-        <is>
-          <t>Profilace fasády — různé tloušťky EPS (kordony, šambrány, rámování oken) — paušál podle pohledů</t>
-        </is>
-      </c>
-      <c r="D124" s="10" t="inlineStr">
-        <is>
-          <t>soubor</t>
-        </is>
-      </c>
-      <c r="E124" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F124" s="11" t="inlineStr">
-        <is>
-          <t>paušál — dle pohledů NCS NZÚ</t>
-        </is>
-      </c>
-      <c r="G124" s="11" t="inlineStr">
-        <is>
-          <t>622221221</t>
-        </is>
-      </c>
-      <c r="H124" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I124" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.005</t>
-        </is>
-      </c>
-      <c r="J124" s="11" t="inlineStr">
-        <is>
-          <t>S01, S12a</t>
-        </is>
-      </c>
-      <c r="K124" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
         </is>
       </c>
     </row>
@@ -7754,112 +7753,117 @@
       </c>
       <c r="C125" s="11" t="inlineStr">
         <is>
+          <t>Profilace fasády — různé tloušťky EPS (kordony, šambrány, rámování oken) — paušál podle pohledů</t>
+        </is>
+      </c>
+      <c r="D125" s="10" t="inlineStr">
+        <is>
+          <t>soubor</t>
+        </is>
+      </c>
+      <c r="E125" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F125" s="11" t="inlineStr">
+        <is>
+          <t>paušál — dle pohledů NCS NZÚ</t>
+        </is>
+      </c>
+      <c r="G125" s="11" t="inlineStr">
+        <is>
+          <t>622221221</t>
+        </is>
+      </c>
+      <c r="H125" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I125" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.005</t>
+        </is>
+      </c>
+      <c r="J125" s="11" t="inlineStr">
+        <is>
+          <t>S01, S12a</t>
+        </is>
+      </c>
+      <c r="K125" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" s="10" t="n">
+        <v>118</v>
+      </c>
+      <c r="B126" s="11" t="inlineStr">
+        <is>
+          <t>HSV-7 Fasáda ETICS</t>
+        </is>
+      </c>
+      <c r="C126" s="11" t="inlineStr">
+        <is>
           <t>Tenkovrstvá pastovitá probarvená omítka, lomená bílá NCS NZÚ — finální vrstva ETICS</t>
         </is>
       </c>
-      <c r="D125" s="10" t="inlineStr">
+      <c r="D126" s="10" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E125" s="12" t="n">
+      <c r="E126" s="12" t="n">
         <v>290.2</v>
       </c>
-      <c r="F125" s="11" t="inlineStr">
+      <c r="F126" s="11" t="inlineStr">
         <is>
           <t>ETICS plocha 276.7 m² + sokl 13.5 m² = 290.2 m²</t>
         </is>
       </c>
-      <c r="G125" s="13" t="inlineStr">
+      <c r="G126" s="13" t="inlineStr">
         <is>
           <t>622521111</t>
         </is>
       </c>
-      <c r="H125" s="10" t="inlineStr">
+      <c r="H126" s="10" t="inlineStr">
         <is>
           <t>⚠ kandidát-verify</t>
         </is>
       </c>
-      <c r="I125" s="11" t="inlineStr">
+      <c r="I126" s="11" t="inlineStr">
         <is>
           <t>260219_dum.HSV7.006</t>
         </is>
       </c>
-      <c r="J125" s="11" t="inlineStr">
+      <c r="J126" s="11" t="inlineStr">
         <is>
           <t>S01, S12a, S12b</t>
         </is>
       </c>
-      <c r="K125" s="11" t="inlineStr">
+      <c r="K126" s="11" t="inlineStr">
         <is>
           <t>Carried 1:1 (atomic — no decomposition needed)</t>
         </is>
       </c>
     </row>
-    <row r="126">
-      <c r="A126" s="8" t="inlineStr">
+    <row r="127">
+      <c r="A127" s="8" t="inlineStr">
         <is>
           <t>━━ HSV-7 Fasáda + zateplení  (5 atomic operací) ━━</t>
         </is>
       </c>
-      <c r="B126" s="9" t="n"/>
-      <c r="C126" s="9" t="n"/>
-      <c r="D126" s="9" t="n"/>
-      <c r="E126" s="9" t="n"/>
-      <c r="F126" s="9" t="n"/>
-      <c r="G126" s="9" t="n"/>
-      <c r="H126" s="9" t="n"/>
-      <c r="I126" s="9" t="n"/>
-      <c r="J126" s="9" t="n"/>
-      <c r="K126" s="9" t="n"/>
-    </row>
-    <row r="127">
-      <c r="A127" s="17" t="n">
-        <v>118</v>
-      </c>
-      <c r="B127" s="18" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda + zateplení</t>
-        </is>
-      </c>
-      <c r="C127" s="18" t="inlineStr">
-        <is>
-          <t>Montáž sanační izolační desky Styrcon 200 + armovací — sokl S03</t>
-        </is>
-      </c>
-      <c r="D127" s="17" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E127" s="19" t="n">
-        <v>23</v>
-      </c>
-      <c r="F127" s="18">
-        <f> obvod 38.7 × 0.6 ≈ 23 (OVĚŘIT)</f>
-        <v/>
-      </c>
-      <c r="G127" s="18" t="inlineStr"/>
-      <c r="H127" s="17" t="inlineStr">
-        <is>
-          <t>❌ blank — ÚRS online</t>
-        </is>
-      </c>
-      <c r="I127" s="18" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.007 → HSV7.007a</t>
-        </is>
-      </c>
-      <c r="J127" s="18" t="inlineStr">
-        <is>
-          <t>S03</t>
-        </is>
-      </c>
-      <c r="K127" s="18" t="inlineStr">
-        <is>
-          <t>Montáž.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
-        </is>
-      </c>
+      <c r="B127" s="9" t="n"/>
+      <c r="C127" s="9" t="n"/>
+      <c r="D127" s="9" t="n"/>
+      <c r="E127" s="9" t="n"/>
+      <c r="F127" s="9" t="n"/>
+      <c r="G127" s="9" t="n"/>
+      <c r="H127" s="9" t="n"/>
+      <c r="I127" s="9" t="n"/>
+      <c r="J127" s="9" t="n"/>
+      <c r="K127" s="9" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="17" t="n">
@@ -7872,7 +7876,7 @@
       </c>
       <c r="C128" s="18" t="inlineStr">
         <is>
-          <t>Sanační deska Styrcon 200 + lepící tmel + armovací stěrka+tkanina — materiál</t>
+          <t>Montáž sanační izolační desky Styrcon 200 + armovací — sokl S03</t>
         </is>
       </c>
       <c r="D128" s="17" t="inlineStr">
@@ -7881,10 +7885,10 @@
         </is>
       </c>
       <c r="E128" s="19" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F128" s="18">
-        <f> 23 × 1.05</f>
+        <f> obvod 38.7 × 0.6 ≈ 23 (OVĚŘIT)</f>
         <v/>
       </c>
       <c r="G128" s="18" t="inlineStr"/>
@@ -7895,7 +7899,7 @@
       </c>
       <c r="I128" s="18" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.007 → HSV7.007b</t>
+          <t>260219_dum.HSV7.007 → HSV7.007a</t>
         </is>
       </c>
       <c r="J128" s="18" t="inlineStr">
@@ -7905,7 +7909,7 @@
       </c>
       <c r="K128" s="18" t="inlineStr">
         <is>
-          <t>Materiál.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+          <t>Montáž.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -7920,7 +7924,7 @@
       </c>
       <c r="C129" s="18" t="inlineStr">
         <is>
-          <t>Drenážní nopová folie 20 mm — dodávka+montáž, sokl pod terénem S03a</t>
+          <t>Sanační deska Styrcon 200 + lepící tmel + armovací stěrka+tkanina — materiál</t>
         </is>
       </c>
       <c r="D129" s="17" t="inlineStr">
@@ -7929,10 +7933,10 @@
         </is>
       </c>
       <c r="E129" s="19" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F129" s="18">
-        <f> 23 × 1.10</f>
+        <f> 23 × 1.05</f>
         <v/>
       </c>
       <c r="G129" s="18" t="inlineStr"/>
@@ -7943,7 +7947,7 @@
       </c>
       <c r="I129" s="18" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.008 → HSV7.008a</t>
+          <t>260219_dum.HSV7.007 → HSV7.007b</t>
         </is>
       </c>
       <c r="J129" s="18" t="inlineStr">
@@ -7953,7 +7957,7 @@
       </c>
       <c r="K129" s="18" t="inlineStr">
         <is>
-          <t>Montáž+materiál.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+          <t>Materiál.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -7968,90 +7972,138 @@
       </c>
       <c r="C130" s="18" t="inlineStr">
         <is>
+          <t>Drenážní nopová folie 20 mm — dodávka+montáž, sokl pod terénem S03a</t>
+        </is>
+      </c>
+      <c r="D130" s="17" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E130" s="19" t="n">
+        <v>25</v>
+      </c>
+      <c r="F130" s="18">
+        <f> 23 × 1.10</f>
+        <v/>
+      </c>
+      <c r="G130" s="18" t="inlineStr"/>
+      <c r="H130" s="17" t="inlineStr">
+        <is>
+          <t>❌ blank — ÚRS online</t>
+        </is>
+      </c>
+      <c r="I130" s="18" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.008 → HSV7.008a</t>
+        </is>
+      </c>
+      <c r="J130" s="18" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="K130" s="18" t="inlineStr">
+        <is>
+          <t>Montáž+materiál.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" s="17" t="n">
+        <v>122</v>
+      </c>
+      <c r="B131" s="18" t="inlineStr">
+        <is>
+          <t>HSV-7 Fasáda + zateplení</t>
+        </is>
+      </c>
+      <c r="C131" s="18" t="inlineStr">
+        <is>
           <t>Kotevní rošt 40 mm provětraného soklu — montáž+materiál S03b</t>
         </is>
       </c>
-      <c r="D130" s="17" t="inlineStr">
+      <c r="D131" s="17" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E130" s="19" t="n">
+      <c r="E131" s="19" t="n">
         <v>23</v>
       </c>
-      <c r="F130" s="18">
+      <c r="F131" s="18">
         <f> 23 (OVĚŘIT)</f>
         <v/>
       </c>
-      <c r="G130" s="18" t="inlineStr"/>
-      <c r="H130" s="17" t="inlineStr">
+      <c r="G131" s="18" t="inlineStr"/>
+      <c r="H131" s="17" t="inlineStr">
         <is>
           <t>❌ blank — ÚRS online</t>
         </is>
       </c>
-      <c r="I130" s="18" t="inlineStr">
+      <c r="I131" s="18" t="inlineStr">
         <is>
           <t>260219_dum.HSV7.009 → HSV7.009a</t>
         </is>
       </c>
-      <c r="J130" s="18" t="inlineStr">
+      <c r="J131" s="18" t="inlineStr">
         <is>
           <t>S03</t>
         </is>
       </c>
-      <c r="K130" s="18" t="inlineStr">
+      <c r="K131" s="18" t="inlineStr">
         <is>
           <t>Rošt.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
-    <row r="131">
-      <c r="A131" s="14" t="n">
-        <v>122</v>
-      </c>
-      <c r="B131" s="15" t="inlineStr">
+    <row r="132">
+      <c r="A132" s="14" t="n">
+        <v>123</v>
+      </c>
+      <c r="B132" s="15" t="inlineStr">
         <is>
           <t>HSV-7 Fasáda + zateplení</t>
         </is>
       </c>
-      <c r="C131" s="15" t="inlineStr">
+      <c r="C132" s="15" t="inlineStr">
         <is>
           <t>Keramický obklad soklu 20 mm — montáž+materiál</t>
         </is>
       </c>
-      <c r="D131" s="14" t="inlineStr">
+      <c r="D132" s="14" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E131" s="16" t="n">
+      <c r="E132" s="16" t="n">
         <v>24</v>
       </c>
-      <c r="F131" s="15">
+      <c r="F132" s="15">
         <f> 23 × 1.05</f>
         <v/>
       </c>
-      <c r="G131" s="15" t="inlineStr">
+      <c r="G132" s="15" t="inlineStr">
         <is>
           <t>781</t>
         </is>
       </c>
-      <c r="H131" s="14" t="inlineStr">
+      <c r="H132" s="14" t="inlineStr">
         <is>
           <t>⚠ família ??? (ÚRS online)</t>
         </is>
       </c>
-      <c r="I131" s="15" t="inlineStr">
+      <c r="I132" s="15" t="inlineStr">
         <is>
           <t>260219_dum.HSV7.009 → HSV7.009b</t>
         </is>
       </c>
-      <c r="J131" s="15" t="inlineStr">
+      <c r="J132" s="15" t="inlineStr">
         <is>
           <t>S03</t>
         </is>
       </c>
-      <c r="K131" s="15" t="inlineStr">
+      <c r="K132" s="15" t="inlineStr">
         <is>
           <t>Obklad.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
@@ -8061,13 +8113,13 @@
   <autoFilter ref="A1:K1"/>
   <mergeCells count="8">
     <mergeCell ref="A22:K22"/>
+    <mergeCell ref="A127:K127"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A98:K98"/>
     <mergeCell ref="A68:K68"/>
     <mergeCell ref="A44:K44"/>
     <mergeCell ref="A116:K116"/>
     <mergeCell ref="A36:K36"/>
-    <mergeCell ref="A126:K126"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -16954,11 +17006,11 @@
         <v>276.7</v>
       </c>
       <c r="F9" s="14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G9" s="15" t="inlineStr">
         <is>
-          <t>HSV7.002a, HSV7.002b</t>
+          <t>HSV7.002a, HSV7.002b, HSV7.002c</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(rd-jachymov): sokl reconcile — výkres S03 (Styrcon+keramický) wins, remove TZ duplicate (233→232)
PD rozpor resolved per investor decision (apply VÝKRES):
- TZ ARS dům text: sokl = XPS + cihelný obklad (HSV7.003)
- výkres S03 + Řez A-A + pohledy C: sokl = sanační Styrcon 200 + keramický obklad

Investor chose VÝKRES → removed HSV7.003 (XPS+cihelný) which double-counted the sokl
obklad (cihelný 13.5 + keramický 23 = 36.5 m² on ~23 m² sokl). Sokl now single S03
treatment (HSV7.007 Styrcon + HSV7.008 nopová folie + HSV7.009 keramický obklad).
Omítka HSV7.006 290.2→276.7 (sokl is keramický obklad, not omítka).

vyjasnění #35 — projektant confirm: výkres (Styrcon+keramický) vs TZ ARS (XPS+cihelný)
+ sokl area should apply řadovka 0.7 (23→~16 m²). HSV7.003 atomic block removed.
10-step regen + assert 31==queue 31. snapshot items_pre_sokl_reconcile.json.

https://claude.ai/code/session_01FskzLAZkXgJAwuN2cQQEdx
</commit_message>
<xml_diff>
--- a/test-data/RD_Jachymov_dum/outputs/Vykaz_vymer_RD_Jachymov_ATOMIC_WORKLIST_2026-05-27.xlsx
+++ b/test-data/RD_Jachymov_dum/outputs/Vykaz_vymer_RD_Jachymov_ATOMIC_WORKLIST_2026-05-27.xlsx
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B5" s="5" t="n">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="B6" s="5" t="n">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C6" s="2">
         <f> carried 1:1 + decomposed children</f>
@@ -603,7 +603,7 @@
         </is>
       </c>
       <c r="B7" s="5" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
@@ -618,7 +618,7 @@
         </is>
       </c>
       <c r="B8" s="5" t="n">
-        <v>90</v>
+        <v>88</v>
       </c>
     </row>
     <row r="9">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="B22" s="5" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
     </row>
     <row r="23">
@@ -1049,7 +1049,7 @@
         </is>
       </c>
       <c r="B53" s="5" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="54">
@@ -1200,7 +1200,7 @@
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>713</t>
+          <t>962</t>
         </is>
       </c>
       <c r="B71" s="5" t="n">
@@ -1210,17 +1210,17 @@
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>962</t>
+          <t>622</t>
         </is>
       </c>
       <c r="B72" s="5" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>622</t>
+          <t>713</t>
         </is>
       </c>
       <c r="B73" s="5" t="n">
@@ -1240,17 +1240,17 @@
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>781</t>
+          <t>210</t>
         </is>
       </c>
       <c r="B75" s="5" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>210</t>
+          <t>764</t>
         </is>
       </c>
       <c r="B76" s="5" t="n">
@@ -1260,7 +1260,7 @@
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>764</t>
+          <t>771</t>
         </is>
       </c>
       <c r="B77" s="5" t="n">
@@ -1270,7 +1270,7 @@
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>771</t>
+          <t>781</t>
         </is>
       </c>
       <c r="B78" s="5" t="n">
@@ -1731,7 +1731,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K132"/>
+  <dimension ref="A1:K130"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -7311,7 +7311,7 @@
     <row r="116">
       <c r="A116" s="8" t="inlineStr">
         <is>
-          <t>━━ HSV-7 Fasáda ETICS  (10 atomic operací) ━━</t>
+          <t>━━ HSV-7 Fasáda ETICS  (8 atomic operací) ━━</t>
         </is>
       </c>
       <c r="B116" s="9" t="n"/>
@@ -7545,24 +7545,24 @@
       </c>
       <c r="C121" s="15" t="inlineStr">
         <is>
-          <t>Lepení + kotvení desek XPS λ=0.034 tl. 120 mm + soklový profil — ETICS sokl</t>
+          <t>Špalety oken — EPS přesah 35-40 mm lepení + kotvení</t>
         </is>
       </c>
       <c r="D121" s="14" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>bm</t>
         </is>
       </c>
       <c r="E121" s="16" t="n">
-        <v>13.5</v>
+        <v>82.2</v>
       </c>
       <c r="F121" s="15">
-        <f> HSV7.003 plocha soklu 13.5 m²</f>
+        <f> HSV7.004 obvod špalet 82.2 bm</f>
         <v/>
       </c>
       <c r="G121" s="15" t="inlineStr">
         <is>
-          <t>713</t>
+          <t>622</t>
         </is>
       </c>
       <c r="H121" s="14" t="inlineStr">
@@ -7572,17 +7572,17 @@
       </c>
       <c r="I121" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.003 → HSV7.003a</t>
+          <t>260219_dum.HSV7.004 → HSV7.004a</t>
         </is>
       </c>
       <c r="J121" s="15" t="inlineStr">
         <is>
-          <t>S01</t>
+          <t>S01, S12a</t>
         </is>
       </c>
       <c r="K121" s="15" t="inlineStr">
         <is>
-          <t>Sokl XPS lepení + soklový profil (713/622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+          <t>Špalety EPS přesah (622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -7597,273 +7597,265 @@
       </c>
       <c r="C122" s="15" t="inlineStr">
         <is>
-          <t>Cihelný obklad soklu spárovaný (na armovací vrstvu)</t>
+          <t>Špalety oken — armovací vrstva síťka + omítka</t>
         </is>
       </c>
       <c r="D122" s="14" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>bm</t>
         </is>
       </c>
       <c r="E122" s="16" t="n">
-        <v>13.5</v>
+        <v>82.2</v>
       </c>
       <c r="F122" s="15">
-        <f> HSV7.003 plocha soklu 13.5 m²</f>
-        <v/>
-      </c>
-      <c r="G122" s="15" t="inlineStr">
-        <is>
-          <t>781</t>
-        </is>
-      </c>
-      <c r="H122" s="14" t="inlineStr">
-        <is>
-          <t>⚠ família ??? (ÚRS online)</t>
-        </is>
-      </c>
-      <c r="I122" s="15" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.003 → HSV7.003b</t>
-        </is>
-      </c>
-      <c r="J122" s="15" t="inlineStr">
-        <is>
-          <t>S01</t>
-        </is>
-      </c>
-      <c r="K122" s="15" t="inlineStr">
-        <is>
-          <t>Cihelný obklad spárovaný (781 família obklady).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
-        </is>
-      </c>
-    </row>
-    <row r="123">
-      <c r="A123" s="14" t="n">
-        <v>115</v>
-      </c>
-      <c r="B123" s="15" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda ETICS</t>
-        </is>
-      </c>
-      <c r="C123" s="15" t="inlineStr">
-        <is>
-          <t>Špalety oken — EPS přesah 35-40 mm lepení + kotvení</t>
-        </is>
-      </c>
-      <c r="D123" s="14" t="inlineStr">
-        <is>
-          <t>bm</t>
-        </is>
-      </c>
-      <c r="E123" s="16" t="n">
-        <v>82.2</v>
-      </c>
-      <c r="F123" s="15">
-        <f> HSV7.004 obvod špalet 82.2 bm</f>
-        <v/>
-      </c>
-      <c r="G123" s="15" t="inlineStr">
-        <is>
-          <t>622</t>
-        </is>
-      </c>
-      <c r="H123" s="14" t="inlineStr">
-        <is>
-          <t>⚠ família ??? (ÚRS online)</t>
-        </is>
-      </c>
-      <c r="I123" s="15" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.004 → HSV7.004a</t>
-        </is>
-      </c>
-      <c r="J123" s="15" t="inlineStr">
-        <is>
-          <t>S01, S12a</t>
-        </is>
-      </c>
-      <c r="K123" s="15" t="inlineStr">
-        <is>
-          <t>Špalety EPS přesah (622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
-        </is>
-      </c>
-    </row>
-    <row r="124">
-      <c r="A124" s="14" t="n">
-        <v>116</v>
-      </c>
-      <c r="B124" s="15" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda ETICS</t>
-        </is>
-      </c>
-      <c r="C124" s="15" t="inlineStr">
-        <is>
-          <t>Špalety oken — armovací vrstva síťka + omítka</t>
-        </is>
-      </c>
-      <c r="D124" s="14" t="inlineStr">
-        <is>
-          <t>bm</t>
-        </is>
-      </c>
-      <c r="E124" s="16" t="n">
-        <v>82.2</v>
-      </c>
-      <c r="F124" s="15">
         <f> HSV7.004 obvod 82.2 bm</f>
         <v/>
       </c>
-      <c r="G124" s="15" t="inlineStr">
+      <c r="G122" s="15" t="inlineStr">
         <is>
           <t>622</t>
         </is>
       </c>
-      <c r="H124" s="14" t="inlineStr">
+      <c r="H122" s="14" t="inlineStr">
         <is>
           <t>⚠ família ??? (ÚRS online)</t>
         </is>
       </c>
-      <c r="I124" s="15" t="inlineStr">
+      <c r="I122" s="15" t="inlineStr">
         <is>
           <t>260219_dum.HSV7.004 → HSV7.004b</t>
         </is>
       </c>
-      <c r="J124" s="15" t="inlineStr">
+      <c r="J122" s="15" t="inlineStr">
         <is>
           <t>S01, S12a</t>
         </is>
       </c>
-      <c r="K124" s="15" t="inlineStr">
+      <c r="K122" s="15" t="inlineStr">
         <is>
           <t>Armovací vrstva + omítka špalet (622 família).  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
+    <row r="123">
+      <c r="A123" s="10" t="n">
+        <v>115</v>
+      </c>
+      <c r="B123" s="11" t="inlineStr">
+        <is>
+          <t>HSV-7 Fasáda ETICS</t>
+        </is>
+      </c>
+      <c r="C123" s="11" t="inlineStr">
+        <is>
+          <t>Profilace fasády — různé tloušťky EPS (kordony, šambrány, rámování oken) — paušál podle pohledů</t>
+        </is>
+      </c>
+      <c r="D123" s="10" t="inlineStr">
+        <is>
+          <t>soubor</t>
+        </is>
+      </c>
+      <c r="E123" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="F123" s="11" t="inlineStr">
+        <is>
+          <t>paušál — dle pohledů NCS NZÚ</t>
+        </is>
+      </c>
+      <c r="G123" s="11" t="inlineStr">
+        <is>
+          <t>622221221</t>
+        </is>
+      </c>
+      <c r="H123" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I123" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.005</t>
+        </is>
+      </c>
+      <c r="J123" s="11" t="inlineStr">
+        <is>
+          <t>S01, S12a</t>
+        </is>
+      </c>
+      <c r="K123" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" s="10" t="n">
+        <v>116</v>
+      </c>
+      <c r="B124" s="11" t="inlineStr">
+        <is>
+          <t>HSV-7 Fasáda ETICS</t>
+        </is>
+      </c>
+      <c r="C124" s="11" t="inlineStr">
+        <is>
+          <t>Tenkovrstvá pastovitá probarvená omítka, lomená bílá NCS NZÚ — finální vrstva ETICS</t>
+        </is>
+      </c>
+      <c r="D124" s="10" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E124" s="12" t="n">
+        <v>276.7</v>
+      </c>
+      <c r="F124" s="11" t="inlineStr">
+        <is>
+          <t>ETICS fasáda 276.7 m² (sokl = keramický obklad S03, NE omítka)</t>
+        </is>
+      </c>
+      <c r="G124" s="13" t="inlineStr">
+        <is>
+          <t>622521111</t>
+        </is>
+      </c>
+      <c r="H124" s="10" t="inlineStr">
+        <is>
+          <t>⚠ kandidát-verify</t>
+        </is>
+      </c>
+      <c r="I124" s="11" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.006</t>
+        </is>
+      </c>
+      <c r="J124" s="11" t="inlineStr">
+        <is>
+          <t>S01, S12a, S12b</t>
+        </is>
+      </c>
+      <c r="K124" s="11" t="inlineStr">
+        <is>
+          <t>Carried 1:1 (atomic — no decomposition needed)</t>
+        </is>
+      </c>
+    </row>
     <row r="125">
-      <c r="A125" s="10" t="n">
+      <c r="A125" s="8" t="inlineStr">
+        <is>
+          <t>━━ HSV-7 Fasáda + zateplení  (5 atomic operací) ━━</t>
+        </is>
+      </c>
+      <c r="B125" s="9" t="n"/>
+      <c r="C125" s="9" t="n"/>
+      <c r="D125" s="9" t="n"/>
+      <c r="E125" s="9" t="n"/>
+      <c r="F125" s="9" t="n"/>
+      <c r="G125" s="9" t="n"/>
+      <c r="H125" s="9" t="n"/>
+      <c r="I125" s="9" t="n"/>
+      <c r="J125" s="9" t="n"/>
+      <c r="K125" s="9" t="n"/>
+    </row>
+    <row r="126">
+      <c r="A126" s="17" t="n">
         <v>117</v>
       </c>
-      <c r="B125" s="11" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda ETICS</t>
-        </is>
-      </c>
-      <c r="C125" s="11" t="inlineStr">
-        <is>
-          <t>Profilace fasády — různé tloušťky EPS (kordony, šambrány, rámování oken) — paušál podle pohledů</t>
-        </is>
-      </c>
-      <c r="D125" s="10" t="inlineStr">
-        <is>
-          <t>soubor</t>
-        </is>
-      </c>
-      <c r="E125" s="12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F125" s="11" t="inlineStr">
-        <is>
-          <t>paušál — dle pohledů NCS NZÚ</t>
-        </is>
-      </c>
-      <c r="G125" s="11" t="inlineStr">
-        <is>
-          <t>622221221</t>
-        </is>
-      </c>
-      <c r="H125" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I125" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.005</t>
-        </is>
-      </c>
-      <c r="J125" s="11" t="inlineStr">
-        <is>
-          <t>S01, S12a</t>
-        </is>
-      </c>
-      <c r="K125" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="126">
-      <c r="A126" s="10" t="n">
+      <c r="B126" s="18" t="inlineStr">
+        <is>
+          <t>HSV-7 Fasáda + zateplení</t>
+        </is>
+      </c>
+      <c r="C126" s="18" t="inlineStr">
+        <is>
+          <t>Montáž sanační izolační desky Styrcon 200 + armovací — sokl S03</t>
+        </is>
+      </c>
+      <c r="D126" s="17" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E126" s="19" t="n">
+        <v>23</v>
+      </c>
+      <c r="F126" s="18">
+        <f> obvod 38.7 × 0.6 ≈ 23 (OVĚŘIT)</f>
+        <v/>
+      </c>
+      <c r="G126" s="18" t="inlineStr"/>
+      <c r="H126" s="17" t="inlineStr">
+        <is>
+          <t>❌ blank — ÚRS online</t>
+        </is>
+      </c>
+      <c r="I126" s="18" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.007 → HSV7.007a</t>
+        </is>
+      </c>
+      <c r="J126" s="18" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="K126" s="18" t="inlineStr">
+        <is>
+          <t>Montáž.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" s="17" t="n">
         <v>118</v>
       </c>
-      <c r="B126" s="11" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda ETICS</t>
-        </is>
-      </c>
-      <c r="C126" s="11" t="inlineStr">
-        <is>
-          <t>Tenkovrstvá pastovitá probarvená omítka, lomená bílá NCS NZÚ — finální vrstva ETICS</t>
-        </is>
-      </c>
-      <c r="D126" s="10" t="inlineStr">
+      <c r="B127" s="18" t="inlineStr">
+        <is>
+          <t>HSV-7 Fasáda + zateplení</t>
+        </is>
+      </c>
+      <c r="C127" s="18" t="inlineStr">
+        <is>
+          <t>Sanační deska Styrcon 200 + lepící tmel + armovací stěrka+tkanina — materiál</t>
+        </is>
+      </c>
+      <c r="D127" s="17" t="inlineStr">
         <is>
           <t>m²</t>
         </is>
       </c>
-      <c r="E126" s="12" t="n">
-        <v>290.2</v>
-      </c>
-      <c r="F126" s="11" t="inlineStr">
-        <is>
-          <t>ETICS plocha 276.7 m² + sokl 13.5 m² = 290.2 m²</t>
-        </is>
-      </c>
-      <c r="G126" s="13" t="inlineStr">
-        <is>
-          <t>622521111</t>
-        </is>
-      </c>
-      <c r="H126" s="10" t="inlineStr">
-        <is>
-          <t>⚠ kandidát-verify</t>
-        </is>
-      </c>
-      <c r="I126" s="11" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.006</t>
-        </is>
-      </c>
-      <c r="J126" s="11" t="inlineStr">
-        <is>
-          <t>S01, S12a, S12b</t>
-        </is>
-      </c>
-      <c r="K126" s="11" t="inlineStr">
-        <is>
-          <t>Carried 1:1 (atomic — no decomposition needed)</t>
-        </is>
-      </c>
-    </row>
-    <row r="127">
-      <c r="A127" s="8" t="inlineStr">
-        <is>
-          <t>━━ HSV-7 Fasáda + zateplení  (5 atomic operací) ━━</t>
-        </is>
-      </c>
-      <c r="B127" s="9" t="n"/>
-      <c r="C127" s="9" t="n"/>
-      <c r="D127" s="9" t="n"/>
-      <c r="E127" s="9" t="n"/>
-      <c r="F127" s="9" t="n"/>
-      <c r="G127" s="9" t="n"/>
-      <c r="H127" s="9" t="n"/>
-      <c r="I127" s="9" t="n"/>
-      <c r="J127" s="9" t="n"/>
-      <c r="K127" s="9" t="n"/>
+      <c r="E127" s="19" t="n">
+        <v>24</v>
+      </c>
+      <c r="F127" s="18">
+        <f> 23 × 1.05</f>
+        <v/>
+      </c>
+      <c r="G127" s="18" t="inlineStr"/>
+      <c r="H127" s="17" t="inlineStr">
+        <is>
+          <t>❌ blank — ÚRS online</t>
+        </is>
+      </c>
+      <c r="I127" s="18" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.007 → HSV7.007b</t>
+        </is>
+      </c>
+      <c r="J127" s="18" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="K127" s="18" t="inlineStr">
+        <is>
+          <t>Materiál.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="17" t="n">
@@ -7876,7 +7868,7 @@
       </c>
       <c r="C128" s="18" t="inlineStr">
         <is>
-          <t>Montáž sanační izolační desky Styrcon 200 + armovací — sokl S03</t>
+          <t>Drenážní nopová folie 20 mm — dodávka+montáž, sokl pod terénem S03a</t>
         </is>
       </c>
       <c r="D128" s="17" t="inlineStr">
@@ -7885,10 +7877,10 @@
         </is>
       </c>
       <c r="E128" s="19" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F128" s="18">
-        <f> obvod 38.7 × 0.6 ≈ 23 (OVĚŘIT)</f>
+        <f> 23 × 1.10</f>
         <v/>
       </c>
       <c r="G128" s="18" t="inlineStr"/>
@@ -7899,7 +7891,7 @@
       </c>
       <c r="I128" s="18" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.007 → HSV7.007a</t>
+          <t>260219_dum.HSV7.008 → HSV7.008a</t>
         </is>
       </c>
       <c r="J128" s="18" t="inlineStr">
@@ -7909,7 +7901,7 @@
       </c>
       <c r="K128" s="18" t="inlineStr">
         <is>
-          <t>Montáž.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+          <t>Montáž+materiál.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
       </c>
     </row>
@@ -7924,7 +7916,7 @@
       </c>
       <c r="C129" s="18" t="inlineStr">
         <is>
-          <t>Sanační deska Styrcon 200 + lepící tmel + armovací stěrka+tkanina — materiál</t>
+          <t>Kotevní rošt 40 mm provětraného soklu — montáž+materiál S03b</t>
         </is>
       </c>
       <c r="D129" s="17" t="inlineStr">
@@ -7933,177 +7925,81 @@
         </is>
       </c>
       <c r="E129" s="19" t="n">
+        <v>23</v>
+      </c>
+      <c r="F129" s="18">
+        <f> 23 (OVĚŘIT)</f>
+        <v/>
+      </c>
+      <c r="G129" s="18" t="inlineStr"/>
+      <c r="H129" s="17" t="inlineStr">
+        <is>
+          <t>❌ blank — ÚRS online</t>
+        </is>
+      </c>
+      <c r="I129" s="18" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.009 → HSV7.009a</t>
+        </is>
+      </c>
+      <c r="J129" s="18" t="inlineStr">
+        <is>
+          <t>S03</t>
+        </is>
+      </c>
+      <c r="K129" s="18" t="inlineStr">
+        <is>
+          <t>Rošt.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" s="14" t="n">
+        <v>121</v>
+      </c>
+      <c r="B130" s="15" t="inlineStr">
+        <is>
+          <t>HSV-7 Fasáda + zateplení</t>
+        </is>
+      </c>
+      <c r="C130" s="15" t="inlineStr">
+        <is>
+          <t>Keramický obklad soklu 20 mm — montáž+materiál</t>
+        </is>
+      </c>
+      <c r="D130" s="14" t="inlineStr">
+        <is>
+          <t>m²</t>
+        </is>
+      </c>
+      <c r="E130" s="16" t="n">
         <v>24</v>
       </c>
-      <c r="F129" s="18">
+      <c r="F130" s="15">
         <f> 23 × 1.05</f>
         <v/>
       </c>
-      <c r="G129" s="18" t="inlineStr"/>
-      <c r="H129" s="17" t="inlineStr">
-        <is>
-          <t>❌ blank — ÚRS online</t>
-        </is>
-      </c>
-      <c r="I129" s="18" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.007 → HSV7.007b</t>
-        </is>
-      </c>
-      <c r="J129" s="18" t="inlineStr">
+      <c r="G130" s="15" t="inlineStr">
+        <is>
+          <t>781</t>
+        </is>
+      </c>
+      <c r="H130" s="14" t="inlineStr">
+        <is>
+          <t>⚠ família ??? (ÚRS online)</t>
+        </is>
+      </c>
+      <c r="I130" s="15" t="inlineStr">
+        <is>
+          <t>260219_dum.HSV7.009 → HSV7.009b</t>
+        </is>
+      </c>
+      <c r="J130" s="15" t="inlineStr">
         <is>
           <t>S03</t>
         </is>
       </c>
-      <c r="K129" s="18" t="inlineStr">
-        <is>
-          <t>Materiál.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
-        </is>
-      </c>
-    </row>
-    <row r="130">
-      <c r="A130" s="17" t="n">
-        <v>121</v>
-      </c>
-      <c r="B130" s="18" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda + zateplení</t>
-        </is>
-      </c>
-      <c r="C130" s="18" t="inlineStr">
-        <is>
-          <t>Drenážní nopová folie 20 mm — dodávka+montáž, sokl pod terénem S03a</t>
-        </is>
-      </c>
-      <c r="D130" s="17" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E130" s="19" t="n">
-        <v>25</v>
-      </c>
-      <c r="F130" s="18">
-        <f> 23 × 1.10</f>
-        <v/>
-      </c>
-      <c r="G130" s="18" t="inlineStr"/>
-      <c r="H130" s="17" t="inlineStr">
-        <is>
-          <t>❌ blank — ÚRS online</t>
-        </is>
-      </c>
-      <c r="I130" s="18" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.008 → HSV7.008a</t>
-        </is>
-      </c>
-      <c r="J130" s="18" t="inlineStr">
-        <is>
-          <t>S03</t>
-        </is>
-      </c>
-      <c r="K130" s="18" t="inlineStr">
-        <is>
-          <t>Montáž+materiál.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
-        </is>
-      </c>
-    </row>
-    <row r="131">
-      <c r="A131" s="17" t="n">
-        <v>122</v>
-      </c>
-      <c r="B131" s="18" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda + zateplení</t>
-        </is>
-      </c>
-      <c r="C131" s="18" t="inlineStr">
-        <is>
-          <t>Kotevní rošt 40 mm provětraného soklu — montáž+materiál S03b</t>
-        </is>
-      </c>
-      <c r="D131" s="17" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E131" s="19" t="n">
-        <v>23</v>
-      </c>
-      <c r="F131" s="18">
-        <f> 23 (OVĚŘIT)</f>
-        <v/>
-      </c>
-      <c r="G131" s="18" t="inlineStr"/>
-      <c r="H131" s="17" t="inlineStr">
-        <is>
-          <t>❌ blank — ÚRS online</t>
-        </is>
-      </c>
-      <c r="I131" s="18" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.009 → HSV7.009a</t>
-        </is>
-      </c>
-      <c r="J131" s="18" t="inlineStr">
-        <is>
-          <t>S03</t>
-        </is>
-      </c>
-      <c r="K131" s="18" t="inlineStr">
-        <is>
-          <t>Rošt.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
-        </is>
-      </c>
-    </row>
-    <row r="132">
-      <c r="A132" s="14" t="n">
-        <v>123</v>
-      </c>
-      <c r="B132" s="15" t="inlineStr">
-        <is>
-          <t>HSV-7 Fasáda + zateplení</t>
-        </is>
-      </c>
-      <c r="C132" s="15" t="inlineStr">
-        <is>
-          <t>Keramický obklad soklu 20 mm — montáž+materiál</t>
-        </is>
-      </c>
-      <c r="D132" s="14" t="inlineStr">
-        <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E132" s="16" t="n">
-        <v>24</v>
-      </c>
-      <c r="F132" s="15">
-        <f> 23 × 1.05</f>
-        <v/>
-      </c>
-      <c r="G132" s="15" t="inlineStr">
-        <is>
-          <t>781</t>
-        </is>
-      </c>
-      <c r="H132" s="14" t="inlineStr">
-        <is>
-          <t>⚠ família ??? (ÚRS online)</t>
-        </is>
-      </c>
-      <c r="I132" s="15" t="inlineStr">
-        <is>
-          <t>260219_dum.HSV7.009 → HSV7.009b</t>
-        </is>
-      </c>
-      <c r="J132" s="15" t="inlineStr">
-        <is>
-          <t>S03</t>
-        </is>
-      </c>
-      <c r="K132" s="15" t="inlineStr">
+      <c r="K130" s="15" t="inlineStr">
         <is>
           <t>Obklad.  Doplnit leaf z CS ÚRS online (app.urs.cz, cen. úroveň 2026 01) dle família + popis + Vzorec.</t>
         </is>
@@ -8113,7 +8009,7 @@
   <autoFilter ref="A1:K1"/>
   <mergeCells count="8">
     <mergeCell ref="A22:K22"/>
-    <mergeCell ref="A127:K127"/>
+    <mergeCell ref="A125:K125"/>
     <mergeCell ref="A2:K2"/>
     <mergeCell ref="A98:K98"/>
     <mergeCell ref="A68:K68"/>
@@ -16701,7 +16597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -17017,7 +16913,7 @@
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.003</t>
+          <t>260219_dum.HSV7.004</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
@@ -17027,40 +16923,40 @@
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
-          <t>ETICS sokl — XPS λ=0.034 tl. 120 mm + soklový profil + cihelný obklad spárovaný</t>
+          <t>Špalety oken — EPS přesah 35-40 mm + síťka + omítka</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>bm</t>
         </is>
       </c>
       <c r="E10" s="16" t="n">
-        <v>13.5</v>
+        <v>82.2</v>
       </c>
       <c r="F10" s="14" t="n">
         <v>2</v>
       </c>
       <c r="G10" s="15" t="inlineStr">
         <is>
-          <t>HSV7.003a, HSV7.003b</t>
+          <t>HSV7.004a, HSV7.004b</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.004</t>
+          <t>260219_dum.PSV76.103</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>HSV-7 Fasáda ETICS</t>
+          <t>PSV-76 Klempíř</t>
         </is>
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>Špalety oken — EPS přesah 35-40 mm + síťka + omítka</t>
+          <t>Dešťové svody Pzn 100 mm + žlaby — 4 svody × ~14 m + žlaby per obvod střechy</t>
         </is>
       </c>
       <c r="D11" s="14" t="inlineStr">
@@ -17069,64 +16965,64 @@
         </is>
       </c>
       <c r="E11" s="16" t="n">
-        <v>82.2</v>
+        <v>43.5</v>
       </c>
       <c r="F11" s="14" t="n">
         <v>2</v>
       </c>
       <c r="G11" s="15" t="inlineStr">
         <is>
-          <t>HSV7.004a, HSV7.004b</t>
+          <t>PSV76.103a, PSV76.103b</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV76.103</t>
+          <t>260219_dum.PSV76.302</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>PSV-76 Klempíř</t>
+          <t>PSV-76 Truhlář</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>Dešťové svody Pzn 100 mm + žlaby — 4 svody × ~14 m + žlaby per obvod střechy</t>
+          <t>Dřevěná terasa za opěrnou stěnou — prkna garapa 145×25 mm na dřevěném roštu z hranolů 50 mm na rektifikovatelných terčíc</t>
         </is>
       </c>
       <c r="D12" s="14" t="inlineStr">
         <is>
-          <t>bm</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E12" s="16" t="n">
-        <v>43.5</v>
+        <v>9.23</v>
       </c>
       <c r="F12" s="14" t="n">
         <v>2</v>
       </c>
       <c r="G12" s="15" t="inlineStr">
         <is>
-          <t>PSV76.103a, PSV76.103b</t>
+          <t>PSV76.302a, PSV76.302b</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV76.302</t>
+          <t>260219_dum.PSV77.002</t>
         </is>
       </c>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>PSV-76 Truhlář</t>
+          <t>PSV-77 Podlahy</t>
         </is>
       </c>
       <c r="C13" s="15" t="inlineStr">
         <is>
-          <t>Dřevěná terasa za opěrnou stěnou — prkna garapa 145×25 mm na dřevěném roštu z hranolů 50 mm na rektifikovatelných terčíc</t>
+          <t>Nášlapná vrstva keramická dlažba lepená — koupelny + WC + spíž + komora (NÁDRŽ NP)</t>
         </is>
       </c>
       <c r="D13" s="14" t="inlineStr">
@@ -17135,21 +17031,21 @@
         </is>
       </c>
       <c r="E13" s="16" t="n">
-        <v>9.23</v>
+        <v>13.5</v>
       </c>
       <c r="F13" s="14" t="n">
         <v>2</v>
       </c>
       <c r="G13" s="15" t="inlineStr">
         <is>
-          <t>PSV76.302a, PSV76.302b</t>
+          <t>PSV77.002a, PSV77.002b</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV77.002</t>
+          <t>260219_dum.PSV77.003</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
@@ -17159,7 +17055,7 @@
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>Nášlapná vrstva keramická dlažba lepená — koupelny + WC + spíž + komora (NÁDRŽ NP)</t>
+          <t>Nášlapná vrstva keramická dlažba — 1.PP technické místnosti (sušárna + sklepy + schodiště + chodba)</t>
         </is>
       </c>
       <c r="D14" s="14" t="inlineStr">
@@ -17168,31 +17064,31 @@
         </is>
       </c>
       <c r="E14" s="16" t="n">
-        <v>13.5</v>
+        <v>32.4</v>
       </c>
       <c r="F14" s="14" t="n">
         <v>2</v>
       </c>
       <c r="G14" s="15" t="inlineStr">
         <is>
-          <t>PSV77.002a, PSV77.002b</t>
+          <t>PSV77.003a, PSV77.003b</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV77.003</t>
+          <t>260219_dum.PSV78.001</t>
         </is>
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>PSV-77 Podlahy</t>
+          <t>PSV-78 Povrchové úpravy</t>
         </is>
       </c>
       <c r="C15" s="15" t="inlineStr">
         <is>
-          <t>Nášlapná vrstva keramická dlažba — 1.PP technické místnosti (sušárna + sklepy + schodiště + chodba)</t>
+          <t>Omítka jádrová vápenocementová tl. 15 mm + štuková povrchová úprava na stěnách 1.PP (stávající vyspravené + nové zděné)</t>
         </is>
       </c>
       <c r="D15" s="14" t="inlineStr">
@@ -17201,21 +17097,21 @@
         </is>
       </c>
       <c r="E15" s="16" t="n">
-        <v>32.4</v>
+        <v>78.2</v>
       </c>
       <c r="F15" s="14" t="n">
         <v>2</v>
       </c>
       <c r="G15" s="15" t="inlineStr">
         <is>
-          <t>PSV77.003a, PSV77.003b</t>
+          <t>PSV78.001a, PSV78.001b</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV78.001</t>
+          <t>260219_dum.PSV78.002</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
@@ -17225,7 +17121,7 @@
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>Omítka jádrová vápenocementová tl. 15 mm + štuková povrchová úprava na stěnách 1.PP (stávající vyspravené + nové zděné)</t>
+          <t>Omítka jádrová vápenocementová tl. 15 mm + štuková povrchová úprava na stěnách 1.NP (stávající vyspravené + nové zděné)</t>
         </is>
       </c>
       <c r="D16" s="14" t="inlineStr">
@@ -17234,21 +17130,21 @@
         </is>
       </c>
       <c r="E16" s="16" t="n">
-        <v>78.2</v>
+        <v>208.4</v>
       </c>
       <c r="F16" s="14" t="n">
         <v>2</v>
       </c>
       <c r="G16" s="15" t="inlineStr">
         <is>
-          <t>PSV78.001a, PSV78.001b</t>
+          <t>PSV78.002a, PSV78.002b</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV78.002</t>
+          <t>260219_dum.PSV78.003</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
@@ -17258,7 +17154,7 @@
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
-          <t>Omítka jádrová vápenocementová tl. 15 mm + štuková povrchová úprava na stěnách 1.NP (stávající vyspravené + nové zděné)</t>
+          <t>Omítka jádrová vápenocementová tl. 15 mm + štuková povrchová úprava na stěnách 2.NP (stávající vyspravené + nové zděné)</t>
         </is>
       </c>
       <c r="D17" s="14" t="inlineStr">
@@ -17267,21 +17163,21 @@
         </is>
       </c>
       <c r="E17" s="16" t="n">
-        <v>208.4</v>
+        <v>201.6</v>
       </c>
       <c r="F17" s="14" t="n">
         <v>2</v>
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
-          <t>PSV78.002a, PSV78.002b</t>
+          <t>PSV78.003a, PSV78.003b</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV78.003</t>
+          <t>260219_dum.PSV78.004</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
@@ -17291,7 +17187,7 @@
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
-          <t>Omítka jádrová vápenocementová tl. 15 mm + štuková povrchová úprava na stěnách 2.NP (stávající vyspravené + nové zděné)</t>
+          <t>Omítka jádrová vápenocementová tl. 15 mm + štuková povrchová úprava na stěnách 3.NP (stávající vyspravené + nové zděné)</t>
         </is>
       </c>
       <c r="D18" s="14" t="inlineStr">
@@ -17300,54 +17196,54 @@
         </is>
       </c>
       <c r="E18" s="16" t="n">
-        <v>201.6</v>
+        <v>179.1</v>
       </c>
       <c r="F18" s="14" t="n">
         <v>2</v>
       </c>
       <c r="G18" s="15" t="inlineStr">
         <is>
-          <t>PSV78.003a, PSV78.003b</t>
+          <t>PSV78.004a, PSV78.004b</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV78.004</t>
+          <t>260219_dum.PSV72.004</t>
         </is>
       </c>
       <c r="B19" s="15" t="inlineStr">
         <is>
-          <t>PSV-78 Povrchové úpravy</t>
+          <t>PSV-72 ZTI</t>
         </is>
       </c>
       <c r="C19" s="15" t="inlineStr">
         <is>
-          <t>Omítka jádrová vápenocementová tl. 15 mm + štuková povrchová úprava na stěnách 3.NP (stávající vyspravené + nové zděné)</t>
+          <t>Sanitární keramika dodávka + montáž v koupelně 1.05 1.NP: 1× vana (DXF) + 1× umyvadlo (DXF) + 1× WC (TZ standard)</t>
         </is>
       </c>
       <c r="D19" s="14" t="inlineStr">
         <is>
-          <t>m²</t>
+          <t>set</t>
         </is>
       </c>
       <c r="E19" s="16" t="n">
-        <v>179.1</v>
+        <v>0</v>
       </c>
       <c r="F19" s="14" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G19" s="15" t="inlineStr">
         <is>
-          <t>PSV78.004a, PSV78.004b</t>
+          <t>PSV72.004a, PSV72.004b, PSV72.004c</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV72.004</t>
+          <t>260219_dum.PSV72.005</t>
         </is>
       </c>
       <c r="B20" s="15" t="inlineStr">
@@ -17357,7 +17253,7 @@
       </c>
       <c r="C20" s="15" t="inlineStr">
         <is>
-          <t>Sanitární keramika dodávka + montáž v koupelně 1.05 1.NP: 1× vana (DXF) + 1× umyvadlo (DXF) + 1× WC (TZ standard)</t>
+          <t>Sanitární keramika dodávka + montáž v koupelně 2.03 2.NP: 1× umyvadlo (DXF) + 1× WC (TZ standard) + 1× sprcha (TZ standa</t>
         </is>
       </c>
       <c r="D20" s="14" t="inlineStr">
@@ -17373,14 +17269,14 @@
       </c>
       <c r="G20" s="15" t="inlineStr">
         <is>
-          <t>PSV72.004a, PSV72.004b, PSV72.004c</t>
+          <t>PSV72.005a, PSV72.005b, PSV72.005c</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV72.005</t>
+          <t>260219_dum.PSV72.006</t>
         </is>
       </c>
       <c r="B21" s="15" t="inlineStr">
@@ -17390,7 +17286,7 @@
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>Sanitární keramika dodávka + montáž v koupelně 2.03 2.NP: 1× umyvadlo (DXF) + 1× WC (TZ standard) + 1× sprcha (TZ standa</t>
+          <t>Sanitární keramika dodávka + montáž v koupelně 3.04 3.NP: 1× WC (DXF) + 1× umyvadlo (TZ standard) + 1× sprcha (TZ standa</t>
         </is>
       </c>
       <c r="D21" s="14" t="inlineStr">
@@ -17406,14 +17302,14 @@
       </c>
       <c r="G21" s="15" t="inlineStr">
         <is>
-          <t>PSV72.005a, PSV72.005b, PSV72.005c</t>
+          <t>PSV72.006a, PSV72.006b, PSV72.006c</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV72.006</t>
+          <t>260219_dum.PSV72.008</t>
         </is>
       </c>
       <c r="B22" s="15" t="inlineStr">
@@ -17423,129 +17319,129 @@
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>Sanitární keramika dodávka + montáž v koupelně 3.04 3.NP: 1× WC (DXF) + 1× umyvadlo (TZ standard) + 1× sprcha (TZ standa</t>
+          <t>Vodovodní baterie (WC ventil + páková umyvadlová + sprchové + dřezové + termostat sprchové) — ~15 ks + drobné instalační</t>
         </is>
       </c>
       <c r="D22" s="14" t="inlineStr">
         <is>
-          <t>set</t>
+          <t>ks</t>
         </is>
       </c>
       <c r="E22" s="16" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="F22" s="14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G22" s="15" t="inlineStr">
         <is>
-          <t>PSV72.006a, PSV72.006b, PSV72.006c</t>
+          <t>PSV72.008a, PSV72.008b, PSV72.008c, PSV72.008d</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.PSV72.008</t>
+          <t>260219_dum.HSV1.015</t>
         </is>
       </c>
       <c r="B23" s="15" t="inlineStr">
         <is>
-          <t>PSV-72 ZTI</t>
+          <t>HSV-1 Zemní práce</t>
         </is>
       </c>
       <c r="C23" s="15" t="inlineStr">
         <is>
-          <t>Vodovodní baterie (WC ventil + páková umyvadlová + sprchové + dřezové + termostat sprchové) — ~15 ks + drobné instalační</t>
+          <t>Drenáž za opěrnou stěnou (bílou vanou) — drenážní trubka DN100 vlnitá perforovaná + štěrkový obsyp 16/32 + geotextilie +</t>
         </is>
       </c>
       <c r="D23" s="14" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>m</t>
         </is>
       </c>
       <c r="E23" s="16" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="F23" s="14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G23" s="15" t="inlineStr">
         <is>
-          <t>PSV72.008a, PSV72.008b, PSV72.008c, PSV72.008d</t>
+          <t>HSV1.015a, HSV1.015b, HSV1.015c</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV1.015</t>
+          <t>260219_dum.HSV5.017</t>
         </is>
       </c>
       <c r="B24" s="15" t="inlineStr">
         <is>
-          <t>HSV-1 Zemní práce</t>
+          <t>HSV-5 Krov + střecha</t>
         </is>
       </c>
       <c r="C24" s="15" t="inlineStr">
         <is>
-          <t>Drenáž za opěrnou stěnou (bílou vanou) — drenážní trubka DN100 vlnitá perforovaná + štěrkový obsyp 16/32 + geotextilie +</t>
+          <t>Montáž svorníků / šroubů tesařských spojů krovu délky přes 150 do 300 mm — spojení kleštin 2×60/180 mm s krokvemi (svorn</t>
         </is>
       </c>
       <c r="D24" s="14" t="inlineStr">
         <is>
-          <t>m</t>
+          <t>ks</t>
         </is>
       </c>
       <c r="E24" s="16" t="n">
-        <v>12</v>
+        <v>50</v>
       </c>
       <c r="F24" s="14" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G24" s="15" t="inlineStr">
         <is>
-          <t>HSV1.015a, HSV1.015b, HSV1.015c</t>
+          <t>HSV5.017a, HSV5.017b, HSV5.017c, HSV5.017d</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.017</t>
+          <t>260219_dum.HSV4.015</t>
         </is>
       </c>
       <c r="B25" s="15" t="inlineStr">
         <is>
-          <t>HSV-5 Krov + střecha</t>
+          <t>HSV-4 Vodorovné</t>
         </is>
       </c>
       <c r="C25" s="15" t="inlineStr">
         <is>
-          <t>Montáž svorníků / šroubů tesařských spojů krovu délky přes 150 do 300 mm — spojení kleštin 2×60/180 mm s krokvemi (svorn</t>
+          <t>Desky kročejové izolace (Isover T-P) tl. 30 mm — trámový strop 1.NP/2.NP</t>
         </is>
       </c>
       <c r="D25" s="14" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>m²</t>
         </is>
       </c>
       <c r="E25" s="16" t="n">
-        <v>50</v>
+        <v>59.5</v>
       </c>
       <c r="F25" s="14" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G25" s="15" t="inlineStr">
         <is>
-          <t>HSV5.017a, HSV5.017b, HSV5.017c, HSV5.017d</t>
+          <t>HSV4.015a, HSV4.015b</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV4.015</t>
+          <t>260219_dum.HSV4.016</t>
         </is>
       </c>
       <c r="B26" s="15" t="inlineStr">
@@ -17555,7 +17451,7 @@
       </c>
       <c r="C26" s="15" t="inlineStr">
         <is>
-          <t>Desky kročejové izolace (Isover T-P) tl. 30 mm — trámový strop 1.NP/2.NP</t>
+          <t>Separační geotextilie pod suchý podsyp — trámový strop 1.NP/2.NP</t>
         </is>
       </c>
       <c r="D26" s="14" t="inlineStr">
@@ -17567,18 +17463,18 @@
         <v>59.5</v>
       </c>
       <c r="F26" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G26" s="15" t="inlineStr">
         <is>
-          <t>HSV4.015a, HSV4.015b</t>
+          <t>HSV4.016a</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV4.016</t>
+          <t>260219_dum.HSV4.017</t>
         </is>
       </c>
       <c r="B27" s="15" t="inlineStr">
@@ -17588,7 +17484,7 @@
       </c>
       <c r="C27" s="15" t="inlineStr">
         <is>
-          <t>Separační geotextilie pod suchý podsyp — trámový strop 1.NP/2.NP</t>
+          <t>Tepelná/akustická izolace minerální vata výplň mezi ocelové nosníky stropu 2.NP/3.NP, tl. 180/200 mm</t>
         </is>
       </c>
       <c r="D27" s="14" t="inlineStr">
@@ -17597,21 +17493,21 @@
         </is>
       </c>
       <c r="E27" s="16" t="n">
-        <v>59.5</v>
+        <v>104.4</v>
       </c>
       <c r="F27" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G27" s="15" t="inlineStr">
         <is>
-          <t>HSV4.016a</t>
+          <t>HSV4.017a, HSV4.017b</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV4.017</t>
+          <t>260219_dum.HSV4.018</t>
         </is>
       </c>
       <c r="B28" s="15" t="inlineStr">
@@ -17621,7 +17517,7 @@
       </c>
       <c r="C28" s="15" t="inlineStr">
         <is>
-          <t>Tepelná/akustická izolace minerální vata výplň mezi ocelové nosníky stropu 2.NP/3.NP, tl. 180/200 mm</t>
+          <t>Roznášecí sádrovláknité dílce Fermacell 2E22 tl. 25 mm — suchá skladba nad cihelnou klembou S08</t>
         </is>
       </c>
       <c r="D28" s="14" t="inlineStr">
@@ -17629,22 +17525,20 @@
           <t>m²</t>
         </is>
       </c>
-      <c r="E28" s="16" t="n">
-        <v>104.4</v>
-      </c>
+      <c r="E28" s="16" t="n"/>
       <c r="F28" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G28" s="15" t="inlineStr">
         <is>
-          <t>HSV4.017a, HSV4.017b</t>
+          <t>HSV4.018a</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV4.018</t>
+          <t>260219_dum.HSV4.019</t>
         </is>
       </c>
       <c r="B29" s="15" t="inlineStr">
@@ -17654,7 +17548,7 @@
       </c>
       <c r="C29" s="15" t="inlineStr">
         <is>
-          <t>Roznášecí sádrovláknité dílce Fermacell 2E22 tl. 25 mm — suchá skladba nad cihelnou klembou S08</t>
+          <t>Desky kročejové izolace (Isover T-P) tl. 30 mm — suchá skladba nad klembou S08</t>
         </is>
       </c>
       <c r="D29" s="14" t="inlineStr">
@@ -17668,14 +17562,14 @@
       </c>
       <c r="G29" s="15" t="inlineStr">
         <is>
-          <t>HSV4.018a</t>
+          <t>HSV4.019a</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV4.019</t>
+          <t>260219_dum.HSV4.020</t>
         </is>
       </c>
       <c r="B30" s="15" t="inlineStr">
@@ -17685,7 +17579,7 @@
       </c>
       <c r="C30" s="15" t="inlineStr">
         <is>
-          <t>Desky kročejové izolace (Isover T-P) tl. 30 mm — suchá skladba nad klembou S08</t>
+          <t>Vyrovnávací suchý podsyp keramzit/liapor + dřevěný rošt tl. 50 mm — nad klembou S08</t>
         </is>
       </c>
       <c r="D30" s="14" t="inlineStr">
@@ -17699,14 +17593,14 @@
       </c>
       <c r="G30" s="15" t="inlineStr">
         <is>
-          <t>HSV4.019a</t>
+          <t>HSV4.020a</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV4.020</t>
+          <t>260219_dum.HSV4.021</t>
         </is>
       </c>
       <c r="B31" s="15" t="inlineStr">
@@ -17716,7 +17610,7 @@
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
-          <t>Vyrovnávací suchý podsyp keramzit/liapor + dřevěný rošt tl. 50 mm — nad klembou S08</t>
+          <t>Separační vrstva pod suchý podsyp — nad cihelnou klembou S08</t>
         </is>
       </c>
       <c r="D31" s="14" t="inlineStr">
@@ -17730,24 +17624,24 @@
       </c>
       <c r="G31" s="15" t="inlineStr">
         <is>
-          <t>HSV4.020a</t>
+          <t>HSV4.021a</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV4.021</t>
+          <t>260219_dum.HSV7.007</t>
         </is>
       </c>
       <c r="B32" s="15" t="inlineStr">
         <is>
-          <t>HSV-4 Vodorovné</t>
+          <t>HSV-7 Fasáda + zateplení</t>
         </is>
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
-          <t>Separační vrstva pod suchý podsyp — nad cihelnou klembou S08</t>
+          <t>Sanační zateplení soklu — sanační izolační deska Styrcon 200 + lepící tmel (Lepstyr plus) + armovací vrstva s tkaninou +</t>
         </is>
       </c>
       <c r="D32" s="14" t="inlineStr">
@@ -17755,20 +17649,22 @@
           <t>m²</t>
         </is>
       </c>
-      <c r="E32" s="16" t="n"/>
+      <c r="E32" s="16" t="n">
+        <v>23</v>
+      </c>
       <c r="F32" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G32" s="15" t="inlineStr">
         <is>
-          <t>HSV4.021a</t>
+          <t>HSV7.007a, HSV7.007b</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.007</t>
+          <t>260219_dum.HSV7.008</t>
         </is>
       </c>
       <c r="B33" s="15" t="inlineStr">
@@ -17778,7 +17674,7 @@
       </c>
       <c r="C33" s="15" t="inlineStr">
         <is>
-          <t>Sanační zateplení soklu — sanační izolační deska Styrcon 200 + lepící tmel (Lepstyr plus) + armovací vrstva s tkaninou +</t>
+          <t>Drenážní vrstva — nopová folie tl. 20 mm na suterénní stěnu pod úrovní terénu</t>
         </is>
       </c>
       <c r="D33" s="14" t="inlineStr">
@@ -17790,18 +17686,18 @@
         <v>23</v>
       </c>
       <c r="F33" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G33" s="15" t="inlineStr">
         <is>
-          <t>HSV7.007a, HSV7.007b</t>
+          <t>HSV7.008a</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.008</t>
+          <t>260219_dum.HSV7.009</t>
         </is>
       </c>
       <c r="B34" s="15" t="inlineStr">
@@ -17811,7 +17707,7 @@
       </c>
       <c r="C34" s="15" t="inlineStr">
         <is>
-          <t>Drenážní vrstva — nopová folie tl. 20 mm na suterénní stěnu pod úrovní terénu</t>
+          <t>Provětrávaná mezera s kotevním roštem 40 mm + keramický obklad 20 mm — sokl nad úrovní terénu</t>
         </is>
       </c>
       <c r="D34" s="14" t="inlineStr">
@@ -17823,28 +17719,28 @@
         <v>23</v>
       </c>
       <c r="F34" s="14" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G34" s="15" t="inlineStr">
         <is>
-          <t>HSV7.008a</t>
+          <t>HSV7.009a, HSV7.009b</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV7.009</t>
+          <t>260219_dum.HSV5.018</t>
         </is>
       </c>
       <c r="B35" s="15" t="inlineStr">
         <is>
-          <t>HSV-7 Fasáda + zateplení</t>
+          <t>HSV-5 Krov + střecha</t>
         </is>
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>Provětrávaná mezera s kotevním roštem 40 mm + keramický obklad 20 mm — sokl nad úrovní terénu</t>
+          <t>Pojistná hydroizolační folie pod hliníkovou falcovanou krytinu (nad celoplošným bedněním)</t>
         </is>
       </c>
       <c r="D35" s="14" t="inlineStr">
@@ -17853,31 +17749,31 @@
         </is>
       </c>
       <c r="E35" s="16" t="n">
-        <v>23</v>
+        <v>140.94</v>
       </c>
       <c r="F35" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G35" s="15" t="inlineStr">
         <is>
-          <t>HSV7.009a, HSV7.009b</t>
+          <t>HSV5.018a</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV5.018</t>
+          <t>260219_dum.HSV6.018</t>
         </is>
       </c>
       <c r="B36" s="15" t="inlineStr">
         <is>
-          <t>HSV-5 Krov + střecha</t>
+          <t>HSV-6 Bourací práce</t>
         </is>
       </c>
       <c r="C36" s="15" t="inlineStr">
         <is>
-          <t>Pojistná hydroizolační folie pod hliníkovou falcovanou krytinu (nad celoplošným bedněním)</t>
+          <t>Demontáž stávajícího vnějšího keramického obkladu suterénní stěny (sokl) tl. 20 mm</t>
         </is>
       </c>
       <c r="D36" s="14" t="inlineStr">
@@ -17886,31 +17782,31 @@
         </is>
       </c>
       <c r="E36" s="16" t="n">
-        <v>140.94</v>
+        <v>23</v>
       </c>
       <c r="F36" s="14" t="n">
         <v>1</v>
       </c>
       <c r="G36" s="15" t="inlineStr">
         <is>
-          <t>HSV5.018a</t>
+          <t>HSV6.018a</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.HSV6.018</t>
+          <t>260217_sklad.HSV5.002</t>
         </is>
       </c>
       <c r="B37" s="15" t="inlineStr">
         <is>
-          <t>HSV-6 Bourací práce</t>
+          <t>HSV-5 Komunikace + vjezd</t>
         </is>
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
-          <t>Demontáž stávajícího vnějšího keramického obkladu suterénní stěny (sokl) tl. 20 mm</t>
+          <t>Napojení vjezdu na ulici Dvořákova — vydláždění z betonových dlaždic + spádování na pozemek investora + odvodnění dešťov</t>
         </is>
       </c>
       <c r="D37" s="14" t="inlineStr">
@@ -17918,68 +17814,68 @@
           <t>m²</t>
         </is>
       </c>
-      <c r="E37" s="16" t="n">
-        <v>23</v>
-      </c>
+      <c r="E37" s="16" t="n"/>
       <c r="F37" s="14" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G37" s="15" t="inlineStr">
         <is>
-          <t>HSV6.018a</t>
+          <t>HSV5.002a, HSV5.002b, HSV5.002c</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="15" t="inlineStr">
         <is>
-          <t>260217_sklad.HSV5.002</t>
+          <t>260217_sklad.PSV76.002</t>
         </is>
       </c>
       <c r="B38" s="15" t="inlineStr">
         <is>
-          <t>HSV-5 Komunikace + vjezd</t>
+          <t>PSV-76 Zámečnictví</t>
         </is>
       </c>
       <c r="C38" s="15" t="inlineStr">
         <is>
-          <t>Napojení vjezdu na ulici Dvořákova — vydláždění z betonových dlaždic + spádování na pozemek investora + odvodnění dešťov</t>
+          <t>Vjezdová brána na pozemku investora (ocelová) — dodávka + montáž</t>
         </is>
       </c>
       <c r="D38" s="14" t="inlineStr">
         <is>
-          <t>m²</t>
-        </is>
-      </c>
-      <c r="E38" s="16" t="n"/>
+          <t>ks</t>
+        </is>
+      </c>
+      <c r="E38" s="16" t="n">
+        <v>1</v>
+      </c>
       <c r="F38" s="14" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G38" s="15" t="inlineStr">
         <is>
-          <t>HSV5.002a, HSV5.002b, HSV5.002c</t>
+          <t>PSV76.002a</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="15" t="inlineStr">
         <is>
-          <t>260217_sklad.PSV76.002</t>
+          <t>260217_sklad.VRN.003</t>
         </is>
       </c>
       <c r="B39" s="15" t="inlineStr">
         <is>
-          <t>PSV-76 Zámečnictví</t>
+          <t>VRN — Geodet / PČR</t>
         </is>
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>Vjezdová brána na pozemku investora (ocelová) — dodávka + montáž</t>
+          <t>Vytyčení + kontrola rozhledových trojúhelníků (Vn=40 km/h, Dz=25 m) dle požadavku DI PČR</t>
         </is>
       </c>
       <c r="D39" s="14" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>soubor</t>
         </is>
       </c>
       <c r="E39" s="16" t="n">
@@ -17990,90 +17886,90 @@
       </c>
       <c r="G39" s="15" t="inlineStr">
         <is>
-          <t>PSV76.002a</t>
+          <t>VRN.003a</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="15" t="inlineStr">
         <is>
-          <t>260217_sklad.VRN.003</t>
+          <t>260219_dum.M24.001</t>
         </is>
       </c>
       <c r="B40" s="15" t="inlineStr">
         <is>
-          <t>VRN — Geodet / PČR</t>
+          <t>M-24 VZT</t>
         </is>
       </c>
       <c r="C40" s="15" t="inlineStr">
         <is>
-          <t>Vytyčení + kontrola rozhledových trojúhelníků (Vn=40 km/h, Dz=25 m) dle požadavku DI PČR</t>
+          <t>Lokální odtah digestoří kuchyní (1.NP + 3.NP) — dodávka + montáž digestoře + prostup fasádou/střechou + zpětná klapka</t>
         </is>
       </c>
       <c r="D40" s="14" t="inlineStr">
         <is>
-          <t>soubor</t>
+          <t>ks</t>
         </is>
       </c>
       <c r="E40" s="16" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F40" s="14" t="n">
         <v>1</v>
       </c>
       <c r="G40" s="15" t="inlineStr">
         <is>
-          <t>VRN.003a</t>
+          <t>M24.001a</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.M24.001</t>
+          <t>260219_dum.M21.008</t>
         </is>
       </c>
       <c r="B41" s="15" t="inlineStr">
         <is>
-          <t>M-24 VZT</t>
+          <t>M-21 ELI silnoproud</t>
         </is>
       </c>
       <c r="C41" s="15" t="inlineStr">
         <is>
-          <t>Lokální odtah digestoří kuchyní (1.NP + 3.NP) — dodávka + montáž digestoře + prostup fasádou/střechou + zpětná klapka</t>
+          <t>Hlavní vypínač elektrické energie TOTAL STOP + požární značení rozvodného zařízení a uzávěrů (voda/elektro)</t>
         </is>
       </c>
       <c r="D41" s="14" t="inlineStr">
         <is>
-          <t>ks</t>
+          <t>soubor</t>
         </is>
       </c>
       <c r="E41" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="F41" s="14" t="n">
         <v>2</v>
       </c>
-      <c r="F41" s="14" t="n">
-        <v>1</v>
-      </c>
       <c r="G41" s="15" t="inlineStr">
         <is>
-          <t>M24.001a</t>
+          <t>M21.008a, M21.008b</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="15" t="inlineStr">
         <is>
-          <t>260219_dum.M21.008</t>
+          <t>260219_dum.PSV95.003</t>
         </is>
       </c>
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>M-21 ELI silnoproud</t>
+          <t>PSV-95 Detekce požární</t>
         </is>
       </c>
       <c r="C42" s="15" t="inlineStr">
         <is>
-          <t>Hlavní vypínač elektrické energie TOTAL STOP + požární značení rozvodného zařízení a uzávěrů (voda/elektro)</t>
+          <t xml:space="preserve">Předávací protokol krbu na tuhá paliva + kontrola bezpečných vzdáleností (800 mm směr sálání / 400 mm strany, nehořlavá </t>
         </is>
       </c>
       <c r="D42" s="14" t="inlineStr">
@@ -18085,42 +17981,9 @@
         <v>1</v>
       </c>
       <c r="F42" s="14" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G42" s="15" t="inlineStr">
-        <is>
-          <t>M21.008a, M21.008b</t>
-        </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="15" t="inlineStr">
-        <is>
-          <t>260219_dum.PSV95.003</t>
-        </is>
-      </c>
-      <c r="B43" s="15" t="inlineStr">
-        <is>
-          <t>PSV-95 Detekce požární</t>
-        </is>
-      </c>
-      <c r="C43" s="15" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Předávací protokol krbu na tuhá paliva + kontrola bezpečných vzdáleností (800 mm směr sálání / 400 mm strany, nehořlavá </t>
-        </is>
-      </c>
-      <c r="D43" s="14" t="inlineStr">
-        <is>
-          <t>soubor</t>
-        </is>
-      </c>
-      <c r="E43" s="16" t="n">
-        <v>1</v>
-      </c>
-      <c r="F43" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="G43" s="15" t="inlineStr">
         <is>
           <t>PSV95.003a</t>
         </is>
@@ -18137,7 +18000,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:E16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -18482,27 +18345,52 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="14" t="inlineStr">
+      <c r="A15" s="17" t="n">
+        <v>35</v>
+      </c>
+      <c r="B15" s="18" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>Sokl — rozpor PD: TZ ARS (XPS + cihelný) vs výkres S03/pohledy (sanační Styrcon + keramický)</t>
+        </is>
+      </c>
+      <c r="D15" s="18" t="inlineStr">
+        <is>
+          <t>NEPŘIDÁNO (verify-first)</t>
+        </is>
+      </c>
+      <c r="E15" s="18" t="inlineStr">
+        <is>
+          <t>Projektante: potvrďte sokl = sanační Styrcon 200 + keramický obklad (výkres), NE XPS + cihelný (TZ ARS text). + délka soklu (řadovka): plocha ≈16 nebo 23 m²?</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>PM05</t>
         </is>
       </c>
-      <c r="B15" s="15" t="inlineStr">
+      <c r="B16" s="15" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
       </c>
-      <c r="C15" s="15" t="inlineStr">
+      <c r="C16" s="15" t="inlineStr">
         <is>
           <t>Okapový chodník + obvodová drenáž domu — NOT_IN_TZ (žádná zmínka v TZ)</t>
         </is>
       </c>
-      <c r="D15" s="15" t="inlineStr">
+      <c r="D16" s="15" t="inlineStr">
         <is>
           <t>SKIP (rekonstrukce — možná existuje)</t>
         </is>
       </c>
-      <c r="E15" s="15" t="inlineStr">
+      <c r="E16" s="15" t="inlineStr">
         <is>
           <t>Volitelné: ověřit zda okapový chodník po obvodu domu je v scope (mimo BV drenáž HSV1.015). Pokud ano → HSV-1 položka.</t>
         </is>

</xml_diff>

<commit_message>
fix(rd-jachymov): sklad patky 7→6 + IPE 7→6 + H-BLOK rozměr potvrzen výkresem
Drawing-confirmed counts from D.1.1.02 (6 patek: řada 785+5×1000+435,
rozteč IPE 1000 mm; 6× IPE180):
- HSV1.004 hloubení patek 1.75→1.5 m³ (6×0.5×0.5×1.0)
- HSV2.002/003 patky spodní/horní 7→6 ks
- HSV2.004 beton zalití formula 6 ks
- HSV1.006 odvoz 32.1→31.85 m³
- HSV4.004 IPE180 921→790 kg (6×7×18.8)
- HSV4.006 žárový zinek 1551→1420 kg
- HSV3.001 H-BLOK: rozměr bloku 1800×600 mm POTVRZEN výkresem D.1.1.02/03
  (provenance upgrade estimate→measured; 18 ks, objem 11.43 m³)

https://claude.ai/code/session_01FskzLAZkXgJAwuN2cQQEdx
</commit_message>
<xml_diff>
--- a/test-data/RD_Jachymov_dum/outputs/Vykaz_vymer_RD_Jachymov_ATOMIC_WORKLIST_2026-05-27.xlsx
+++ b/test-data/RD_Jachymov_dum/outputs/Vykaz_vymer_RD_Jachymov_ATOMIC_WORKLIST_2026-05-27.xlsx
@@ -18038,7 +18038,7 @@
       </c>
       <c r="C6" s="11" t="inlineStr">
         <is>
-          <t>Hloubení patek pro stojky IPE180 zastřešení parkingu, 500×500 mm × 1.0 m hl. × 7 ks</t>
+          <t>Hloubení patek pro stojky IPE180 zastřešení parkingu, 500×500 mm × 1.0 m hl. × 6 ks</t>
         </is>
       </c>
       <c r="D6" s="10" t="inlineStr">
@@ -18047,11 +18047,11 @@
         </is>
       </c>
       <c r="E6" s="12" t="n">
-        <v>1.75</v>
+        <v>1.5</v>
       </c>
       <c r="F6" s="11" t="inlineStr">
         <is>
-          <t>DXF: 7 patek × 0.5 × 0.5 × 1.0 (TZ rozteč 1000 mm × 7 m parking)</t>
+          <t>6 patek × 0.5 × 0.5 × 1.0 m hl. = 1.5 m³</t>
         </is>
       </c>
       <c r="G6" s="11" t="inlineStr">
@@ -18149,10 +18149,10 @@
         </is>
       </c>
       <c r="E8" s="19" t="n">
-        <v>32.1</v>
+        <v>31.85</v>
       </c>
       <c r="F8" s="18">
-        <f> součet hloubení sklad + figura + patky (25.5+4.85+1.75)</f>
+        <f> součet hloubení sklad + figura + patky (25.5+4.85+1.5)</f>
         <v/>
       </c>
       <c r="G8" s="18" t="inlineStr"/>
@@ -18250,7 +18250,7 @@
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Dvoustupňové patky pro IPE180 zastřešení parkingu — spodní část prostý beton C16/20 500×500×500 mm × 7 ks</t>
+          <t>Dvoustupňové patky pro IPE180 zastřešení parkingu — spodní část prostý beton C16/20 500×500×500 mm × 6 ks</t>
         </is>
       </c>
       <c r="D11" s="10" t="inlineStr">
@@ -18259,11 +18259,11 @@
         </is>
       </c>
       <c r="E11" s="12" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>DXF: 7 ks (rozteč 1000 mm × 7000 mm parking délka)</t>
+          <t>6 ks (výkres D.1.1.02 — 6 štvercových patek pod IPE180)</t>
         </is>
       </c>
       <c r="G11" s="13" t="inlineStr">
@@ -18299,7 +18299,7 @@
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Montáž — Dvoustupňové patky pro IPE180 — horní část z tvarovek ztraceného bednění 300×300 mm × 7 ks</t>
+          <t>Montáž — Dvoustupňové patky pro IPE180 — horní část z tvarovek ztraceného bednění 300×300 mm × 6 ks</t>
         </is>
       </c>
       <c r="D12" s="10" t="inlineStr">
@@ -18308,11 +18308,11 @@
         </is>
       </c>
       <c r="E12" s="12" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>7 ks (= spodní)</t>
+          <t>6 ks (= spodní, výkres D.1.1.02)</t>
         </is>
       </c>
       <c r="G12" s="11" t="inlineStr">
@@ -18357,7 +18357,7 @@
         </is>
       </c>
       <c r="E13" s="19" t="n">
-        <v>7.21</v>
+        <v>6.18</v>
       </c>
       <c r="F13" s="18">
         <f> montáž × 1.03</f>
@@ -18401,11 +18401,11 @@
         </is>
       </c>
       <c r="E14" s="12" t="n">
-        <v>1.8</v>
+        <v>1.75</v>
       </c>
       <c r="F14" s="11" t="inlineStr">
         <is>
-          <t>patky horní (0.3×0.3×0.5×7) + zídka (odhad ~1 m³)</t>
+          <t>patky horní (0.3×0.3×0.5×6 = 0.27) + zídka lemující + věnec nad patkami (odhad ~1.5 m³) = ~1.75 m³</t>
         </is>
       </c>
       <c r="G14" s="11" t="inlineStr">
@@ -18577,7 +18577,7 @@
       </c>
       <c r="F18" s="11" t="inlineStr">
         <is>
-          <t>S04 líc 6.35 × 3.0 m = 19.05 m² (řez A-A measured) ÷ ~1.08 m²/blok = 17.6 → 18 ks. POZOR: rozměr bloku 1800×600 mm je ODHAD z analogie (web BB6 stejných gabaritů + AI-souhrn), NE z Herkul tech. listu napřímo (hblok.cz nedostupný). H-BLOK má interlocking profil — modul může být jiný. OVĚŘIT u Herkul.</t>
+          <t>S04 líc 6.35 × 3.0 m = 19.05 m²; blok 1800×600 mm (výkres D.1.1.02/03: délka 1800, 5 řad × 600 výška = 3000) → 3 celé (1800×3=5400) + 1 kus 950 mm na řadu, vazba na zámek; 5 řad × ~3.5 bloku ≈ 18 ks</t>
         </is>
       </c>
       <c r="G18" s="11" t="inlineStr">
@@ -19234,7 +19234,7 @@
       </c>
       <c r="C32" s="11" t="inlineStr">
         <is>
-          <t>Montáž — Sekundární zastřešení parkingu — IPE180 v rozteči 1000 mm × délka 7 m × 7 ks</t>
+          <t>Montáž — Sekundární zastřešení parkingu — IPE180 v rozteči 1000 mm × délka 6 m × 6 ks</t>
         </is>
       </c>
       <c r="D32" s="10" t="inlineStr">
@@ -19243,11 +19243,11 @@
         </is>
       </c>
       <c r="E32" s="12" t="n">
-        <v>921</v>
+        <v>790</v>
       </c>
       <c r="F32" s="11" t="inlineStr">
         <is>
-          <t>7 ks × 7 m × 18.8 kg/m = 921</t>
+          <t>6 ks IPE180 × 7.0 m × 18.8 kg/m = 789.6 → 790 kg (výkres D.1.1.02: 6 nosníků)</t>
         </is>
       </c>
       <c r="G32" s="11" t="inlineStr">
@@ -19296,7 +19296,7 @@
         </is>
       </c>
       <c r="E33" s="19" t="n">
-        <v>948.63</v>
+        <v>813.7</v>
       </c>
       <c r="F33" s="18">
         <f> montáž × 1.03</f>
@@ -19397,11 +19397,12 @@
         </is>
       </c>
       <c r="E35" s="12" t="n">
-        <v>1551</v>
-      </c>
-      <c r="F35" s="11">
-        <f> hmotnost IPE180 (921 kg) + odhad pororoštů (21 m² × 30 kg/m²) = ~1551</f>
-        <v/>
+        <v>1420</v>
+      </c>
+      <c r="F35" s="11" t="inlineStr">
+        <is>
+          <t>IPE 790 kg + pororošt 630 kg = 1420 kg žárově zinkováno (IPE 6 ks)</t>
+        </is>
       </c>
       <c r="G35" s="11" t="inlineStr">
         <is>
@@ -19449,7 +19450,7 @@
         </is>
       </c>
       <c r="E36" s="19" t="n">
-        <v>1582.02</v>
+        <v>1448.4</v>
       </c>
       <c r="F36" s="18">
         <f> montáž × 1.02</f>
@@ -20591,7 +20592,7 @@
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
-          <t>Dvoustupňové patky pro IPE180 — horní část z tvarovek ztraceného bednění 300×300 mm × 7 ks</t>
+          <t>Dvoustupňové patky pro IPE180 — horní část z tvarovek ztraceného bednění 300×300 mm × 6 ks</t>
         </is>
       </c>
       <c r="D10" s="14" t="inlineStr">
@@ -20600,7 +20601,7 @@
         </is>
       </c>
       <c r="E10" s="16" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F10" s="14" t="n">
         <v>2</v>
@@ -20987,7 +20988,7 @@
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>Sekundární zastřešení parkingu — IPE180 v rozteči 1000 mm × délka 7 m × 7 ks</t>
+          <t>Sekundární zastřešení parkingu — IPE180 v rozteči 1000 mm × délka 6 m × 6 ks</t>
         </is>
       </c>
       <c r="D22" s="14" t="inlineStr">
@@ -20996,7 +20997,7 @@
         </is>
       </c>
       <c r="E22" s="16" t="n">
-        <v>921</v>
+        <v>790</v>
       </c>
       <c r="F22" s="14" t="n">
         <v>2</v>
@@ -21029,7 +21030,7 @@
         </is>
       </c>
       <c r="E23" s="16" t="n">
-        <v>1551</v>
+        <v>1420</v>
       </c>
       <c r="F23" s="14" t="n">
         <v>2</v>

</xml_diff>